<commit_message>
Download Excel uses the designed template
- Excel download fills the designed template (Dashboard with formulas and chart,
  Client, Policies, new Review notes sheet) instead of plain sheets
- Dashboard counts paid-up policies like the app; single premium not annualised
- Chart shows category labels and RM scale

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Policy_Review_Template.xlsx
+++ b/Policy_Review_Template.xlsx
@@ -10,8 +10,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Client" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Policies" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="5" state="hidden" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review notes" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lists" sheetId="6" state="hidden" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -123,7 +124,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -154,6 +155,9 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -327,6 +331,7 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
@@ -338,6 +343,7 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
         <majorGridlines/>
         <numFmt formatCode="#,##0" sourceLinked="0"/>
@@ -364,7 +370,7 @@
       <row>24</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="5760000" cy="2700000"/>
+    <ext cx="6480000" cy="3240000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="1" name="Chart 1"/>
@@ -672,7 +678,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E43"/>
+  <dimension ref="A1:E46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -693,7 +699,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Auto-calculated from 'Client' and 'Policies'. Only INFORCE policies count toward coverage.</t>
+          <t>Auto-calculated from 'Client' and 'Policies'. Inforce and paid-up policies count toward coverage.</t>
         </is>
       </c>
     </row>
@@ -751,7 +757,7 @@
         </is>
       </c>
       <c r="B6" s="7">
-        <f>SUMIFS(Policies!$L$2:$L$100,Policies!$G$2:$G$100,"Inforce")</f>
+        <f>SUMIFS(Policies!$L$2:$L$100,Policies!$G$2:$G$100,"Inforce")+SUMIFS(Policies!$L$2:$L$100,Policies!$G$2:$G$100,"Paid-up")</f>
         <v/>
       </c>
       <c r="C6" s="7">
@@ -774,7 +780,7 @@
         </is>
       </c>
       <c r="B7" s="9">
-        <f>SUMIFS(Policies!$M$2:$M$100,Policies!$G$2:$G$100,"Inforce")</f>
+        <f>SUMIFS(Policies!$M$2:$M$100,Policies!$G$2:$G$100,"Inforce")+SUMIFS(Policies!$M$2:$M$100,Policies!$G$2:$G$100,"Paid-up")</f>
         <v/>
       </c>
       <c r="C7" s="9">
@@ -797,7 +803,7 @@
         </is>
       </c>
       <c r="B8" s="7">
-        <f>SUMIFS(Policies!$N$2:$N$100,Policies!$G$2:$G$100,"Inforce")</f>
+        <f>SUMIFS(Policies!$N$2:$N$100,Policies!$G$2:$G$100,"Inforce")+SUMIFS(Policies!$N$2:$N$100,Policies!$G$2:$G$100,"Paid-up")</f>
         <v/>
       </c>
       <c r="C8" s="7">
@@ -820,7 +826,7 @@
         </is>
       </c>
       <c r="B9" s="9">
-        <f>SUMIFS(Policies!$Y$2:$Y$100,Policies!$G$2:$G$100,"Inforce")+N(Client!B21)+N(Client!B22)</f>
+        <f>SUMIFS(Policies!$Y$2:$Y$100,Policies!$G$2:$G$100,"Inforce")+SUMIFS(Policies!$Y$2:$Y$100,Policies!$G$2:$G$100,"Paid-up")+N(Client!B21)+N(Client!B22)</f>
         <v/>
       </c>
       <c r="C9" s="9">
@@ -843,7 +849,7 @@
         </is>
       </c>
       <c r="B10" s="7">
-        <f>_xlfn.MAXIFS(Policies!$P$2:$P$100,Policies!$G$2:$G$100,"Inforce")</f>
+        <f>MAX(_xlfn.MAXIFS(Policies!$P$2:$P$100,Policies!$G$2:$G$100,"Inforce"),_xlfn.MAXIFS(Policies!$P$2:$P$100,Policies!$G$2:$G$100,"Paid-up"))</f>
         <v/>
       </c>
       <c r="C10" s="7">
@@ -866,7 +872,7 @@
         </is>
       </c>
       <c r="B11" s="9">
-        <f>_xlfn.MAXIFS(Policies!$Q$2:$Q$100,Policies!$G$2:$G$100,"Inforce")</f>
+        <f>MAX(_xlfn.MAXIFS(Policies!$Q$2:$Q$100,Policies!$G$2:$G$100,"Inforce"),_xlfn.MAXIFS(Policies!$Q$2:$Q$100,Policies!$G$2:$G$100,"Paid-up"))</f>
         <v/>
       </c>
       <c r="C11" s="9">
@@ -889,7 +895,7 @@
         </is>
       </c>
       <c r="B12" s="7">
-        <f>SUMIFS(Policies!$R$2:$R$100,Policies!$G$2:$G$100,"Inforce")</f>
+        <f>SUMIFS(Policies!$R$2:$R$100,Policies!$G$2:$G$100,"Inforce")+SUMIFS(Policies!$R$2:$R$100,Policies!$G$2:$G$100,"Paid-up")</f>
         <v/>
       </c>
       <c r="C12" s="7" t="inlineStr">
@@ -918,11 +924,11 @@
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>Total annual premium (inforce)  年缴总保费</t>
+          <t>Total annual premium (inforce + paid-up)  年缴总保费</t>
         </is>
       </c>
       <c r="B15" s="9">
-        <f>SUMIFS(Policies!$Z$2:$Z$100,Policies!$G$2:$G$100,"Inforce")</f>
+        <f>SUMIFS(Policies!$Z$2:$Z$100,Policies!$G$2:$G$100,"Inforce")+SUMIFS(Policies!$Z$2:$Z$100,Policies!$G$2:$G$100,"Paid-up")</f>
         <v/>
       </c>
     </row>
@@ -969,11 +975,11 @@
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>Inforce policies  有效保单</t>
+          <t>Inforce / paid-up policies  有效保单</t>
         </is>
       </c>
       <c r="B21" s="12">
-        <f>COUNTIFS(Policies!$G$2:$G$100,"Inforce")</f>
+        <f>COUNTIFS(Policies!$G$2:$G$100,"Inforce")+COUNTIFS(Policies!$G$2:$G$100,"Paid-up")</f>
         <v/>
       </c>
     </row>
@@ -995,22 +1001,22 @@
         </is>
       </c>
       <c r="B23" s="12">
-        <f>COUNTIFS(Policies!$G$2:$G$100,"Inforce",Policies!$T$2:$T$100,"",Policies!$A$2:$A$100,"&lt;&gt;")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" s="13" t="inlineStr">
+        <f>COUNTIFS(Policies!$G$2:$G$100,"Inforce",Policies!$T$2:$T$100,"",Policies!$A$2:$A$100,"&lt;&gt;")+COUNTIFS(Policies!$G$2:$G$100,"Paid-up",Policies!$T$2:$T$100,"",Policies!$A$2:$A$100,"&lt;&gt;")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="13" t="inlineStr">
         <is>
           <t>Disclaimer: Summary based on policy information provided as at review date. Benefits are subject to the terms of each policy contract. Review standards are planning benchmarks, not recommendations or official figures.</t>
         </is>
       </c>
     </row>
-    <row r="42"/>
-    <row r="43"/>
+    <row r="45"/>
+    <row r="46"/>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A41:E43"/>
+    <mergeCell ref="A44:E46"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -1483,11 +1489,11 @@
       <c r="M2" s="9" t="n">
         <v>200000</v>
       </c>
-      <c r="N2" s="12" t="n"/>
-      <c r="O2" s="12" t="n"/>
-      <c r="P2" s="12" t="n"/>
-      <c r="Q2" s="12" t="n"/>
-      <c r="R2" s="12" t="n"/>
+      <c r="N2" s="9" t="n"/>
+      <c r="O2" s="9" t="n"/>
+      <c r="P2" s="9" t="n"/>
+      <c r="Q2" s="9" t="n"/>
+      <c r="R2" s="9" t="n"/>
       <c r="S2" s="12" t="inlineStr">
         <is>
           <t>Yes</t>
@@ -1514,8 +1520,9 @@
         </is>
       </c>
       <c r="X2" s="12" t="inlineStr"/>
+      <c r="Y2" s="9" t="n"/>
       <c r="Z2" s="21">
-        <f>IF(J2="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J2,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,1},MATCH(K2,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
+        <f>IF(J2="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J2,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K2,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
     </row>
@@ -1575,15 +1582,15 @@
       <c r="M3" s="9" t="n">
         <v>50000</v>
       </c>
-      <c r="N3" s="12" t="n"/>
-      <c r="O3" s="12" t="n"/>
+      <c r="N3" s="9" t="n"/>
+      <c r="O3" s="9" t="n"/>
       <c r="P3" s="9" t="n">
         <v>150000</v>
       </c>
       <c r="Q3" s="9" t="n">
         <v>150</v>
       </c>
-      <c r="R3" s="12" t="n"/>
+      <c r="R3" s="9" t="n"/>
       <c r="S3" s="12" t="inlineStr">
         <is>
           <t>No</t>
@@ -1602,8 +1609,9 @@
           <t>Nominee not recorded - to confirm</t>
         </is>
       </c>
+      <c r="Y3" s="9" t="n"/>
       <c r="Z3" s="21">
-        <f>IF(J3="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J3,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,1},MATCH(K3,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
+        <f>IF(J3="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J3,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K3,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
     </row>
@@ -1649,7 +1657,7 @@
       <c r="I4" s="20" t="n">
         <v>58450</v>
       </c>
-      <c r="J4" s="12" t="inlineStr">
+      <c r="J4" s="9" t="inlineStr">
         <is>
           <t>RM 1,800.00</t>
         </is>
@@ -1662,14 +1670,14 @@
       <c r="L4" s="9" t="n">
         <v>100000</v>
       </c>
-      <c r="M4" s="12" t="n"/>
+      <c r="M4" s="9" t="n"/>
       <c r="N4" s="9" t="n">
         <v>100000</v>
       </c>
-      <c r="O4" s="12" t="n"/>
-      <c r="P4" s="12" t="n"/>
-      <c r="Q4" s="12" t="n"/>
-      <c r="R4" s="12" t="n"/>
+      <c r="O4" s="9" t="n"/>
+      <c r="P4" s="9" t="n"/>
+      <c r="Q4" s="9" t="n"/>
+      <c r="R4" s="9" t="n"/>
       <c r="S4" s="12" t="inlineStr">
         <is>
           <t>No</t>
@@ -1696,8 +1704,9 @@
         </is>
       </c>
       <c r="X4" s="12" t="inlineStr"/>
+      <c r="Y4" s="9" t="n"/>
       <c r="Z4" s="21">
-        <f>IF(J4="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J4,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,1},MATCH(K4,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
+        <f>IF(J4="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J4,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K4,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
     </row>
@@ -1751,12 +1760,12 @@
           <t>Yearly</t>
         </is>
       </c>
-      <c r="L5" s="12" t="n"/>
-      <c r="M5" s="12" t="n"/>
-      <c r="N5" s="12" t="n"/>
-      <c r="O5" s="12" t="n"/>
-      <c r="P5" s="12" t="n"/>
-      <c r="Q5" s="12" t="n"/>
+      <c r="L5" s="9" t="n"/>
+      <c r="M5" s="9" t="n"/>
+      <c r="N5" s="9" t="n"/>
+      <c r="O5" s="9" t="n"/>
+      <c r="P5" s="9" t="n"/>
+      <c r="Q5" s="9" t="n"/>
       <c r="R5" s="9" t="n">
         <v>100000</v>
       </c>
@@ -1778,8 +1787,9 @@
           <t>Yearly renewable</t>
         </is>
       </c>
+      <c r="Y5" s="9" t="n"/>
       <c r="Z5" s="21">
-        <f>IF(J5="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J5,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,1},MATCH(K5,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
+        <f>IF(J5="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J5,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K5,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
     </row>
@@ -1836,12 +1846,12 @@
       <c r="L6" s="9" t="n">
         <v>30000</v>
       </c>
-      <c r="M6" s="12" t="n"/>
-      <c r="N6" s="12" t="n"/>
-      <c r="O6" s="12" t="n"/>
-      <c r="P6" s="12" t="n"/>
-      <c r="Q6" s="12" t="n"/>
-      <c r="R6" s="12" t="n"/>
+      <c r="M6" s="9" t="n"/>
+      <c r="N6" s="9" t="n"/>
+      <c r="O6" s="9" t="n"/>
+      <c r="P6" s="9" t="n"/>
+      <c r="Q6" s="9" t="n"/>
+      <c r="R6" s="9" t="n"/>
       <c r="S6" s="12" t="inlineStr">
         <is>
           <t>No</t>
@@ -1872,572 +1882,2923 @@
           <t>Lapsed 2021 - discuss reinstatement?</t>
         </is>
       </c>
+      <c r="Y6" s="9" t="n"/>
       <c r="Z6" s="21">
-        <f>IF(J6="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J6,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,1},MATCH(K6,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
+        <f>IF(J6="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J6,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K6,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
     </row>
     <row r="7">
+      <c r="A7" s="12" t="n"/>
+      <c r="B7" s="12" t="n"/>
+      <c r="C7" s="12" t="n"/>
+      <c r="D7" s="12" t="n"/>
+      <c r="E7" s="12" t="n"/>
+      <c r="F7" s="12" t="n"/>
+      <c r="G7" s="12" t="n"/>
+      <c r="H7" s="20" t="n"/>
+      <c r="I7" s="20" t="n"/>
+      <c r="J7" s="9" t="n"/>
+      <c r="K7" s="12" t="n"/>
+      <c r="L7" s="9" t="n"/>
+      <c r="M7" s="9" t="n"/>
+      <c r="N7" s="9" t="n"/>
+      <c r="O7" s="9" t="n"/>
+      <c r="P7" s="9" t="n"/>
+      <c r="Q7" s="9" t="n"/>
+      <c r="R7" s="9" t="n"/>
+      <c r="S7" s="12" t="n"/>
+      <c r="T7" s="12" t="n"/>
+      <c r="U7" s="12" t="n"/>
+      <c r="V7" s="12" t="n"/>
+      <c r="W7" s="12" t="n"/>
+      <c r="X7" s="12" t="n"/>
+      <c r="Y7" s="9" t="n"/>
       <c r="Z7" s="21">
-        <f>IF(J7="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J7,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,1},MATCH(K7,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
+        <f>IF(J7="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J7,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K7,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
     </row>
     <row r="8">
+      <c r="A8" s="12" t="n"/>
+      <c r="B8" s="12" t="n"/>
+      <c r="C8" s="12" t="n"/>
+      <c r="D8" s="12" t="n"/>
+      <c r="E8" s="12" t="n"/>
+      <c r="F8" s="12" t="n"/>
+      <c r="G8" s="12" t="n"/>
+      <c r="H8" s="20" t="n"/>
+      <c r="I8" s="20" t="n"/>
+      <c r="J8" s="9" t="n"/>
+      <c r="K8" s="12" t="n"/>
+      <c r="L8" s="9" t="n"/>
+      <c r="M8" s="9" t="n"/>
+      <c r="N8" s="9" t="n"/>
+      <c r="O8" s="9" t="n"/>
+      <c r="P8" s="9" t="n"/>
+      <c r="Q8" s="9" t="n"/>
+      <c r="R8" s="9" t="n"/>
+      <c r="S8" s="12" t="n"/>
+      <c r="T8" s="12" t="n"/>
+      <c r="U8" s="12" t="n"/>
+      <c r="V8" s="12" t="n"/>
+      <c r="W8" s="12" t="n"/>
+      <c r="X8" s="12" t="n"/>
+      <c r="Y8" s="9" t="n"/>
       <c r="Z8" s="21">
-        <f>IF(J8="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J8,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,1},MATCH(K8,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
+        <f>IF(J8="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J8,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K8,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
     </row>
     <row r="9">
+      <c r="A9" s="12" t="n"/>
+      <c r="B9" s="12" t="n"/>
+      <c r="C9" s="12" t="n"/>
+      <c r="D9" s="12" t="n"/>
+      <c r="E9" s="12" t="n"/>
+      <c r="F9" s="12" t="n"/>
+      <c r="G9" s="12" t="n"/>
+      <c r="H9" s="20" t="n"/>
+      <c r="I9" s="20" t="n"/>
+      <c r="J9" s="9" t="n"/>
+      <c r="K9" s="12" t="n"/>
+      <c r="L9" s="9" t="n"/>
+      <c r="M9" s="9" t="n"/>
+      <c r="N9" s="9" t="n"/>
+      <c r="O9" s="9" t="n"/>
+      <c r="P9" s="9" t="n"/>
+      <c r="Q9" s="9" t="n"/>
+      <c r="R9" s="9" t="n"/>
+      <c r="S9" s="12" t="n"/>
+      <c r="T9" s="12" t="n"/>
+      <c r="U9" s="12" t="n"/>
+      <c r="V9" s="12" t="n"/>
+      <c r="W9" s="12" t="n"/>
+      <c r="X9" s="12" t="n"/>
+      <c r="Y9" s="9" t="n"/>
       <c r="Z9" s="21">
-        <f>IF(J9="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J9,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,1},MATCH(K9,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
+        <f>IF(J9="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J9,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K9,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
     </row>
     <row r="10">
+      <c r="A10" s="12" t="n"/>
+      <c r="B10" s="12" t="n"/>
+      <c r="C10" s="12" t="n"/>
+      <c r="D10" s="12" t="n"/>
+      <c r="E10" s="12" t="n"/>
+      <c r="F10" s="12" t="n"/>
+      <c r="G10" s="12" t="n"/>
+      <c r="H10" s="20" t="n"/>
+      <c r="I10" s="20" t="n"/>
+      <c r="J10" s="9" t="n"/>
+      <c r="K10" s="12" t="n"/>
+      <c r="L10" s="9" t="n"/>
+      <c r="M10" s="9" t="n"/>
+      <c r="N10" s="9" t="n"/>
+      <c r="O10" s="9" t="n"/>
+      <c r="P10" s="9" t="n"/>
+      <c r="Q10" s="9" t="n"/>
+      <c r="R10" s="9" t="n"/>
+      <c r="S10" s="12" t="n"/>
+      <c r="T10" s="12" t="n"/>
+      <c r="U10" s="12" t="n"/>
+      <c r="V10" s="12" t="n"/>
+      <c r="W10" s="12" t="n"/>
+      <c r="X10" s="12" t="n"/>
+      <c r="Y10" s="9" t="n"/>
       <c r="Z10" s="21">
-        <f>IF(J10="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J10,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,1},MATCH(K10,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
+        <f>IF(J10="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J10,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K10,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
     </row>
     <row r="11">
+      <c r="A11" s="12" t="n"/>
+      <c r="B11" s="12" t="n"/>
+      <c r="C11" s="12" t="n"/>
+      <c r="D11" s="12" t="n"/>
+      <c r="E11" s="12" t="n"/>
+      <c r="F11" s="12" t="n"/>
+      <c r="G11" s="12" t="n"/>
+      <c r="H11" s="20" t="n"/>
+      <c r="I11" s="20" t="n"/>
+      <c r="J11" s="9" t="n"/>
+      <c r="K11" s="12" t="n"/>
+      <c r="L11" s="9" t="n"/>
+      <c r="M11" s="9" t="n"/>
+      <c r="N11" s="9" t="n"/>
+      <c r="O11" s="9" t="n"/>
+      <c r="P11" s="9" t="n"/>
+      <c r="Q11" s="9" t="n"/>
+      <c r="R11" s="9" t="n"/>
+      <c r="S11" s="12" t="n"/>
+      <c r="T11" s="12" t="n"/>
+      <c r="U11" s="12" t="n"/>
+      <c r="V11" s="12" t="n"/>
+      <c r="W11" s="12" t="n"/>
+      <c r="X11" s="12" t="n"/>
+      <c r="Y11" s="9" t="n"/>
       <c r="Z11" s="21">
-        <f>IF(J11="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J11,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,1},MATCH(K11,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
+        <f>IF(J11="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J11,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K11,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
     </row>
     <row r="12">
+      <c r="A12" s="12" t="n"/>
+      <c r="B12" s="12" t="n"/>
+      <c r="C12" s="12" t="n"/>
+      <c r="D12" s="12" t="n"/>
+      <c r="E12" s="12" t="n"/>
+      <c r="F12" s="12" t="n"/>
+      <c r="G12" s="12" t="n"/>
+      <c r="H12" s="20" t="n"/>
+      <c r="I12" s="20" t="n"/>
+      <c r="J12" s="9" t="n"/>
+      <c r="K12" s="12" t="n"/>
+      <c r="L12" s="9" t="n"/>
+      <c r="M12" s="9" t="n"/>
+      <c r="N12" s="9" t="n"/>
+      <c r="O12" s="9" t="n"/>
+      <c r="P12" s="9" t="n"/>
+      <c r="Q12" s="9" t="n"/>
+      <c r="R12" s="9" t="n"/>
+      <c r="S12" s="12" t="n"/>
+      <c r="T12" s="12" t="n"/>
+      <c r="U12" s="12" t="n"/>
+      <c r="V12" s="12" t="n"/>
+      <c r="W12" s="12" t="n"/>
+      <c r="X12" s="12" t="n"/>
+      <c r="Y12" s="9" t="n"/>
       <c r="Z12" s="21">
-        <f>IF(J12="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J12,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,1},MATCH(K12,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
+        <f>IF(J12="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J12,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K12,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
     </row>
     <row r="13">
+      <c r="A13" s="12" t="n"/>
+      <c r="B13" s="12" t="n"/>
+      <c r="C13" s="12" t="n"/>
+      <c r="D13" s="12" t="n"/>
+      <c r="E13" s="12" t="n"/>
+      <c r="F13" s="12" t="n"/>
+      <c r="G13" s="12" t="n"/>
+      <c r="H13" s="20" t="n"/>
+      <c r="I13" s="20" t="n"/>
+      <c r="J13" s="9" t="n"/>
+      <c r="K13" s="12" t="n"/>
+      <c r="L13" s="9" t="n"/>
+      <c r="M13" s="9" t="n"/>
+      <c r="N13" s="9" t="n"/>
+      <c r="O13" s="9" t="n"/>
+      <c r="P13" s="9" t="n"/>
+      <c r="Q13" s="9" t="n"/>
+      <c r="R13" s="9" t="n"/>
+      <c r="S13" s="12" t="n"/>
+      <c r="T13" s="12" t="n"/>
+      <c r="U13" s="12" t="n"/>
+      <c r="V13" s="12" t="n"/>
+      <c r="W13" s="12" t="n"/>
+      <c r="X13" s="12" t="n"/>
+      <c r="Y13" s="9" t="n"/>
       <c r="Z13" s="21">
-        <f>IF(J13="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J13,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,1},MATCH(K13,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
+        <f>IF(J13="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J13,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K13,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
     </row>
     <row r="14">
+      <c r="A14" s="12" t="n"/>
+      <c r="B14" s="12" t="n"/>
+      <c r="C14" s="12" t="n"/>
+      <c r="D14" s="12" t="n"/>
+      <c r="E14" s="12" t="n"/>
+      <c r="F14" s="12" t="n"/>
+      <c r="G14" s="12" t="n"/>
+      <c r="H14" s="20" t="n"/>
+      <c r="I14" s="20" t="n"/>
+      <c r="J14" s="9" t="n"/>
+      <c r="K14" s="12" t="n"/>
+      <c r="L14" s="9" t="n"/>
+      <c r="M14" s="9" t="n"/>
+      <c r="N14" s="9" t="n"/>
+      <c r="O14" s="9" t="n"/>
+      <c r="P14" s="9" t="n"/>
+      <c r="Q14" s="9" t="n"/>
+      <c r="R14" s="9" t="n"/>
+      <c r="S14" s="12" t="n"/>
+      <c r="T14" s="12" t="n"/>
+      <c r="U14" s="12" t="n"/>
+      <c r="V14" s="12" t="n"/>
+      <c r="W14" s="12" t="n"/>
+      <c r="X14" s="12" t="n"/>
+      <c r="Y14" s="9" t="n"/>
       <c r="Z14" s="21">
-        <f>IF(J14="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J14,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,1},MATCH(K14,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
+        <f>IF(J14="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J14,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K14,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
     </row>
     <row r="15">
+      <c r="A15" s="12" t="n"/>
+      <c r="B15" s="12" t="n"/>
+      <c r="C15" s="12" t="n"/>
+      <c r="D15" s="12" t="n"/>
+      <c r="E15" s="12" t="n"/>
+      <c r="F15" s="12" t="n"/>
+      <c r="G15" s="12" t="n"/>
+      <c r="H15" s="20" t="n"/>
+      <c r="I15" s="20" t="n"/>
+      <c r="J15" s="9" t="n"/>
+      <c r="K15" s="12" t="n"/>
+      <c r="L15" s="9" t="n"/>
+      <c r="M15" s="9" t="n"/>
+      <c r="N15" s="9" t="n"/>
+      <c r="O15" s="9" t="n"/>
+      <c r="P15" s="9" t="n"/>
+      <c r="Q15" s="9" t="n"/>
+      <c r="R15" s="9" t="n"/>
+      <c r="S15" s="12" t="n"/>
+      <c r="T15" s="12" t="n"/>
+      <c r="U15" s="12" t="n"/>
+      <c r="V15" s="12" t="n"/>
+      <c r="W15" s="12" t="n"/>
+      <c r="X15" s="12" t="n"/>
+      <c r="Y15" s="9" t="n"/>
       <c r="Z15" s="21">
-        <f>IF(J15="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J15,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,1},MATCH(K15,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
+        <f>IF(J15="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J15,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K15,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
     </row>
     <row r="16">
+      <c r="A16" s="12" t="n"/>
+      <c r="B16" s="12" t="n"/>
+      <c r="C16" s="12" t="n"/>
+      <c r="D16" s="12" t="n"/>
+      <c r="E16" s="12" t="n"/>
+      <c r="F16" s="12" t="n"/>
+      <c r="G16" s="12" t="n"/>
+      <c r="H16" s="20" t="n"/>
+      <c r="I16" s="20" t="n"/>
+      <c r="J16" s="9" t="n"/>
+      <c r="K16" s="12" t="n"/>
+      <c r="L16" s="9" t="n"/>
+      <c r="M16" s="9" t="n"/>
+      <c r="N16" s="9" t="n"/>
+      <c r="O16" s="9" t="n"/>
+      <c r="P16" s="9" t="n"/>
+      <c r="Q16" s="9" t="n"/>
+      <c r="R16" s="9" t="n"/>
+      <c r="S16" s="12" t="n"/>
+      <c r="T16" s="12" t="n"/>
+      <c r="U16" s="12" t="n"/>
+      <c r="V16" s="12" t="n"/>
+      <c r="W16" s="12" t="n"/>
+      <c r="X16" s="12" t="n"/>
+      <c r="Y16" s="9" t="n"/>
       <c r="Z16" s="21">
-        <f>IF(J16="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J16,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,1},MATCH(K16,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
+        <f>IF(J16="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J16,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K16,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
     </row>
     <row r="17">
+      <c r="A17" s="12" t="n"/>
+      <c r="B17" s="12" t="n"/>
+      <c r="C17" s="12" t="n"/>
+      <c r="D17" s="12" t="n"/>
+      <c r="E17" s="12" t="n"/>
+      <c r="F17" s="12" t="n"/>
+      <c r="G17" s="12" t="n"/>
+      <c r="H17" s="20" t="n"/>
+      <c r="I17" s="20" t="n"/>
+      <c r="J17" s="9" t="n"/>
+      <c r="K17" s="12" t="n"/>
+      <c r="L17" s="9" t="n"/>
+      <c r="M17" s="9" t="n"/>
+      <c r="N17" s="9" t="n"/>
+      <c r="O17" s="9" t="n"/>
+      <c r="P17" s="9" t="n"/>
+      <c r="Q17" s="9" t="n"/>
+      <c r="R17" s="9" t="n"/>
+      <c r="S17" s="12" t="n"/>
+      <c r="T17" s="12" t="n"/>
+      <c r="U17" s="12" t="n"/>
+      <c r="V17" s="12" t="n"/>
+      <c r="W17" s="12" t="n"/>
+      <c r="X17" s="12" t="n"/>
+      <c r="Y17" s="9" t="n"/>
       <c r="Z17" s="21">
-        <f>IF(J17="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J17,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,1},MATCH(K17,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
+        <f>IF(J17="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J17,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K17,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
     </row>
     <row r="18">
+      <c r="A18" s="12" t="n"/>
+      <c r="B18" s="12" t="n"/>
+      <c r="C18" s="12" t="n"/>
+      <c r="D18" s="12" t="n"/>
+      <c r="E18" s="12" t="n"/>
+      <c r="F18" s="12" t="n"/>
+      <c r="G18" s="12" t="n"/>
+      <c r="H18" s="20" t="n"/>
+      <c r="I18" s="20" t="n"/>
+      <c r="J18" s="9" t="n"/>
+      <c r="K18" s="12" t="n"/>
+      <c r="L18" s="9" t="n"/>
+      <c r="M18" s="9" t="n"/>
+      <c r="N18" s="9" t="n"/>
+      <c r="O18" s="9" t="n"/>
+      <c r="P18" s="9" t="n"/>
+      <c r="Q18" s="9" t="n"/>
+      <c r="R18" s="9" t="n"/>
+      <c r="S18" s="12" t="n"/>
+      <c r="T18" s="12" t="n"/>
+      <c r="U18" s="12" t="n"/>
+      <c r="V18" s="12" t="n"/>
+      <c r="W18" s="12" t="n"/>
+      <c r="X18" s="12" t="n"/>
+      <c r="Y18" s="9" t="n"/>
       <c r="Z18" s="21">
-        <f>IF(J18="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J18,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,1},MATCH(K18,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
+        <f>IF(J18="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J18,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K18,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
     </row>
     <row r="19">
+      <c r="A19" s="12" t="n"/>
+      <c r="B19" s="12" t="n"/>
+      <c r="C19" s="12" t="n"/>
+      <c r="D19" s="12" t="n"/>
+      <c r="E19" s="12" t="n"/>
+      <c r="F19" s="12" t="n"/>
+      <c r="G19" s="12" t="n"/>
+      <c r="H19" s="20" t="n"/>
+      <c r="I19" s="20" t="n"/>
+      <c r="J19" s="9" t="n"/>
+      <c r="K19" s="12" t="n"/>
+      <c r="L19" s="9" t="n"/>
+      <c r="M19" s="9" t="n"/>
+      <c r="N19" s="9" t="n"/>
+      <c r="O19" s="9" t="n"/>
+      <c r="P19" s="9" t="n"/>
+      <c r="Q19" s="9" t="n"/>
+      <c r="R19" s="9" t="n"/>
+      <c r="S19" s="12" t="n"/>
+      <c r="T19" s="12" t="n"/>
+      <c r="U19" s="12" t="n"/>
+      <c r="V19" s="12" t="n"/>
+      <c r="W19" s="12" t="n"/>
+      <c r="X19" s="12" t="n"/>
+      <c r="Y19" s="9" t="n"/>
       <c r="Z19" s="21">
-        <f>IF(J19="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J19,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,1},MATCH(K19,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
+        <f>IF(J19="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J19,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K19,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
     </row>
     <row r="20">
+      <c r="A20" s="12" t="n"/>
+      <c r="B20" s="12" t="n"/>
+      <c r="C20" s="12" t="n"/>
+      <c r="D20" s="12" t="n"/>
+      <c r="E20" s="12" t="n"/>
+      <c r="F20" s="12" t="n"/>
+      <c r="G20" s="12" t="n"/>
+      <c r="H20" s="20" t="n"/>
+      <c r="I20" s="20" t="n"/>
+      <c r="J20" s="9" t="n"/>
+      <c r="K20" s="12" t="n"/>
+      <c r="L20" s="9" t="n"/>
+      <c r="M20" s="9" t="n"/>
+      <c r="N20" s="9" t="n"/>
+      <c r="O20" s="9" t="n"/>
+      <c r="P20" s="9" t="n"/>
+      <c r="Q20" s="9" t="n"/>
+      <c r="R20" s="9" t="n"/>
+      <c r="S20" s="12" t="n"/>
+      <c r="T20" s="12" t="n"/>
+      <c r="U20" s="12" t="n"/>
+      <c r="V20" s="12" t="n"/>
+      <c r="W20" s="12" t="n"/>
+      <c r="X20" s="12" t="n"/>
+      <c r="Y20" s="9" t="n"/>
       <c r="Z20" s="21">
-        <f>IF(J20="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J20,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,1},MATCH(K20,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
+        <f>IF(J20="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J20,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K20,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
     </row>
     <row r="21">
+      <c r="A21" s="12" t="n"/>
+      <c r="B21" s="12" t="n"/>
+      <c r="C21" s="12" t="n"/>
+      <c r="D21" s="12" t="n"/>
+      <c r="E21" s="12" t="n"/>
+      <c r="F21" s="12" t="n"/>
+      <c r="G21" s="12" t="n"/>
+      <c r="H21" s="20" t="n"/>
+      <c r="I21" s="20" t="n"/>
+      <c r="J21" s="9" t="n"/>
+      <c r="K21" s="12" t="n"/>
+      <c r="L21" s="9" t="n"/>
+      <c r="M21" s="9" t="n"/>
+      <c r="N21" s="9" t="n"/>
+      <c r="O21" s="9" t="n"/>
+      <c r="P21" s="9" t="n"/>
+      <c r="Q21" s="9" t="n"/>
+      <c r="R21" s="9" t="n"/>
+      <c r="S21" s="12" t="n"/>
+      <c r="T21" s="12" t="n"/>
+      <c r="U21" s="12" t="n"/>
+      <c r="V21" s="12" t="n"/>
+      <c r="W21" s="12" t="n"/>
+      <c r="X21" s="12" t="n"/>
+      <c r="Y21" s="9" t="n"/>
       <c r="Z21" s="21">
-        <f>IF(J21="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J21,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,1},MATCH(K21,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
+        <f>IF(J21="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J21,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K21,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
     </row>
     <row r="22">
+      <c r="A22" s="12" t="n"/>
+      <c r="B22" s="12" t="n"/>
+      <c r="C22" s="12" t="n"/>
+      <c r="D22" s="12" t="n"/>
+      <c r="E22" s="12" t="n"/>
+      <c r="F22" s="12" t="n"/>
+      <c r="G22" s="12" t="n"/>
+      <c r="H22" s="20" t="n"/>
+      <c r="I22" s="20" t="n"/>
+      <c r="J22" s="9" t="n"/>
+      <c r="K22" s="12" t="n"/>
+      <c r="L22" s="9" t="n"/>
+      <c r="M22" s="9" t="n"/>
+      <c r="N22" s="9" t="n"/>
+      <c r="O22" s="9" t="n"/>
+      <c r="P22" s="9" t="n"/>
+      <c r="Q22" s="9" t="n"/>
+      <c r="R22" s="9" t="n"/>
+      <c r="S22" s="12" t="n"/>
+      <c r="T22" s="12" t="n"/>
+      <c r="U22" s="12" t="n"/>
+      <c r="V22" s="12" t="n"/>
+      <c r="W22" s="12" t="n"/>
+      <c r="X22" s="12" t="n"/>
+      <c r="Y22" s="9" t="n"/>
       <c r="Z22" s="21">
-        <f>IF(J22="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J22,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,1},MATCH(K22,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
+        <f>IF(J22="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J22,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K22,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
     </row>
     <row r="23">
+      <c r="A23" s="12" t="n"/>
+      <c r="B23" s="12" t="n"/>
+      <c r="C23" s="12" t="n"/>
+      <c r="D23" s="12" t="n"/>
+      <c r="E23" s="12" t="n"/>
+      <c r="F23" s="12" t="n"/>
+      <c r="G23" s="12" t="n"/>
+      <c r="H23" s="20" t="n"/>
+      <c r="I23" s="20" t="n"/>
+      <c r="J23" s="9" t="n"/>
+      <c r="K23" s="12" t="n"/>
+      <c r="L23" s="9" t="n"/>
+      <c r="M23" s="9" t="n"/>
+      <c r="N23" s="9" t="n"/>
+      <c r="O23" s="9" t="n"/>
+      <c r="P23" s="9" t="n"/>
+      <c r="Q23" s="9" t="n"/>
+      <c r="R23" s="9" t="n"/>
+      <c r="S23" s="12" t="n"/>
+      <c r="T23" s="12" t="n"/>
+      <c r="U23" s="12" t="n"/>
+      <c r="V23" s="12" t="n"/>
+      <c r="W23" s="12" t="n"/>
+      <c r="X23" s="12" t="n"/>
+      <c r="Y23" s="9" t="n"/>
       <c r="Z23" s="21">
-        <f>IF(J23="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J23,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,1},MATCH(K23,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
+        <f>IF(J23="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J23,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K23,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
     </row>
     <row r="24">
+      <c r="A24" s="12" t="n"/>
+      <c r="B24" s="12" t="n"/>
+      <c r="C24" s="12" t="n"/>
+      <c r="D24" s="12" t="n"/>
+      <c r="E24" s="12" t="n"/>
+      <c r="F24" s="12" t="n"/>
+      <c r="G24" s="12" t="n"/>
+      <c r="H24" s="20" t="n"/>
+      <c r="I24" s="20" t="n"/>
+      <c r="J24" s="9" t="n"/>
+      <c r="K24" s="12" t="n"/>
+      <c r="L24" s="9" t="n"/>
+      <c r="M24" s="9" t="n"/>
+      <c r="N24" s="9" t="n"/>
+      <c r="O24" s="9" t="n"/>
+      <c r="P24" s="9" t="n"/>
+      <c r="Q24" s="9" t="n"/>
+      <c r="R24" s="9" t="n"/>
+      <c r="S24" s="12" t="n"/>
+      <c r="T24" s="12" t="n"/>
+      <c r="U24" s="12" t="n"/>
+      <c r="V24" s="12" t="n"/>
+      <c r="W24" s="12" t="n"/>
+      <c r="X24" s="12" t="n"/>
+      <c r="Y24" s="9" t="n"/>
       <c r="Z24" s="21">
-        <f>IF(J24="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J24,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,1},MATCH(K24,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
+        <f>IF(J24="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J24,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K24,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
     </row>
     <row r="25">
+      <c r="A25" s="12" t="n"/>
+      <c r="B25" s="12" t="n"/>
+      <c r="C25" s="12" t="n"/>
+      <c r="D25" s="12" t="n"/>
+      <c r="E25" s="12" t="n"/>
+      <c r="F25" s="12" t="n"/>
+      <c r="G25" s="12" t="n"/>
+      <c r="H25" s="20" t="n"/>
+      <c r="I25" s="20" t="n"/>
+      <c r="J25" s="9" t="n"/>
+      <c r="K25" s="12" t="n"/>
+      <c r="L25" s="9" t="n"/>
+      <c r="M25" s="9" t="n"/>
+      <c r="N25" s="9" t="n"/>
+      <c r="O25" s="9" t="n"/>
+      <c r="P25" s="9" t="n"/>
+      <c r="Q25" s="9" t="n"/>
+      <c r="R25" s="9" t="n"/>
+      <c r="S25" s="12" t="n"/>
+      <c r="T25" s="12" t="n"/>
+      <c r="U25" s="12" t="n"/>
+      <c r="V25" s="12" t="n"/>
+      <c r="W25" s="12" t="n"/>
+      <c r="X25" s="12" t="n"/>
+      <c r="Y25" s="9" t="n"/>
       <c r="Z25" s="21">
-        <f>IF(J25="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J25,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,1},MATCH(K25,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
+        <f>IF(J25="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J25,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K25,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
     </row>
     <row r="26">
+      <c r="A26" s="12" t="n"/>
+      <c r="B26" s="12" t="n"/>
+      <c r="C26" s="12" t="n"/>
+      <c r="D26" s="12" t="n"/>
+      <c r="E26" s="12" t="n"/>
+      <c r="F26" s="12" t="n"/>
+      <c r="G26" s="12" t="n"/>
+      <c r="H26" s="20" t="n"/>
+      <c r="I26" s="20" t="n"/>
+      <c r="J26" s="9" t="n"/>
+      <c r="K26" s="12" t="n"/>
+      <c r="L26" s="9" t="n"/>
+      <c r="M26" s="9" t="n"/>
+      <c r="N26" s="9" t="n"/>
+      <c r="O26" s="9" t="n"/>
+      <c r="P26" s="9" t="n"/>
+      <c r="Q26" s="9" t="n"/>
+      <c r="R26" s="9" t="n"/>
+      <c r="S26" s="12" t="n"/>
+      <c r="T26" s="12" t="n"/>
+      <c r="U26" s="12" t="n"/>
+      <c r="V26" s="12" t="n"/>
+      <c r="W26" s="12" t="n"/>
+      <c r="X26" s="12" t="n"/>
+      <c r="Y26" s="9" t="n"/>
       <c r="Z26" s="21">
-        <f>IF(J26="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J26,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,1},MATCH(K26,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
+        <f>IF(J26="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J26,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K26,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
     </row>
     <row r="27">
+      <c r="A27" s="12" t="n"/>
+      <c r="B27" s="12" t="n"/>
+      <c r="C27" s="12" t="n"/>
+      <c r="D27" s="12" t="n"/>
+      <c r="E27" s="12" t="n"/>
+      <c r="F27" s="12" t="n"/>
+      <c r="G27" s="12" t="n"/>
+      <c r="H27" s="20" t="n"/>
+      <c r="I27" s="20" t="n"/>
+      <c r="J27" s="9" t="n"/>
+      <c r="K27" s="12" t="n"/>
+      <c r="L27" s="9" t="n"/>
+      <c r="M27" s="9" t="n"/>
+      <c r="N27" s="9" t="n"/>
+      <c r="O27" s="9" t="n"/>
+      <c r="P27" s="9" t="n"/>
+      <c r="Q27" s="9" t="n"/>
+      <c r="R27" s="9" t="n"/>
+      <c r="S27" s="12" t="n"/>
+      <c r="T27" s="12" t="n"/>
+      <c r="U27" s="12" t="n"/>
+      <c r="V27" s="12" t="n"/>
+      <c r="W27" s="12" t="n"/>
+      <c r="X27" s="12" t="n"/>
+      <c r="Y27" s="9" t="n"/>
       <c r="Z27" s="21">
-        <f>IF(J27="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J27,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,1},MATCH(K27,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
+        <f>IF(J27="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J27,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K27,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
     </row>
     <row r="28">
+      <c r="A28" s="12" t="n"/>
+      <c r="B28" s="12" t="n"/>
+      <c r="C28" s="12" t="n"/>
+      <c r="D28" s="12" t="n"/>
+      <c r="E28" s="12" t="n"/>
+      <c r="F28" s="12" t="n"/>
+      <c r="G28" s="12" t="n"/>
+      <c r="H28" s="20" t="n"/>
+      <c r="I28" s="20" t="n"/>
+      <c r="J28" s="9" t="n"/>
+      <c r="K28" s="12" t="n"/>
+      <c r="L28" s="9" t="n"/>
+      <c r="M28" s="9" t="n"/>
+      <c r="N28" s="9" t="n"/>
+      <c r="O28" s="9" t="n"/>
+      <c r="P28" s="9" t="n"/>
+      <c r="Q28" s="9" t="n"/>
+      <c r="R28" s="9" t="n"/>
+      <c r="S28" s="12" t="n"/>
+      <c r="T28" s="12" t="n"/>
+      <c r="U28" s="12" t="n"/>
+      <c r="V28" s="12" t="n"/>
+      <c r="W28" s="12" t="n"/>
+      <c r="X28" s="12" t="n"/>
+      <c r="Y28" s="9" t="n"/>
       <c r="Z28" s="21">
-        <f>IF(J28="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J28,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,1},MATCH(K28,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
+        <f>IF(J28="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J28,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K28,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
     </row>
     <row r="29">
+      <c r="A29" s="12" t="n"/>
+      <c r="B29" s="12" t="n"/>
+      <c r="C29" s="12" t="n"/>
+      <c r="D29" s="12" t="n"/>
+      <c r="E29" s="12" t="n"/>
+      <c r="F29" s="12" t="n"/>
+      <c r="G29" s="12" t="n"/>
+      <c r="H29" s="20" t="n"/>
+      <c r="I29" s="20" t="n"/>
+      <c r="J29" s="9" t="n"/>
+      <c r="K29" s="12" t="n"/>
+      <c r="L29" s="9" t="n"/>
+      <c r="M29" s="9" t="n"/>
+      <c r="N29" s="9" t="n"/>
+      <c r="O29" s="9" t="n"/>
+      <c r="P29" s="9" t="n"/>
+      <c r="Q29" s="9" t="n"/>
+      <c r="R29" s="9" t="n"/>
+      <c r="S29" s="12" t="n"/>
+      <c r="T29" s="12" t="n"/>
+      <c r="U29" s="12" t="n"/>
+      <c r="V29" s="12" t="n"/>
+      <c r="W29" s="12" t="n"/>
+      <c r="X29" s="12" t="n"/>
+      <c r="Y29" s="9" t="n"/>
       <c r="Z29" s="21">
-        <f>IF(J29="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J29,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,1},MATCH(K29,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
+        <f>IF(J29="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J29,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K29,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
     </row>
     <row r="30">
+      <c r="A30" s="12" t="n"/>
+      <c r="B30" s="12" t="n"/>
+      <c r="C30" s="12" t="n"/>
+      <c r="D30" s="12" t="n"/>
+      <c r="E30" s="12" t="n"/>
+      <c r="F30" s="12" t="n"/>
+      <c r="G30" s="12" t="n"/>
+      <c r="H30" s="20" t="n"/>
+      <c r="I30" s="20" t="n"/>
+      <c r="J30" s="9" t="n"/>
+      <c r="K30" s="12" t="n"/>
+      <c r="L30" s="9" t="n"/>
+      <c r="M30" s="9" t="n"/>
+      <c r="N30" s="9" t="n"/>
+      <c r="O30" s="9" t="n"/>
+      <c r="P30" s="9" t="n"/>
+      <c r="Q30" s="9" t="n"/>
+      <c r="R30" s="9" t="n"/>
+      <c r="S30" s="12" t="n"/>
+      <c r="T30" s="12" t="n"/>
+      <c r="U30" s="12" t="n"/>
+      <c r="V30" s="12" t="n"/>
+      <c r="W30" s="12" t="n"/>
+      <c r="X30" s="12" t="n"/>
+      <c r="Y30" s="9" t="n"/>
       <c r="Z30" s="21">
-        <f>IF(J30="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J30,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,1},MATCH(K30,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
+        <f>IF(J30="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J30,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K30,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
     </row>
     <row r="31">
+      <c r="A31" s="12" t="n"/>
+      <c r="B31" s="12" t="n"/>
+      <c r="C31" s="12" t="n"/>
+      <c r="D31" s="12" t="n"/>
+      <c r="E31" s="12" t="n"/>
+      <c r="F31" s="12" t="n"/>
+      <c r="G31" s="12" t="n"/>
+      <c r="H31" s="20" t="n"/>
+      <c r="I31" s="20" t="n"/>
+      <c r="J31" s="9" t="n"/>
+      <c r="K31" s="12" t="n"/>
+      <c r="L31" s="9" t="n"/>
+      <c r="M31" s="9" t="n"/>
+      <c r="N31" s="9" t="n"/>
+      <c r="O31" s="9" t="n"/>
+      <c r="P31" s="9" t="n"/>
+      <c r="Q31" s="9" t="n"/>
+      <c r="R31" s="9" t="n"/>
+      <c r="S31" s="12" t="n"/>
+      <c r="T31" s="12" t="n"/>
+      <c r="U31" s="12" t="n"/>
+      <c r="V31" s="12" t="n"/>
+      <c r="W31" s="12" t="n"/>
+      <c r="X31" s="12" t="n"/>
+      <c r="Y31" s="9" t="n"/>
       <c r="Z31" s="21">
-        <f>IF(J31="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J31,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,1},MATCH(K31,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
+        <f>IF(J31="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J31,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K31,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
     </row>
     <row r="32">
+      <c r="A32" s="12" t="n"/>
+      <c r="B32" s="12" t="n"/>
+      <c r="C32" s="12" t="n"/>
+      <c r="D32" s="12" t="n"/>
+      <c r="E32" s="12" t="n"/>
+      <c r="F32" s="12" t="n"/>
+      <c r="G32" s="12" t="n"/>
+      <c r="H32" s="20" t="n"/>
+      <c r="I32" s="20" t="n"/>
+      <c r="J32" s="9" t="n"/>
+      <c r="K32" s="12" t="n"/>
+      <c r="L32" s="9" t="n"/>
+      <c r="M32" s="9" t="n"/>
+      <c r="N32" s="9" t="n"/>
+      <c r="O32" s="9" t="n"/>
+      <c r="P32" s="9" t="n"/>
+      <c r="Q32" s="9" t="n"/>
+      <c r="R32" s="9" t="n"/>
+      <c r="S32" s="12" t="n"/>
+      <c r="T32" s="12" t="n"/>
+      <c r="U32" s="12" t="n"/>
+      <c r="V32" s="12" t="n"/>
+      <c r="W32" s="12" t="n"/>
+      <c r="X32" s="12" t="n"/>
+      <c r="Y32" s="9" t="n"/>
       <c r="Z32" s="21">
-        <f>IF(J32="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J32,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,1},MATCH(K32,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
+        <f>IF(J32="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J32,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K32,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
     </row>
     <row r="33">
+      <c r="A33" s="12" t="n"/>
+      <c r="B33" s="12" t="n"/>
+      <c r="C33" s="12" t="n"/>
+      <c r="D33" s="12" t="n"/>
+      <c r="E33" s="12" t="n"/>
+      <c r="F33" s="12" t="n"/>
+      <c r="G33" s="12" t="n"/>
+      <c r="H33" s="20" t="n"/>
+      <c r="I33" s="20" t="n"/>
+      <c r="J33" s="9" t="n"/>
+      <c r="K33" s="12" t="n"/>
+      <c r="L33" s="9" t="n"/>
+      <c r="M33" s="9" t="n"/>
+      <c r="N33" s="9" t="n"/>
+      <c r="O33" s="9" t="n"/>
+      <c r="P33" s="9" t="n"/>
+      <c r="Q33" s="9" t="n"/>
+      <c r="R33" s="9" t="n"/>
+      <c r="S33" s="12" t="n"/>
+      <c r="T33" s="12" t="n"/>
+      <c r="U33" s="12" t="n"/>
+      <c r="V33" s="12" t="n"/>
+      <c r="W33" s="12" t="n"/>
+      <c r="X33" s="12" t="n"/>
+      <c r="Y33" s="9" t="n"/>
       <c r="Z33" s="21">
-        <f>IF(J33="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J33,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,1},MATCH(K33,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
+        <f>IF(J33="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J33,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K33,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
     </row>
     <row r="34">
+      <c r="A34" s="12" t="n"/>
+      <c r="B34" s="12" t="n"/>
+      <c r="C34" s="12" t="n"/>
+      <c r="D34" s="12" t="n"/>
+      <c r="E34" s="12" t="n"/>
+      <c r="F34" s="12" t="n"/>
+      <c r="G34" s="12" t="n"/>
+      <c r="H34" s="20" t="n"/>
+      <c r="I34" s="20" t="n"/>
+      <c r="J34" s="9" t="n"/>
+      <c r="K34" s="12" t="n"/>
+      <c r="L34" s="9" t="n"/>
+      <c r="M34" s="9" t="n"/>
+      <c r="N34" s="9" t="n"/>
+      <c r="O34" s="9" t="n"/>
+      <c r="P34" s="9" t="n"/>
+      <c r="Q34" s="9" t="n"/>
+      <c r="R34" s="9" t="n"/>
+      <c r="S34" s="12" t="n"/>
+      <c r="T34" s="12" t="n"/>
+      <c r="U34" s="12" t="n"/>
+      <c r="V34" s="12" t="n"/>
+      <c r="W34" s="12" t="n"/>
+      <c r="X34" s="12" t="n"/>
+      <c r="Y34" s="9" t="n"/>
       <c r="Z34" s="21">
-        <f>IF(J34="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J34,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,1},MATCH(K34,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
+        <f>IF(J34="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J34,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K34,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
     </row>
     <row r="35">
+      <c r="A35" s="12" t="n"/>
+      <c r="B35" s="12" t="n"/>
+      <c r="C35" s="12" t="n"/>
+      <c r="D35" s="12" t="n"/>
+      <c r="E35" s="12" t="n"/>
+      <c r="F35" s="12" t="n"/>
+      <c r="G35" s="12" t="n"/>
+      <c r="H35" s="20" t="n"/>
+      <c r="I35" s="20" t="n"/>
+      <c r="J35" s="9" t="n"/>
+      <c r="K35" s="12" t="n"/>
+      <c r="L35" s="9" t="n"/>
+      <c r="M35" s="9" t="n"/>
+      <c r="N35" s="9" t="n"/>
+      <c r="O35" s="9" t="n"/>
+      <c r="P35" s="9" t="n"/>
+      <c r="Q35" s="9" t="n"/>
+      <c r="R35" s="9" t="n"/>
+      <c r="S35" s="12" t="n"/>
+      <c r="T35" s="12" t="n"/>
+      <c r="U35" s="12" t="n"/>
+      <c r="V35" s="12" t="n"/>
+      <c r="W35" s="12" t="n"/>
+      <c r="X35" s="12" t="n"/>
+      <c r="Y35" s="9" t="n"/>
       <c r="Z35" s="21">
-        <f>IF(J35="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J35,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,1},MATCH(K35,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
+        <f>IF(J35="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J35,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K35,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
     </row>
     <row r="36">
+      <c r="A36" s="12" t="n"/>
+      <c r="B36" s="12" t="n"/>
+      <c r="C36" s="12" t="n"/>
+      <c r="D36" s="12" t="n"/>
+      <c r="E36" s="12" t="n"/>
+      <c r="F36" s="12" t="n"/>
+      <c r="G36" s="12" t="n"/>
+      <c r="H36" s="20" t="n"/>
+      <c r="I36" s="20" t="n"/>
+      <c r="J36" s="9" t="n"/>
+      <c r="K36" s="12" t="n"/>
+      <c r="L36" s="9" t="n"/>
+      <c r="M36" s="9" t="n"/>
+      <c r="N36" s="9" t="n"/>
+      <c r="O36" s="9" t="n"/>
+      <c r="P36" s="9" t="n"/>
+      <c r="Q36" s="9" t="n"/>
+      <c r="R36" s="9" t="n"/>
+      <c r="S36" s="12" t="n"/>
+      <c r="T36" s="12" t="n"/>
+      <c r="U36" s="12" t="n"/>
+      <c r="V36" s="12" t="n"/>
+      <c r="W36" s="12" t="n"/>
+      <c r="X36" s="12" t="n"/>
+      <c r="Y36" s="9" t="n"/>
       <c r="Z36" s="21">
-        <f>IF(J36="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J36,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,1},MATCH(K36,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
+        <f>IF(J36="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J36,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K36,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
     </row>
     <row r="37">
+      <c r="A37" s="12" t="n"/>
+      <c r="B37" s="12" t="n"/>
+      <c r="C37" s="12" t="n"/>
+      <c r="D37" s="12" t="n"/>
+      <c r="E37" s="12" t="n"/>
+      <c r="F37" s="12" t="n"/>
+      <c r="G37" s="12" t="n"/>
+      <c r="H37" s="20" t="n"/>
+      <c r="I37" s="20" t="n"/>
+      <c r="J37" s="9" t="n"/>
+      <c r="K37" s="12" t="n"/>
+      <c r="L37" s="9" t="n"/>
+      <c r="M37" s="9" t="n"/>
+      <c r="N37" s="9" t="n"/>
+      <c r="O37" s="9" t="n"/>
+      <c r="P37" s="9" t="n"/>
+      <c r="Q37" s="9" t="n"/>
+      <c r="R37" s="9" t="n"/>
+      <c r="S37" s="12" t="n"/>
+      <c r="T37" s="12" t="n"/>
+      <c r="U37" s="12" t="n"/>
+      <c r="V37" s="12" t="n"/>
+      <c r="W37" s="12" t="n"/>
+      <c r="X37" s="12" t="n"/>
+      <c r="Y37" s="9" t="n"/>
       <c r="Z37" s="21">
-        <f>IF(J37="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J37,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,1},MATCH(K37,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
+        <f>IF(J37="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J37,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K37,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
     </row>
     <row r="38">
+      <c r="A38" s="12" t="n"/>
+      <c r="B38" s="12" t="n"/>
+      <c r="C38" s="12" t="n"/>
+      <c r="D38" s="12" t="n"/>
+      <c r="E38" s="12" t="n"/>
+      <c r="F38" s="12" t="n"/>
+      <c r="G38" s="12" t="n"/>
+      <c r="H38" s="20" t="n"/>
+      <c r="I38" s="20" t="n"/>
+      <c r="J38" s="9" t="n"/>
+      <c r="K38" s="12" t="n"/>
+      <c r="L38" s="9" t="n"/>
+      <c r="M38" s="9" t="n"/>
+      <c r="N38" s="9" t="n"/>
+      <c r="O38" s="9" t="n"/>
+      <c r="P38" s="9" t="n"/>
+      <c r="Q38" s="9" t="n"/>
+      <c r="R38" s="9" t="n"/>
+      <c r="S38" s="12" t="n"/>
+      <c r="T38" s="12" t="n"/>
+      <c r="U38" s="12" t="n"/>
+      <c r="V38" s="12" t="n"/>
+      <c r="W38" s="12" t="n"/>
+      <c r="X38" s="12" t="n"/>
+      <c r="Y38" s="9" t="n"/>
       <c r="Z38" s="21">
-        <f>IF(J38="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J38,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,1},MATCH(K38,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
+        <f>IF(J38="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J38,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K38,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
     </row>
     <row r="39">
+      <c r="A39" s="12" t="n"/>
+      <c r="B39" s="12" t="n"/>
+      <c r="C39" s="12" t="n"/>
+      <c r="D39" s="12" t="n"/>
+      <c r="E39" s="12" t="n"/>
+      <c r="F39" s="12" t="n"/>
+      <c r="G39" s="12" t="n"/>
+      <c r="H39" s="20" t="n"/>
+      <c r="I39" s="20" t="n"/>
+      <c r="J39" s="9" t="n"/>
+      <c r="K39" s="12" t="n"/>
+      <c r="L39" s="9" t="n"/>
+      <c r="M39" s="9" t="n"/>
+      <c r="N39" s="9" t="n"/>
+      <c r="O39" s="9" t="n"/>
+      <c r="P39" s="9" t="n"/>
+      <c r="Q39" s="9" t="n"/>
+      <c r="R39" s="9" t="n"/>
+      <c r="S39" s="12" t="n"/>
+      <c r="T39" s="12" t="n"/>
+      <c r="U39" s="12" t="n"/>
+      <c r="V39" s="12" t="n"/>
+      <c r="W39" s="12" t="n"/>
+      <c r="X39" s="12" t="n"/>
+      <c r="Y39" s="9" t="n"/>
       <c r="Z39" s="21">
-        <f>IF(J39="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J39,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,1},MATCH(K39,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
+        <f>IF(J39="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J39,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K39,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
     </row>
     <row r="40">
+      <c r="A40" s="12" t="n"/>
+      <c r="B40" s="12" t="n"/>
+      <c r="C40" s="12" t="n"/>
+      <c r="D40" s="12" t="n"/>
+      <c r="E40" s="12" t="n"/>
+      <c r="F40" s="12" t="n"/>
+      <c r="G40" s="12" t="n"/>
+      <c r="H40" s="20" t="n"/>
+      <c r="I40" s="20" t="n"/>
+      <c r="J40" s="9" t="n"/>
+      <c r="K40" s="12" t="n"/>
+      <c r="L40" s="9" t="n"/>
+      <c r="M40" s="9" t="n"/>
+      <c r="N40" s="9" t="n"/>
+      <c r="O40" s="9" t="n"/>
+      <c r="P40" s="9" t="n"/>
+      <c r="Q40" s="9" t="n"/>
+      <c r="R40" s="9" t="n"/>
+      <c r="S40" s="12" t="n"/>
+      <c r="T40" s="12" t="n"/>
+      <c r="U40" s="12" t="n"/>
+      <c r="V40" s="12" t="n"/>
+      <c r="W40" s="12" t="n"/>
+      <c r="X40" s="12" t="n"/>
+      <c r="Y40" s="9" t="n"/>
       <c r="Z40" s="21">
-        <f>IF(J40="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J40,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,1},MATCH(K40,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
+        <f>IF(J40="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J40,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K40,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
     </row>
     <row r="41">
+      <c r="A41" s="12" t="n"/>
+      <c r="B41" s="12" t="n"/>
+      <c r="C41" s="12" t="n"/>
+      <c r="D41" s="12" t="n"/>
+      <c r="E41" s="12" t="n"/>
+      <c r="F41" s="12" t="n"/>
+      <c r="G41" s="12" t="n"/>
+      <c r="H41" s="20" t="n"/>
+      <c r="I41" s="20" t="n"/>
+      <c r="J41" s="9" t="n"/>
+      <c r="K41" s="12" t="n"/>
+      <c r="L41" s="9" t="n"/>
+      <c r="M41" s="9" t="n"/>
+      <c r="N41" s="9" t="n"/>
+      <c r="O41" s="9" t="n"/>
+      <c r="P41" s="9" t="n"/>
+      <c r="Q41" s="9" t="n"/>
+      <c r="R41" s="9" t="n"/>
+      <c r="S41" s="12" t="n"/>
+      <c r="T41" s="12" t="n"/>
+      <c r="U41" s="12" t="n"/>
+      <c r="V41" s="12" t="n"/>
+      <c r="W41" s="12" t="n"/>
+      <c r="X41" s="12" t="n"/>
+      <c r="Y41" s="9" t="n"/>
       <c r="Z41" s="21">
-        <f>IF(J41="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J41,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,1},MATCH(K41,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
+        <f>IF(J41="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J41,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K41,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
     </row>
     <row r="42">
+      <c r="A42" s="12" t="n"/>
+      <c r="B42" s="12" t="n"/>
+      <c r="C42" s="12" t="n"/>
+      <c r="D42" s="12" t="n"/>
+      <c r="E42" s="12" t="n"/>
+      <c r="F42" s="12" t="n"/>
+      <c r="G42" s="12" t="n"/>
+      <c r="H42" s="20" t="n"/>
+      <c r="I42" s="20" t="n"/>
+      <c r="J42" s="9" t="n"/>
+      <c r="K42" s="12" t="n"/>
+      <c r="L42" s="9" t="n"/>
+      <c r="M42" s="9" t="n"/>
+      <c r="N42" s="9" t="n"/>
+      <c r="O42" s="9" t="n"/>
+      <c r="P42" s="9" t="n"/>
+      <c r="Q42" s="9" t="n"/>
+      <c r="R42" s="9" t="n"/>
+      <c r="S42" s="12" t="n"/>
+      <c r="T42" s="12" t="n"/>
+      <c r="U42" s="12" t="n"/>
+      <c r="V42" s="12" t="n"/>
+      <c r="W42" s="12" t="n"/>
+      <c r="X42" s="12" t="n"/>
+      <c r="Y42" s="9" t="n"/>
       <c r="Z42" s="21">
-        <f>IF(J42="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J42,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,1},MATCH(K42,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
+        <f>IF(J42="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J42,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K42,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
     </row>
     <row r="43">
+      <c r="A43" s="12" t="n"/>
+      <c r="B43" s="12" t="n"/>
+      <c r="C43" s="12" t="n"/>
+      <c r="D43" s="12" t="n"/>
+      <c r="E43" s="12" t="n"/>
+      <c r="F43" s="12" t="n"/>
+      <c r="G43" s="12" t="n"/>
+      <c r="H43" s="20" t="n"/>
+      <c r="I43" s="20" t="n"/>
+      <c r="J43" s="9" t="n"/>
+      <c r="K43" s="12" t="n"/>
+      <c r="L43" s="9" t="n"/>
+      <c r="M43" s="9" t="n"/>
+      <c r="N43" s="9" t="n"/>
+      <c r="O43" s="9" t="n"/>
+      <c r="P43" s="9" t="n"/>
+      <c r="Q43" s="9" t="n"/>
+      <c r="R43" s="9" t="n"/>
+      <c r="S43" s="12" t="n"/>
+      <c r="T43" s="12" t="n"/>
+      <c r="U43" s="12" t="n"/>
+      <c r="V43" s="12" t="n"/>
+      <c r="W43" s="12" t="n"/>
+      <c r="X43" s="12" t="n"/>
+      <c r="Y43" s="9" t="n"/>
       <c r="Z43" s="21">
-        <f>IF(J43="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J43,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,1},MATCH(K43,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
+        <f>IF(J43="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J43,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K43,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
     </row>
     <row r="44">
+      <c r="A44" s="12" t="n"/>
+      <c r="B44" s="12" t="n"/>
+      <c r="C44" s="12" t="n"/>
+      <c r="D44" s="12" t="n"/>
+      <c r="E44" s="12" t="n"/>
+      <c r="F44" s="12" t="n"/>
+      <c r="G44" s="12" t="n"/>
+      <c r="H44" s="20" t="n"/>
+      <c r="I44" s="20" t="n"/>
+      <c r="J44" s="9" t="n"/>
+      <c r="K44" s="12" t="n"/>
+      <c r="L44" s="9" t="n"/>
+      <c r="M44" s="9" t="n"/>
+      <c r="N44" s="9" t="n"/>
+      <c r="O44" s="9" t="n"/>
+      <c r="P44" s="9" t="n"/>
+      <c r="Q44" s="9" t="n"/>
+      <c r="R44" s="9" t="n"/>
+      <c r="S44" s="12" t="n"/>
+      <c r="T44" s="12" t="n"/>
+      <c r="U44" s="12" t="n"/>
+      <c r="V44" s="12" t="n"/>
+      <c r="W44" s="12" t="n"/>
+      <c r="X44" s="12" t="n"/>
+      <c r="Y44" s="9" t="n"/>
       <c r="Z44" s="21">
-        <f>IF(J44="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J44,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,1},MATCH(K44,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
+        <f>IF(J44="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J44,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K44,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
     </row>
     <row r="45">
+      <c r="A45" s="12" t="n"/>
+      <c r="B45" s="12" t="n"/>
+      <c r="C45" s="12" t="n"/>
+      <c r="D45" s="12" t="n"/>
+      <c r="E45" s="12" t="n"/>
+      <c r="F45" s="12" t="n"/>
+      <c r="G45" s="12" t="n"/>
+      <c r="H45" s="20" t="n"/>
+      <c r="I45" s="20" t="n"/>
+      <c r="J45" s="9" t="n"/>
+      <c r="K45" s="12" t="n"/>
+      <c r="L45" s="9" t="n"/>
+      <c r="M45" s="9" t="n"/>
+      <c r="N45" s="9" t="n"/>
+      <c r="O45" s="9" t="n"/>
+      <c r="P45" s="9" t="n"/>
+      <c r="Q45" s="9" t="n"/>
+      <c r="R45" s="9" t="n"/>
+      <c r="S45" s="12" t="n"/>
+      <c r="T45" s="12" t="n"/>
+      <c r="U45" s="12" t="n"/>
+      <c r="V45" s="12" t="n"/>
+      <c r="W45" s="12" t="n"/>
+      <c r="X45" s="12" t="n"/>
+      <c r="Y45" s="9" t="n"/>
       <c r="Z45" s="21">
-        <f>IF(J45="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J45,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,1},MATCH(K45,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
+        <f>IF(J45="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J45,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K45,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
     </row>
     <row r="46">
+      <c r="A46" s="12" t="n"/>
+      <c r="B46" s="12" t="n"/>
+      <c r="C46" s="12" t="n"/>
+      <c r="D46" s="12" t="n"/>
+      <c r="E46" s="12" t="n"/>
+      <c r="F46" s="12" t="n"/>
+      <c r="G46" s="12" t="n"/>
+      <c r="H46" s="20" t="n"/>
+      <c r="I46" s="20" t="n"/>
+      <c r="J46" s="9" t="n"/>
+      <c r="K46" s="12" t="n"/>
+      <c r="L46" s="9" t="n"/>
+      <c r="M46" s="9" t="n"/>
+      <c r="N46" s="9" t="n"/>
+      <c r="O46" s="9" t="n"/>
+      <c r="P46" s="9" t="n"/>
+      <c r="Q46" s="9" t="n"/>
+      <c r="R46" s="9" t="n"/>
+      <c r="S46" s="12" t="n"/>
+      <c r="T46" s="12" t="n"/>
+      <c r="U46" s="12" t="n"/>
+      <c r="V46" s="12" t="n"/>
+      <c r="W46" s="12" t="n"/>
+      <c r="X46" s="12" t="n"/>
+      <c r="Y46" s="9" t="n"/>
       <c r="Z46" s="21">
-        <f>IF(J46="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J46,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,1},MATCH(K46,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
+        <f>IF(J46="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J46,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K46,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
     </row>
     <row r="47">
+      <c r="A47" s="12" t="n"/>
+      <c r="B47" s="12" t="n"/>
+      <c r="C47" s="12" t="n"/>
+      <c r="D47" s="12" t="n"/>
+      <c r="E47" s="12" t="n"/>
+      <c r="F47" s="12" t="n"/>
+      <c r="G47" s="12" t="n"/>
+      <c r="H47" s="20" t="n"/>
+      <c r="I47" s="20" t="n"/>
+      <c r="J47" s="9" t="n"/>
+      <c r="K47" s="12" t="n"/>
+      <c r="L47" s="9" t="n"/>
+      <c r="M47" s="9" t="n"/>
+      <c r="N47" s="9" t="n"/>
+      <c r="O47" s="9" t="n"/>
+      <c r="P47" s="9" t="n"/>
+      <c r="Q47" s="9" t="n"/>
+      <c r="R47" s="9" t="n"/>
+      <c r="S47" s="12" t="n"/>
+      <c r="T47" s="12" t="n"/>
+      <c r="U47" s="12" t="n"/>
+      <c r="V47" s="12" t="n"/>
+      <c r="W47" s="12" t="n"/>
+      <c r="X47" s="12" t="n"/>
+      <c r="Y47" s="9" t="n"/>
       <c r="Z47" s="21">
-        <f>IF(J47="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J47,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,1},MATCH(K47,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
+        <f>IF(J47="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J47,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K47,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
     </row>
     <row r="48">
+      <c r="A48" s="12" t="n"/>
+      <c r="B48" s="12" t="n"/>
+      <c r="C48" s="12" t="n"/>
+      <c r="D48" s="12" t="n"/>
+      <c r="E48" s="12" t="n"/>
+      <c r="F48" s="12" t="n"/>
+      <c r="G48" s="12" t="n"/>
+      <c r="H48" s="20" t="n"/>
+      <c r="I48" s="20" t="n"/>
+      <c r="J48" s="9" t="n"/>
+      <c r="K48" s="12" t="n"/>
+      <c r="L48" s="9" t="n"/>
+      <c r="M48" s="9" t="n"/>
+      <c r="N48" s="9" t="n"/>
+      <c r="O48" s="9" t="n"/>
+      <c r="P48" s="9" t="n"/>
+      <c r="Q48" s="9" t="n"/>
+      <c r="R48" s="9" t="n"/>
+      <c r="S48" s="12" t="n"/>
+      <c r="T48" s="12" t="n"/>
+      <c r="U48" s="12" t="n"/>
+      <c r="V48" s="12" t="n"/>
+      <c r="W48" s="12" t="n"/>
+      <c r="X48" s="12" t="n"/>
+      <c r="Y48" s="9" t="n"/>
       <c r="Z48" s="21">
-        <f>IF(J48="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J48,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,1},MATCH(K48,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
+        <f>IF(J48="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J48,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K48,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
     </row>
     <row r="49">
+      <c r="A49" s="12" t="n"/>
+      <c r="B49" s="12" t="n"/>
+      <c r="C49" s="12" t="n"/>
+      <c r="D49" s="12" t="n"/>
+      <c r="E49" s="12" t="n"/>
+      <c r="F49" s="12" t="n"/>
+      <c r="G49" s="12" t="n"/>
+      <c r="H49" s="20" t="n"/>
+      <c r="I49" s="20" t="n"/>
+      <c r="J49" s="9" t="n"/>
+      <c r="K49" s="12" t="n"/>
+      <c r="L49" s="9" t="n"/>
+      <c r="M49" s="9" t="n"/>
+      <c r="N49" s="9" t="n"/>
+      <c r="O49" s="9" t="n"/>
+      <c r="P49" s="9" t="n"/>
+      <c r="Q49" s="9" t="n"/>
+      <c r="R49" s="9" t="n"/>
+      <c r="S49" s="12" t="n"/>
+      <c r="T49" s="12" t="n"/>
+      <c r="U49" s="12" t="n"/>
+      <c r="V49" s="12" t="n"/>
+      <c r="W49" s="12" t="n"/>
+      <c r="X49" s="12" t="n"/>
+      <c r="Y49" s="9" t="n"/>
       <c r="Z49" s="21">
-        <f>IF(J49="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J49,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,1},MATCH(K49,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
+        <f>IF(J49="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J49,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K49,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
     </row>
     <row r="50">
+      <c r="A50" s="12" t="n"/>
+      <c r="B50" s="12" t="n"/>
+      <c r="C50" s="12" t="n"/>
+      <c r="D50" s="12" t="n"/>
+      <c r="E50" s="12" t="n"/>
+      <c r="F50" s="12" t="n"/>
+      <c r="G50" s="12" t="n"/>
+      <c r="H50" s="20" t="n"/>
+      <c r="I50" s="20" t="n"/>
+      <c r="J50" s="9" t="n"/>
+      <c r="K50" s="12" t="n"/>
+      <c r="L50" s="9" t="n"/>
+      <c r="M50" s="9" t="n"/>
+      <c r="N50" s="9" t="n"/>
+      <c r="O50" s="9" t="n"/>
+      <c r="P50" s="9" t="n"/>
+      <c r="Q50" s="9" t="n"/>
+      <c r="R50" s="9" t="n"/>
+      <c r="S50" s="12" t="n"/>
+      <c r="T50" s="12" t="n"/>
+      <c r="U50" s="12" t="n"/>
+      <c r="V50" s="12" t="n"/>
+      <c r="W50" s="12" t="n"/>
+      <c r="X50" s="12" t="n"/>
+      <c r="Y50" s="9" t="n"/>
       <c r="Z50" s="21">
-        <f>IF(J50="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J50,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,1},MATCH(K50,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
+        <f>IF(J50="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J50,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K50,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
     </row>
     <row r="51">
+      <c r="A51" s="12" t="n"/>
+      <c r="B51" s="12" t="n"/>
+      <c r="C51" s="12" t="n"/>
+      <c r="D51" s="12" t="n"/>
+      <c r="E51" s="12" t="n"/>
+      <c r="F51" s="12" t="n"/>
+      <c r="G51" s="12" t="n"/>
+      <c r="H51" s="20" t="n"/>
+      <c r="I51" s="20" t="n"/>
+      <c r="J51" s="9" t="n"/>
+      <c r="K51" s="12" t="n"/>
+      <c r="L51" s="9" t="n"/>
+      <c r="M51" s="9" t="n"/>
+      <c r="N51" s="9" t="n"/>
+      <c r="O51" s="9" t="n"/>
+      <c r="P51" s="9" t="n"/>
+      <c r="Q51" s="9" t="n"/>
+      <c r="R51" s="9" t="n"/>
+      <c r="S51" s="12" t="n"/>
+      <c r="T51" s="12" t="n"/>
+      <c r="U51" s="12" t="n"/>
+      <c r="V51" s="12" t="n"/>
+      <c r="W51" s="12" t="n"/>
+      <c r="X51" s="12" t="n"/>
+      <c r="Y51" s="9" t="n"/>
       <c r="Z51" s="21">
-        <f>IF(J51="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J51,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,1},MATCH(K51,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
+        <f>IF(J51="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J51,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K51,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
     </row>
     <row r="52">
+      <c r="A52" s="12" t="n"/>
+      <c r="B52" s="12" t="n"/>
+      <c r="C52" s="12" t="n"/>
+      <c r="D52" s="12" t="n"/>
+      <c r="E52" s="12" t="n"/>
+      <c r="F52" s="12" t="n"/>
+      <c r="G52" s="12" t="n"/>
+      <c r="H52" s="20" t="n"/>
+      <c r="I52" s="20" t="n"/>
+      <c r="J52" s="9" t="n"/>
+      <c r="K52" s="12" t="n"/>
+      <c r="L52" s="9" t="n"/>
+      <c r="M52" s="9" t="n"/>
+      <c r="N52" s="9" t="n"/>
+      <c r="O52" s="9" t="n"/>
+      <c r="P52" s="9" t="n"/>
+      <c r="Q52" s="9" t="n"/>
+      <c r="R52" s="9" t="n"/>
+      <c r="S52" s="12" t="n"/>
+      <c r="T52" s="12" t="n"/>
+      <c r="U52" s="12" t="n"/>
+      <c r="V52" s="12" t="n"/>
+      <c r="W52" s="12" t="n"/>
+      <c r="X52" s="12" t="n"/>
+      <c r="Y52" s="9" t="n"/>
       <c r="Z52" s="21">
-        <f>IF(J52="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J52,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,1},MATCH(K52,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
+        <f>IF(J52="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J52,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K52,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
     </row>
     <row r="53">
+      <c r="A53" s="12" t="n"/>
+      <c r="B53" s="12" t="n"/>
+      <c r="C53" s="12" t="n"/>
+      <c r="D53" s="12" t="n"/>
+      <c r="E53" s="12" t="n"/>
+      <c r="F53" s="12" t="n"/>
+      <c r="G53" s="12" t="n"/>
+      <c r="H53" s="20" t="n"/>
+      <c r="I53" s="20" t="n"/>
+      <c r="J53" s="9" t="n"/>
+      <c r="K53" s="12" t="n"/>
+      <c r="L53" s="9" t="n"/>
+      <c r="M53" s="9" t="n"/>
+      <c r="N53" s="9" t="n"/>
+      <c r="O53" s="9" t="n"/>
+      <c r="P53" s="9" t="n"/>
+      <c r="Q53" s="9" t="n"/>
+      <c r="R53" s="9" t="n"/>
+      <c r="S53" s="12" t="n"/>
+      <c r="T53" s="12" t="n"/>
+      <c r="U53" s="12" t="n"/>
+      <c r="V53" s="12" t="n"/>
+      <c r="W53" s="12" t="n"/>
+      <c r="X53" s="12" t="n"/>
+      <c r="Y53" s="9" t="n"/>
       <c r="Z53" s="21">
-        <f>IF(J53="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J53,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,1},MATCH(K53,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
+        <f>IF(J53="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J53,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K53,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
     </row>
     <row r="54">
+      <c r="A54" s="12" t="n"/>
+      <c r="B54" s="12" t="n"/>
+      <c r="C54" s="12" t="n"/>
+      <c r="D54" s="12" t="n"/>
+      <c r="E54" s="12" t="n"/>
+      <c r="F54" s="12" t="n"/>
+      <c r="G54" s="12" t="n"/>
+      <c r="H54" s="20" t="n"/>
+      <c r="I54" s="20" t="n"/>
+      <c r="J54" s="9" t="n"/>
+      <c r="K54" s="12" t="n"/>
+      <c r="L54" s="9" t="n"/>
+      <c r="M54" s="9" t="n"/>
+      <c r="N54" s="9" t="n"/>
+      <c r="O54" s="9" t="n"/>
+      <c r="P54" s="9" t="n"/>
+      <c r="Q54" s="9" t="n"/>
+      <c r="R54" s="9" t="n"/>
+      <c r="S54" s="12" t="n"/>
+      <c r="T54" s="12" t="n"/>
+      <c r="U54" s="12" t="n"/>
+      <c r="V54" s="12" t="n"/>
+      <c r="W54" s="12" t="n"/>
+      <c r="X54" s="12" t="n"/>
+      <c r="Y54" s="9" t="n"/>
       <c r="Z54" s="21">
-        <f>IF(J54="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J54,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,1},MATCH(K54,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
+        <f>IF(J54="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J54,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K54,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
     </row>
     <row r="55">
+      <c r="A55" s="12" t="n"/>
+      <c r="B55" s="12" t="n"/>
+      <c r="C55" s="12" t="n"/>
+      <c r="D55" s="12" t="n"/>
+      <c r="E55" s="12" t="n"/>
+      <c r="F55" s="12" t="n"/>
+      <c r="G55" s="12" t="n"/>
+      <c r="H55" s="20" t="n"/>
+      <c r="I55" s="20" t="n"/>
+      <c r="J55" s="9" t="n"/>
+      <c r="K55" s="12" t="n"/>
+      <c r="L55" s="9" t="n"/>
+      <c r="M55" s="9" t="n"/>
+      <c r="N55" s="9" t="n"/>
+      <c r="O55" s="9" t="n"/>
+      <c r="P55" s="9" t="n"/>
+      <c r="Q55" s="9" t="n"/>
+      <c r="R55" s="9" t="n"/>
+      <c r="S55" s="12" t="n"/>
+      <c r="T55" s="12" t="n"/>
+      <c r="U55" s="12" t="n"/>
+      <c r="V55" s="12" t="n"/>
+      <c r="W55" s="12" t="n"/>
+      <c r="X55" s="12" t="n"/>
+      <c r="Y55" s="9" t="n"/>
       <c r="Z55" s="21">
-        <f>IF(J55="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J55,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,1},MATCH(K55,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
+        <f>IF(J55="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J55,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K55,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
     </row>
     <row r="56">
+      <c r="A56" s="12" t="n"/>
+      <c r="B56" s="12" t="n"/>
+      <c r="C56" s="12" t="n"/>
+      <c r="D56" s="12" t="n"/>
+      <c r="E56" s="12" t="n"/>
+      <c r="F56" s="12" t="n"/>
+      <c r="G56" s="12" t="n"/>
+      <c r="H56" s="20" t="n"/>
+      <c r="I56" s="20" t="n"/>
+      <c r="J56" s="9" t="n"/>
+      <c r="K56" s="12" t="n"/>
+      <c r="L56" s="9" t="n"/>
+      <c r="M56" s="9" t="n"/>
+      <c r="N56" s="9" t="n"/>
+      <c r="O56" s="9" t="n"/>
+      <c r="P56" s="9" t="n"/>
+      <c r="Q56" s="9" t="n"/>
+      <c r="R56" s="9" t="n"/>
+      <c r="S56" s="12" t="n"/>
+      <c r="T56" s="12" t="n"/>
+      <c r="U56" s="12" t="n"/>
+      <c r="V56" s="12" t="n"/>
+      <c r="W56" s="12" t="n"/>
+      <c r="X56" s="12" t="n"/>
+      <c r="Y56" s="9" t="n"/>
       <c r="Z56" s="21">
-        <f>IF(J56="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J56,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,1},MATCH(K56,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
+        <f>IF(J56="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J56,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K56,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
     </row>
     <row r="57">
+      <c r="A57" s="12" t="n"/>
+      <c r="B57" s="12" t="n"/>
+      <c r="C57" s="12" t="n"/>
+      <c r="D57" s="12" t="n"/>
+      <c r="E57" s="12" t="n"/>
+      <c r="F57" s="12" t="n"/>
+      <c r="G57" s="12" t="n"/>
+      <c r="H57" s="20" t="n"/>
+      <c r="I57" s="20" t="n"/>
+      <c r="J57" s="9" t="n"/>
+      <c r="K57" s="12" t="n"/>
+      <c r="L57" s="9" t="n"/>
+      <c r="M57" s="9" t="n"/>
+      <c r="N57" s="9" t="n"/>
+      <c r="O57" s="9" t="n"/>
+      <c r="P57" s="9" t="n"/>
+      <c r="Q57" s="9" t="n"/>
+      <c r="R57" s="9" t="n"/>
+      <c r="S57" s="12" t="n"/>
+      <c r="T57" s="12" t="n"/>
+      <c r="U57" s="12" t="n"/>
+      <c r="V57" s="12" t="n"/>
+      <c r="W57" s="12" t="n"/>
+      <c r="X57" s="12" t="n"/>
+      <c r="Y57" s="9" t="n"/>
       <c r="Z57" s="21">
-        <f>IF(J57="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J57,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,1},MATCH(K57,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
+        <f>IF(J57="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J57,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K57,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
     </row>
     <row r="58">
+      <c r="A58" s="12" t="n"/>
+      <c r="B58" s="12" t="n"/>
+      <c r="C58" s="12" t="n"/>
+      <c r="D58" s="12" t="n"/>
+      <c r="E58" s="12" t="n"/>
+      <c r="F58" s="12" t="n"/>
+      <c r="G58" s="12" t="n"/>
+      <c r="H58" s="20" t="n"/>
+      <c r="I58" s="20" t="n"/>
+      <c r="J58" s="9" t="n"/>
+      <c r="K58" s="12" t="n"/>
+      <c r="L58" s="9" t="n"/>
+      <c r="M58" s="9" t="n"/>
+      <c r="N58" s="9" t="n"/>
+      <c r="O58" s="9" t="n"/>
+      <c r="P58" s="9" t="n"/>
+      <c r="Q58" s="9" t="n"/>
+      <c r="R58" s="9" t="n"/>
+      <c r="S58" s="12" t="n"/>
+      <c r="T58" s="12" t="n"/>
+      <c r="U58" s="12" t="n"/>
+      <c r="V58" s="12" t="n"/>
+      <c r="W58" s="12" t="n"/>
+      <c r="X58" s="12" t="n"/>
+      <c r="Y58" s="9" t="n"/>
       <c r="Z58" s="21">
-        <f>IF(J58="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J58,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,1},MATCH(K58,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
+        <f>IF(J58="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J58,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K58,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
     </row>
     <row r="59">
+      <c r="A59" s="12" t="n"/>
+      <c r="B59" s="12" t="n"/>
+      <c r="C59" s="12" t="n"/>
+      <c r="D59" s="12" t="n"/>
+      <c r="E59" s="12" t="n"/>
+      <c r="F59" s="12" t="n"/>
+      <c r="G59" s="12" t="n"/>
+      <c r="H59" s="20" t="n"/>
+      <c r="I59" s="20" t="n"/>
+      <c r="J59" s="9" t="n"/>
+      <c r="K59" s="12" t="n"/>
+      <c r="L59" s="9" t="n"/>
+      <c r="M59" s="9" t="n"/>
+      <c r="N59" s="9" t="n"/>
+      <c r="O59" s="9" t="n"/>
+      <c r="P59" s="9" t="n"/>
+      <c r="Q59" s="9" t="n"/>
+      <c r="R59" s="9" t="n"/>
+      <c r="S59" s="12" t="n"/>
+      <c r="T59" s="12" t="n"/>
+      <c r="U59" s="12" t="n"/>
+      <c r="V59" s="12" t="n"/>
+      <c r="W59" s="12" t="n"/>
+      <c r="X59" s="12" t="n"/>
+      <c r="Y59" s="9" t="n"/>
       <c r="Z59" s="21">
-        <f>IF(J59="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J59,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,1},MATCH(K59,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
+        <f>IF(J59="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J59,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K59,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
     </row>
     <row r="60">
+      <c r="A60" s="12" t="n"/>
+      <c r="B60" s="12" t="n"/>
+      <c r="C60" s="12" t="n"/>
+      <c r="D60" s="12" t="n"/>
+      <c r="E60" s="12" t="n"/>
+      <c r="F60" s="12" t="n"/>
+      <c r="G60" s="12" t="n"/>
+      <c r="H60" s="20" t="n"/>
+      <c r="I60" s="20" t="n"/>
+      <c r="J60" s="9" t="n"/>
+      <c r="K60" s="12" t="n"/>
+      <c r="L60" s="9" t="n"/>
+      <c r="M60" s="9" t="n"/>
+      <c r="N60" s="9" t="n"/>
+      <c r="O60" s="9" t="n"/>
+      <c r="P60" s="9" t="n"/>
+      <c r="Q60" s="9" t="n"/>
+      <c r="R60" s="9" t="n"/>
+      <c r="S60" s="12" t="n"/>
+      <c r="T60" s="12" t="n"/>
+      <c r="U60" s="12" t="n"/>
+      <c r="V60" s="12" t="n"/>
+      <c r="W60" s="12" t="n"/>
+      <c r="X60" s="12" t="n"/>
+      <c r="Y60" s="9" t="n"/>
       <c r="Z60" s="21">
-        <f>IF(J60="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J60,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,1},MATCH(K60,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
+        <f>IF(J60="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J60,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K60,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
     </row>
     <row r="61">
+      <c r="A61" s="12" t="n"/>
+      <c r="B61" s="12" t="n"/>
+      <c r="C61" s="12" t="n"/>
+      <c r="D61" s="12" t="n"/>
+      <c r="E61" s="12" t="n"/>
+      <c r="F61" s="12" t="n"/>
+      <c r="G61" s="12" t="n"/>
+      <c r="H61" s="20" t="n"/>
+      <c r="I61" s="20" t="n"/>
+      <c r="J61" s="9" t="n"/>
+      <c r="K61" s="12" t="n"/>
+      <c r="L61" s="9" t="n"/>
+      <c r="M61" s="9" t="n"/>
+      <c r="N61" s="9" t="n"/>
+      <c r="O61" s="9" t="n"/>
+      <c r="P61" s="9" t="n"/>
+      <c r="Q61" s="9" t="n"/>
+      <c r="R61" s="9" t="n"/>
+      <c r="S61" s="12" t="n"/>
+      <c r="T61" s="12" t="n"/>
+      <c r="U61" s="12" t="n"/>
+      <c r="V61" s="12" t="n"/>
+      <c r="W61" s="12" t="n"/>
+      <c r="X61" s="12" t="n"/>
+      <c r="Y61" s="9" t="n"/>
       <c r="Z61" s="21">
-        <f>IF(J61="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J61,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,1},MATCH(K61,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
+        <f>IF(J61="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J61,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K61,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
     </row>
     <row r="62">
+      <c r="A62" s="12" t="n"/>
+      <c r="B62" s="12" t="n"/>
+      <c r="C62" s="12" t="n"/>
+      <c r="D62" s="12" t="n"/>
+      <c r="E62" s="12" t="n"/>
+      <c r="F62" s="12" t="n"/>
+      <c r="G62" s="12" t="n"/>
+      <c r="H62" s="20" t="n"/>
+      <c r="I62" s="20" t="n"/>
+      <c r="J62" s="9" t="n"/>
+      <c r="K62" s="12" t="n"/>
+      <c r="L62" s="9" t="n"/>
+      <c r="M62" s="9" t="n"/>
+      <c r="N62" s="9" t="n"/>
+      <c r="O62" s="9" t="n"/>
+      <c r="P62" s="9" t="n"/>
+      <c r="Q62" s="9" t="n"/>
+      <c r="R62" s="9" t="n"/>
+      <c r="S62" s="12" t="n"/>
+      <c r="T62" s="12" t="n"/>
+      <c r="U62" s="12" t="n"/>
+      <c r="V62" s="12" t="n"/>
+      <c r="W62" s="12" t="n"/>
+      <c r="X62" s="12" t="n"/>
+      <c r="Y62" s="9" t="n"/>
       <c r="Z62" s="21">
-        <f>IF(J62="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J62,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,1},MATCH(K62,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
+        <f>IF(J62="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J62,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K62,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
     </row>
     <row r="63">
+      <c r="A63" s="12" t="n"/>
+      <c r="B63" s="12" t="n"/>
+      <c r="C63" s="12" t="n"/>
+      <c r="D63" s="12" t="n"/>
+      <c r="E63" s="12" t="n"/>
+      <c r="F63" s="12" t="n"/>
+      <c r="G63" s="12" t="n"/>
+      <c r="H63" s="20" t="n"/>
+      <c r="I63" s="20" t="n"/>
+      <c r="J63" s="9" t="n"/>
+      <c r="K63" s="12" t="n"/>
+      <c r="L63" s="9" t="n"/>
+      <c r="M63" s="9" t="n"/>
+      <c r="N63" s="9" t="n"/>
+      <c r="O63" s="9" t="n"/>
+      <c r="P63" s="9" t="n"/>
+      <c r="Q63" s="9" t="n"/>
+      <c r="R63" s="9" t="n"/>
+      <c r="S63" s="12" t="n"/>
+      <c r="T63" s="12" t="n"/>
+      <c r="U63" s="12" t="n"/>
+      <c r="V63" s="12" t="n"/>
+      <c r="W63" s="12" t="n"/>
+      <c r="X63" s="12" t="n"/>
+      <c r="Y63" s="9" t="n"/>
       <c r="Z63" s="21">
-        <f>IF(J63="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J63,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,1},MATCH(K63,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
+        <f>IF(J63="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J63,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K63,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
     </row>
     <row r="64">
+      <c r="A64" s="12" t="n"/>
+      <c r="B64" s="12" t="n"/>
+      <c r="C64" s="12" t="n"/>
+      <c r="D64" s="12" t="n"/>
+      <c r="E64" s="12" t="n"/>
+      <c r="F64" s="12" t="n"/>
+      <c r="G64" s="12" t="n"/>
+      <c r="H64" s="20" t="n"/>
+      <c r="I64" s="20" t="n"/>
+      <c r="J64" s="9" t="n"/>
+      <c r="K64" s="12" t="n"/>
+      <c r="L64" s="9" t="n"/>
+      <c r="M64" s="9" t="n"/>
+      <c r="N64" s="9" t="n"/>
+      <c r="O64" s="9" t="n"/>
+      <c r="P64" s="9" t="n"/>
+      <c r="Q64" s="9" t="n"/>
+      <c r="R64" s="9" t="n"/>
+      <c r="S64" s="12" t="n"/>
+      <c r="T64" s="12" t="n"/>
+      <c r="U64" s="12" t="n"/>
+      <c r="V64" s="12" t="n"/>
+      <c r="W64" s="12" t="n"/>
+      <c r="X64" s="12" t="n"/>
+      <c r="Y64" s="9" t="n"/>
       <c r="Z64" s="21">
-        <f>IF(J64="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J64,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,1},MATCH(K64,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
+        <f>IF(J64="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J64,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K64,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
     </row>
     <row r="65">
+      <c r="A65" s="12" t="n"/>
+      <c r="B65" s="12" t="n"/>
+      <c r="C65" s="12" t="n"/>
+      <c r="D65" s="12" t="n"/>
+      <c r="E65" s="12" t="n"/>
+      <c r="F65" s="12" t="n"/>
+      <c r="G65" s="12" t="n"/>
+      <c r="H65" s="20" t="n"/>
+      <c r="I65" s="20" t="n"/>
+      <c r="J65" s="9" t="n"/>
+      <c r="K65" s="12" t="n"/>
+      <c r="L65" s="9" t="n"/>
+      <c r="M65" s="9" t="n"/>
+      <c r="N65" s="9" t="n"/>
+      <c r="O65" s="9" t="n"/>
+      <c r="P65" s="9" t="n"/>
+      <c r="Q65" s="9" t="n"/>
+      <c r="R65" s="9" t="n"/>
+      <c r="S65" s="12" t="n"/>
+      <c r="T65" s="12" t="n"/>
+      <c r="U65" s="12" t="n"/>
+      <c r="V65" s="12" t="n"/>
+      <c r="W65" s="12" t="n"/>
+      <c r="X65" s="12" t="n"/>
+      <c r="Y65" s="9" t="n"/>
       <c r="Z65" s="21">
-        <f>IF(J65="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J65,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,1},MATCH(K65,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
+        <f>IF(J65="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J65,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K65,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
     </row>
     <row r="66">
+      <c r="A66" s="12" t="n"/>
+      <c r="B66" s="12" t="n"/>
+      <c r="C66" s="12" t="n"/>
+      <c r="D66" s="12" t="n"/>
+      <c r="E66" s="12" t="n"/>
+      <c r="F66" s="12" t="n"/>
+      <c r="G66" s="12" t="n"/>
+      <c r="H66" s="20" t="n"/>
+      <c r="I66" s="20" t="n"/>
+      <c r="J66" s="9" t="n"/>
+      <c r="K66" s="12" t="n"/>
+      <c r="L66" s="9" t="n"/>
+      <c r="M66" s="9" t="n"/>
+      <c r="N66" s="9" t="n"/>
+      <c r="O66" s="9" t="n"/>
+      <c r="P66" s="9" t="n"/>
+      <c r="Q66" s="9" t="n"/>
+      <c r="R66" s="9" t="n"/>
+      <c r="S66" s="12" t="n"/>
+      <c r="T66" s="12" t="n"/>
+      <c r="U66" s="12" t="n"/>
+      <c r="V66" s="12" t="n"/>
+      <c r="W66" s="12" t="n"/>
+      <c r="X66" s="12" t="n"/>
+      <c r="Y66" s="9" t="n"/>
       <c r="Z66" s="21">
-        <f>IF(J66="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J66,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,1},MATCH(K66,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
+        <f>IF(J66="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J66,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K66,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
     </row>
     <row r="67">
+      <c r="A67" s="12" t="n"/>
+      <c r="B67" s="12" t="n"/>
+      <c r="C67" s="12" t="n"/>
+      <c r="D67" s="12" t="n"/>
+      <c r="E67" s="12" t="n"/>
+      <c r="F67" s="12" t="n"/>
+      <c r="G67" s="12" t="n"/>
+      <c r="H67" s="20" t="n"/>
+      <c r="I67" s="20" t="n"/>
+      <c r="J67" s="9" t="n"/>
+      <c r="K67" s="12" t="n"/>
+      <c r="L67" s="9" t="n"/>
+      <c r="M67" s="9" t="n"/>
+      <c r="N67" s="9" t="n"/>
+      <c r="O67" s="9" t="n"/>
+      <c r="P67" s="9" t="n"/>
+      <c r="Q67" s="9" t="n"/>
+      <c r="R67" s="9" t="n"/>
+      <c r="S67" s="12" t="n"/>
+      <c r="T67" s="12" t="n"/>
+      <c r="U67" s="12" t="n"/>
+      <c r="V67" s="12" t="n"/>
+      <c r="W67" s="12" t="n"/>
+      <c r="X67" s="12" t="n"/>
+      <c r="Y67" s="9" t="n"/>
       <c r="Z67" s="21">
-        <f>IF(J67="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J67,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,1},MATCH(K67,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
+        <f>IF(J67="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J67,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K67,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
     </row>
     <row r="68">
+      <c r="A68" s="12" t="n"/>
+      <c r="B68" s="12" t="n"/>
+      <c r="C68" s="12" t="n"/>
+      <c r="D68" s="12" t="n"/>
+      <c r="E68" s="12" t="n"/>
+      <c r="F68" s="12" t="n"/>
+      <c r="G68" s="12" t="n"/>
+      <c r="H68" s="20" t="n"/>
+      <c r="I68" s="20" t="n"/>
+      <c r="J68" s="9" t="n"/>
+      <c r="K68" s="12" t="n"/>
+      <c r="L68" s="9" t="n"/>
+      <c r="M68" s="9" t="n"/>
+      <c r="N68" s="9" t="n"/>
+      <c r="O68" s="9" t="n"/>
+      <c r="P68" s="9" t="n"/>
+      <c r="Q68" s="9" t="n"/>
+      <c r="R68" s="9" t="n"/>
+      <c r="S68" s="12" t="n"/>
+      <c r="T68" s="12" t="n"/>
+      <c r="U68" s="12" t="n"/>
+      <c r="V68" s="12" t="n"/>
+      <c r="W68" s="12" t="n"/>
+      <c r="X68" s="12" t="n"/>
+      <c r="Y68" s="9" t="n"/>
       <c r="Z68" s="21">
-        <f>IF(J68="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J68,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,1},MATCH(K68,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
+        <f>IF(J68="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J68,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K68,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
     </row>
     <row r="69">
+      <c r="A69" s="12" t="n"/>
+      <c r="B69" s="12" t="n"/>
+      <c r="C69" s="12" t="n"/>
+      <c r="D69" s="12" t="n"/>
+      <c r="E69" s="12" t="n"/>
+      <c r="F69" s="12" t="n"/>
+      <c r="G69" s="12" t="n"/>
+      <c r="H69" s="20" t="n"/>
+      <c r="I69" s="20" t="n"/>
+      <c r="J69" s="9" t="n"/>
+      <c r="K69" s="12" t="n"/>
+      <c r="L69" s="9" t="n"/>
+      <c r="M69" s="9" t="n"/>
+      <c r="N69" s="9" t="n"/>
+      <c r="O69" s="9" t="n"/>
+      <c r="P69" s="9" t="n"/>
+      <c r="Q69" s="9" t="n"/>
+      <c r="R69" s="9" t="n"/>
+      <c r="S69" s="12" t="n"/>
+      <c r="T69" s="12" t="n"/>
+      <c r="U69" s="12" t="n"/>
+      <c r="V69" s="12" t="n"/>
+      <c r="W69" s="12" t="n"/>
+      <c r="X69" s="12" t="n"/>
+      <c r="Y69" s="9" t="n"/>
       <c r="Z69" s="21">
-        <f>IF(J69="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J69,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,1},MATCH(K69,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
+        <f>IF(J69="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J69,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K69,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
     </row>
     <row r="70">
+      <c r="A70" s="12" t="n"/>
+      <c r="B70" s="12" t="n"/>
+      <c r="C70" s="12" t="n"/>
+      <c r="D70" s="12" t="n"/>
+      <c r="E70" s="12" t="n"/>
+      <c r="F70" s="12" t="n"/>
+      <c r="G70" s="12" t="n"/>
+      <c r="H70" s="20" t="n"/>
+      <c r="I70" s="20" t="n"/>
+      <c r="J70" s="9" t="n"/>
+      <c r="K70" s="12" t="n"/>
+      <c r="L70" s="9" t="n"/>
+      <c r="M70" s="9" t="n"/>
+      <c r="N70" s="9" t="n"/>
+      <c r="O70" s="9" t="n"/>
+      <c r="P70" s="9" t="n"/>
+      <c r="Q70" s="9" t="n"/>
+      <c r="R70" s="9" t="n"/>
+      <c r="S70" s="12" t="n"/>
+      <c r="T70" s="12" t="n"/>
+      <c r="U70" s="12" t="n"/>
+      <c r="V70" s="12" t="n"/>
+      <c r="W70" s="12" t="n"/>
+      <c r="X70" s="12" t="n"/>
+      <c r="Y70" s="9" t="n"/>
       <c r="Z70" s="21">
-        <f>IF(J70="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J70,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,1},MATCH(K70,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
+        <f>IF(J70="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J70,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K70,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
     </row>
     <row r="71">
+      <c r="A71" s="12" t="n"/>
+      <c r="B71" s="12" t="n"/>
+      <c r="C71" s="12" t="n"/>
+      <c r="D71" s="12" t="n"/>
+      <c r="E71" s="12" t="n"/>
+      <c r="F71" s="12" t="n"/>
+      <c r="G71" s="12" t="n"/>
+      <c r="H71" s="20" t="n"/>
+      <c r="I71" s="20" t="n"/>
+      <c r="J71" s="9" t="n"/>
+      <c r="K71" s="12" t="n"/>
+      <c r="L71" s="9" t="n"/>
+      <c r="M71" s="9" t="n"/>
+      <c r="N71" s="9" t="n"/>
+      <c r="O71" s="9" t="n"/>
+      <c r="P71" s="9" t="n"/>
+      <c r="Q71" s="9" t="n"/>
+      <c r="R71" s="9" t="n"/>
+      <c r="S71" s="12" t="n"/>
+      <c r="T71" s="12" t="n"/>
+      <c r="U71" s="12" t="n"/>
+      <c r="V71" s="12" t="n"/>
+      <c r="W71" s="12" t="n"/>
+      <c r="X71" s="12" t="n"/>
+      <c r="Y71" s="9" t="n"/>
       <c r="Z71" s="21">
-        <f>IF(J71="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J71,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,1},MATCH(K71,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
+        <f>IF(J71="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J71,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K71,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
     </row>
     <row r="72">
+      <c r="A72" s="12" t="n"/>
+      <c r="B72" s="12" t="n"/>
+      <c r="C72" s="12" t="n"/>
+      <c r="D72" s="12" t="n"/>
+      <c r="E72" s="12" t="n"/>
+      <c r="F72" s="12" t="n"/>
+      <c r="G72" s="12" t="n"/>
+      <c r="H72" s="20" t="n"/>
+      <c r="I72" s="20" t="n"/>
+      <c r="J72" s="9" t="n"/>
+      <c r="K72" s="12" t="n"/>
+      <c r="L72" s="9" t="n"/>
+      <c r="M72" s="9" t="n"/>
+      <c r="N72" s="9" t="n"/>
+      <c r="O72" s="9" t="n"/>
+      <c r="P72" s="9" t="n"/>
+      <c r="Q72" s="9" t="n"/>
+      <c r="R72" s="9" t="n"/>
+      <c r="S72" s="12" t="n"/>
+      <c r="T72" s="12" t="n"/>
+      <c r="U72" s="12" t="n"/>
+      <c r="V72" s="12" t="n"/>
+      <c r="W72" s="12" t="n"/>
+      <c r="X72" s="12" t="n"/>
+      <c r="Y72" s="9" t="n"/>
       <c r="Z72" s="21">
-        <f>IF(J72="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J72,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,1},MATCH(K72,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
+        <f>IF(J72="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J72,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K72,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
     </row>
     <row r="73">
+      <c r="A73" s="12" t="n"/>
+      <c r="B73" s="12" t="n"/>
+      <c r="C73" s="12" t="n"/>
+      <c r="D73" s="12" t="n"/>
+      <c r="E73" s="12" t="n"/>
+      <c r="F73" s="12" t="n"/>
+      <c r="G73" s="12" t="n"/>
+      <c r="H73" s="20" t="n"/>
+      <c r="I73" s="20" t="n"/>
+      <c r="J73" s="9" t="n"/>
+      <c r="K73" s="12" t="n"/>
+      <c r="L73" s="9" t="n"/>
+      <c r="M73" s="9" t="n"/>
+      <c r="N73" s="9" t="n"/>
+      <c r="O73" s="9" t="n"/>
+      <c r="P73" s="9" t="n"/>
+      <c r="Q73" s="9" t="n"/>
+      <c r="R73" s="9" t="n"/>
+      <c r="S73" s="12" t="n"/>
+      <c r="T73" s="12" t="n"/>
+      <c r="U73" s="12" t="n"/>
+      <c r="V73" s="12" t="n"/>
+      <c r="W73" s="12" t="n"/>
+      <c r="X73" s="12" t="n"/>
+      <c r="Y73" s="9" t="n"/>
       <c r="Z73" s="21">
-        <f>IF(J73="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J73,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,1},MATCH(K73,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
+        <f>IF(J73="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J73,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K73,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
     </row>
     <row r="74">
+      <c r="A74" s="12" t="n"/>
+      <c r="B74" s="12" t="n"/>
+      <c r="C74" s="12" t="n"/>
+      <c r="D74" s="12" t="n"/>
+      <c r="E74" s="12" t="n"/>
+      <c r="F74" s="12" t="n"/>
+      <c r="G74" s="12" t="n"/>
+      <c r="H74" s="20" t="n"/>
+      <c r="I74" s="20" t="n"/>
+      <c r="J74" s="9" t="n"/>
+      <c r="K74" s="12" t="n"/>
+      <c r="L74" s="9" t="n"/>
+      <c r="M74" s="9" t="n"/>
+      <c r="N74" s="9" t="n"/>
+      <c r="O74" s="9" t="n"/>
+      <c r="P74" s="9" t="n"/>
+      <c r="Q74" s="9" t="n"/>
+      <c r="R74" s="9" t="n"/>
+      <c r="S74" s="12" t="n"/>
+      <c r="T74" s="12" t="n"/>
+      <c r="U74" s="12" t="n"/>
+      <c r="V74" s="12" t="n"/>
+      <c r="W74" s="12" t="n"/>
+      <c r="X74" s="12" t="n"/>
+      <c r="Y74" s="9" t="n"/>
       <c r="Z74" s="21">
-        <f>IF(J74="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J74,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,1},MATCH(K74,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
+        <f>IF(J74="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J74,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K74,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
     </row>
     <row r="75">
+      <c r="A75" s="12" t="n"/>
+      <c r="B75" s="12" t="n"/>
+      <c r="C75" s="12" t="n"/>
+      <c r="D75" s="12" t="n"/>
+      <c r="E75" s="12" t="n"/>
+      <c r="F75" s="12" t="n"/>
+      <c r="G75" s="12" t="n"/>
+      <c r="H75" s="20" t="n"/>
+      <c r="I75" s="20" t="n"/>
+      <c r="J75" s="9" t="n"/>
+      <c r="K75" s="12" t="n"/>
+      <c r="L75" s="9" t="n"/>
+      <c r="M75" s="9" t="n"/>
+      <c r="N75" s="9" t="n"/>
+      <c r="O75" s="9" t="n"/>
+      <c r="P75" s="9" t="n"/>
+      <c r="Q75" s="9" t="n"/>
+      <c r="R75" s="9" t="n"/>
+      <c r="S75" s="12" t="n"/>
+      <c r="T75" s="12" t="n"/>
+      <c r="U75" s="12" t="n"/>
+      <c r="V75" s="12" t="n"/>
+      <c r="W75" s="12" t="n"/>
+      <c r="X75" s="12" t="n"/>
+      <c r="Y75" s="9" t="n"/>
       <c r="Z75" s="21">
-        <f>IF(J75="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J75,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,1},MATCH(K75,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
+        <f>IF(J75="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J75,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K75,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
     </row>
     <row r="76">
+      <c r="A76" s="12" t="n"/>
+      <c r="B76" s="12" t="n"/>
+      <c r="C76" s="12" t="n"/>
+      <c r="D76" s="12" t="n"/>
+      <c r="E76" s="12" t="n"/>
+      <c r="F76" s="12" t="n"/>
+      <c r="G76" s="12" t="n"/>
+      <c r="H76" s="20" t="n"/>
+      <c r="I76" s="20" t="n"/>
+      <c r="J76" s="9" t="n"/>
+      <c r="K76" s="12" t="n"/>
+      <c r="L76" s="9" t="n"/>
+      <c r="M76" s="9" t="n"/>
+      <c r="N76" s="9" t="n"/>
+      <c r="O76" s="9" t="n"/>
+      <c r="P76" s="9" t="n"/>
+      <c r="Q76" s="9" t="n"/>
+      <c r="R76" s="9" t="n"/>
+      <c r="S76" s="12" t="n"/>
+      <c r="T76" s="12" t="n"/>
+      <c r="U76" s="12" t="n"/>
+      <c r="V76" s="12" t="n"/>
+      <c r="W76" s="12" t="n"/>
+      <c r="X76" s="12" t="n"/>
+      <c r="Y76" s="9" t="n"/>
       <c r="Z76" s="21">
-        <f>IF(J76="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J76,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,1},MATCH(K76,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
+        <f>IF(J76="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J76,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K76,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
     </row>
     <row r="77">
+      <c r="A77" s="12" t="n"/>
+      <c r="B77" s="12" t="n"/>
+      <c r="C77" s="12" t="n"/>
+      <c r="D77" s="12" t="n"/>
+      <c r="E77" s="12" t="n"/>
+      <c r="F77" s="12" t="n"/>
+      <c r="G77" s="12" t="n"/>
+      <c r="H77" s="20" t="n"/>
+      <c r="I77" s="20" t="n"/>
+      <c r="J77" s="9" t="n"/>
+      <c r="K77" s="12" t="n"/>
+      <c r="L77" s="9" t="n"/>
+      <c r="M77" s="9" t="n"/>
+      <c r="N77" s="9" t="n"/>
+      <c r="O77" s="9" t="n"/>
+      <c r="P77" s="9" t="n"/>
+      <c r="Q77" s="9" t="n"/>
+      <c r="R77" s="9" t="n"/>
+      <c r="S77" s="12" t="n"/>
+      <c r="T77" s="12" t="n"/>
+      <c r="U77" s="12" t="n"/>
+      <c r="V77" s="12" t="n"/>
+      <c r="W77" s="12" t="n"/>
+      <c r="X77" s="12" t="n"/>
+      <c r="Y77" s="9" t="n"/>
       <c r="Z77" s="21">
-        <f>IF(J77="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J77,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,1},MATCH(K77,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
+        <f>IF(J77="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J77,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K77,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
     </row>
     <row r="78">
+      <c r="A78" s="12" t="n"/>
+      <c r="B78" s="12" t="n"/>
+      <c r="C78" s="12" t="n"/>
+      <c r="D78" s="12" t="n"/>
+      <c r="E78" s="12" t="n"/>
+      <c r="F78" s="12" t="n"/>
+      <c r="G78" s="12" t="n"/>
+      <c r="H78" s="20" t="n"/>
+      <c r="I78" s="20" t="n"/>
+      <c r="J78" s="9" t="n"/>
+      <c r="K78" s="12" t="n"/>
+      <c r="L78" s="9" t="n"/>
+      <c r="M78" s="9" t="n"/>
+      <c r="N78" s="9" t="n"/>
+      <c r="O78" s="9" t="n"/>
+      <c r="P78" s="9" t="n"/>
+      <c r="Q78" s="9" t="n"/>
+      <c r="R78" s="9" t="n"/>
+      <c r="S78" s="12" t="n"/>
+      <c r="T78" s="12" t="n"/>
+      <c r="U78" s="12" t="n"/>
+      <c r="V78" s="12" t="n"/>
+      <c r="W78" s="12" t="n"/>
+      <c r="X78" s="12" t="n"/>
+      <c r="Y78" s="9" t="n"/>
       <c r="Z78" s="21">
-        <f>IF(J78="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J78,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,1},MATCH(K78,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
+        <f>IF(J78="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J78,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K78,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
     </row>
     <row r="79">
+      <c r="A79" s="12" t="n"/>
+      <c r="B79" s="12" t="n"/>
+      <c r="C79" s="12" t="n"/>
+      <c r="D79" s="12" t="n"/>
+      <c r="E79" s="12" t="n"/>
+      <c r="F79" s="12" t="n"/>
+      <c r="G79" s="12" t="n"/>
+      <c r="H79" s="20" t="n"/>
+      <c r="I79" s="20" t="n"/>
+      <c r="J79" s="9" t="n"/>
+      <c r="K79" s="12" t="n"/>
+      <c r="L79" s="9" t="n"/>
+      <c r="M79" s="9" t="n"/>
+      <c r="N79" s="9" t="n"/>
+      <c r="O79" s="9" t="n"/>
+      <c r="P79" s="9" t="n"/>
+      <c r="Q79" s="9" t="n"/>
+      <c r="R79" s="9" t="n"/>
+      <c r="S79" s="12" t="n"/>
+      <c r="T79" s="12" t="n"/>
+      <c r="U79" s="12" t="n"/>
+      <c r="V79" s="12" t="n"/>
+      <c r="W79" s="12" t="n"/>
+      <c r="X79" s="12" t="n"/>
+      <c r="Y79" s="9" t="n"/>
       <c r="Z79" s="21">
-        <f>IF(J79="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J79,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,1},MATCH(K79,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
+        <f>IF(J79="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J79,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K79,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
     </row>
     <row r="80">
+      <c r="A80" s="12" t="n"/>
+      <c r="B80" s="12" t="n"/>
+      <c r="C80" s="12" t="n"/>
+      <c r="D80" s="12" t="n"/>
+      <c r="E80" s="12" t="n"/>
+      <c r="F80" s="12" t="n"/>
+      <c r="G80" s="12" t="n"/>
+      <c r="H80" s="20" t="n"/>
+      <c r="I80" s="20" t="n"/>
+      <c r="J80" s="9" t="n"/>
+      <c r="K80" s="12" t="n"/>
+      <c r="L80" s="9" t="n"/>
+      <c r="M80" s="9" t="n"/>
+      <c r="N80" s="9" t="n"/>
+      <c r="O80" s="9" t="n"/>
+      <c r="P80" s="9" t="n"/>
+      <c r="Q80" s="9" t="n"/>
+      <c r="R80" s="9" t="n"/>
+      <c r="S80" s="12" t="n"/>
+      <c r="T80" s="12" t="n"/>
+      <c r="U80" s="12" t="n"/>
+      <c r="V80" s="12" t="n"/>
+      <c r="W80" s="12" t="n"/>
+      <c r="X80" s="12" t="n"/>
+      <c r="Y80" s="9" t="n"/>
       <c r="Z80" s="21">
-        <f>IF(J80="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J80,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,1},MATCH(K80,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
+        <f>IF(J80="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J80,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K80,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
     </row>
     <row r="81">
+      <c r="A81" s="12" t="n"/>
+      <c r="B81" s="12" t="n"/>
+      <c r="C81" s="12" t="n"/>
+      <c r="D81" s="12" t="n"/>
+      <c r="E81" s="12" t="n"/>
+      <c r="F81" s="12" t="n"/>
+      <c r="G81" s="12" t="n"/>
+      <c r="H81" s="20" t="n"/>
+      <c r="I81" s="20" t="n"/>
+      <c r="J81" s="9" t="n"/>
+      <c r="K81" s="12" t="n"/>
+      <c r="L81" s="9" t="n"/>
+      <c r="M81" s="9" t="n"/>
+      <c r="N81" s="9" t="n"/>
+      <c r="O81" s="9" t="n"/>
+      <c r="P81" s="9" t="n"/>
+      <c r="Q81" s="9" t="n"/>
+      <c r="R81" s="9" t="n"/>
+      <c r="S81" s="12" t="n"/>
+      <c r="T81" s="12" t="n"/>
+      <c r="U81" s="12" t="n"/>
+      <c r="V81" s="12" t="n"/>
+      <c r="W81" s="12" t="n"/>
+      <c r="X81" s="12" t="n"/>
+      <c r="Y81" s="9" t="n"/>
       <c r="Z81" s="21">
-        <f>IF(J81="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J81,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,1},MATCH(K81,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
+        <f>IF(J81="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J81,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K81,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
     </row>
     <row r="82">
+      <c r="A82" s="12" t="n"/>
+      <c r="B82" s="12" t="n"/>
+      <c r="C82" s="12" t="n"/>
+      <c r="D82" s="12" t="n"/>
+      <c r="E82" s="12" t="n"/>
+      <c r="F82" s="12" t="n"/>
+      <c r="G82" s="12" t="n"/>
+      <c r="H82" s="20" t="n"/>
+      <c r="I82" s="20" t="n"/>
+      <c r="J82" s="9" t="n"/>
+      <c r="K82" s="12" t="n"/>
+      <c r="L82" s="9" t="n"/>
+      <c r="M82" s="9" t="n"/>
+      <c r="N82" s="9" t="n"/>
+      <c r="O82" s="9" t="n"/>
+      <c r="P82" s="9" t="n"/>
+      <c r="Q82" s="9" t="n"/>
+      <c r="R82" s="9" t="n"/>
+      <c r="S82" s="12" t="n"/>
+      <c r="T82" s="12" t="n"/>
+      <c r="U82" s="12" t="n"/>
+      <c r="V82" s="12" t="n"/>
+      <c r="W82" s="12" t="n"/>
+      <c r="X82" s="12" t="n"/>
+      <c r="Y82" s="9" t="n"/>
       <c r="Z82" s="21">
-        <f>IF(J82="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J82,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,1},MATCH(K82,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
+        <f>IF(J82="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J82,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K82,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
     </row>
     <row r="83">
+      <c r="A83" s="12" t="n"/>
+      <c r="B83" s="12" t="n"/>
+      <c r="C83" s="12" t="n"/>
+      <c r="D83" s="12" t="n"/>
+      <c r="E83" s="12" t="n"/>
+      <c r="F83" s="12" t="n"/>
+      <c r="G83" s="12" t="n"/>
+      <c r="H83" s="20" t="n"/>
+      <c r="I83" s="20" t="n"/>
+      <c r="J83" s="9" t="n"/>
+      <c r="K83" s="12" t="n"/>
+      <c r="L83" s="9" t="n"/>
+      <c r="M83" s="9" t="n"/>
+      <c r="N83" s="9" t="n"/>
+      <c r="O83" s="9" t="n"/>
+      <c r="P83" s="9" t="n"/>
+      <c r="Q83" s="9" t="n"/>
+      <c r="R83" s="9" t="n"/>
+      <c r="S83" s="12" t="n"/>
+      <c r="T83" s="12" t="n"/>
+      <c r="U83" s="12" t="n"/>
+      <c r="V83" s="12" t="n"/>
+      <c r="W83" s="12" t="n"/>
+      <c r="X83" s="12" t="n"/>
+      <c r="Y83" s="9" t="n"/>
       <c r="Z83" s="21">
-        <f>IF(J83="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J83,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,1},MATCH(K83,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
+        <f>IF(J83="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J83,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K83,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
     </row>
     <row r="84">
+      <c r="A84" s="12" t="n"/>
+      <c r="B84" s="12" t="n"/>
+      <c r="C84" s="12" t="n"/>
+      <c r="D84" s="12" t="n"/>
+      <c r="E84" s="12" t="n"/>
+      <c r="F84" s="12" t="n"/>
+      <c r="G84" s="12" t="n"/>
+      <c r="H84" s="20" t="n"/>
+      <c r="I84" s="20" t="n"/>
+      <c r="J84" s="9" t="n"/>
+      <c r="K84" s="12" t="n"/>
+      <c r="L84" s="9" t="n"/>
+      <c r="M84" s="9" t="n"/>
+      <c r="N84" s="9" t="n"/>
+      <c r="O84" s="9" t="n"/>
+      <c r="P84" s="9" t="n"/>
+      <c r="Q84" s="9" t="n"/>
+      <c r="R84" s="9" t="n"/>
+      <c r="S84" s="12" t="n"/>
+      <c r="T84" s="12" t="n"/>
+      <c r="U84" s="12" t="n"/>
+      <c r="V84" s="12" t="n"/>
+      <c r="W84" s="12" t="n"/>
+      <c r="X84" s="12" t="n"/>
+      <c r="Y84" s="9" t="n"/>
       <c r="Z84" s="21">
-        <f>IF(J84="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J84,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,1},MATCH(K84,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
+        <f>IF(J84="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J84,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K84,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
     </row>
     <row r="85">
+      <c r="A85" s="12" t="n"/>
+      <c r="B85" s="12" t="n"/>
+      <c r="C85" s="12" t="n"/>
+      <c r="D85" s="12" t="n"/>
+      <c r="E85" s="12" t="n"/>
+      <c r="F85" s="12" t="n"/>
+      <c r="G85" s="12" t="n"/>
+      <c r="H85" s="20" t="n"/>
+      <c r="I85" s="20" t="n"/>
+      <c r="J85" s="9" t="n"/>
+      <c r="K85" s="12" t="n"/>
+      <c r="L85" s="9" t="n"/>
+      <c r="M85" s="9" t="n"/>
+      <c r="N85" s="9" t="n"/>
+      <c r="O85" s="9" t="n"/>
+      <c r="P85" s="9" t="n"/>
+      <c r="Q85" s="9" t="n"/>
+      <c r="R85" s="9" t="n"/>
+      <c r="S85" s="12" t="n"/>
+      <c r="T85" s="12" t="n"/>
+      <c r="U85" s="12" t="n"/>
+      <c r="V85" s="12" t="n"/>
+      <c r="W85" s="12" t="n"/>
+      <c r="X85" s="12" t="n"/>
+      <c r="Y85" s="9" t="n"/>
       <c r="Z85" s="21">
-        <f>IF(J85="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J85,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,1},MATCH(K85,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
+        <f>IF(J85="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J85,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K85,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
     </row>
     <row r="86">
+      <c r="A86" s="12" t="n"/>
+      <c r="B86" s="12" t="n"/>
+      <c r="C86" s="12" t="n"/>
+      <c r="D86" s="12" t="n"/>
+      <c r="E86" s="12" t="n"/>
+      <c r="F86" s="12" t="n"/>
+      <c r="G86" s="12" t="n"/>
+      <c r="H86" s="20" t="n"/>
+      <c r="I86" s="20" t="n"/>
+      <c r="J86" s="9" t="n"/>
+      <c r="K86" s="12" t="n"/>
+      <c r="L86" s="9" t="n"/>
+      <c r="M86" s="9" t="n"/>
+      <c r="N86" s="9" t="n"/>
+      <c r="O86" s="9" t="n"/>
+      <c r="P86" s="9" t="n"/>
+      <c r="Q86" s="9" t="n"/>
+      <c r="R86" s="9" t="n"/>
+      <c r="S86" s="12" t="n"/>
+      <c r="T86" s="12" t="n"/>
+      <c r="U86" s="12" t="n"/>
+      <c r="V86" s="12" t="n"/>
+      <c r="W86" s="12" t="n"/>
+      <c r="X86" s="12" t="n"/>
+      <c r="Y86" s="9" t="n"/>
       <c r="Z86" s="21">
-        <f>IF(J86="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J86,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,1},MATCH(K86,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
+        <f>IF(J86="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J86,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K86,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
     </row>
     <row r="87">
+      <c r="A87" s="12" t="n"/>
+      <c r="B87" s="12" t="n"/>
+      <c r="C87" s="12" t="n"/>
+      <c r="D87" s="12" t="n"/>
+      <c r="E87" s="12" t="n"/>
+      <c r="F87" s="12" t="n"/>
+      <c r="G87" s="12" t="n"/>
+      <c r="H87" s="20" t="n"/>
+      <c r="I87" s="20" t="n"/>
+      <c r="J87" s="9" t="n"/>
+      <c r="K87" s="12" t="n"/>
+      <c r="L87" s="9" t="n"/>
+      <c r="M87" s="9" t="n"/>
+      <c r="N87" s="9" t="n"/>
+      <c r="O87" s="9" t="n"/>
+      <c r="P87" s="9" t="n"/>
+      <c r="Q87" s="9" t="n"/>
+      <c r="R87" s="9" t="n"/>
+      <c r="S87" s="12" t="n"/>
+      <c r="T87" s="12" t="n"/>
+      <c r="U87" s="12" t="n"/>
+      <c r="V87" s="12" t="n"/>
+      <c r="W87" s="12" t="n"/>
+      <c r="X87" s="12" t="n"/>
+      <c r="Y87" s="9" t="n"/>
       <c r="Z87" s="21">
-        <f>IF(J87="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J87,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,1},MATCH(K87,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
+        <f>IF(J87="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J87,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K87,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
     </row>
     <row r="88">
+      <c r="A88" s="12" t="n"/>
+      <c r="B88" s="12" t="n"/>
+      <c r="C88" s="12" t="n"/>
+      <c r="D88" s="12" t="n"/>
+      <c r="E88" s="12" t="n"/>
+      <c r="F88" s="12" t="n"/>
+      <c r="G88" s="12" t="n"/>
+      <c r="H88" s="20" t="n"/>
+      <c r="I88" s="20" t="n"/>
+      <c r="J88" s="9" t="n"/>
+      <c r="K88" s="12" t="n"/>
+      <c r="L88" s="9" t="n"/>
+      <c r="M88" s="9" t="n"/>
+      <c r="N88" s="9" t="n"/>
+      <c r="O88" s="9" t="n"/>
+      <c r="P88" s="9" t="n"/>
+      <c r="Q88" s="9" t="n"/>
+      <c r="R88" s="9" t="n"/>
+      <c r="S88" s="12" t="n"/>
+      <c r="T88" s="12" t="n"/>
+      <c r="U88" s="12" t="n"/>
+      <c r="V88" s="12" t="n"/>
+      <c r="W88" s="12" t="n"/>
+      <c r="X88" s="12" t="n"/>
+      <c r="Y88" s="9" t="n"/>
       <c r="Z88" s="21">
-        <f>IF(J88="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J88,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,1},MATCH(K88,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
+        <f>IF(J88="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J88,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K88,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
     </row>
     <row r="89">
+      <c r="A89" s="12" t="n"/>
+      <c r="B89" s="12" t="n"/>
+      <c r="C89" s="12" t="n"/>
+      <c r="D89" s="12" t="n"/>
+      <c r="E89" s="12" t="n"/>
+      <c r="F89" s="12" t="n"/>
+      <c r="G89" s="12" t="n"/>
+      <c r="H89" s="20" t="n"/>
+      <c r="I89" s="20" t="n"/>
+      <c r="J89" s="9" t="n"/>
+      <c r="K89" s="12" t="n"/>
+      <c r="L89" s="9" t="n"/>
+      <c r="M89" s="9" t="n"/>
+      <c r="N89" s="9" t="n"/>
+      <c r="O89" s="9" t="n"/>
+      <c r="P89" s="9" t="n"/>
+      <c r="Q89" s="9" t="n"/>
+      <c r="R89" s="9" t="n"/>
+      <c r="S89" s="12" t="n"/>
+      <c r="T89" s="12" t="n"/>
+      <c r="U89" s="12" t="n"/>
+      <c r="V89" s="12" t="n"/>
+      <c r="W89" s="12" t="n"/>
+      <c r="X89" s="12" t="n"/>
+      <c r="Y89" s="9" t="n"/>
       <c r="Z89" s="21">
-        <f>IF(J89="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J89,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,1},MATCH(K89,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
+        <f>IF(J89="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J89,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K89,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
     </row>
     <row r="90">
+      <c r="A90" s="12" t="n"/>
+      <c r="B90" s="12" t="n"/>
+      <c r="C90" s="12" t="n"/>
+      <c r="D90" s="12" t="n"/>
+      <c r="E90" s="12" t="n"/>
+      <c r="F90" s="12" t="n"/>
+      <c r="G90" s="12" t="n"/>
+      <c r="H90" s="20" t="n"/>
+      <c r="I90" s="20" t="n"/>
+      <c r="J90" s="9" t="n"/>
+      <c r="K90" s="12" t="n"/>
+      <c r="L90" s="9" t="n"/>
+      <c r="M90" s="9" t="n"/>
+      <c r="N90" s="9" t="n"/>
+      <c r="O90" s="9" t="n"/>
+      <c r="P90" s="9" t="n"/>
+      <c r="Q90" s="9" t="n"/>
+      <c r="R90" s="9" t="n"/>
+      <c r="S90" s="12" t="n"/>
+      <c r="T90" s="12" t="n"/>
+      <c r="U90" s="12" t="n"/>
+      <c r="V90" s="12" t="n"/>
+      <c r="W90" s="12" t="n"/>
+      <c r="X90" s="12" t="n"/>
+      <c r="Y90" s="9" t="n"/>
       <c r="Z90" s="21">
-        <f>IF(J90="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J90,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,1},MATCH(K90,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
+        <f>IF(J90="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J90,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K90,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
     </row>
     <row r="91">
+      <c r="A91" s="12" t="n"/>
+      <c r="B91" s="12" t="n"/>
+      <c r="C91" s="12" t="n"/>
+      <c r="D91" s="12" t="n"/>
+      <c r="E91" s="12" t="n"/>
+      <c r="F91" s="12" t="n"/>
+      <c r="G91" s="12" t="n"/>
+      <c r="H91" s="20" t="n"/>
+      <c r="I91" s="20" t="n"/>
+      <c r="J91" s="9" t="n"/>
+      <c r="K91" s="12" t="n"/>
+      <c r="L91" s="9" t="n"/>
+      <c r="M91" s="9" t="n"/>
+      <c r="N91" s="9" t="n"/>
+      <c r="O91" s="9" t="n"/>
+      <c r="P91" s="9" t="n"/>
+      <c r="Q91" s="9" t="n"/>
+      <c r="R91" s="9" t="n"/>
+      <c r="S91" s="12" t="n"/>
+      <c r="T91" s="12" t="n"/>
+      <c r="U91" s="12" t="n"/>
+      <c r="V91" s="12" t="n"/>
+      <c r="W91" s="12" t="n"/>
+      <c r="X91" s="12" t="n"/>
+      <c r="Y91" s="9" t="n"/>
       <c r="Z91" s="21">
-        <f>IF(J91="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J91,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,1},MATCH(K91,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
+        <f>IF(J91="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J91,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K91,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
     </row>
     <row r="92">
+      <c r="A92" s="12" t="n"/>
+      <c r="B92" s="12" t="n"/>
+      <c r="C92" s="12" t="n"/>
+      <c r="D92" s="12" t="n"/>
+      <c r="E92" s="12" t="n"/>
+      <c r="F92" s="12" t="n"/>
+      <c r="G92" s="12" t="n"/>
+      <c r="H92" s="20" t="n"/>
+      <c r="I92" s="20" t="n"/>
+      <c r="J92" s="9" t="n"/>
+      <c r="K92" s="12" t="n"/>
+      <c r="L92" s="9" t="n"/>
+      <c r="M92" s="9" t="n"/>
+      <c r="N92" s="9" t="n"/>
+      <c r="O92" s="9" t="n"/>
+      <c r="P92" s="9" t="n"/>
+      <c r="Q92" s="9" t="n"/>
+      <c r="R92" s="9" t="n"/>
+      <c r="S92" s="12" t="n"/>
+      <c r="T92" s="12" t="n"/>
+      <c r="U92" s="12" t="n"/>
+      <c r="V92" s="12" t="n"/>
+      <c r="W92" s="12" t="n"/>
+      <c r="X92" s="12" t="n"/>
+      <c r="Y92" s="9" t="n"/>
       <c r="Z92" s="21">
-        <f>IF(J92="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J92,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,1},MATCH(K92,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
+        <f>IF(J92="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J92,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K92,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
     </row>
     <row r="93">
+      <c r="A93" s="12" t="n"/>
+      <c r="B93" s="12" t="n"/>
+      <c r="C93" s="12" t="n"/>
+      <c r="D93" s="12" t="n"/>
+      <c r="E93" s="12" t="n"/>
+      <c r="F93" s="12" t="n"/>
+      <c r="G93" s="12" t="n"/>
+      <c r="H93" s="20" t="n"/>
+      <c r="I93" s="20" t="n"/>
+      <c r="J93" s="9" t="n"/>
+      <c r="K93" s="12" t="n"/>
+      <c r="L93" s="9" t="n"/>
+      <c r="M93" s="9" t="n"/>
+      <c r="N93" s="9" t="n"/>
+      <c r="O93" s="9" t="n"/>
+      <c r="P93" s="9" t="n"/>
+      <c r="Q93" s="9" t="n"/>
+      <c r="R93" s="9" t="n"/>
+      <c r="S93" s="12" t="n"/>
+      <c r="T93" s="12" t="n"/>
+      <c r="U93" s="12" t="n"/>
+      <c r="V93" s="12" t="n"/>
+      <c r="W93" s="12" t="n"/>
+      <c r="X93" s="12" t="n"/>
+      <c r="Y93" s="9" t="n"/>
       <c r="Z93" s="21">
-        <f>IF(J93="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J93,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,1},MATCH(K93,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
+        <f>IF(J93="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J93,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K93,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
     </row>
     <row r="94">
+      <c r="A94" s="12" t="n"/>
+      <c r="B94" s="12" t="n"/>
+      <c r="C94" s="12" t="n"/>
+      <c r="D94" s="12" t="n"/>
+      <c r="E94" s="12" t="n"/>
+      <c r="F94" s="12" t="n"/>
+      <c r="G94" s="12" t="n"/>
+      <c r="H94" s="20" t="n"/>
+      <c r="I94" s="20" t="n"/>
+      <c r="J94" s="9" t="n"/>
+      <c r="K94" s="12" t="n"/>
+      <c r="L94" s="9" t="n"/>
+      <c r="M94" s="9" t="n"/>
+      <c r="N94" s="9" t="n"/>
+      <c r="O94" s="9" t="n"/>
+      <c r="P94" s="9" t="n"/>
+      <c r="Q94" s="9" t="n"/>
+      <c r="R94" s="9" t="n"/>
+      <c r="S94" s="12" t="n"/>
+      <c r="T94" s="12" t="n"/>
+      <c r="U94" s="12" t="n"/>
+      <c r="V94" s="12" t="n"/>
+      <c r="W94" s="12" t="n"/>
+      <c r="X94" s="12" t="n"/>
+      <c r="Y94" s="9" t="n"/>
       <c r="Z94" s="21">
-        <f>IF(J94="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J94,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,1},MATCH(K94,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
+        <f>IF(J94="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J94,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K94,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
     </row>
     <row r="95">
+      <c r="A95" s="12" t="n"/>
+      <c r="B95" s="12" t="n"/>
+      <c r="C95" s="12" t="n"/>
+      <c r="D95" s="12" t="n"/>
+      <c r="E95" s="12" t="n"/>
+      <c r="F95" s="12" t="n"/>
+      <c r="G95" s="12" t="n"/>
+      <c r="H95" s="20" t="n"/>
+      <c r="I95" s="20" t="n"/>
+      <c r="J95" s="9" t="n"/>
+      <c r="K95" s="12" t="n"/>
+      <c r="L95" s="9" t="n"/>
+      <c r="M95" s="9" t="n"/>
+      <c r="N95" s="9" t="n"/>
+      <c r="O95" s="9" t="n"/>
+      <c r="P95" s="9" t="n"/>
+      <c r="Q95" s="9" t="n"/>
+      <c r="R95" s="9" t="n"/>
+      <c r="S95" s="12" t="n"/>
+      <c r="T95" s="12" t="n"/>
+      <c r="U95" s="12" t="n"/>
+      <c r="V95" s="12" t="n"/>
+      <c r="W95" s="12" t="n"/>
+      <c r="X95" s="12" t="n"/>
+      <c r="Y95" s="9" t="n"/>
       <c r="Z95" s="21">
-        <f>IF(J95="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J95,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,1},MATCH(K95,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
+        <f>IF(J95="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J95,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K95,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
     </row>
     <row r="96">
+      <c r="A96" s="12" t="n"/>
+      <c r="B96" s="12" t="n"/>
+      <c r="C96" s="12" t="n"/>
+      <c r="D96" s="12" t="n"/>
+      <c r="E96" s="12" t="n"/>
+      <c r="F96" s="12" t="n"/>
+      <c r="G96" s="12" t="n"/>
+      <c r="H96" s="20" t="n"/>
+      <c r="I96" s="20" t="n"/>
+      <c r="J96" s="9" t="n"/>
+      <c r="K96" s="12" t="n"/>
+      <c r="L96" s="9" t="n"/>
+      <c r="M96" s="9" t="n"/>
+      <c r="N96" s="9" t="n"/>
+      <c r="O96" s="9" t="n"/>
+      <c r="P96" s="9" t="n"/>
+      <c r="Q96" s="9" t="n"/>
+      <c r="R96" s="9" t="n"/>
+      <c r="S96" s="12" t="n"/>
+      <c r="T96" s="12" t="n"/>
+      <c r="U96" s="12" t="n"/>
+      <c r="V96" s="12" t="n"/>
+      <c r="W96" s="12" t="n"/>
+      <c r="X96" s="12" t="n"/>
+      <c r="Y96" s="9" t="n"/>
       <c r="Z96" s="21">
-        <f>IF(J96="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J96,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,1},MATCH(K96,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
+        <f>IF(J96="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J96,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K96,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
     </row>
     <row r="97">
+      <c r="A97" s="12" t="n"/>
+      <c r="B97" s="12" t="n"/>
+      <c r="C97" s="12" t="n"/>
+      <c r="D97" s="12" t="n"/>
+      <c r="E97" s="12" t="n"/>
+      <c r="F97" s="12" t="n"/>
+      <c r="G97" s="12" t="n"/>
+      <c r="H97" s="20" t="n"/>
+      <c r="I97" s="20" t="n"/>
+      <c r="J97" s="9" t="n"/>
+      <c r="K97" s="12" t="n"/>
+      <c r="L97" s="9" t="n"/>
+      <c r="M97" s="9" t="n"/>
+      <c r="N97" s="9" t="n"/>
+      <c r="O97" s="9" t="n"/>
+      <c r="P97" s="9" t="n"/>
+      <c r="Q97" s="9" t="n"/>
+      <c r="R97" s="9" t="n"/>
+      <c r="S97" s="12" t="n"/>
+      <c r="T97" s="12" t="n"/>
+      <c r="U97" s="12" t="n"/>
+      <c r="V97" s="12" t="n"/>
+      <c r="W97" s="12" t="n"/>
+      <c r="X97" s="12" t="n"/>
+      <c r="Y97" s="9" t="n"/>
       <c r="Z97" s="21">
-        <f>IF(J97="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J97,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,1},MATCH(K97,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
+        <f>IF(J97="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J97,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K97,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
     </row>
     <row r="98">
+      <c r="A98" s="12" t="n"/>
+      <c r="B98" s="12" t="n"/>
+      <c r="C98" s="12" t="n"/>
+      <c r="D98" s="12" t="n"/>
+      <c r="E98" s="12" t="n"/>
+      <c r="F98" s="12" t="n"/>
+      <c r="G98" s="12" t="n"/>
+      <c r="H98" s="20" t="n"/>
+      <c r="I98" s="20" t="n"/>
+      <c r="J98" s="9" t="n"/>
+      <c r="K98" s="12" t="n"/>
+      <c r="L98" s="9" t="n"/>
+      <c r="M98" s="9" t="n"/>
+      <c r="N98" s="9" t="n"/>
+      <c r="O98" s="9" t="n"/>
+      <c r="P98" s="9" t="n"/>
+      <c r="Q98" s="9" t="n"/>
+      <c r="R98" s="9" t="n"/>
+      <c r="S98" s="12" t="n"/>
+      <c r="T98" s="12" t="n"/>
+      <c r="U98" s="12" t="n"/>
+      <c r="V98" s="12" t="n"/>
+      <c r="W98" s="12" t="n"/>
+      <c r="X98" s="12" t="n"/>
+      <c r="Y98" s="9" t="n"/>
       <c r="Z98" s="21">
-        <f>IF(J98="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J98,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,1},MATCH(K98,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
+        <f>IF(J98="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J98,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K98,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
     </row>
     <row r="99">
+      <c r="A99" s="12" t="n"/>
+      <c r="B99" s="12" t="n"/>
+      <c r="C99" s="12" t="n"/>
+      <c r="D99" s="12" t="n"/>
+      <c r="E99" s="12" t="n"/>
+      <c r="F99" s="12" t="n"/>
+      <c r="G99" s="12" t="n"/>
+      <c r="H99" s="20" t="n"/>
+      <c r="I99" s="20" t="n"/>
+      <c r="J99" s="9" t="n"/>
+      <c r="K99" s="12" t="n"/>
+      <c r="L99" s="9" t="n"/>
+      <c r="M99" s="9" t="n"/>
+      <c r="N99" s="9" t="n"/>
+      <c r="O99" s="9" t="n"/>
+      <c r="P99" s="9" t="n"/>
+      <c r="Q99" s="9" t="n"/>
+      <c r="R99" s="9" t="n"/>
+      <c r="S99" s="12" t="n"/>
+      <c r="T99" s="12" t="n"/>
+      <c r="U99" s="12" t="n"/>
+      <c r="V99" s="12" t="n"/>
+      <c r="W99" s="12" t="n"/>
+      <c r="X99" s="12" t="n"/>
+      <c r="Y99" s="9" t="n"/>
       <c r="Z99" s="21">
-        <f>IF(J99="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J99,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,1},MATCH(K99,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
+        <f>IF(J99="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J99,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K99,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
     </row>
     <row r="100">
+      <c r="A100" s="12" t="n"/>
+      <c r="B100" s="12" t="n"/>
+      <c r="C100" s="12" t="n"/>
+      <c r="D100" s="12" t="n"/>
+      <c r="E100" s="12" t="n"/>
+      <c r="F100" s="12" t="n"/>
+      <c r="G100" s="12" t="n"/>
+      <c r="H100" s="20" t="n"/>
+      <c r="I100" s="20" t="n"/>
+      <c r="J100" s="9" t="n"/>
+      <c r="K100" s="12" t="n"/>
+      <c r="L100" s="9" t="n"/>
+      <c r="M100" s="9" t="n"/>
+      <c r="N100" s="9" t="n"/>
+      <c r="O100" s="9" t="n"/>
+      <c r="P100" s="9" t="n"/>
+      <c r="Q100" s="9" t="n"/>
+      <c r="R100" s="9" t="n"/>
+      <c r="S100" s="12" t="n"/>
+      <c r="T100" s="12" t="n"/>
+      <c r="U100" s="12" t="n"/>
+      <c r="V100" s="12" t="n"/>
+      <c r="W100" s="12" t="n"/>
+      <c r="X100" s="12" t="n"/>
+      <c r="Y100" s="9" t="n"/>
       <c r="Z100" s="21">
-        <f>IF(J100="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J100,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,1},MATCH(K100,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
+        <f>IF(J100="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J100,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K100,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
     </row>
@@ -2477,80 +4838,1412 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="008A63C2"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A10"/>
+  <dimension ref="A1:E200"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="110" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="22" t="inlineStr">
-        <is>
-          <t>HOW TO USE  使用方法</t>
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Review notes  检视记录</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="23" t="inlineStr">
-        <is>
-          <t>1. Client sheet: fill client name, income, review date. Review standard is RM1m for Life, CI, Retirement, Medical - adjust if needed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="23" t="inlineStr">
-        <is>
-          <t>2. Policies sheet: one row per policy. Use the dropdowns for Type, Status, Payment Mode.</t>
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Filled by the app: areas to discuss, data checks and the change log.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="23" t="inlineStr">
-        <is>
-          <t>3. Leave a cell BLANK if you don't know it. Never type a guess - the app flags blanks for you to confirm.</t>
-        </is>
-      </c>
+      <c r="A4" s="22" t="n"/>
+      <c r="B4" s="22" t="n"/>
+      <c r="C4" s="22" t="n"/>
+      <c r="D4" s="22" t="n"/>
+      <c r="E4" s="22" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="23" t="inlineStr">
-        <is>
-          <t>4. Dashboard sheet updates automatically (Excel-only version).</t>
-        </is>
-      </c>
+      <c r="A5" s="22" t="n"/>
+      <c r="B5" s="22" t="n"/>
+      <c r="C5" s="22" t="n"/>
+      <c r="D5" s="22" t="n"/>
+      <c r="E5" s="22" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="23" t="inlineStr">
-        <is>
-          <t>5. For the visual PDF report: open 'Policy Review Snapshot.html', load this file, click 'Generate'.</t>
-        </is>
-      </c>
+      <c r="A6" s="22" t="n"/>
+      <c r="B6" s="22" t="n"/>
+      <c r="C6" s="22" t="n"/>
+      <c r="D6" s="22" t="n"/>
+      <c r="E6" s="22" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="23" t="inlineStr"/>
+      <c r="A7" s="22" t="n"/>
+      <c r="B7" s="22" t="n"/>
+      <c r="C7" s="22" t="n"/>
+      <c r="D7" s="22" t="n"/>
+      <c r="E7" s="22" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="23" t="inlineStr">
-        <is>
-          <t>Pink nominee cell = inforce policy without nominee recorded.</t>
-        </is>
-      </c>
+      <c r="A8" s="22" t="n"/>
+      <c r="B8" s="22" t="n"/>
+      <c r="C8" s="22" t="n"/>
+      <c r="D8" s="22" t="n"/>
+      <c r="E8" s="22" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="23" t="inlineStr">
-        <is>
-          <t>Only Inforce policies count toward coverage totals. Lapsed/Paid-up are listed separately.</t>
-        </is>
-      </c>
+      <c r="A9" s="22" t="n"/>
+      <c r="B9" s="22" t="n"/>
+      <c r="C9" s="22" t="n"/>
+      <c r="D9" s="22" t="n"/>
+      <c r="E9" s="22" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="23" t="inlineStr">
-        <is>
-          <t>The rows marked (sample) are fictional - delete them before using with a real client.</t>
-        </is>
-      </c>
+      <c r="A10" s="22" t="n"/>
+      <c r="B10" s="22" t="n"/>
+      <c r="C10" s="22" t="n"/>
+      <c r="D10" s="22" t="n"/>
+      <c r="E10" s="22" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="22" t="n"/>
+      <c r="B11" s="22" t="n"/>
+      <c r="C11" s="22" t="n"/>
+      <c r="D11" s="22" t="n"/>
+      <c r="E11" s="22" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="22" t="n"/>
+      <c r="B12" s="22" t="n"/>
+      <c r="C12" s="22" t="n"/>
+      <c r="D12" s="22" t="n"/>
+      <c r="E12" s="22" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="22" t="n"/>
+      <c r="B13" s="22" t="n"/>
+      <c r="C13" s="22" t="n"/>
+      <c r="D13" s="22" t="n"/>
+      <c r="E13" s="22" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="22" t="n"/>
+      <c r="B14" s="22" t="n"/>
+      <c r="C14" s="22" t="n"/>
+      <c r="D14" s="22" t="n"/>
+      <c r="E14" s="22" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="22" t="n"/>
+      <c r="B15" s="22" t="n"/>
+      <c r="C15" s="22" t="n"/>
+      <c r="D15" s="22" t="n"/>
+      <c r="E15" s="22" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="22" t="n"/>
+      <c r="B16" s="22" t="n"/>
+      <c r="C16" s="22" t="n"/>
+      <c r="D16" s="22" t="n"/>
+      <c r="E16" s="22" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="22" t="n"/>
+      <c r="B17" s="22" t="n"/>
+      <c r="C17" s="22" t="n"/>
+      <c r="D17" s="22" t="n"/>
+      <c r="E17" s="22" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="22" t="n"/>
+      <c r="B18" s="22" t="n"/>
+      <c r="C18" s="22" t="n"/>
+      <c r="D18" s="22" t="n"/>
+      <c r="E18" s="22" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="22" t="n"/>
+      <c r="B19" s="22" t="n"/>
+      <c r="C19" s="22" t="n"/>
+      <c r="D19" s="22" t="n"/>
+      <c r="E19" s="22" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="22" t="n"/>
+      <c r="B20" s="22" t="n"/>
+      <c r="C20" s="22" t="n"/>
+      <c r="D20" s="22" t="n"/>
+      <c r="E20" s="22" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="22" t="n"/>
+      <c r="B21" s="22" t="n"/>
+      <c r="C21" s="22" t="n"/>
+      <c r="D21" s="22" t="n"/>
+      <c r="E21" s="22" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="22" t="n"/>
+      <c r="B22" s="22" t="n"/>
+      <c r="C22" s="22" t="n"/>
+      <c r="D22" s="22" t="n"/>
+      <c r="E22" s="22" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="22" t="n"/>
+      <c r="B23" s="22" t="n"/>
+      <c r="C23" s="22" t="n"/>
+      <c r="D23" s="22" t="n"/>
+      <c r="E23" s="22" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="22" t="n"/>
+      <c r="B24" s="22" t="n"/>
+      <c r="C24" s="22" t="n"/>
+      <c r="D24" s="22" t="n"/>
+      <c r="E24" s="22" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="22" t="n"/>
+      <c r="B25" s="22" t="n"/>
+      <c r="C25" s="22" t="n"/>
+      <c r="D25" s="22" t="n"/>
+      <c r="E25" s="22" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="22" t="n"/>
+      <c r="B26" s="22" t="n"/>
+      <c r="C26" s="22" t="n"/>
+      <c r="D26" s="22" t="n"/>
+      <c r="E26" s="22" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="22" t="n"/>
+      <c r="B27" s="22" t="n"/>
+      <c r="C27" s="22" t="n"/>
+      <c r="D27" s="22" t="n"/>
+      <c r="E27" s="22" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="22" t="n"/>
+      <c r="B28" s="22" t="n"/>
+      <c r="C28" s="22" t="n"/>
+      <c r="D28" s="22" t="n"/>
+      <c r="E28" s="22" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="22" t="n"/>
+      <c r="B29" s="22" t="n"/>
+      <c r="C29" s="22" t="n"/>
+      <c r="D29" s="22" t="n"/>
+      <c r="E29" s="22" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="22" t="n"/>
+      <c r="B30" s="22" t="n"/>
+      <c r="C30" s="22" t="n"/>
+      <c r="D30" s="22" t="n"/>
+      <c r="E30" s="22" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="22" t="n"/>
+      <c r="B31" s="22" t="n"/>
+      <c r="C31" s="22" t="n"/>
+      <c r="D31" s="22" t="n"/>
+      <c r="E31" s="22" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="22" t="n"/>
+      <c r="B32" s="22" t="n"/>
+      <c r="C32" s="22" t="n"/>
+      <c r="D32" s="22" t="n"/>
+      <c r="E32" s="22" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="22" t="n"/>
+      <c r="B33" s="22" t="n"/>
+      <c r="C33" s="22" t="n"/>
+      <c r="D33" s="22" t="n"/>
+      <c r="E33" s="22" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="22" t="n"/>
+      <c r="B34" s="22" t="n"/>
+      <c r="C34" s="22" t="n"/>
+      <c r="D34" s="22" t="n"/>
+      <c r="E34" s="22" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="22" t="n"/>
+      <c r="B35" s="22" t="n"/>
+      <c r="C35" s="22" t="n"/>
+      <c r="D35" s="22" t="n"/>
+      <c r="E35" s="22" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="22" t="n"/>
+      <c r="B36" s="22" t="n"/>
+      <c r="C36" s="22" t="n"/>
+      <c r="D36" s="22" t="n"/>
+      <c r="E36" s="22" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="22" t="n"/>
+      <c r="B37" s="22" t="n"/>
+      <c r="C37" s="22" t="n"/>
+      <c r="D37" s="22" t="n"/>
+      <c r="E37" s="22" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="22" t="n"/>
+      <c r="B38" s="22" t="n"/>
+      <c r="C38" s="22" t="n"/>
+      <c r="D38" s="22" t="n"/>
+      <c r="E38" s="22" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="22" t="n"/>
+      <c r="B39" s="22" t="n"/>
+      <c r="C39" s="22" t="n"/>
+      <c r="D39" s="22" t="n"/>
+      <c r="E39" s="22" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="22" t="n"/>
+      <c r="B40" s="22" t="n"/>
+      <c r="C40" s="22" t="n"/>
+      <c r="D40" s="22" t="n"/>
+      <c r="E40" s="22" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="22" t="n"/>
+      <c r="B41" s="22" t="n"/>
+      <c r="C41" s="22" t="n"/>
+      <c r="D41" s="22" t="n"/>
+      <c r="E41" s="22" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="22" t="n"/>
+      <c r="B42" s="22" t="n"/>
+      <c r="C42" s="22" t="n"/>
+      <c r="D42" s="22" t="n"/>
+      <c r="E42" s="22" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="22" t="n"/>
+      <c r="B43" s="22" t="n"/>
+      <c r="C43" s="22" t="n"/>
+      <c r="D43" s="22" t="n"/>
+      <c r="E43" s="22" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="22" t="n"/>
+      <c r="B44" s="22" t="n"/>
+      <c r="C44" s="22" t="n"/>
+      <c r="D44" s="22" t="n"/>
+      <c r="E44" s="22" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="22" t="n"/>
+      <c r="B45" s="22" t="n"/>
+      <c r="C45" s="22" t="n"/>
+      <c r="D45" s="22" t="n"/>
+      <c r="E45" s="22" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="22" t="n"/>
+      <c r="B46" s="22" t="n"/>
+      <c r="C46" s="22" t="n"/>
+      <c r="D46" s="22" t="n"/>
+      <c r="E46" s="22" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="22" t="n"/>
+      <c r="B47" s="22" t="n"/>
+      <c r="C47" s="22" t="n"/>
+      <c r="D47" s="22" t="n"/>
+      <c r="E47" s="22" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="22" t="n"/>
+      <c r="B48" s="22" t="n"/>
+      <c r="C48" s="22" t="n"/>
+      <c r="D48" s="22" t="n"/>
+      <c r="E48" s="22" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="22" t="n"/>
+      <c r="B49" s="22" t="n"/>
+      <c r="C49" s="22" t="n"/>
+      <c r="D49" s="22" t="n"/>
+      <c r="E49" s="22" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="22" t="n"/>
+      <c r="B50" s="22" t="n"/>
+      <c r="C50" s="22" t="n"/>
+      <c r="D50" s="22" t="n"/>
+      <c r="E50" s="22" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="22" t="n"/>
+      <c r="B51" s="22" t="n"/>
+      <c r="C51" s="22" t="n"/>
+      <c r="D51" s="22" t="n"/>
+      <c r="E51" s="22" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="22" t="n"/>
+      <c r="B52" s="22" t="n"/>
+      <c r="C52" s="22" t="n"/>
+      <c r="D52" s="22" t="n"/>
+      <c r="E52" s="22" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="22" t="n"/>
+      <c r="B53" s="22" t="n"/>
+      <c r="C53" s="22" t="n"/>
+      <c r="D53" s="22" t="n"/>
+      <c r="E53" s="22" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="22" t="n"/>
+      <c r="B54" s="22" t="n"/>
+      <c r="C54" s="22" t="n"/>
+      <c r="D54" s="22" t="n"/>
+      <c r="E54" s="22" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="22" t="n"/>
+      <c r="B55" s="22" t="n"/>
+      <c r="C55" s="22" t="n"/>
+      <c r="D55" s="22" t="n"/>
+      <c r="E55" s="22" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="22" t="n"/>
+      <c r="B56" s="22" t="n"/>
+      <c r="C56" s="22" t="n"/>
+      <c r="D56" s="22" t="n"/>
+      <c r="E56" s="22" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="22" t="n"/>
+      <c r="B57" s="22" t="n"/>
+      <c r="C57" s="22" t="n"/>
+      <c r="D57" s="22" t="n"/>
+      <c r="E57" s="22" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="22" t="n"/>
+      <c r="B58" s="22" t="n"/>
+      <c r="C58" s="22" t="n"/>
+      <c r="D58" s="22" t="n"/>
+      <c r="E58" s="22" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="22" t="n"/>
+      <c r="B59" s="22" t="n"/>
+      <c r="C59" s="22" t="n"/>
+      <c r="D59" s="22" t="n"/>
+      <c r="E59" s="22" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="22" t="n"/>
+      <c r="B60" s="22" t="n"/>
+      <c r="C60" s="22" t="n"/>
+      <c r="D60" s="22" t="n"/>
+      <c r="E60" s="22" t="n"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="22" t="n"/>
+      <c r="B61" s="22" t="n"/>
+      <c r="C61" s="22" t="n"/>
+      <c r="D61" s="22" t="n"/>
+      <c r="E61" s="22" t="n"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="22" t="n"/>
+      <c r="B62" s="22" t="n"/>
+      <c r="C62" s="22" t="n"/>
+      <c r="D62" s="22" t="n"/>
+      <c r="E62" s="22" t="n"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="22" t="n"/>
+      <c r="B63" s="22" t="n"/>
+      <c r="C63" s="22" t="n"/>
+      <c r="D63" s="22" t="n"/>
+      <c r="E63" s="22" t="n"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="22" t="n"/>
+      <c r="B64" s="22" t="n"/>
+      <c r="C64" s="22" t="n"/>
+      <c r="D64" s="22" t="n"/>
+      <c r="E64" s="22" t="n"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="22" t="n"/>
+      <c r="B65" s="22" t="n"/>
+      <c r="C65" s="22" t="n"/>
+      <c r="D65" s="22" t="n"/>
+      <c r="E65" s="22" t="n"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="22" t="n"/>
+      <c r="B66" s="22" t="n"/>
+      <c r="C66" s="22" t="n"/>
+      <c r="D66" s="22" t="n"/>
+      <c r="E66" s="22" t="n"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="22" t="n"/>
+      <c r="B67" s="22" t="n"/>
+      <c r="C67" s="22" t="n"/>
+      <c r="D67" s="22" t="n"/>
+      <c r="E67" s="22" t="n"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="22" t="n"/>
+      <c r="B68" s="22" t="n"/>
+      <c r="C68" s="22" t="n"/>
+      <c r="D68" s="22" t="n"/>
+      <c r="E68" s="22" t="n"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="22" t="n"/>
+      <c r="B69" s="22" t="n"/>
+      <c r="C69" s="22" t="n"/>
+      <c r="D69" s="22" t="n"/>
+      <c r="E69" s="22" t="n"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="22" t="n"/>
+      <c r="B70" s="22" t="n"/>
+      <c r="C70" s="22" t="n"/>
+      <c r="D70" s="22" t="n"/>
+      <c r="E70" s="22" t="n"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="22" t="n"/>
+      <c r="B71" s="22" t="n"/>
+      <c r="C71" s="22" t="n"/>
+      <c r="D71" s="22" t="n"/>
+      <c r="E71" s="22" t="n"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="22" t="n"/>
+      <c r="B72" s="22" t="n"/>
+      <c r="C72" s="22" t="n"/>
+      <c r="D72" s="22" t="n"/>
+      <c r="E72" s="22" t="n"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="22" t="n"/>
+      <c r="B73" s="22" t="n"/>
+      <c r="C73" s="22" t="n"/>
+      <c r="D73" s="22" t="n"/>
+      <c r="E73" s="22" t="n"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="22" t="n"/>
+      <c r="B74" s="22" t="n"/>
+      <c r="C74" s="22" t="n"/>
+      <c r="D74" s="22" t="n"/>
+      <c r="E74" s="22" t="n"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="22" t="n"/>
+      <c r="B75" s="22" t="n"/>
+      <c r="C75" s="22" t="n"/>
+      <c r="D75" s="22" t="n"/>
+      <c r="E75" s="22" t="n"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="22" t="n"/>
+      <c r="B76" s="22" t="n"/>
+      <c r="C76" s="22" t="n"/>
+      <c r="D76" s="22" t="n"/>
+      <c r="E76" s="22" t="n"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="22" t="n"/>
+      <c r="B77" s="22" t="n"/>
+      <c r="C77" s="22" t="n"/>
+      <c r="D77" s="22" t="n"/>
+      <c r="E77" s="22" t="n"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="22" t="n"/>
+      <c r="B78" s="22" t="n"/>
+      <c r="C78" s="22" t="n"/>
+      <c r="D78" s="22" t="n"/>
+      <c r="E78" s="22" t="n"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="22" t="n"/>
+      <c r="B79" s="22" t="n"/>
+      <c r="C79" s="22" t="n"/>
+      <c r="D79" s="22" t="n"/>
+      <c r="E79" s="22" t="n"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="22" t="n"/>
+      <c r="B80" s="22" t="n"/>
+      <c r="C80" s="22" t="n"/>
+      <c r="D80" s="22" t="n"/>
+      <c r="E80" s="22" t="n"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="22" t="n"/>
+      <c r="B81" s="22" t="n"/>
+      <c r="C81" s="22" t="n"/>
+      <c r="D81" s="22" t="n"/>
+      <c r="E81" s="22" t="n"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="22" t="n"/>
+      <c r="B82" s="22" t="n"/>
+      <c r="C82" s="22" t="n"/>
+      <c r="D82" s="22" t="n"/>
+      <c r="E82" s="22" t="n"/>
+    </row>
+    <row r="83">
+      <c r="A83" s="22" t="n"/>
+      <c r="B83" s="22" t="n"/>
+      <c r="C83" s="22" t="n"/>
+      <c r="D83" s="22" t="n"/>
+      <c r="E83" s="22" t="n"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="22" t="n"/>
+      <c r="B84" s="22" t="n"/>
+      <c r="C84" s="22" t="n"/>
+      <c r="D84" s="22" t="n"/>
+      <c r="E84" s="22" t="n"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="22" t="n"/>
+      <c r="B85" s="22" t="n"/>
+      <c r="C85" s="22" t="n"/>
+      <c r="D85" s="22" t="n"/>
+      <c r="E85" s="22" t="n"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="22" t="n"/>
+      <c r="B86" s="22" t="n"/>
+      <c r="C86" s="22" t="n"/>
+      <c r="D86" s="22" t="n"/>
+      <c r="E86" s="22" t="n"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="22" t="n"/>
+      <c r="B87" s="22" t="n"/>
+      <c r="C87" s="22" t="n"/>
+      <c r="D87" s="22" t="n"/>
+      <c r="E87" s="22" t="n"/>
+    </row>
+    <row r="88">
+      <c r="A88" s="22" t="n"/>
+      <c r="B88" s="22" t="n"/>
+      <c r="C88" s="22" t="n"/>
+      <c r="D88" s="22" t="n"/>
+      <c r="E88" s="22" t="n"/>
+    </row>
+    <row r="89">
+      <c r="A89" s="22" t="n"/>
+      <c r="B89" s="22" t="n"/>
+      <c r="C89" s="22" t="n"/>
+      <c r="D89" s="22" t="n"/>
+      <c r="E89" s="22" t="n"/>
+    </row>
+    <row r="90">
+      <c r="A90" s="22" t="n"/>
+      <c r="B90" s="22" t="n"/>
+      <c r="C90" s="22" t="n"/>
+      <c r="D90" s="22" t="n"/>
+      <c r="E90" s="22" t="n"/>
+    </row>
+    <row r="91">
+      <c r="A91" s="22" t="n"/>
+      <c r="B91" s="22" t="n"/>
+      <c r="C91" s="22" t="n"/>
+      <c r="D91" s="22" t="n"/>
+      <c r="E91" s="22" t="n"/>
+    </row>
+    <row r="92">
+      <c r="A92" s="22" t="n"/>
+      <c r="B92" s="22" t="n"/>
+      <c r="C92" s="22" t="n"/>
+      <c r="D92" s="22" t="n"/>
+      <c r="E92" s="22" t="n"/>
+    </row>
+    <row r="93">
+      <c r="A93" s="22" t="n"/>
+      <c r="B93" s="22" t="n"/>
+      <c r="C93" s="22" t="n"/>
+      <c r="D93" s="22" t="n"/>
+      <c r="E93" s="22" t="n"/>
+    </row>
+    <row r="94">
+      <c r="A94" s="22" t="n"/>
+      <c r="B94" s="22" t="n"/>
+      <c r="C94" s="22" t="n"/>
+      <c r="D94" s="22" t="n"/>
+      <c r="E94" s="22" t="n"/>
+    </row>
+    <row r="95">
+      <c r="A95" s="22" t="n"/>
+      <c r="B95" s="22" t="n"/>
+      <c r="C95" s="22" t="n"/>
+      <c r="D95" s="22" t="n"/>
+      <c r="E95" s="22" t="n"/>
+    </row>
+    <row r="96">
+      <c r="A96" s="22" t="n"/>
+      <c r="B96" s="22" t="n"/>
+      <c r="C96" s="22" t="n"/>
+      <c r="D96" s="22" t="n"/>
+      <c r="E96" s="22" t="n"/>
+    </row>
+    <row r="97">
+      <c r="A97" s="22" t="n"/>
+      <c r="B97" s="22" t="n"/>
+      <c r="C97" s="22" t="n"/>
+      <c r="D97" s="22" t="n"/>
+      <c r="E97" s="22" t="n"/>
+    </row>
+    <row r="98">
+      <c r="A98" s="22" t="n"/>
+      <c r="B98" s="22" t="n"/>
+      <c r="C98" s="22" t="n"/>
+      <c r="D98" s="22" t="n"/>
+      <c r="E98" s="22" t="n"/>
+    </row>
+    <row r="99">
+      <c r="A99" s="22" t="n"/>
+      <c r="B99" s="22" t="n"/>
+      <c r="C99" s="22" t="n"/>
+      <c r="D99" s="22" t="n"/>
+      <c r="E99" s="22" t="n"/>
+    </row>
+    <row r="100">
+      <c r="A100" s="22" t="n"/>
+      <c r="B100" s="22" t="n"/>
+      <c r="C100" s="22" t="n"/>
+      <c r="D100" s="22" t="n"/>
+      <c r="E100" s="22" t="n"/>
+    </row>
+    <row r="101">
+      <c r="A101" s="22" t="n"/>
+      <c r="B101" s="22" t="n"/>
+      <c r="C101" s="22" t="n"/>
+      <c r="D101" s="22" t="n"/>
+      <c r="E101" s="22" t="n"/>
+    </row>
+    <row r="102">
+      <c r="A102" s="22" t="n"/>
+      <c r="B102" s="22" t="n"/>
+      <c r="C102" s="22" t="n"/>
+      <c r="D102" s="22" t="n"/>
+      <c r="E102" s="22" t="n"/>
+    </row>
+    <row r="103">
+      <c r="A103" s="22" t="n"/>
+      <c r="B103" s="22" t="n"/>
+      <c r="C103" s="22" t="n"/>
+      <c r="D103" s="22" t="n"/>
+      <c r="E103" s="22" t="n"/>
+    </row>
+    <row r="104">
+      <c r="A104" s="22" t="n"/>
+      <c r="B104" s="22" t="n"/>
+      <c r="C104" s="22" t="n"/>
+      <c r="D104" s="22" t="n"/>
+      <c r="E104" s="22" t="n"/>
+    </row>
+    <row r="105">
+      <c r="A105" s="22" t="n"/>
+      <c r="B105" s="22" t="n"/>
+      <c r="C105" s="22" t="n"/>
+      <c r="D105" s="22" t="n"/>
+      <c r="E105" s="22" t="n"/>
+    </row>
+    <row r="106">
+      <c r="A106" s="22" t="n"/>
+      <c r="B106" s="22" t="n"/>
+      <c r="C106" s="22" t="n"/>
+      <c r="D106" s="22" t="n"/>
+      <c r="E106" s="22" t="n"/>
+    </row>
+    <row r="107">
+      <c r="A107" s="22" t="n"/>
+      <c r="B107" s="22" t="n"/>
+      <c r="C107" s="22" t="n"/>
+      <c r="D107" s="22" t="n"/>
+      <c r="E107" s="22" t="n"/>
+    </row>
+    <row r="108">
+      <c r="A108" s="22" t="n"/>
+      <c r="B108" s="22" t="n"/>
+      <c r="C108" s="22" t="n"/>
+      <c r="D108" s="22" t="n"/>
+      <c r="E108" s="22" t="n"/>
+    </row>
+    <row r="109">
+      <c r="A109" s="22" t="n"/>
+      <c r="B109" s="22" t="n"/>
+      <c r="C109" s="22" t="n"/>
+      <c r="D109" s="22" t="n"/>
+      <c r="E109" s="22" t="n"/>
+    </row>
+    <row r="110">
+      <c r="A110" s="22" t="n"/>
+      <c r="B110" s="22" t="n"/>
+      <c r="C110" s="22" t="n"/>
+      <c r="D110" s="22" t="n"/>
+      <c r="E110" s="22" t="n"/>
+    </row>
+    <row r="111">
+      <c r="A111" s="22" t="n"/>
+      <c r="B111" s="22" t="n"/>
+      <c r="C111" s="22" t="n"/>
+      <c r="D111" s="22" t="n"/>
+      <c r="E111" s="22" t="n"/>
+    </row>
+    <row r="112">
+      <c r="A112" s="22" t="n"/>
+      <c r="B112" s="22" t="n"/>
+      <c r="C112" s="22" t="n"/>
+      <c r="D112" s="22" t="n"/>
+      <c r="E112" s="22" t="n"/>
+    </row>
+    <row r="113">
+      <c r="A113" s="22" t="n"/>
+      <c r="B113" s="22" t="n"/>
+      <c r="C113" s="22" t="n"/>
+      <c r="D113" s="22" t="n"/>
+      <c r="E113" s="22" t="n"/>
+    </row>
+    <row r="114">
+      <c r="A114" s="22" t="n"/>
+      <c r="B114" s="22" t="n"/>
+      <c r="C114" s="22" t="n"/>
+      <c r="D114" s="22" t="n"/>
+      <c r="E114" s="22" t="n"/>
+    </row>
+    <row r="115">
+      <c r="A115" s="22" t="n"/>
+      <c r="B115" s="22" t="n"/>
+      <c r="C115" s="22" t="n"/>
+      <c r="D115" s="22" t="n"/>
+      <c r="E115" s="22" t="n"/>
+    </row>
+    <row r="116">
+      <c r="A116" s="22" t="n"/>
+      <c r="B116" s="22" t="n"/>
+      <c r="C116" s="22" t="n"/>
+      <c r="D116" s="22" t="n"/>
+      <c r="E116" s="22" t="n"/>
+    </row>
+    <row r="117">
+      <c r="A117" s="22" t="n"/>
+      <c r="B117" s="22" t="n"/>
+      <c r="C117" s="22" t="n"/>
+      <c r="D117" s="22" t="n"/>
+      <c r="E117" s="22" t="n"/>
+    </row>
+    <row r="118">
+      <c r="A118" s="22" t="n"/>
+      <c r="B118" s="22" t="n"/>
+      <c r="C118" s="22" t="n"/>
+      <c r="D118" s="22" t="n"/>
+      <c r="E118" s="22" t="n"/>
+    </row>
+    <row r="119">
+      <c r="A119" s="22" t="n"/>
+      <c r="B119" s="22" t="n"/>
+      <c r="C119" s="22" t="n"/>
+      <c r="D119" s="22" t="n"/>
+      <c r="E119" s="22" t="n"/>
+    </row>
+    <row r="120">
+      <c r="A120" s="22" t="n"/>
+      <c r="B120" s="22" t="n"/>
+      <c r="C120" s="22" t="n"/>
+      <c r="D120" s="22" t="n"/>
+      <c r="E120" s="22" t="n"/>
+    </row>
+    <row r="121">
+      <c r="A121" s="22" t="n"/>
+      <c r="B121" s="22" t="n"/>
+      <c r="C121" s="22" t="n"/>
+      <c r="D121" s="22" t="n"/>
+      <c r="E121" s="22" t="n"/>
+    </row>
+    <row r="122">
+      <c r="A122" s="22" t="n"/>
+      <c r="B122" s="22" t="n"/>
+      <c r="C122" s="22" t="n"/>
+      <c r="D122" s="22" t="n"/>
+      <c r="E122" s="22" t="n"/>
+    </row>
+    <row r="123">
+      <c r="A123" s="22" t="n"/>
+      <c r="B123" s="22" t="n"/>
+      <c r="C123" s="22" t="n"/>
+      <c r="D123" s="22" t="n"/>
+      <c r="E123" s="22" t="n"/>
+    </row>
+    <row r="124">
+      <c r="A124" s="22" t="n"/>
+      <c r="B124" s="22" t="n"/>
+      <c r="C124" s="22" t="n"/>
+      <c r="D124" s="22" t="n"/>
+      <c r="E124" s="22" t="n"/>
+    </row>
+    <row r="125">
+      <c r="A125" s="22" t="n"/>
+      <c r="B125" s="22" t="n"/>
+      <c r="C125" s="22" t="n"/>
+      <c r="D125" s="22" t="n"/>
+      <c r="E125" s="22" t="n"/>
+    </row>
+    <row r="126">
+      <c r="A126" s="22" t="n"/>
+      <c r="B126" s="22" t="n"/>
+      <c r="C126" s="22" t="n"/>
+      <c r="D126" s="22" t="n"/>
+      <c r="E126" s="22" t="n"/>
+    </row>
+    <row r="127">
+      <c r="A127" s="22" t="n"/>
+      <c r="B127" s="22" t="n"/>
+      <c r="C127" s="22" t="n"/>
+      <c r="D127" s="22" t="n"/>
+      <c r="E127" s="22" t="n"/>
+    </row>
+    <row r="128">
+      <c r="A128" s="22" t="n"/>
+      <c r="B128" s="22" t="n"/>
+      <c r="C128" s="22" t="n"/>
+      <c r="D128" s="22" t="n"/>
+      <c r="E128" s="22" t="n"/>
+    </row>
+    <row r="129">
+      <c r="A129" s="22" t="n"/>
+      <c r="B129" s="22" t="n"/>
+      <c r="C129" s="22" t="n"/>
+      <c r="D129" s="22" t="n"/>
+      <c r="E129" s="22" t="n"/>
+    </row>
+    <row r="130">
+      <c r="A130" s="22" t="n"/>
+      <c r="B130" s="22" t="n"/>
+      <c r="C130" s="22" t="n"/>
+      <c r="D130" s="22" t="n"/>
+      <c r="E130" s="22" t="n"/>
+    </row>
+    <row r="131">
+      <c r="A131" s="22" t="n"/>
+      <c r="B131" s="22" t="n"/>
+      <c r="C131" s="22" t="n"/>
+      <c r="D131" s="22" t="n"/>
+      <c r="E131" s="22" t="n"/>
+    </row>
+    <row r="132">
+      <c r="A132" s="22" t="n"/>
+      <c r="B132" s="22" t="n"/>
+      <c r="C132" s="22" t="n"/>
+      <c r="D132" s="22" t="n"/>
+      <c r="E132" s="22" t="n"/>
+    </row>
+    <row r="133">
+      <c r="A133" s="22" t="n"/>
+      <c r="B133" s="22" t="n"/>
+      <c r="C133" s="22" t="n"/>
+      <c r="D133" s="22" t="n"/>
+      <c r="E133" s="22" t="n"/>
+    </row>
+    <row r="134">
+      <c r="A134" s="22" t="n"/>
+      <c r="B134" s="22" t="n"/>
+      <c r="C134" s="22" t="n"/>
+      <c r="D134" s="22" t="n"/>
+      <c r="E134" s="22" t="n"/>
+    </row>
+    <row r="135">
+      <c r="A135" s="22" t="n"/>
+      <c r="B135" s="22" t="n"/>
+      <c r="C135" s="22" t="n"/>
+      <c r="D135" s="22" t="n"/>
+      <c r="E135" s="22" t="n"/>
+    </row>
+    <row r="136">
+      <c r="A136" s="22" t="n"/>
+      <c r="B136" s="22" t="n"/>
+      <c r="C136" s="22" t="n"/>
+      <c r="D136" s="22" t="n"/>
+      <c r="E136" s="22" t="n"/>
+    </row>
+    <row r="137">
+      <c r="A137" s="22" t="n"/>
+      <c r="B137" s="22" t="n"/>
+      <c r="C137" s="22" t="n"/>
+      <c r="D137" s="22" t="n"/>
+      <c r="E137" s="22" t="n"/>
+    </row>
+    <row r="138">
+      <c r="A138" s="22" t="n"/>
+      <c r="B138" s="22" t="n"/>
+      <c r="C138" s="22" t="n"/>
+      <c r="D138" s="22" t="n"/>
+      <c r="E138" s="22" t="n"/>
+    </row>
+    <row r="139">
+      <c r="A139" s="22" t="n"/>
+      <c r="B139" s="22" t="n"/>
+      <c r="C139" s="22" t="n"/>
+      <c r="D139" s="22" t="n"/>
+      <c r="E139" s="22" t="n"/>
+    </row>
+    <row r="140">
+      <c r="A140" s="22" t="n"/>
+      <c r="B140" s="22" t="n"/>
+      <c r="C140" s="22" t="n"/>
+      <c r="D140" s="22" t="n"/>
+      <c r="E140" s="22" t="n"/>
+    </row>
+    <row r="141">
+      <c r="A141" s="22" t="n"/>
+      <c r="B141" s="22" t="n"/>
+      <c r="C141" s="22" t="n"/>
+      <c r="D141" s="22" t="n"/>
+      <c r="E141" s="22" t="n"/>
+    </row>
+    <row r="142">
+      <c r="A142" s="22" t="n"/>
+      <c r="B142" s="22" t="n"/>
+      <c r="C142" s="22" t="n"/>
+      <c r="D142" s="22" t="n"/>
+      <c r="E142" s="22" t="n"/>
+    </row>
+    <row r="143">
+      <c r="A143" s="22" t="n"/>
+      <c r="B143" s="22" t="n"/>
+      <c r="C143" s="22" t="n"/>
+      <c r="D143" s="22" t="n"/>
+      <c r="E143" s="22" t="n"/>
+    </row>
+    <row r="144">
+      <c r="A144" s="22" t="n"/>
+      <c r="B144" s="22" t="n"/>
+      <c r="C144" s="22" t="n"/>
+      <c r="D144" s="22" t="n"/>
+      <c r="E144" s="22" t="n"/>
+    </row>
+    <row r="145">
+      <c r="A145" s="22" t="n"/>
+      <c r="B145" s="22" t="n"/>
+      <c r="C145" s="22" t="n"/>
+      <c r="D145" s="22" t="n"/>
+      <c r="E145" s="22" t="n"/>
+    </row>
+    <row r="146">
+      <c r="A146" s="22" t="n"/>
+      <c r="B146" s="22" t="n"/>
+      <c r="C146" s="22" t="n"/>
+      <c r="D146" s="22" t="n"/>
+      <c r="E146" s="22" t="n"/>
+    </row>
+    <row r="147">
+      <c r="A147" s="22" t="n"/>
+      <c r="B147" s="22" t="n"/>
+      <c r="C147" s="22" t="n"/>
+      <c r="D147" s="22" t="n"/>
+      <c r="E147" s="22" t="n"/>
+    </row>
+    <row r="148">
+      <c r="A148" s="22" t="n"/>
+      <c r="B148" s="22" t="n"/>
+      <c r="C148" s="22" t="n"/>
+      <c r="D148" s="22" t="n"/>
+      <c r="E148" s="22" t="n"/>
+    </row>
+    <row r="149">
+      <c r="A149" s="22" t="n"/>
+      <c r="B149" s="22" t="n"/>
+      <c r="C149" s="22" t="n"/>
+      <c r="D149" s="22" t="n"/>
+      <c r="E149" s="22" t="n"/>
+    </row>
+    <row r="150">
+      <c r="A150" s="22" t="n"/>
+      <c r="B150" s="22" t="n"/>
+      <c r="C150" s="22" t="n"/>
+      <c r="D150" s="22" t="n"/>
+      <c r="E150" s="22" t="n"/>
+    </row>
+    <row r="151">
+      <c r="A151" s="22" t="n"/>
+      <c r="B151" s="22" t="n"/>
+      <c r="C151" s="22" t="n"/>
+      <c r="D151" s="22" t="n"/>
+      <c r="E151" s="22" t="n"/>
+    </row>
+    <row r="152">
+      <c r="A152" s="22" t="n"/>
+      <c r="B152" s="22" t="n"/>
+      <c r="C152" s="22" t="n"/>
+      <c r="D152" s="22" t="n"/>
+      <c r="E152" s="22" t="n"/>
+    </row>
+    <row r="153">
+      <c r="A153" s="22" t="n"/>
+      <c r="B153" s="22" t="n"/>
+      <c r="C153" s="22" t="n"/>
+      <c r="D153" s="22" t="n"/>
+      <c r="E153" s="22" t="n"/>
+    </row>
+    <row r="154">
+      <c r="A154" s="22" t="n"/>
+      <c r="B154" s="22" t="n"/>
+      <c r="C154" s="22" t="n"/>
+      <c r="D154" s="22" t="n"/>
+      <c r="E154" s="22" t="n"/>
+    </row>
+    <row r="155">
+      <c r="A155" s="22" t="n"/>
+      <c r="B155" s="22" t="n"/>
+      <c r="C155" s="22" t="n"/>
+      <c r="D155" s="22" t="n"/>
+      <c r="E155" s="22" t="n"/>
+    </row>
+    <row r="156">
+      <c r="A156" s="22" t="n"/>
+      <c r="B156" s="22" t="n"/>
+      <c r="C156" s="22" t="n"/>
+      <c r="D156" s="22" t="n"/>
+      <c r="E156" s="22" t="n"/>
+    </row>
+    <row r="157">
+      <c r="A157" s="22" t="n"/>
+      <c r="B157" s="22" t="n"/>
+      <c r="C157" s="22" t="n"/>
+      <c r="D157" s="22" t="n"/>
+      <c r="E157" s="22" t="n"/>
+    </row>
+    <row r="158">
+      <c r="A158" s="22" t="n"/>
+      <c r="B158" s="22" t="n"/>
+      <c r="C158" s="22" t="n"/>
+      <c r="D158" s="22" t="n"/>
+      <c r="E158" s="22" t="n"/>
+    </row>
+    <row r="159">
+      <c r="A159" s="22" t="n"/>
+      <c r="B159" s="22" t="n"/>
+      <c r="C159" s="22" t="n"/>
+      <c r="D159" s="22" t="n"/>
+      <c r="E159" s="22" t="n"/>
+    </row>
+    <row r="160">
+      <c r="A160" s="22" t="n"/>
+      <c r="B160" s="22" t="n"/>
+      <c r="C160" s="22" t="n"/>
+      <c r="D160" s="22" t="n"/>
+      <c r="E160" s="22" t="n"/>
+    </row>
+    <row r="161">
+      <c r="A161" s="22" t="n"/>
+      <c r="B161" s="22" t="n"/>
+      <c r="C161" s="22" t="n"/>
+      <c r="D161" s="22" t="n"/>
+      <c r="E161" s="22" t="n"/>
+    </row>
+    <row r="162">
+      <c r="A162" s="22" t="n"/>
+      <c r="B162" s="22" t="n"/>
+      <c r="C162" s="22" t="n"/>
+      <c r="D162" s="22" t="n"/>
+      <c r="E162" s="22" t="n"/>
+    </row>
+    <row r="163">
+      <c r="A163" s="22" t="n"/>
+      <c r="B163" s="22" t="n"/>
+      <c r="C163" s="22" t="n"/>
+      <c r="D163" s="22" t="n"/>
+      <c r="E163" s="22" t="n"/>
+    </row>
+    <row r="164">
+      <c r="A164" s="22" t="n"/>
+      <c r="B164" s="22" t="n"/>
+      <c r="C164" s="22" t="n"/>
+      <c r="D164" s="22" t="n"/>
+      <c r="E164" s="22" t="n"/>
+    </row>
+    <row r="165">
+      <c r="A165" s="22" t="n"/>
+      <c r="B165" s="22" t="n"/>
+      <c r="C165" s="22" t="n"/>
+      <c r="D165" s="22" t="n"/>
+      <c r="E165" s="22" t="n"/>
+    </row>
+    <row r="166">
+      <c r="A166" s="22" t="n"/>
+      <c r="B166" s="22" t="n"/>
+      <c r="C166" s="22" t="n"/>
+      <c r="D166" s="22" t="n"/>
+      <c r="E166" s="22" t="n"/>
+    </row>
+    <row r="167">
+      <c r="A167" s="22" t="n"/>
+      <c r="B167" s="22" t="n"/>
+      <c r="C167" s="22" t="n"/>
+      <c r="D167" s="22" t="n"/>
+      <c r="E167" s="22" t="n"/>
+    </row>
+    <row r="168">
+      <c r="A168" s="22" t="n"/>
+      <c r="B168" s="22" t="n"/>
+      <c r="C168" s="22" t="n"/>
+      <c r="D168" s="22" t="n"/>
+      <c r="E168" s="22" t="n"/>
+    </row>
+    <row r="169">
+      <c r="A169" s="22" t="n"/>
+      <c r="B169" s="22" t="n"/>
+      <c r="C169" s="22" t="n"/>
+      <c r="D169" s="22" t="n"/>
+      <c r="E169" s="22" t="n"/>
+    </row>
+    <row r="170">
+      <c r="A170" s="22" t="n"/>
+      <c r="B170" s="22" t="n"/>
+      <c r="C170" s="22" t="n"/>
+      <c r="D170" s="22" t="n"/>
+      <c r="E170" s="22" t="n"/>
+    </row>
+    <row r="171">
+      <c r="A171" s="22" t="n"/>
+      <c r="B171" s="22" t="n"/>
+      <c r="C171" s="22" t="n"/>
+      <c r="D171" s="22" t="n"/>
+      <c r="E171" s="22" t="n"/>
+    </row>
+    <row r="172">
+      <c r="A172" s="22" t="n"/>
+      <c r="B172" s="22" t="n"/>
+      <c r="C172" s="22" t="n"/>
+      <c r="D172" s="22" t="n"/>
+      <c r="E172" s="22" t="n"/>
+    </row>
+    <row r="173">
+      <c r="A173" s="22" t="n"/>
+      <c r="B173" s="22" t="n"/>
+      <c r="C173" s="22" t="n"/>
+      <c r="D173" s="22" t="n"/>
+      <c r="E173" s="22" t="n"/>
+    </row>
+    <row r="174">
+      <c r="A174" s="22" t="n"/>
+      <c r="B174" s="22" t="n"/>
+      <c r="C174" s="22" t="n"/>
+      <c r="D174" s="22" t="n"/>
+      <c r="E174" s="22" t="n"/>
+    </row>
+    <row r="175">
+      <c r="A175" s="22" t="n"/>
+      <c r="B175" s="22" t="n"/>
+      <c r="C175" s="22" t="n"/>
+      <c r="D175" s="22" t="n"/>
+      <c r="E175" s="22" t="n"/>
+    </row>
+    <row r="176">
+      <c r="A176" s="22" t="n"/>
+      <c r="B176" s="22" t="n"/>
+      <c r="C176" s="22" t="n"/>
+      <c r="D176" s="22" t="n"/>
+      <c r="E176" s="22" t="n"/>
+    </row>
+    <row r="177">
+      <c r="A177" s="22" t="n"/>
+      <c r="B177" s="22" t="n"/>
+      <c r="C177" s="22" t="n"/>
+      <c r="D177" s="22" t="n"/>
+      <c r="E177" s="22" t="n"/>
+    </row>
+    <row r="178">
+      <c r="A178" s="22" t="n"/>
+      <c r="B178" s="22" t="n"/>
+      <c r="C178" s="22" t="n"/>
+      <c r="D178" s="22" t="n"/>
+      <c r="E178" s="22" t="n"/>
+    </row>
+    <row r="179">
+      <c r="A179" s="22" t="n"/>
+      <c r="B179" s="22" t="n"/>
+      <c r="C179" s="22" t="n"/>
+      <c r="D179" s="22" t="n"/>
+      <c r="E179" s="22" t="n"/>
+    </row>
+    <row r="180">
+      <c r="A180" s="22" t="n"/>
+      <c r="B180" s="22" t="n"/>
+      <c r="C180" s="22" t="n"/>
+      <c r="D180" s="22" t="n"/>
+      <c r="E180" s="22" t="n"/>
+    </row>
+    <row r="181">
+      <c r="A181" s="22" t="n"/>
+      <c r="B181" s="22" t="n"/>
+      <c r="C181" s="22" t="n"/>
+      <c r="D181" s="22" t="n"/>
+      <c r="E181" s="22" t="n"/>
+    </row>
+    <row r="182">
+      <c r="A182" s="22" t="n"/>
+      <c r="B182" s="22" t="n"/>
+      <c r="C182" s="22" t="n"/>
+      <c r="D182" s="22" t="n"/>
+      <c r="E182" s="22" t="n"/>
+    </row>
+    <row r="183">
+      <c r="A183" s="22" t="n"/>
+      <c r="B183" s="22" t="n"/>
+      <c r="C183" s="22" t="n"/>
+      <c r="D183" s="22" t="n"/>
+      <c r="E183" s="22" t="n"/>
+    </row>
+    <row r="184">
+      <c r="A184" s="22" t="n"/>
+      <c r="B184" s="22" t="n"/>
+      <c r="C184" s="22" t="n"/>
+      <c r="D184" s="22" t="n"/>
+      <c r="E184" s="22" t="n"/>
+    </row>
+    <row r="185">
+      <c r="A185" s="22" t="n"/>
+      <c r="B185" s="22" t="n"/>
+      <c r="C185" s="22" t="n"/>
+      <c r="D185" s="22" t="n"/>
+      <c r="E185" s="22" t="n"/>
+    </row>
+    <row r="186">
+      <c r="A186" s="22" t="n"/>
+      <c r="B186" s="22" t="n"/>
+      <c r="C186" s="22" t="n"/>
+      <c r="D186" s="22" t="n"/>
+      <c r="E186" s="22" t="n"/>
+    </row>
+    <row r="187">
+      <c r="A187" s="22" t="n"/>
+      <c r="B187" s="22" t="n"/>
+      <c r="C187" s="22" t="n"/>
+      <c r="D187" s="22" t="n"/>
+      <c r="E187" s="22" t="n"/>
+    </row>
+    <row r="188">
+      <c r="A188" s="22" t="n"/>
+      <c r="B188" s="22" t="n"/>
+      <c r="C188" s="22" t="n"/>
+      <c r="D188" s="22" t="n"/>
+      <c r="E188" s="22" t="n"/>
+    </row>
+    <row r="189">
+      <c r="A189" s="22" t="n"/>
+      <c r="B189" s="22" t="n"/>
+      <c r="C189" s="22" t="n"/>
+      <c r="D189" s="22" t="n"/>
+      <c r="E189" s="22" t="n"/>
+    </row>
+    <row r="190">
+      <c r="A190" s="22" t="n"/>
+      <c r="B190" s="22" t="n"/>
+      <c r="C190" s="22" t="n"/>
+      <c r="D190" s="22" t="n"/>
+      <c r="E190" s="22" t="n"/>
+    </row>
+    <row r="191">
+      <c r="A191" s="22" t="n"/>
+      <c r="B191" s="22" t="n"/>
+      <c r="C191" s="22" t="n"/>
+      <c r="D191" s="22" t="n"/>
+      <c r="E191" s="22" t="n"/>
+    </row>
+    <row r="192">
+      <c r="A192" s="22" t="n"/>
+      <c r="B192" s="22" t="n"/>
+      <c r="C192" s="22" t="n"/>
+      <c r="D192" s="22" t="n"/>
+      <c r="E192" s="22" t="n"/>
+    </row>
+    <row r="193">
+      <c r="A193" s="22" t="n"/>
+      <c r="B193" s="22" t="n"/>
+      <c r="C193" s="22" t="n"/>
+      <c r="D193" s="22" t="n"/>
+      <c r="E193" s="22" t="n"/>
+    </row>
+    <row r="194">
+      <c r="A194" s="22" t="n"/>
+      <c r="B194" s="22" t="n"/>
+      <c r="C194" s="22" t="n"/>
+      <c r="D194" s="22" t="n"/>
+      <c r="E194" s="22" t="n"/>
+    </row>
+    <row r="195">
+      <c r="A195" s="22" t="n"/>
+      <c r="B195" s="22" t="n"/>
+      <c r="C195" s="22" t="n"/>
+      <c r="D195" s="22" t="n"/>
+      <c r="E195" s="22" t="n"/>
+    </row>
+    <row r="196">
+      <c r="A196" s="22" t="n"/>
+      <c r="B196" s="22" t="n"/>
+      <c r="C196" s="22" t="n"/>
+      <c r="D196" s="22" t="n"/>
+      <c r="E196" s="22" t="n"/>
+    </row>
+    <row r="197">
+      <c r="A197" s="22" t="n"/>
+      <c r="B197" s="22" t="n"/>
+      <c r="C197" s="22" t="n"/>
+      <c r="D197" s="22" t="n"/>
+      <c r="E197" s="22" t="n"/>
+    </row>
+    <row r="198">
+      <c r="A198" s="22" t="n"/>
+      <c r="B198" s="22" t="n"/>
+      <c r="C198" s="22" t="n"/>
+      <c r="D198" s="22" t="n"/>
+      <c r="E198" s="22" t="n"/>
+    </row>
+    <row r="199">
+      <c r="A199" s="22" t="n"/>
+      <c r="B199" s="22" t="n"/>
+      <c r="C199" s="22" t="n"/>
+      <c r="D199" s="22" t="n"/>
+      <c r="E199" s="22" t="n"/>
+    </row>
+    <row r="200">
+      <c r="A200" s="22" t="n"/>
+      <c r="B200" s="22" t="n"/>
+      <c r="C200" s="22" t="n"/>
+      <c r="D200" s="22" t="n"/>
+      <c r="E200" s="22" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2563,6 +6256,89 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:A10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="110" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="23" t="inlineStr">
+        <is>
+          <t>HOW TO USE  使用方法</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="24" t="inlineStr">
+        <is>
+          <t>1. Client sheet: fill client name, income, review date. Review standard is RM1m for Life, CI, Retirement, Medical - adjust if needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="24" t="inlineStr">
+        <is>
+          <t>2. Policies sheet: one row per policy. Use the dropdowns for Type, Status, Payment Mode.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="24" t="inlineStr">
+        <is>
+          <t>3. Leave a cell BLANK if you don't know it. Never type a guess - the app flags blanks for you to confirm.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="24" t="inlineStr">
+        <is>
+          <t>4. Dashboard sheet updates automatically (Excel-only version).</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="24" t="inlineStr">
+        <is>
+          <t>5. For the visual PDF report: open 'Policy Review Snapshot.html', load this file, click 'Generate'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="24" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="24" t="inlineStr">
+        <is>
+          <t>Pink nominee cell = inforce policy without nominee recorded.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="24" t="inlineStr">
+        <is>
+          <t>Only Inforce policies count toward coverage totals. Lapsed/Paid-up are listed separately.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="24" t="inlineStr">
+        <is>
+          <t>The rows marked (sample) are fictional - delete them before using with a real client.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:A26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>

</xml_diff>

<commit_message>
Add Trust Created (Yes / No / Not sure)
- New column in the template (Z) with a dropdown; ePartner Y/N values are read
- Pick it per policy in step 5; shown on each policy card
- Discussion point for policies with a nominee where trust is No / Not sure

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Policy_Review_Template.xlsx
+++ b/Policy_Review_Template.xlsx
@@ -928,7 +928,7 @@
         </is>
       </c>
       <c r="B15" s="9">
-        <f>SUMIFS(Policies!$Z$2:$Z$100,Policies!$G$2:$G$100,"Inforce")+SUMIFS(Policies!$Z$2:$Z$100,Policies!$G$2:$G$100,"Paid-up")</f>
+        <f>SUMIFS(Policies!$AA$2:$AA$100,Policies!$G$2:$G$100,"Inforce")+SUMIFS(Policies!$AA$2:$AA$100,Policies!$G$2:$G$100,"Paid-up")</f>
         <v/>
       </c>
     </row>
@@ -1270,7 +1270,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z100"/>
+  <dimension ref="A1:AA100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1298,7 +1298,8 @@
     <col width="30" customWidth="1" min="23" max="23"/>
     <col width="28" customWidth="1" min="24" max="24"/>
     <col width="15" customWidth="1" min="25" max="25"/>
-    <col width="14" customWidth="1" min="26" max="26"/>
+    <col width="12" customWidth="1" min="26" max="26"/>
+    <col width="14" customWidth="1" min="27" max="27"/>
   </cols>
   <sheetData>
     <row r="1" ht="42" customHeight="1">
@@ -1427,7 +1428,12 @@
           <t>Retirement Fund (RM)</t>
         </is>
       </c>
-      <c r="Z1" s="19" t="inlineStr">
+      <c r="Z1" s="18" t="inlineStr">
+        <is>
+          <t>Trust Created</t>
+        </is>
+      </c>
+      <c r="AA1" s="19" t="inlineStr">
         <is>
           <t>Annual Premium (auto)</t>
         </is>
@@ -1521,7 +1527,8 @@
       </c>
       <c r="X2" s="12" t="inlineStr"/>
       <c r="Y2" s="9" t="n"/>
-      <c r="Z2" s="21">
+      <c r="Z2" s="12" t="n"/>
+      <c r="AA2" s="21">
         <f>IF(J2="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J2,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K2,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -1610,7 +1617,8 @@
         </is>
       </c>
       <c r="Y3" s="9" t="n"/>
-      <c r="Z3" s="21">
+      <c r="Z3" s="12" t="n"/>
+      <c r="AA3" s="21">
         <f>IF(J3="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J3,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K3,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -1705,7 +1713,8 @@
       </c>
       <c r="X4" s="12" t="inlineStr"/>
       <c r="Y4" s="9" t="n"/>
-      <c r="Z4" s="21">
+      <c r="Z4" s="12" t="n"/>
+      <c r="AA4" s="21">
         <f>IF(J4="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J4,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K4,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -1788,7 +1797,8 @@
         </is>
       </c>
       <c r="Y5" s="9" t="n"/>
-      <c r="Z5" s="21">
+      <c r="Z5" s="12" t="n"/>
+      <c r="AA5" s="21">
         <f>IF(J5="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J5,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K5,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -1883,7 +1893,8 @@
         </is>
       </c>
       <c r="Y6" s="9" t="n"/>
-      <c r="Z6" s="21">
+      <c r="Z6" s="12" t="n"/>
+      <c r="AA6" s="21">
         <f>IF(J6="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J6,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K6,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -1914,7 +1925,8 @@
       <c r="W7" s="12" t="n"/>
       <c r="X7" s="12" t="n"/>
       <c r="Y7" s="9" t="n"/>
-      <c r="Z7" s="21">
+      <c r="Z7" s="12" t="n"/>
+      <c r="AA7" s="21">
         <f>IF(J7="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J7,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K7,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -1945,7 +1957,8 @@
       <c r="W8" s="12" t="n"/>
       <c r="X8" s="12" t="n"/>
       <c r="Y8" s="9" t="n"/>
-      <c r="Z8" s="21">
+      <c r="Z8" s="12" t="n"/>
+      <c r="AA8" s="21">
         <f>IF(J8="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J8,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K8,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -1976,7 +1989,8 @@
       <c r="W9" s="12" t="n"/>
       <c r="X9" s="12" t="n"/>
       <c r="Y9" s="9" t="n"/>
-      <c r="Z9" s="21">
+      <c r="Z9" s="12" t="n"/>
+      <c r="AA9" s="21">
         <f>IF(J9="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J9,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K9,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2007,7 +2021,8 @@
       <c r="W10" s="12" t="n"/>
       <c r="X10" s="12" t="n"/>
       <c r="Y10" s="9" t="n"/>
-      <c r="Z10" s="21">
+      <c r="Z10" s="12" t="n"/>
+      <c r="AA10" s="21">
         <f>IF(J10="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J10,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K10,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2038,7 +2053,8 @@
       <c r="W11" s="12" t="n"/>
       <c r="X11" s="12" t="n"/>
       <c r="Y11" s="9" t="n"/>
-      <c r="Z11" s="21">
+      <c r="Z11" s="12" t="n"/>
+      <c r="AA11" s="21">
         <f>IF(J11="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J11,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K11,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2069,7 +2085,8 @@
       <c r="W12" s="12" t="n"/>
       <c r="X12" s="12" t="n"/>
       <c r="Y12" s="9" t="n"/>
-      <c r="Z12" s="21">
+      <c r="Z12" s="12" t="n"/>
+      <c r="AA12" s="21">
         <f>IF(J12="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J12,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K12,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2100,7 +2117,8 @@
       <c r="W13" s="12" t="n"/>
       <c r="X13" s="12" t="n"/>
       <c r="Y13" s="9" t="n"/>
-      <c r="Z13" s="21">
+      <c r="Z13" s="12" t="n"/>
+      <c r="AA13" s="21">
         <f>IF(J13="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J13,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K13,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2131,7 +2149,8 @@
       <c r="W14" s="12" t="n"/>
       <c r="X14" s="12" t="n"/>
       <c r="Y14" s="9" t="n"/>
-      <c r="Z14" s="21">
+      <c r="Z14" s="12" t="n"/>
+      <c r="AA14" s="21">
         <f>IF(J14="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J14,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K14,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2162,7 +2181,8 @@
       <c r="W15" s="12" t="n"/>
       <c r="X15" s="12" t="n"/>
       <c r="Y15" s="9" t="n"/>
-      <c r="Z15" s="21">
+      <c r="Z15" s="12" t="n"/>
+      <c r="AA15" s="21">
         <f>IF(J15="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J15,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K15,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2193,7 +2213,8 @@
       <c r="W16" s="12" t="n"/>
       <c r="X16" s="12" t="n"/>
       <c r="Y16" s="9" t="n"/>
-      <c r="Z16" s="21">
+      <c r="Z16" s="12" t="n"/>
+      <c r="AA16" s="21">
         <f>IF(J16="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J16,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K16,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2224,7 +2245,8 @@
       <c r="W17" s="12" t="n"/>
       <c r="X17" s="12" t="n"/>
       <c r="Y17" s="9" t="n"/>
-      <c r="Z17" s="21">
+      <c r="Z17" s="12" t="n"/>
+      <c r="AA17" s="21">
         <f>IF(J17="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J17,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K17,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2255,7 +2277,8 @@
       <c r="W18" s="12" t="n"/>
       <c r="X18" s="12" t="n"/>
       <c r="Y18" s="9" t="n"/>
-      <c r="Z18" s="21">
+      <c r="Z18" s="12" t="n"/>
+      <c r="AA18" s="21">
         <f>IF(J18="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J18,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K18,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2286,7 +2309,8 @@
       <c r="W19" s="12" t="n"/>
       <c r="X19" s="12" t="n"/>
       <c r="Y19" s="9" t="n"/>
-      <c r="Z19" s="21">
+      <c r="Z19" s="12" t="n"/>
+      <c r="AA19" s="21">
         <f>IF(J19="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J19,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K19,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2317,7 +2341,8 @@
       <c r="W20" s="12" t="n"/>
       <c r="X20" s="12" t="n"/>
       <c r="Y20" s="9" t="n"/>
-      <c r="Z20" s="21">
+      <c r="Z20" s="12" t="n"/>
+      <c r="AA20" s="21">
         <f>IF(J20="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J20,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K20,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2348,7 +2373,8 @@
       <c r="W21" s="12" t="n"/>
       <c r="X21" s="12" t="n"/>
       <c r="Y21" s="9" t="n"/>
-      <c r="Z21" s="21">
+      <c r="Z21" s="12" t="n"/>
+      <c r="AA21" s="21">
         <f>IF(J21="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J21,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K21,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2379,7 +2405,8 @@
       <c r="W22" s="12" t="n"/>
       <c r="X22" s="12" t="n"/>
       <c r="Y22" s="9" t="n"/>
-      <c r="Z22" s="21">
+      <c r="Z22" s="12" t="n"/>
+      <c r="AA22" s="21">
         <f>IF(J22="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J22,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K22,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2410,7 +2437,8 @@
       <c r="W23" s="12" t="n"/>
       <c r="X23" s="12" t="n"/>
       <c r="Y23" s="9" t="n"/>
-      <c r="Z23" s="21">
+      <c r="Z23" s="12" t="n"/>
+      <c r="AA23" s="21">
         <f>IF(J23="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J23,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K23,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2441,7 +2469,8 @@
       <c r="W24" s="12" t="n"/>
       <c r="X24" s="12" t="n"/>
       <c r="Y24" s="9" t="n"/>
-      <c r="Z24" s="21">
+      <c r="Z24" s="12" t="n"/>
+      <c r="AA24" s="21">
         <f>IF(J24="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J24,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K24,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2472,7 +2501,8 @@
       <c r="W25" s="12" t="n"/>
       <c r="X25" s="12" t="n"/>
       <c r="Y25" s="9" t="n"/>
-      <c r="Z25" s="21">
+      <c r="Z25" s="12" t="n"/>
+      <c r="AA25" s="21">
         <f>IF(J25="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J25,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K25,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2503,7 +2533,8 @@
       <c r="W26" s="12" t="n"/>
       <c r="X26" s="12" t="n"/>
       <c r="Y26" s="9" t="n"/>
-      <c r="Z26" s="21">
+      <c r="Z26" s="12" t="n"/>
+      <c r="AA26" s="21">
         <f>IF(J26="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J26,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K26,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2534,7 +2565,8 @@
       <c r="W27" s="12" t="n"/>
       <c r="X27" s="12" t="n"/>
       <c r="Y27" s="9" t="n"/>
-      <c r="Z27" s="21">
+      <c r="Z27" s="12" t="n"/>
+      <c r="AA27" s="21">
         <f>IF(J27="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J27,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K27,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2565,7 +2597,8 @@
       <c r="W28" s="12" t="n"/>
       <c r="X28" s="12" t="n"/>
       <c r="Y28" s="9" t="n"/>
-      <c r="Z28" s="21">
+      <c r="Z28" s="12" t="n"/>
+      <c r="AA28" s="21">
         <f>IF(J28="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J28,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K28,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2596,7 +2629,8 @@
       <c r="W29" s="12" t="n"/>
       <c r="X29" s="12" t="n"/>
       <c r="Y29" s="9" t="n"/>
-      <c r="Z29" s="21">
+      <c r="Z29" s="12" t="n"/>
+      <c r="AA29" s="21">
         <f>IF(J29="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J29,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K29,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2627,7 +2661,8 @@
       <c r="W30" s="12" t="n"/>
       <c r="X30" s="12" t="n"/>
       <c r="Y30" s="9" t="n"/>
-      <c r="Z30" s="21">
+      <c r="Z30" s="12" t="n"/>
+      <c r="AA30" s="21">
         <f>IF(J30="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J30,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K30,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2658,7 +2693,8 @@
       <c r="W31" s="12" t="n"/>
       <c r="X31" s="12" t="n"/>
       <c r="Y31" s="9" t="n"/>
-      <c r="Z31" s="21">
+      <c r="Z31" s="12" t="n"/>
+      <c r="AA31" s="21">
         <f>IF(J31="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J31,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K31,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2689,7 +2725,8 @@
       <c r="W32" s="12" t="n"/>
       <c r="X32" s="12" t="n"/>
       <c r="Y32" s="9" t="n"/>
-      <c r="Z32" s="21">
+      <c r="Z32" s="12" t="n"/>
+      <c r="AA32" s="21">
         <f>IF(J32="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J32,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K32,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2720,7 +2757,8 @@
       <c r="W33" s="12" t="n"/>
       <c r="X33" s="12" t="n"/>
       <c r="Y33" s="9" t="n"/>
-      <c r="Z33" s="21">
+      <c r="Z33" s="12" t="n"/>
+      <c r="AA33" s="21">
         <f>IF(J33="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J33,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K33,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2751,7 +2789,8 @@
       <c r="W34" s="12" t="n"/>
       <c r="X34" s="12" t="n"/>
       <c r="Y34" s="9" t="n"/>
-      <c r="Z34" s="21">
+      <c r="Z34" s="12" t="n"/>
+      <c r="AA34" s="21">
         <f>IF(J34="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J34,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K34,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2782,7 +2821,8 @@
       <c r="W35" s="12" t="n"/>
       <c r="X35" s="12" t="n"/>
       <c r="Y35" s="9" t="n"/>
-      <c r="Z35" s="21">
+      <c r="Z35" s="12" t="n"/>
+      <c r="AA35" s="21">
         <f>IF(J35="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J35,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K35,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2813,7 +2853,8 @@
       <c r="W36" s="12" t="n"/>
       <c r="X36" s="12" t="n"/>
       <c r="Y36" s="9" t="n"/>
-      <c r="Z36" s="21">
+      <c r="Z36" s="12" t="n"/>
+      <c r="AA36" s="21">
         <f>IF(J36="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J36,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K36,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2844,7 +2885,8 @@
       <c r="W37" s="12" t="n"/>
       <c r="X37" s="12" t="n"/>
       <c r="Y37" s="9" t="n"/>
-      <c r="Z37" s="21">
+      <c r="Z37" s="12" t="n"/>
+      <c r="AA37" s="21">
         <f>IF(J37="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J37,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K37,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2875,7 +2917,8 @@
       <c r="W38" s="12" t="n"/>
       <c r="X38" s="12" t="n"/>
       <c r="Y38" s="9" t="n"/>
-      <c r="Z38" s="21">
+      <c r="Z38" s="12" t="n"/>
+      <c r="AA38" s="21">
         <f>IF(J38="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J38,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K38,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2906,7 +2949,8 @@
       <c r="W39" s="12" t="n"/>
       <c r="X39" s="12" t="n"/>
       <c r="Y39" s="9" t="n"/>
-      <c r="Z39" s="21">
+      <c r="Z39" s="12" t="n"/>
+      <c r="AA39" s="21">
         <f>IF(J39="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J39,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K39,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2937,7 +2981,8 @@
       <c r="W40" s="12" t="n"/>
       <c r="X40" s="12" t="n"/>
       <c r="Y40" s="9" t="n"/>
-      <c r="Z40" s="21">
+      <c r="Z40" s="12" t="n"/>
+      <c r="AA40" s="21">
         <f>IF(J40="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J40,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K40,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2968,7 +3013,8 @@
       <c r="W41" s="12" t="n"/>
       <c r="X41" s="12" t="n"/>
       <c r="Y41" s="9" t="n"/>
-      <c r="Z41" s="21">
+      <c r="Z41" s="12" t="n"/>
+      <c r="AA41" s="21">
         <f>IF(J41="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J41,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K41,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2999,7 +3045,8 @@
       <c r="W42" s="12" t="n"/>
       <c r="X42" s="12" t="n"/>
       <c r="Y42" s="9" t="n"/>
-      <c r="Z42" s="21">
+      <c r="Z42" s="12" t="n"/>
+      <c r="AA42" s="21">
         <f>IF(J42="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J42,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K42,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3030,7 +3077,8 @@
       <c r="W43" s="12" t="n"/>
       <c r="X43" s="12" t="n"/>
       <c r="Y43" s="9" t="n"/>
-      <c r="Z43" s="21">
+      <c r="Z43" s="12" t="n"/>
+      <c r="AA43" s="21">
         <f>IF(J43="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J43,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K43,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3061,7 +3109,8 @@
       <c r="W44" s="12" t="n"/>
       <c r="X44" s="12" t="n"/>
       <c r="Y44" s="9" t="n"/>
-      <c r="Z44" s="21">
+      <c r="Z44" s="12" t="n"/>
+      <c r="AA44" s="21">
         <f>IF(J44="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J44,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K44,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3092,7 +3141,8 @@
       <c r="W45" s="12" t="n"/>
       <c r="X45" s="12" t="n"/>
       <c r="Y45" s="9" t="n"/>
-      <c r="Z45" s="21">
+      <c r="Z45" s="12" t="n"/>
+      <c r="AA45" s="21">
         <f>IF(J45="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J45,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K45,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3123,7 +3173,8 @@
       <c r="W46" s="12" t="n"/>
       <c r="X46" s="12" t="n"/>
       <c r="Y46" s="9" t="n"/>
-      <c r="Z46" s="21">
+      <c r="Z46" s="12" t="n"/>
+      <c r="AA46" s="21">
         <f>IF(J46="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J46,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K46,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3154,7 +3205,8 @@
       <c r="W47" s="12" t="n"/>
       <c r="X47" s="12" t="n"/>
       <c r="Y47" s="9" t="n"/>
-      <c r="Z47" s="21">
+      <c r="Z47" s="12" t="n"/>
+      <c r="AA47" s="21">
         <f>IF(J47="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J47,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K47,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3185,7 +3237,8 @@
       <c r="W48" s="12" t="n"/>
       <c r="X48" s="12" t="n"/>
       <c r="Y48" s="9" t="n"/>
-      <c r="Z48" s="21">
+      <c r="Z48" s="12" t="n"/>
+      <c r="AA48" s="21">
         <f>IF(J48="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J48,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K48,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3216,7 +3269,8 @@
       <c r="W49" s="12" t="n"/>
       <c r="X49" s="12" t="n"/>
       <c r="Y49" s="9" t="n"/>
-      <c r="Z49" s="21">
+      <c r="Z49" s="12" t="n"/>
+      <c r="AA49" s="21">
         <f>IF(J49="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J49,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K49,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3247,7 +3301,8 @@
       <c r="W50" s="12" t="n"/>
       <c r="X50" s="12" t="n"/>
       <c r="Y50" s="9" t="n"/>
-      <c r="Z50" s="21">
+      <c r="Z50" s="12" t="n"/>
+      <c r="AA50" s="21">
         <f>IF(J50="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J50,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K50,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3278,7 +3333,8 @@
       <c r="W51" s="12" t="n"/>
       <c r="X51" s="12" t="n"/>
       <c r="Y51" s="9" t="n"/>
-      <c r="Z51" s="21">
+      <c r="Z51" s="12" t="n"/>
+      <c r="AA51" s="21">
         <f>IF(J51="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J51,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K51,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3309,7 +3365,8 @@
       <c r="W52" s="12" t="n"/>
       <c r="X52" s="12" t="n"/>
       <c r="Y52" s="9" t="n"/>
-      <c r="Z52" s="21">
+      <c r="Z52" s="12" t="n"/>
+      <c r="AA52" s="21">
         <f>IF(J52="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J52,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K52,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3340,7 +3397,8 @@
       <c r="W53" s="12" t="n"/>
       <c r="X53" s="12" t="n"/>
       <c r="Y53" s="9" t="n"/>
-      <c r="Z53" s="21">
+      <c r="Z53" s="12" t="n"/>
+      <c r="AA53" s="21">
         <f>IF(J53="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J53,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K53,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3371,7 +3429,8 @@
       <c r="W54" s="12" t="n"/>
       <c r="X54" s="12" t="n"/>
       <c r="Y54" s="9" t="n"/>
-      <c r="Z54" s="21">
+      <c r="Z54" s="12" t="n"/>
+      <c r="AA54" s="21">
         <f>IF(J54="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J54,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K54,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3402,7 +3461,8 @@
       <c r="W55" s="12" t="n"/>
       <c r="X55" s="12" t="n"/>
       <c r="Y55" s="9" t="n"/>
-      <c r="Z55" s="21">
+      <c r="Z55" s="12" t="n"/>
+      <c r="AA55" s="21">
         <f>IF(J55="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J55,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K55,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3433,7 +3493,8 @@
       <c r="W56" s="12" t="n"/>
       <c r="X56" s="12" t="n"/>
       <c r="Y56" s="9" t="n"/>
-      <c r="Z56" s="21">
+      <c r="Z56" s="12" t="n"/>
+      <c r="AA56" s="21">
         <f>IF(J56="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J56,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K56,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3464,7 +3525,8 @@
       <c r="W57" s="12" t="n"/>
       <c r="X57" s="12" t="n"/>
       <c r="Y57" s="9" t="n"/>
-      <c r="Z57" s="21">
+      <c r="Z57" s="12" t="n"/>
+      <c r="AA57" s="21">
         <f>IF(J57="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J57,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K57,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3495,7 +3557,8 @@
       <c r="W58" s="12" t="n"/>
       <c r="X58" s="12" t="n"/>
       <c r="Y58" s="9" t="n"/>
-      <c r="Z58" s="21">
+      <c r="Z58" s="12" t="n"/>
+      <c r="AA58" s="21">
         <f>IF(J58="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J58,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K58,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3526,7 +3589,8 @@
       <c r="W59" s="12" t="n"/>
       <c r="X59" s="12" t="n"/>
       <c r="Y59" s="9" t="n"/>
-      <c r="Z59" s="21">
+      <c r="Z59" s="12" t="n"/>
+      <c r="AA59" s="21">
         <f>IF(J59="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J59,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K59,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3557,7 +3621,8 @@
       <c r="W60" s="12" t="n"/>
       <c r="X60" s="12" t="n"/>
       <c r="Y60" s="9" t="n"/>
-      <c r="Z60" s="21">
+      <c r="Z60" s="12" t="n"/>
+      <c r="AA60" s="21">
         <f>IF(J60="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J60,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K60,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3588,7 +3653,8 @@
       <c r="W61" s="12" t="n"/>
       <c r="X61" s="12" t="n"/>
       <c r="Y61" s="9" t="n"/>
-      <c r="Z61" s="21">
+      <c r="Z61" s="12" t="n"/>
+      <c r="AA61" s="21">
         <f>IF(J61="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J61,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K61,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3619,7 +3685,8 @@
       <c r="W62" s="12" t="n"/>
       <c r="X62" s="12" t="n"/>
       <c r="Y62" s="9" t="n"/>
-      <c r="Z62" s="21">
+      <c r="Z62" s="12" t="n"/>
+      <c r="AA62" s="21">
         <f>IF(J62="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J62,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K62,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3650,7 +3717,8 @@
       <c r="W63" s="12" t="n"/>
       <c r="X63" s="12" t="n"/>
       <c r="Y63" s="9" t="n"/>
-      <c r="Z63" s="21">
+      <c r="Z63" s="12" t="n"/>
+      <c r="AA63" s="21">
         <f>IF(J63="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J63,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K63,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3681,7 +3749,8 @@
       <c r="W64" s="12" t="n"/>
       <c r="X64" s="12" t="n"/>
       <c r="Y64" s="9" t="n"/>
-      <c r="Z64" s="21">
+      <c r="Z64" s="12" t="n"/>
+      <c r="AA64" s="21">
         <f>IF(J64="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J64,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K64,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3712,7 +3781,8 @@
       <c r="W65" s="12" t="n"/>
       <c r="X65" s="12" t="n"/>
       <c r="Y65" s="9" t="n"/>
-      <c r="Z65" s="21">
+      <c r="Z65" s="12" t="n"/>
+      <c r="AA65" s="21">
         <f>IF(J65="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J65,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K65,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3743,7 +3813,8 @@
       <c r="W66" s="12" t="n"/>
       <c r="X66" s="12" t="n"/>
       <c r="Y66" s="9" t="n"/>
-      <c r="Z66" s="21">
+      <c r="Z66" s="12" t="n"/>
+      <c r="AA66" s="21">
         <f>IF(J66="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J66,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K66,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3774,7 +3845,8 @@
       <c r="W67" s="12" t="n"/>
       <c r="X67" s="12" t="n"/>
       <c r="Y67" s="9" t="n"/>
-      <c r="Z67" s="21">
+      <c r="Z67" s="12" t="n"/>
+      <c r="AA67" s="21">
         <f>IF(J67="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J67,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K67,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3805,7 +3877,8 @@
       <c r="W68" s="12" t="n"/>
       <c r="X68" s="12" t="n"/>
       <c r="Y68" s="9" t="n"/>
-      <c r="Z68" s="21">
+      <c r="Z68" s="12" t="n"/>
+      <c r="AA68" s="21">
         <f>IF(J68="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J68,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K68,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3836,7 +3909,8 @@
       <c r="W69" s="12" t="n"/>
       <c r="X69" s="12" t="n"/>
       <c r="Y69" s="9" t="n"/>
-      <c r="Z69" s="21">
+      <c r="Z69" s="12" t="n"/>
+      <c r="AA69" s="21">
         <f>IF(J69="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J69,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K69,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3867,7 +3941,8 @@
       <c r="W70" s="12" t="n"/>
       <c r="X70" s="12" t="n"/>
       <c r="Y70" s="9" t="n"/>
-      <c r="Z70" s="21">
+      <c r="Z70" s="12" t="n"/>
+      <c r="AA70" s="21">
         <f>IF(J70="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J70,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K70,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3898,7 +3973,8 @@
       <c r="W71" s="12" t="n"/>
       <c r="X71" s="12" t="n"/>
       <c r="Y71" s="9" t="n"/>
-      <c r="Z71" s="21">
+      <c r="Z71" s="12" t="n"/>
+      <c r="AA71" s="21">
         <f>IF(J71="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J71,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K71,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3929,7 +4005,8 @@
       <c r="W72" s="12" t="n"/>
       <c r="X72" s="12" t="n"/>
       <c r="Y72" s="9" t="n"/>
-      <c r="Z72" s="21">
+      <c r="Z72" s="12" t="n"/>
+      <c r="AA72" s="21">
         <f>IF(J72="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J72,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K72,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3960,7 +4037,8 @@
       <c r="W73" s="12" t="n"/>
       <c r="X73" s="12" t="n"/>
       <c r="Y73" s="9" t="n"/>
-      <c r="Z73" s="21">
+      <c r="Z73" s="12" t="n"/>
+      <c r="AA73" s="21">
         <f>IF(J73="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J73,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K73,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3991,7 +4069,8 @@
       <c r="W74" s="12" t="n"/>
       <c r="X74" s="12" t="n"/>
       <c r="Y74" s="9" t="n"/>
-      <c r="Z74" s="21">
+      <c r="Z74" s="12" t="n"/>
+      <c r="AA74" s="21">
         <f>IF(J74="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J74,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K74,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -4022,7 +4101,8 @@
       <c r="W75" s="12" t="n"/>
       <c r="X75" s="12" t="n"/>
       <c r="Y75" s="9" t="n"/>
-      <c r="Z75" s="21">
+      <c r="Z75" s="12" t="n"/>
+      <c r="AA75" s="21">
         <f>IF(J75="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J75,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K75,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -4053,7 +4133,8 @@
       <c r="W76" s="12" t="n"/>
       <c r="X76" s="12" t="n"/>
       <c r="Y76" s="9" t="n"/>
-      <c r="Z76" s="21">
+      <c r="Z76" s="12" t="n"/>
+      <c r="AA76" s="21">
         <f>IF(J76="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J76,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K76,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -4084,7 +4165,8 @@
       <c r="W77" s="12" t="n"/>
       <c r="X77" s="12" t="n"/>
       <c r="Y77" s="9" t="n"/>
-      <c r="Z77" s="21">
+      <c r="Z77" s="12" t="n"/>
+      <c r="AA77" s="21">
         <f>IF(J77="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J77,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K77,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -4115,7 +4197,8 @@
       <c r="W78" s="12" t="n"/>
       <c r="X78" s="12" t="n"/>
       <c r="Y78" s="9" t="n"/>
-      <c r="Z78" s="21">
+      <c r="Z78" s="12" t="n"/>
+      <c r="AA78" s="21">
         <f>IF(J78="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J78,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K78,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -4146,7 +4229,8 @@
       <c r="W79" s="12" t="n"/>
       <c r="X79" s="12" t="n"/>
       <c r="Y79" s="9" t="n"/>
-      <c r="Z79" s="21">
+      <c r="Z79" s="12" t="n"/>
+      <c r="AA79" s="21">
         <f>IF(J79="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J79,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K79,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -4177,7 +4261,8 @@
       <c r="W80" s="12" t="n"/>
       <c r="X80" s="12" t="n"/>
       <c r="Y80" s="9" t="n"/>
-      <c r="Z80" s="21">
+      <c r="Z80" s="12" t="n"/>
+      <c r="AA80" s="21">
         <f>IF(J80="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J80,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K80,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -4208,7 +4293,8 @@
       <c r="W81" s="12" t="n"/>
       <c r="X81" s="12" t="n"/>
       <c r="Y81" s="9" t="n"/>
-      <c r="Z81" s="21">
+      <c r="Z81" s="12" t="n"/>
+      <c r="AA81" s="21">
         <f>IF(J81="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J81,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K81,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -4239,7 +4325,8 @@
       <c r="W82" s="12" t="n"/>
       <c r="X82" s="12" t="n"/>
       <c r="Y82" s="9" t="n"/>
-      <c r="Z82" s="21">
+      <c r="Z82" s="12" t="n"/>
+      <c r="AA82" s="21">
         <f>IF(J82="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J82,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K82,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -4270,7 +4357,8 @@
       <c r="W83" s="12" t="n"/>
       <c r="X83" s="12" t="n"/>
       <c r="Y83" s="9" t="n"/>
-      <c r="Z83" s="21">
+      <c r="Z83" s="12" t="n"/>
+      <c r="AA83" s="21">
         <f>IF(J83="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J83,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K83,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -4301,7 +4389,8 @@
       <c r="W84" s="12" t="n"/>
       <c r="X84" s="12" t="n"/>
       <c r="Y84" s="9" t="n"/>
-      <c r="Z84" s="21">
+      <c r="Z84" s="12" t="n"/>
+      <c r="AA84" s="21">
         <f>IF(J84="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J84,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K84,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -4332,7 +4421,8 @@
       <c r="W85" s="12" t="n"/>
       <c r="X85" s="12" t="n"/>
       <c r="Y85" s="9" t="n"/>
-      <c r="Z85" s="21">
+      <c r="Z85" s="12" t="n"/>
+      <c r="AA85" s="21">
         <f>IF(J85="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J85,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K85,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -4363,7 +4453,8 @@
       <c r="W86" s="12" t="n"/>
       <c r="X86" s="12" t="n"/>
       <c r="Y86" s="9" t="n"/>
-      <c r="Z86" s="21">
+      <c r="Z86" s="12" t="n"/>
+      <c r="AA86" s="21">
         <f>IF(J86="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J86,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K86,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -4394,7 +4485,8 @@
       <c r="W87" s="12" t="n"/>
       <c r="X87" s="12" t="n"/>
       <c r="Y87" s="9" t="n"/>
-      <c r="Z87" s="21">
+      <c r="Z87" s="12" t="n"/>
+      <c r="AA87" s="21">
         <f>IF(J87="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J87,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K87,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -4425,7 +4517,8 @@
       <c r="W88" s="12" t="n"/>
       <c r="X88" s="12" t="n"/>
       <c r="Y88" s="9" t="n"/>
-      <c r="Z88" s="21">
+      <c r="Z88" s="12" t="n"/>
+      <c r="AA88" s="21">
         <f>IF(J88="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J88,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K88,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -4456,7 +4549,8 @@
       <c r="W89" s="12" t="n"/>
       <c r="X89" s="12" t="n"/>
       <c r="Y89" s="9" t="n"/>
-      <c r="Z89" s="21">
+      <c r="Z89" s="12" t="n"/>
+      <c r="AA89" s="21">
         <f>IF(J89="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J89,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K89,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -4487,7 +4581,8 @@
       <c r="W90" s="12" t="n"/>
       <c r="X90" s="12" t="n"/>
       <c r="Y90" s="9" t="n"/>
-      <c r="Z90" s="21">
+      <c r="Z90" s="12" t="n"/>
+      <c r="AA90" s="21">
         <f>IF(J90="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J90,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K90,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -4518,7 +4613,8 @@
       <c r="W91" s="12" t="n"/>
       <c r="X91" s="12" t="n"/>
       <c r="Y91" s="9" t="n"/>
-      <c r="Z91" s="21">
+      <c r="Z91" s="12" t="n"/>
+      <c r="AA91" s="21">
         <f>IF(J91="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J91,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K91,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -4549,7 +4645,8 @@
       <c r="W92" s="12" t="n"/>
       <c r="X92" s="12" t="n"/>
       <c r="Y92" s="9" t="n"/>
-      <c r="Z92" s="21">
+      <c r="Z92" s="12" t="n"/>
+      <c r="AA92" s="21">
         <f>IF(J92="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J92,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K92,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -4580,7 +4677,8 @@
       <c r="W93" s="12" t="n"/>
       <c r="X93" s="12" t="n"/>
       <c r="Y93" s="9" t="n"/>
-      <c r="Z93" s="21">
+      <c r="Z93" s="12" t="n"/>
+      <c r="AA93" s="21">
         <f>IF(J93="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J93,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K93,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -4611,7 +4709,8 @@
       <c r="W94" s="12" t="n"/>
       <c r="X94" s="12" t="n"/>
       <c r="Y94" s="9" t="n"/>
-      <c r="Z94" s="21">
+      <c r="Z94" s="12" t="n"/>
+      <c r="AA94" s="21">
         <f>IF(J94="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J94,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K94,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -4642,7 +4741,8 @@
       <c r="W95" s="12" t="n"/>
       <c r="X95" s="12" t="n"/>
       <c r="Y95" s="9" t="n"/>
-      <c r="Z95" s="21">
+      <c r="Z95" s="12" t="n"/>
+      <c r="AA95" s="21">
         <f>IF(J95="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J95,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K95,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -4673,7 +4773,8 @@
       <c r="W96" s="12" t="n"/>
       <c r="X96" s="12" t="n"/>
       <c r="Y96" s="9" t="n"/>
-      <c r="Z96" s="21">
+      <c r="Z96" s="12" t="n"/>
+      <c r="AA96" s="21">
         <f>IF(J96="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J96,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K96,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -4704,7 +4805,8 @@
       <c r="W97" s="12" t="n"/>
       <c r="X97" s="12" t="n"/>
       <c r="Y97" s="9" t="n"/>
-      <c r="Z97" s="21">
+      <c r="Z97" s="12" t="n"/>
+      <c r="AA97" s="21">
         <f>IF(J97="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J97,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K97,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -4735,7 +4837,8 @@
       <c r="W98" s="12" t="n"/>
       <c r="X98" s="12" t="n"/>
       <c r="Y98" s="9" t="n"/>
-      <c r="Z98" s="21">
+      <c r="Z98" s="12" t="n"/>
+      <c r="AA98" s="21">
         <f>IF(J98="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J98,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K98,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -4766,7 +4869,8 @@
       <c r="W99" s="12" t="n"/>
       <c r="X99" s="12" t="n"/>
       <c r="Y99" s="9" t="n"/>
-      <c r="Z99" s="21">
+      <c r="Z99" s="12" t="n"/>
+      <c r="AA99" s="21">
         <f>IF(J99="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J99,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K99,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -4797,7 +4901,8 @@
       <c r="W100" s="12" t="n"/>
       <c r="X100" s="12" t="n"/>
       <c r="Y100" s="9" t="n"/>
-      <c r="Z100" s="21">
+      <c r="Z100" s="12" t="n"/>
+      <c r="AA100" s="21">
         <f>IF(J100="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J100,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K100,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -4808,7 +4913,7 @@
       <formula>AND($G2="Inforce",$T2="",$A2&lt;&gt;"")</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="7">
+  <dataValidations count="8">
     <dataValidation sqref="D2:D100" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Whole Life,Term Life,Investment-Linked,Medical,Critical Illness,Personal Accident,Endowment / Savings,Other"</formula1>
     </dataValidation>
@@ -4823,6 +4928,9 @@
     </dataValidation>
     <dataValidation sqref="V2:V100" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Beneficiary,Hibah,Trustee,Conditional Hibah,None"</formula1>
+    </dataValidation>
+    <dataValidation sqref="Z2:Z100" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Yes,No,Not sure"</formula1>
     </dataValidation>
     <dataValidation sqref="W2:W100" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Family income protection,Medical &amp; hospital bills,Critical illness recovery,Retirement,Children's education,Savings &amp; wealth,Mortgage / loan protection,Estate &amp; legacy,Accident cover,Business protection"</formula1>

</xml_diff>

<commit_message>
Client phone, birthday and family members (not on report)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Policy_Review_Template.xlsx
+++ b/Policy_Review_Template.xlsx
@@ -124,7 +124,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -147,13 +147,16 @@
     <xf numFmtId="164" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="9" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="49" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -1029,12 +1032,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C22"/>
+  <dimension ref="A1:E45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
     <col width="26" customWidth="1" min="2" max="2"/>
     <col width="40" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1258,7 +1263,185 @@
         </is>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" s="10" t="inlineStr">
+        <is>
+          <t>Contact  联络资料</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>Phone  电话</t>
+        </is>
+      </c>
+      <c r="B25" s="18" t="n"/>
+      <c r="C25" s="16" t="inlineStr">
+        <is>
+          <t>Not shown on the client report</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>Date of birth  生日</t>
+        </is>
+      </c>
+      <c r="B26" s="15" t="n"/>
+      <c r="C26" s="16" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="10" t="inlineStr">
+        <is>
+          <t>Family members  家人</t>
+        </is>
+      </c>
+      <c r="C29" s="16" t="inlineStr">
+        <is>
+          <t>For birthdays and follow-up. Not shown on the client report.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="19" t="inlineStr">
+        <is>
+          <t>Name  姓名</t>
+        </is>
+      </c>
+      <c r="B30" s="19" t="inlineStr">
+        <is>
+          <t>Relationship  关系</t>
+        </is>
+      </c>
+      <c r="C30" s="19" t="inlineStr">
+        <is>
+          <t>Birthday  生日</t>
+        </is>
+      </c>
+      <c r="D30" s="19" t="inlineStr">
+        <is>
+          <t>Phone  电话</t>
+        </is>
+      </c>
+      <c r="E30" s="19" t="inlineStr">
+        <is>
+          <t>Notes  备注</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="12" t="n"/>
+      <c r="B31" s="12" t="n"/>
+      <c r="C31" s="20" t="n"/>
+      <c r="D31" s="21" t="n"/>
+      <c r="E31" s="12" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="12" t="n"/>
+      <c r="B32" s="12" t="n"/>
+      <c r="C32" s="20" t="n"/>
+      <c r="D32" s="21" t="n"/>
+      <c r="E32" s="12" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="12" t="n"/>
+      <c r="B33" s="12" t="n"/>
+      <c r="C33" s="20" t="n"/>
+      <c r="D33" s="21" t="n"/>
+      <c r="E33" s="12" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="12" t="n"/>
+      <c r="B34" s="12" t="n"/>
+      <c r="C34" s="20" t="n"/>
+      <c r="D34" s="21" t="n"/>
+      <c r="E34" s="12" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="12" t="n"/>
+      <c r="B35" s="12" t="n"/>
+      <c r="C35" s="20" t="n"/>
+      <c r="D35" s="21" t="n"/>
+      <c r="E35" s="12" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="12" t="n"/>
+      <c r="B36" s="12" t="n"/>
+      <c r="C36" s="20" t="n"/>
+      <c r="D36" s="21" t="n"/>
+      <c r="E36" s="12" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="12" t="n"/>
+      <c r="B37" s="12" t="n"/>
+      <c r="C37" s="20" t="n"/>
+      <c r="D37" s="21" t="n"/>
+      <c r="E37" s="12" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="12" t="n"/>
+      <c r="B38" s="12" t="n"/>
+      <c r="C38" s="20" t="n"/>
+      <c r="D38" s="21" t="n"/>
+      <c r="E38" s="12" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="12" t="n"/>
+      <c r="B39" s="12" t="n"/>
+      <c r="C39" s="20" t="n"/>
+      <c r="D39" s="21" t="n"/>
+      <c r="E39" s="12" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="12" t="n"/>
+      <c r="B40" s="12" t="n"/>
+      <c r="C40" s="20" t="n"/>
+      <c r="D40" s="21" t="n"/>
+      <c r="E40" s="12" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="12" t="n"/>
+      <c r="B41" s="12" t="n"/>
+      <c r="C41" s="20" t="n"/>
+      <c r="D41" s="21" t="n"/>
+      <c r="E41" s="12" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="12" t="n"/>
+      <c r="B42" s="12" t="n"/>
+      <c r="C42" s="20" t="n"/>
+      <c r="D42" s="21" t="n"/>
+      <c r="E42" s="12" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="12" t="n"/>
+      <c r="B43" s="12" t="n"/>
+      <c r="C43" s="20" t="n"/>
+      <c r="D43" s="21" t="n"/>
+      <c r="E43" s="12" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="12" t="n"/>
+      <c r="B44" s="12" t="n"/>
+      <c r="C44" s="20" t="n"/>
+      <c r="D44" s="21" t="n"/>
+      <c r="E44" s="12" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="12" t="n"/>
+      <c r="B45" s="12" t="n"/>
+      <c r="C45" s="20" t="n"/>
+      <c r="D45" s="21" t="n"/>
+      <c r="E45" s="12" t="n"/>
+    </row>
   </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="B31 B32 B33 B34 B35 B36 B37 B38 B39 B40 B41 B42 B43 B44 B45" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Spouse 配偶,Son 儿子,Daughter 女儿,Father 父亲,Mother 母亲,Brother 兄弟,Sister 姐妹,Other 其他"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1303,137 +1486,137 @@
   </cols>
   <sheetData>
     <row r="1" ht="42" customHeight="1">
-      <c r="A1" s="18" t="inlineStr">
+      <c r="A1" s="22" t="inlineStr">
         <is>
           <t>Policy No</t>
         </is>
       </c>
-      <c r="B1" s="18" t="inlineStr">
+      <c r="B1" s="22" t="inlineStr">
         <is>
           <t>Insurer</t>
         </is>
       </c>
-      <c r="C1" s="18" t="inlineStr">
+      <c r="C1" s="22" t="inlineStr">
         <is>
           <t>Plan Name</t>
         </is>
       </c>
-      <c r="D1" s="18" t="inlineStr">
+      <c r="D1" s="22" t="inlineStr">
         <is>
           <t>Policy Type</t>
         </is>
       </c>
-      <c r="E1" s="18" t="inlineStr">
+      <c r="E1" s="22" t="inlineStr">
         <is>
           <t>Life Assured</t>
         </is>
       </c>
-      <c r="F1" s="18" t="inlineStr">
+      <c r="F1" s="22" t="inlineStr">
         <is>
           <t>Policy Owner</t>
         </is>
       </c>
-      <c r="G1" s="18" t="inlineStr">
+      <c r="G1" s="22" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="H1" s="18" t="inlineStr">
+      <c r="H1" s="22" t="inlineStr">
         <is>
           <t>Commencement Date</t>
         </is>
       </c>
-      <c r="I1" s="18" t="inlineStr">
+      <c r="I1" s="22" t="inlineStr">
         <is>
           <t>Expiry Date</t>
         </is>
       </c>
-      <c r="J1" s="18" t="inlineStr">
+      <c r="J1" s="22" t="inlineStr">
         <is>
           <t>Premium (RM)</t>
         </is>
       </c>
-      <c r="K1" s="18" t="inlineStr">
+      <c r="K1" s="22" t="inlineStr">
         <is>
           <t>Payment Mode</t>
         </is>
       </c>
-      <c r="L1" s="18" t="inlineStr">
+      <c r="L1" s="22" t="inlineStr">
         <is>
           <t>Death (RM)</t>
         </is>
       </c>
-      <c r="M1" s="18" t="inlineStr">
+      <c r="M1" s="22" t="inlineStr">
         <is>
           <t>TPD (RM)</t>
         </is>
       </c>
-      <c r="N1" s="18" t="inlineStr">
+      <c r="N1" s="22" t="inlineStr">
         <is>
           <t>Critical Illness (RM)</t>
         </is>
       </c>
-      <c r="O1" s="18" t="inlineStr">
+      <c r="O1" s="22" t="inlineStr">
         <is>
           <t>Early CI (RM)</t>
         </is>
       </c>
-      <c r="P1" s="18" t="inlineStr">
+      <c r="P1" s="22" t="inlineStr">
         <is>
           <t>Medical Annual Limit (RM)</t>
         </is>
       </c>
-      <c r="Q1" s="18" t="inlineStr">
+      <c r="Q1" s="22" t="inlineStr">
         <is>
           <t>Room &amp; Board (RM/day)</t>
         </is>
       </c>
-      <c r="R1" s="18" t="inlineStr">
+      <c r="R1" s="22" t="inlineStr">
         <is>
           <t>Personal Accident (RM)</t>
         </is>
       </c>
-      <c r="S1" s="18" t="inlineStr">
+      <c r="S1" s="22" t="inlineStr">
         <is>
           <t>Waiver of Premium</t>
         </is>
       </c>
-      <c r="T1" s="18" t="inlineStr">
+      <c r="T1" s="22" t="inlineStr">
         <is>
           <t>Nominee Name</t>
         </is>
       </c>
-      <c r="U1" s="18" t="inlineStr">
+      <c r="U1" s="22" t="inlineStr">
         <is>
           <t>Nominee Relationship</t>
         </is>
       </c>
-      <c r="V1" s="18" t="inlineStr">
+      <c r="V1" s="22" t="inlineStr">
         <is>
           <t>Nomination Type</t>
         </is>
       </c>
-      <c r="W1" s="18" t="inlineStr">
+      <c r="W1" s="22" t="inlineStr">
         <is>
           <t>Purpose</t>
         </is>
       </c>
-      <c r="X1" s="18" t="inlineStr">
+      <c r="X1" s="22" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="Y1" s="18" t="inlineStr">
+      <c r="Y1" s="22" t="inlineStr">
         <is>
           <t>Retirement Fund (RM)</t>
         </is>
       </c>
-      <c r="Z1" s="18" t="inlineStr">
+      <c r="Z1" s="22" t="inlineStr">
         <is>
           <t>Trust Created</t>
         </is>
       </c>
-      <c r="AA1" s="19" t="inlineStr">
+      <c r="AA1" s="23" t="inlineStr">
         <is>
           <t>Annual Premium (auto)</t>
         </is>
@@ -1528,7 +1711,7 @@
       <c r="X2" s="12" t="inlineStr"/>
       <c r="Y2" s="9" t="n"/>
       <c r="Z2" s="12" t="n"/>
-      <c r="AA2" s="21">
+      <c r="AA2" s="24">
         <f>IF(J2="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J2,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K2,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -1618,7 +1801,7 @@
       </c>
       <c r="Y3" s="9" t="n"/>
       <c r="Z3" s="12" t="n"/>
-      <c r="AA3" s="21">
+      <c r="AA3" s="24">
         <f>IF(J3="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J3,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K3,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -1714,7 +1897,7 @@
       <c r="X4" s="12" t="inlineStr"/>
       <c r="Y4" s="9" t="n"/>
       <c r="Z4" s="12" t="n"/>
-      <c r="AA4" s="21">
+      <c r="AA4" s="24">
         <f>IF(J4="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J4,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K4,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -1798,7 +1981,7 @@
       </c>
       <c r="Y5" s="9" t="n"/>
       <c r="Z5" s="12" t="n"/>
-      <c r="AA5" s="21">
+      <c r="AA5" s="24">
         <f>IF(J5="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J5,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K5,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -1894,7 +2077,7 @@
       </c>
       <c r="Y6" s="9" t="n"/>
       <c r="Z6" s="12" t="n"/>
-      <c r="AA6" s="21">
+      <c r="AA6" s="24">
         <f>IF(J6="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J6,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K6,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -1926,7 +2109,7 @@
       <c r="X7" s="12" t="n"/>
       <c r="Y7" s="9" t="n"/>
       <c r="Z7" s="12" t="n"/>
-      <c r="AA7" s="21">
+      <c r="AA7" s="24">
         <f>IF(J7="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J7,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K7,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -1958,7 +2141,7 @@
       <c r="X8" s="12" t="n"/>
       <c r="Y8" s="9" t="n"/>
       <c r="Z8" s="12" t="n"/>
-      <c r="AA8" s="21">
+      <c r="AA8" s="24">
         <f>IF(J8="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J8,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K8,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -1990,7 +2173,7 @@
       <c r="X9" s="12" t="n"/>
       <c r="Y9" s="9" t="n"/>
       <c r="Z9" s="12" t="n"/>
-      <c r="AA9" s="21">
+      <c r="AA9" s="24">
         <f>IF(J9="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J9,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K9,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2022,7 +2205,7 @@
       <c r="X10" s="12" t="n"/>
       <c r="Y10" s="9" t="n"/>
       <c r="Z10" s="12" t="n"/>
-      <c r="AA10" s="21">
+      <c r="AA10" s="24">
         <f>IF(J10="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J10,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K10,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2054,7 +2237,7 @@
       <c r="X11" s="12" t="n"/>
       <c r="Y11" s="9" t="n"/>
       <c r="Z11" s="12" t="n"/>
-      <c r="AA11" s="21">
+      <c r="AA11" s="24">
         <f>IF(J11="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J11,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K11,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2086,7 +2269,7 @@
       <c r="X12" s="12" t="n"/>
       <c r="Y12" s="9" t="n"/>
       <c r="Z12" s="12" t="n"/>
-      <c r="AA12" s="21">
+      <c r="AA12" s="24">
         <f>IF(J12="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J12,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K12,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2118,7 +2301,7 @@
       <c r="X13" s="12" t="n"/>
       <c r="Y13" s="9" t="n"/>
       <c r="Z13" s="12" t="n"/>
-      <c r="AA13" s="21">
+      <c r="AA13" s="24">
         <f>IF(J13="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J13,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K13,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2150,7 +2333,7 @@
       <c r="X14" s="12" t="n"/>
       <c r="Y14" s="9" t="n"/>
       <c r="Z14" s="12" t="n"/>
-      <c r="AA14" s="21">
+      <c r="AA14" s="24">
         <f>IF(J14="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J14,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K14,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2182,7 +2365,7 @@
       <c r="X15" s="12" t="n"/>
       <c r="Y15" s="9" t="n"/>
       <c r="Z15" s="12" t="n"/>
-      <c r="AA15" s="21">
+      <c r="AA15" s="24">
         <f>IF(J15="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J15,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K15,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2214,7 +2397,7 @@
       <c r="X16" s="12" t="n"/>
       <c r="Y16" s="9" t="n"/>
       <c r="Z16" s="12" t="n"/>
-      <c r="AA16" s="21">
+      <c r="AA16" s="24">
         <f>IF(J16="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J16,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K16,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2246,7 +2429,7 @@
       <c r="X17" s="12" t="n"/>
       <c r="Y17" s="9" t="n"/>
       <c r="Z17" s="12" t="n"/>
-      <c r="AA17" s="21">
+      <c r="AA17" s="24">
         <f>IF(J17="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J17,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K17,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2278,7 +2461,7 @@
       <c r="X18" s="12" t="n"/>
       <c r="Y18" s="9" t="n"/>
       <c r="Z18" s="12" t="n"/>
-      <c r="AA18" s="21">
+      <c r="AA18" s="24">
         <f>IF(J18="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J18,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K18,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2310,7 +2493,7 @@
       <c r="X19" s="12" t="n"/>
       <c r="Y19" s="9" t="n"/>
       <c r="Z19" s="12" t="n"/>
-      <c r="AA19" s="21">
+      <c r="AA19" s="24">
         <f>IF(J19="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J19,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K19,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2342,7 +2525,7 @@
       <c r="X20" s="12" t="n"/>
       <c r="Y20" s="9" t="n"/>
       <c r="Z20" s="12" t="n"/>
-      <c r="AA20" s="21">
+      <c r="AA20" s="24">
         <f>IF(J20="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J20,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K20,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2374,7 +2557,7 @@
       <c r="X21" s="12" t="n"/>
       <c r="Y21" s="9" t="n"/>
       <c r="Z21" s="12" t="n"/>
-      <c r="AA21" s="21">
+      <c r="AA21" s="24">
         <f>IF(J21="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J21,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K21,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2406,7 +2589,7 @@
       <c r="X22" s="12" t="n"/>
       <c r="Y22" s="9" t="n"/>
       <c r="Z22" s="12" t="n"/>
-      <c r="AA22" s="21">
+      <c r="AA22" s="24">
         <f>IF(J22="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J22,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K22,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2438,7 +2621,7 @@
       <c r="X23" s="12" t="n"/>
       <c r="Y23" s="9" t="n"/>
       <c r="Z23" s="12" t="n"/>
-      <c r="AA23" s="21">
+      <c r="AA23" s="24">
         <f>IF(J23="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J23,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K23,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2470,7 +2653,7 @@
       <c r="X24" s="12" t="n"/>
       <c r="Y24" s="9" t="n"/>
       <c r="Z24" s="12" t="n"/>
-      <c r="AA24" s="21">
+      <c r="AA24" s="24">
         <f>IF(J24="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J24,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K24,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2502,7 +2685,7 @@
       <c r="X25" s="12" t="n"/>
       <c r="Y25" s="9" t="n"/>
       <c r="Z25" s="12" t="n"/>
-      <c r="AA25" s="21">
+      <c r="AA25" s="24">
         <f>IF(J25="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J25,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K25,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2534,7 +2717,7 @@
       <c r="X26" s="12" t="n"/>
       <c r="Y26" s="9" t="n"/>
       <c r="Z26" s="12" t="n"/>
-      <c r="AA26" s="21">
+      <c r="AA26" s="24">
         <f>IF(J26="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J26,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K26,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2566,7 +2749,7 @@
       <c r="X27" s="12" t="n"/>
       <c r="Y27" s="9" t="n"/>
       <c r="Z27" s="12" t="n"/>
-      <c r="AA27" s="21">
+      <c r="AA27" s="24">
         <f>IF(J27="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J27,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K27,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2598,7 +2781,7 @@
       <c r="X28" s="12" t="n"/>
       <c r="Y28" s="9" t="n"/>
       <c r="Z28" s="12" t="n"/>
-      <c r="AA28" s="21">
+      <c r="AA28" s="24">
         <f>IF(J28="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J28,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K28,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2630,7 +2813,7 @@
       <c r="X29" s="12" t="n"/>
       <c r="Y29" s="9" t="n"/>
       <c r="Z29" s="12" t="n"/>
-      <c r="AA29" s="21">
+      <c r="AA29" s="24">
         <f>IF(J29="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J29,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K29,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2662,7 +2845,7 @@
       <c r="X30" s="12" t="n"/>
       <c r="Y30" s="9" t="n"/>
       <c r="Z30" s="12" t="n"/>
-      <c r="AA30" s="21">
+      <c r="AA30" s="24">
         <f>IF(J30="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J30,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K30,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2694,7 +2877,7 @@
       <c r="X31" s="12" t="n"/>
       <c r="Y31" s="9" t="n"/>
       <c r="Z31" s="12" t="n"/>
-      <c r="AA31" s="21">
+      <c r="AA31" s="24">
         <f>IF(J31="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J31,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K31,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2726,7 +2909,7 @@
       <c r="X32" s="12" t="n"/>
       <c r="Y32" s="9" t="n"/>
       <c r="Z32" s="12" t="n"/>
-      <c r="AA32" s="21">
+      <c r="AA32" s="24">
         <f>IF(J32="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J32,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K32,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2758,7 +2941,7 @@
       <c r="X33" s="12" t="n"/>
       <c r="Y33" s="9" t="n"/>
       <c r="Z33" s="12" t="n"/>
-      <c r="AA33" s="21">
+      <c r="AA33" s="24">
         <f>IF(J33="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J33,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K33,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2790,7 +2973,7 @@
       <c r="X34" s="12" t="n"/>
       <c r="Y34" s="9" t="n"/>
       <c r="Z34" s="12" t="n"/>
-      <c r="AA34" s="21">
+      <c r="AA34" s="24">
         <f>IF(J34="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J34,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K34,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2822,7 +3005,7 @@
       <c r="X35" s="12" t="n"/>
       <c r="Y35" s="9" t="n"/>
       <c r="Z35" s="12" t="n"/>
-      <c r="AA35" s="21">
+      <c r="AA35" s="24">
         <f>IF(J35="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J35,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K35,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2854,7 +3037,7 @@
       <c r="X36" s="12" t="n"/>
       <c r="Y36" s="9" t="n"/>
       <c r="Z36" s="12" t="n"/>
-      <c r="AA36" s="21">
+      <c r="AA36" s="24">
         <f>IF(J36="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J36,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K36,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2886,7 +3069,7 @@
       <c r="X37" s="12" t="n"/>
       <c r="Y37" s="9" t="n"/>
       <c r="Z37" s="12" t="n"/>
-      <c r="AA37" s="21">
+      <c r="AA37" s="24">
         <f>IF(J37="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J37,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K37,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2918,7 +3101,7 @@
       <c r="X38" s="12" t="n"/>
       <c r="Y38" s="9" t="n"/>
       <c r="Z38" s="12" t="n"/>
-      <c r="AA38" s="21">
+      <c r="AA38" s="24">
         <f>IF(J38="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J38,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K38,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2950,7 +3133,7 @@
       <c r="X39" s="12" t="n"/>
       <c r="Y39" s="9" t="n"/>
       <c r="Z39" s="12" t="n"/>
-      <c r="AA39" s="21">
+      <c r="AA39" s="24">
         <f>IF(J39="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J39,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K39,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2982,7 +3165,7 @@
       <c r="X40" s="12" t="n"/>
       <c r="Y40" s="9" t="n"/>
       <c r="Z40" s="12" t="n"/>
-      <c r="AA40" s="21">
+      <c r="AA40" s="24">
         <f>IF(J40="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J40,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K40,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3014,7 +3197,7 @@
       <c r="X41" s="12" t="n"/>
       <c r="Y41" s="9" t="n"/>
       <c r="Z41" s="12" t="n"/>
-      <c r="AA41" s="21">
+      <c r="AA41" s="24">
         <f>IF(J41="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J41,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K41,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3046,7 +3229,7 @@
       <c r="X42" s="12" t="n"/>
       <c r="Y42" s="9" t="n"/>
       <c r="Z42" s="12" t="n"/>
-      <c r="AA42" s="21">
+      <c r="AA42" s="24">
         <f>IF(J42="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J42,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K42,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3078,7 +3261,7 @@
       <c r="X43" s="12" t="n"/>
       <c r="Y43" s="9" t="n"/>
       <c r="Z43" s="12" t="n"/>
-      <c r="AA43" s="21">
+      <c r="AA43" s="24">
         <f>IF(J43="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J43,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K43,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3110,7 +3293,7 @@
       <c r="X44" s="12" t="n"/>
       <c r="Y44" s="9" t="n"/>
       <c r="Z44" s="12" t="n"/>
-      <c r="AA44" s="21">
+      <c r="AA44" s="24">
         <f>IF(J44="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J44,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K44,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3142,7 +3325,7 @@
       <c r="X45" s="12" t="n"/>
       <c r="Y45" s="9" t="n"/>
       <c r="Z45" s="12" t="n"/>
-      <c r="AA45" s="21">
+      <c r="AA45" s="24">
         <f>IF(J45="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J45,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K45,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3174,7 +3357,7 @@
       <c r="X46" s="12" t="n"/>
       <c r="Y46" s="9" t="n"/>
       <c r="Z46" s="12" t="n"/>
-      <c r="AA46" s="21">
+      <c r="AA46" s="24">
         <f>IF(J46="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J46,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K46,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3206,7 +3389,7 @@
       <c r="X47" s="12" t="n"/>
       <c r="Y47" s="9" t="n"/>
       <c r="Z47" s="12" t="n"/>
-      <c r="AA47" s="21">
+      <c r="AA47" s="24">
         <f>IF(J47="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J47,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K47,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3238,7 +3421,7 @@
       <c r="X48" s="12" t="n"/>
       <c r="Y48" s="9" t="n"/>
       <c r="Z48" s="12" t="n"/>
-      <c r="AA48" s="21">
+      <c r="AA48" s="24">
         <f>IF(J48="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J48,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K48,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3270,7 +3453,7 @@
       <c r="X49" s="12" t="n"/>
       <c r="Y49" s="9" t="n"/>
       <c r="Z49" s="12" t="n"/>
-      <c r="AA49" s="21">
+      <c r="AA49" s="24">
         <f>IF(J49="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J49,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K49,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3302,7 +3485,7 @@
       <c r="X50" s="12" t="n"/>
       <c r="Y50" s="9" t="n"/>
       <c r="Z50" s="12" t="n"/>
-      <c r="AA50" s="21">
+      <c r="AA50" s="24">
         <f>IF(J50="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J50,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K50,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3334,7 +3517,7 @@
       <c r="X51" s="12" t="n"/>
       <c r="Y51" s="9" t="n"/>
       <c r="Z51" s="12" t="n"/>
-      <c r="AA51" s="21">
+      <c r="AA51" s="24">
         <f>IF(J51="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J51,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K51,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3366,7 +3549,7 @@
       <c r="X52" s="12" t="n"/>
       <c r="Y52" s="9" t="n"/>
       <c r="Z52" s="12" t="n"/>
-      <c r="AA52" s="21">
+      <c r="AA52" s="24">
         <f>IF(J52="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J52,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K52,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3398,7 +3581,7 @@
       <c r="X53" s="12" t="n"/>
       <c r="Y53" s="9" t="n"/>
       <c r="Z53" s="12" t="n"/>
-      <c r="AA53" s="21">
+      <c r="AA53" s="24">
         <f>IF(J53="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J53,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K53,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3430,7 +3613,7 @@
       <c r="X54" s="12" t="n"/>
       <c r="Y54" s="9" t="n"/>
       <c r="Z54" s="12" t="n"/>
-      <c r="AA54" s="21">
+      <c r="AA54" s="24">
         <f>IF(J54="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J54,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K54,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3462,7 +3645,7 @@
       <c r="X55" s="12" t="n"/>
       <c r="Y55" s="9" t="n"/>
       <c r="Z55" s="12" t="n"/>
-      <c r="AA55" s="21">
+      <c r="AA55" s="24">
         <f>IF(J55="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J55,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K55,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3494,7 +3677,7 @@
       <c r="X56" s="12" t="n"/>
       <c r="Y56" s="9" t="n"/>
       <c r="Z56" s="12" t="n"/>
-      <c r="AA56" s="21">
+      <c r="AA56" s="24">
         <f>IF(J56="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J56,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K56,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3526,7 +3709,7 @@
       <c r="X57" s="12" t="n"/>
       <c r="Y57" s="9" t="n"/>
       <c r="Z57" s="12" t="n"/>
-      <c r="AA57" s="21">
+      <c r="AA57" s="24">
         <f>IF(J57="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J57,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K57,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3558,7 +3741,7 @@
       <c r="X58" s="12" t="n"/>
       <c r="Y58" s="9" t="n"/>
       <c r="Z58" s="12" t="n"/>
-      <c r="AA58" s="21">
+      <c r="AA58" s="24">
         <f>IF(J58="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J58,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K58,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3590,7 +3773,7 @@
       <c r="X59" s="12" t="n"/>
       <c r="Y59" s="9" t="n"/>
       <c r="Z59" s="12" t="n"/>
-      <c r="AA59" s="21">
+      <c r="AA59" s="24">
         <f>IF(J59="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J59,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K59,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3622,7 +3805,7 @@
       <c r="X60" s="12" t="n"/>
       <c r="Y60" s="9" t="n"/>
       <c r="Z60" s="12" t="n"/>
-      <c r="AA60" s="21">
+      <c r="AA60" s="24">
         <f>IF(J60="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J60,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K60,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3654,7 +3837,7 @@
       <c r="X61" s="12" t="n"/>
       <c r="Y61" s="9" t="n"/>
       <c r="Z61" s="12" t="n"/>
-      <c r="AA61" s="21">
+      <c r="AA61" s="24">
         <f>IF(J61="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J61,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K61,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3686,7 +3869,7 @@
       <c r="X62" s="12" t="n"/>
       <c r="Y62" s="9" t="n"/>
       <c r="Z62" s="12" t="n"/>
-      <c r="AA62" s="21">
+      <c r="AA62" s="24">
         <f>IF(J62="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J62,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K62,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3718,7 +3901,7 @@
       <c r="X63" s="12" t="n"/>
       <c r="Y63" s="9" t="n"/>
       <c r="Z63" s="12" t="n"/>
-      <c r="AA63" s="21">
+      <c r="AA63" s="24">
         <f>IF(J63="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J63,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K63,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3750,7 +3933,7 @@
       <c r="X64" s="12" t="n"/>
       <c r="Y64" s="9" t="n"/>
       <c r="Z64" s="12" t="n"/>
-      <c r="AA64" s="21">
+      <c r="AA64" s="24">
         <f>IF(J64="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J64,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K64,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3782,7 +3965,7 @@
       <c r="X65" s="12" t="n"/>
       <c r="Y65" s="9" t="n"/>
       <c r="Z65" s="12" t="n"/>
-      <c r="AA65" s="21">
+      <c r="AA65" s="24">
         <f>IF(J65="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J65,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K65,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3814,7 +3997,7 @@
       <c r="X66" s="12" t="n"/>
       <c r="Y66" s="9" t="n"/>
       <c r="Z66" s="12" t="n"/>
-      <c r="AA66" s="21">
+      <c r="AA66" s="24">
         <f>IF(J66="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J66,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K66,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3846,7 +4029,7 @@
       <c r="X67" s="12" t="n"/>
       <c r="Y67" s="9" t="n"/>
       <c r="Z67" s="12" t="n"/>
-      <c r="AA67" s="21">
+      <c r="AA67" s="24">
         <f>IF(J67="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J67,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K67,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3878,7 +4061,7 @@
       <c r="X68" s="12" t="n"/>
       <c r="Y68" s="9" t="n"/>
       <c r="Z68" s="12" t="n"/>
-      <c r="AA68" s="21">
+      <c r="AA68" s="24">
         <f>IF(J68="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J68,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K68,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3910,7 +4093,7 @@
       <c r="X69" s="12" t="n"/>
       <c r="Y69" s="9" t="n"/>
       <c r="Z69" s="12" t="n"/>
-      <c r="AA69" s="21">
+      <c r="AA69" s="24">
         <f>IF(J69="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J69,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K69,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3942,7 +4125,7 @@
       <c r="X70" s="12" t="n"/>
       <c r="Y70" s="9" t="n"/>
       <c r="Z70" s="12" t="n"/>
-      <c r="AA70" s="21">
+      <c r="AA70" s="24">
         <f>IF(J70="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J70,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K70,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3974,7 +4157,7 @@
       <c r="X71" s="12" t="n"/>
       <c r="Y71" s="9" t="n"/>
       <c r="Z71" s="12" t="n"/>
-      <c r="AA71" s="21">
+      <c r="AA71" s="24">
         <f>IF(J71="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J71,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K71,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -4006,7 +4189,7 @@
       <c r="X72" s="12" t="n"/>
       <c r="Y72" s="9" t="n"/>
       <c r="Z72" s="12" t="n"/>
-      <c r="AA72" s="21">
+      <c r="AA72" s="24">
         <f>IF(J72="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J72,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K72,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -4038,7 +4221,7 @@
       <c r="X73" s="12" t="n"/>
       <c r="Y73" s="9" t="n"/>
       <c r="Z73" s="12" t="n"/>
-      <c r="AA73" s="21">
+      <c r="AA73" s="24">
         <f>IF(J73="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J73,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K73,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -4070,7 +4253,7 @@
       <c r="X74" s="12" t="n"/>
       <c r="Y74" s="9" t="n"/>
       <c r="Z74" s="12" t="n"/>
-      <c r="AA74" s="21">
+      <c r="AA74" s="24">
         <f>IF(J74="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J74,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K74,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -4102,7 +4285,7 @@
       <c r="X75" s="12" t="n"/>
       <c r="Y75" s="9" t="n"/>
       <c r="Z75" s="12" t="n"/>
-      <c r="AA75" s="21">
+      <c r="AA75" s="24">
         <f>IF(J75="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J75,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K75,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -4134,7 +4317,7 @@
       <c r="X76" s="12" t="n"/>
       <c r="Y76" s="9" t="n"/>
       <c r="Z76" s="12" t="n"/>
-      <c r="AA76" s="21">
+      <c r="AA76" s="24">
         <f>IF(J76="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J76,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K76,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -4166,7 +4349,7 @@
       <c r="X77" s="12" t="n"/>
       <c r="Y77" s="9" t="n"/>
       <c r="Z77" s="12" t="n"/>
-      <c r="AA77" s="21">
+      <c r="AA77" s="24">
         <f>IF(J77="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J77,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K77,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -4198,7 +4381,7 @@
       <c r="X78" s="12" t="n"/>
       <c r="Y78" s="9" t="n"/>
       <c r="Z78" s="12" t="n"/>
-      <c r="AA78" s="21">
+      <c r="AA78" s="24">
         <f>IF(J78="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J78,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K78,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -4230,7 +4413,7 @@
       <c r="X79" s="12" t="n"/>
       <c r="Y79" s="9" t="n"/>
       <c r="Z79" s="12" t="n"/>
-      <c r="AA79" s="21">
+      <c r="AA79" s="24">
         <f>IF(J79="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J79,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K79,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -4262,7 +4445,7 @@
       <c r="X80" s="12" t="n"/>
       <c r="Y80" s="9" t="n"/>
       <c r="Z80" s="12" t="n"/>
-      <c r="AA80" s="21">
+      <c r="AA80" s="24">
         <f>IF(J80="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J80,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K80,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -4294,7 +4477,7 @@
       <c r="X81" s="12" t="n"/>
       <c r="Y81" s="9" t="n"/>
       <c r="Z81" s="12" t="n"/>
-      <c r="AA81" s="21">
+      <c r="AA81" s="24">
         <f>IF(J81="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J81,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K81,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -4326,7 +4509,7 @@
       <c r="X82" s="12" t="n"/>
       <c r="Y82" s="9" t="n"/>
       <c r="Z82" s="12" t="n"/>
-      <c r="AA82" s="21">
+      <c r="AA82" s="24">
         <f>IF(J82="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J82,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K82,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -4358,7 +4541,7 @@
       <c r="X83" s="12" t="n"/>
       <c r="Y83" s="9" t="n"/>
       <c r="Z83" s="12" t="n"/>
-      <c r="AA83" s="21">
+      <c r="AA83" s="24">
         <f>IF(J83="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J83,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K83,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -4390,7 +4573,7 @@
       <c r="X84" s="12" t="n"/>
       <c r="Y84" s="9" t="n"/>
       <c r="Z84" s="12" t="n"/>
-      <c r="AA84" s="21">
+      <c r="AA84" s="24">
         <f>IF(J84="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J84,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K84,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -4422,7 +4605,7 @@
       <c r="X85" s="12" t="n"/>
       <c r="Y85" s="9" t="n"/>
       <c r="Z85" s="12" t="n"/>
-      <c r="AA85" s="21">
+      <c r="AA85" s="24">
         <f>IF(J85="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J85,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K85,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -4454,7 +4637,7 @@
       <c r="X86" s="12" t="n"/>
       <c r="Y86" s="9" t="n"/>
       <c r="Z86" s="12" t="n"/>
-      <c r="AA86" s="21">
+      <c r="AA86" s="24">
         <f>IF(J86="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J86,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K86,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -4486,7 +4669,7 @@
       <c r="X87" s="12" t="n"/>
       <c r="Y87" s="9" t="n"/>
       <c r="Z87" s="12" t="n"/>
-      <c r="AA87" s="21">
+      <c r="AA87" s="24">
         <f>IF(J87="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J87,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K87,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -4518,7 +4701,7 @@
       <c r="X88" s="12" t="n"/>
       <c r="Y88" s="9" t="n"/>
       <c r="Z88" s="12" t="n"/>
-      <c r="AA88" s="21">
+      <c r="AA88" s="24">
         <f>IF(J88="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J88,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K88,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -4550,7 +4733,7 @@
       <c r="X89" s="12" t="n"/>
       <c r="Y89" s="9" t="n"/>
       <c r="Z89" s="12" t="n"/>
-      <c r="AA89" s="21">
+      <c r="AA89" s="24">
         <f>IF(J89="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J89,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K89,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -4582,7 +4765,7 @@
       <c r="X90" s="12" t="n"/>
       <c r="Y90" s="9" t="n"/>
       <c r="Z90" s="12" t="n"/>
-      <c r="AA90" s="21">
+      <c r="AA90" s="24">
         <f>IF(J90="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J90,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K90,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -4614,7 +4797,7 @@
       <c r="X91" s="12" t="n"/>
       <c r="Y91" s="9" t="n"/>
       <c r="Z91" s="12" t="n"/>
-      <c r="AA91" s="21">
+      <c r="AA91" s="24">
         <f>IF(J91="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J91,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K91,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -4646,7 +4829,7 @@
       <c r="X92" s="12" t="n"/>
       <c r="Y92" s="9" t="n"/>
       <c r="Z92" s="12" t="n"/>
-      <c r="AA92" s="21">
+      <c r="AA92" s="24">
         <f>IF(J92="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J92,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K92,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -4678,7 +4861,7 @@
       <c r="X93" s="12" t="n"/>
       <c r="Y93" s="9" t="n"/>
       <c r="Z93" s="12" t="n"/>
-      <c r="AA93" s="21">
+      <c r="AA93" s="24">
         <f>IF(J93="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J93,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K93,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -4710,7 +4893,7 @@
       <c r="X94" s="12" t="n"/>
       <c r="Y94" s="9" t="n"/>
       <c r="Z94" s="12" t="n"/>
-      <c r="AA94" s="21">
+      <c r="AA94" s="24">
         <f>IF(J94="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J94,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K94,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -4742,7 +4925,7 @@
       <c r="X95" s="12" t="n"/>
       <c r="Y95" s="9" t="n"/>
       <c r="Z95" s="12" t="n"/>
-      <c r="AA95" s="21">
+      <c r="AA95" s="24">
         <f>IF(J95="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J95,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K95,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -4774,7 +4957,7 @@
       <c r="X96" s="12" t="n"/>
       <c r="Y96" s="9" t="n"/>
       <c r="Z96" s="12" t="n"/>
-      <c r="AA96" s="21">
+      <c r="AA96" s="24">
         <f>IF(J96="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J96,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K96,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -4806,7 +4989,7 @@
       <c r="X97" s="12" t="n"/>
       <c r="Y97" s="9" t="n"/>
       <c r="Z97" s="12" t="n"/>
-      <c r="AA97" s="21">
+      <c r="AA97" s="24">
         <f>IF(J97="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J97,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K97,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -4838,7 +5021,7 @@
       <c r="X98" s="12" t="n"/>
       <c r="Y98" s="9" t="n"/>
       <c r="Z98" s="12" t="n"/>
-      <c r="AA98" s="21">
+      <c r="AA98" s="24">
         <f>IF(J98="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J98,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K98,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -4870,7 +5053,7 @@
       <c r="X99" s="12" t="n"/>
       <c r="Y99" s="9" t="n"/>
       <c r="Z99" s="12" t="n"/>
-      <c r="AA99" s="21">
+      <c r="AA99" s="24">
         <f>IF(J99="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J99,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K99,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -4902,7 +5085,7 @@
       <c r="X100" s="12" t="n"/>
       <c r="Y100" s="9" t="n"/>
       <c r="Z100" s="12" t="n"/>
-      <c r="AA100" s="21">
+      <c r="AA100" s="24">
         <f>IF(J100="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J100,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K100,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -4975,1383 +5158,1383 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="22" t="n"/>
-      <c r="B4" s="22" t="n"/>
-      <c r="C4" s="22" t="n"/>
-      <c r="D4" s="22" t="n"/>
-      <c r="E4" s="22" t="n"/>
+      <c r="A4" s="25" t="n"/>
+      <c r="B4" s="25" t="n"/>
+      <c r="C4" s="25" t="n"/>
+      <c r="D4" s="25" t="n"/>
+      <c r="E4" s="25" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="22" t="n"/>
-      <c r="B5" s="22" t="n"/>
-      <c r="C5" s="22" t="n"/>
-      <c r="D5" s="22" t="n"/>
-      <c r="E5" s="22" t="n"/>
+      <c r="A5" s="25" t="n"/>
+      <c r="B5" s="25" t="n"/>
+      <c r="C5" s="25" t="n"/>
+      <c r="D5" s="25" t="n"/>
+      <c r="E5" s="25" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="22" t="n"/>
-      <c r="B6" s="22" t="n"/>
-      <c r="C6" s="22" t="n"/>
-      <c r="D6" s="22" t="n"/>
-      <c r="E6" s="22" t="n"/>
+      <c r="A6" s="25" t="n"/>
+      <c r="B6" s="25" t="n"/>
+      <c r="C6" s="25" t="n"/>
+      <c r="D6" s="25" t="n"/>
+      <c r="E6" s="25" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="22" t="n"/>
-      <c r="B7" s="22" t="n"/>
-      <c r="C7" s="22" t="n"/>
-      <c r="D7" s="22" t="n"/>
-      <c r="E7" s="22" t="n"/>
+      <c r="A7" s="25" t="n"/>
+      <c r="B7" s="25" t="n"/>
+      <c r="C7" s="25" t="n"/>
+      <c r="D7" s="25" t="n"/>
+      <c r="E7" s="25" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="22" t="n"/>
-      <c r="B8" s="22" t="n"/>
-      <c r="C8" s="22" t="n"/>
-      <c r="D8" s="22" t="n"/>
-      <c r="E8" s="22" t="n"/>
+      <c r="A8" s="25" t="n"/>
+      <c r="B8" s="25" t="n"/>
+      <c r="C8" s="25" t="n"/>
+      <c r="D8" s="25" t="n"/>
+      <c r="E8" s="25" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="22" t="n"/>
-      <c r="B9" s="22" t="n"/>
-      <c r="C9" s="22" t="n"/>
-      <c r="D9" s="22" t="n"/>
-      <c r="E9" s="22" t="n"/>
+      <c r="A9" s="25" t="n"/>
+      <c r="B9" s="25" t="n"/>
+      <c r="C9" s="25" t="n"/>
+      <c r="D9" s="25" t="n"/>
+      <c r="E9" s="25" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="22" t="n"/>
-      <c r="B10" s="22" t="n"/>
-      <c r="C10" s="22" t="n"/>
-      <c r="D10" s="22" t="n"/>
-      <c r="E10" s="22" t="n"/>
+      <c r="A10" s="25" t="n"/>
+      <c r="B10" s="25" t="n"/>
+      <c r="C10" s="25" t="n"/>
+      <c r="D10" s="25" t="n"/>
+      <c r="E10" s="25" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="22" t="n"/>
-      <c r="B11" s="22" t="n"/>
-      <c r="C11" s="22" t="n"/>
-      <c r="D11" s="22" t="n"/>
-      <c r="E11" s="22" t="n"/>
+      <c r="A11" s="25" t="n"/>
+      <c r="B11" s="25" t="n"/>
+      <c r="C11" s="25" t="n"/>
+      <c r="D11" s="25" t="n"/>
+      <c r="E11" s="25" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="22" t="n"/>
-      <c r="B12" s="22" t="n"/>
-      <c r="C12" s="22" t="n"/>
-      <c r="D12" s="22" t="n"/>
-      <c r="E12" s="22" t="n"/>
+      <c r="A12" s="25" t="n"/>
+      <c r="B12" s="25" t="n"/>
+      <c r="C12" s="25" t="n"/>
+      <c r="D12" s="25" t="n"/>
+      <c r="E12" s="25" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="22" t="n"/>
-      <c r="B13" s="22" t="n"/>
-      <c r="C13" s="22" t="n"/>
-      <c r="D13" s="22" t="n"/>
-      <c r="E13" s="22" t="n"/>
+      <c r="A13" s="25" t="n"/>
+      <c r="B13" s="25" t="n"/>
+      <c r="C13" s="25" t="n"/>
+      <c r="D13" s="25" t="n"/>
+      <c r="E13" s="25" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="22" t="n"/>
-      <c r="B14" s="22" t="n"/>
-      <c r="C14" s="22" t="n"/>
-      <c r="D14" s="22" t="n"/>
-      <c r="E14" s="22" t="n"/>
+      <c r="A14" s="25" t="n"/>
+      <c r="B14" s="25" t="n"/>
+      <c r="C14" s="25" t="n"/>
+      <c r="D14" s="25" t="n"/>
+      <c r="E14" s="25" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="22" t="n"/>
-      <c r="B15" s="22" t="n"/>
-      <c r="C15" s="22" t="n"/>
-      <c r="D15" s="22" t="n"/>
-      <c r="E15" s="22" t="n"/>
+      <c r="A15" s="25" t="n"/>
+      <c r="B15" s="25" t="n"/>
+      <c r="C15" s="25" t="n"/>
+      <c r="D15" s="25" t="n"/>
+      <c r="E15" s="25" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="22" t="n"/>
-      <c r="B16" s="22" t="n"/>
-      <c r="C16" s="22" t="n"/>
-      <c r="D16" s="22" t="n"/>
-      <c r="E16" s="22" t="n"/>
+      <c r="A16" s="25" t="n"/>
+      <c r="B16" s="25" t="n"/>
+      <c r="C16" s="25" t="n"/>
+      <c r="D16" s="25" t="n"/>
+      <c r="E16" s="25" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="22" t="n"/>
-      <c r="B17" s="22" t="n"/>
-      <c r="C17" s="22" t="n"/>
-      <c r="D17" s="22" t="n"/>
-      <c r="E17" s="22" t="n"/>
+      <c r="A17" s="25" t="n"/>
+      <c r="B17" s="25" t="n"/>
+      <c r="C17" s="25" t="n"/>
+      <c r="D17" s="25" t="n"/>
+      <c r="E17" s="25" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="22" t="n"/>
-      <c r="B18" s="22" t="n"/>
-      <c r="C18" s="22" t="n"/>
-      <c r="D18" s="22" t="n"/>
-      <c r="E18" s="22" t="n"/>
+      <c r="A18" s="25" t="n"/>
+      <c r="B18" s="25" t="n"/>
+      <c r="C18" s="25" t="n"/>
+      <c r="D18" s="25" t="n"/>
+      <c r="E18" s="25" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="22" t="n"/>
-      <c r="B19" s="22" t="n"/>
-      <c r="C19" s="22" t="n"/>
-      <c r="D19" s="22" t="n"/>
-      <c r="E19" s="22" t="n"/>
+      <c r="A19" s="25" t="n"/>
+      <c r="B19" s="25" t="n"/>
+      <c r="C19" s="25" t="n"/>
+      <c r="D19" s="25" t="n"/>
+      <c r="E19" s="25" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="22" t="n"/>
-      <c r="B20" s="22" t="n"/>
-      <c r="C20" s="22" t="n"/>
-      <c r="D20" s="22" t="n"/>
-      <c r="E20" s="22" t="n"/>
+      <c r="A20" s="25" t="n"/>
+      <c r="B20" s="25" t="n"/>
+      <c r="C20" s="25" t="n"/>
+      <c r="D20" s="25" t="n"/>
+      <c r="E20" s="25" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="22" t="n"/>
-      <c r="B21" s="22" t="n"/>
-      <c r="C21" s="22" t="n"/>
-      <c r="D21" s="22" t="n"/>
-      <c r="E21" s="22" t="n"/>
+      <c r="A21" s="25" t="n"/>
+      <c r="B21" s="25" t="n"/>
+      <c r="C21" s="25" t="n"/>
+      <c r="D21" s="25" t="n"/>
+      <c r="E21" s="25" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="22" t="n"/>
-      <c r="B22" s="22" t="n"/>
-      <c r="C22" s="22" t="n"/>
-      <c r="D22" s="22" t="n"/>
-      <c r="E22" s="22" t="n"/>
+      <c r="A22" s="25" t="n"/>
+      <c r="B22" s="25" t="n"/>
+      <c r="C22" s="25" t="n"/>
+      <c r="D22" s="25" t="n"/>
+      <c r="E22" s="25" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="22" t="n"/>
-      <c r="B23" s="22" t="n"/>
-      <c r="C23" s="22" t="n"/>
-      <c r="D23" s="22" t="n"/>
-      <c r="E23" s="22" t="n"/>
+      <c r="A23" s="25" t="n"/>
+      <c r="B23" s="25" t="n"/>
+      <c r="C23" s="25" t="n"/>
+      <c r="D23" s="25" t="n"/>
+      <c r="E23" s="25" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="22" t="n"/>
-      <c r="B24" s="22" t="n"/>
-      <c r="C24" s="22" t="n"/>
-      <c r="D24" s="22" t="n"/>
-      <c r="E24" s="22" t="n"/>
+      <c r="A24" s="25" t="n"/>
+      <c r="B24" s="25" t="n"/>
+      <c r="C24" s="25" t="n"/>
+      <c r="D24" s="25" t="n"/>
+      <c r="E24" s="25" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="22" t="n"/>
-      <c r="B25" s="22" t="n"/>
-      <c r="C25" s="22" t="n"/>
-      <c r="D25" s="22" t="n"/>
-      <c r="E25" s="22" t="n"/>
+      <c r="A25" s="25" t="n"/>
+      <c r="B25" s="25" t="n"/>
+      <c r="C25" s="25" t="n"/>
+      <c r="D25" s="25" t="n"/>
+      <c r="E25" s="25" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="22" t="n"/>
-      <c r="B26" s="22" t="n"/>
-      <c r="C26" s="22" t="n"/>
-      <c r="D26" s="22" t="n"/>
-      <c r="E26" s="22" t="n"/>
+      <c r="A26" s="25" t="n"/>
+      <c r="B26" s="25" t="n"/>
+      <c r="C26" s="25" t="n"/>
+      <c r="D26" s="25" t="n"/>
+      <c r="E26" s="25" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="22" t="n"/>
-      <c r="B27" s="22" t="n"/>
-      <c r="C27" s="22" t="n"/>
-      <c r="D27" s="22" t="n"/>
-      <c r="E27" s="22" t="n"/>
+      <c r="A27" s="25" t="n"/>
+      <c r="B27" s="25" t="n"/>
+      <c r="C27" s="25" t="n"/>
+      <c r="D27" s="25" t="n"/>
+      <c r="E27" s="25" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="22" t="n"/>
-      <c r="B28" s="22" t="n"/>
-      <c r="C28" s="22" t="n"/>
-      <c r="D28" s="22" t="n"/>
-      <c r="E28" s="22" t="n"/>
+      <c r="A28" s="25" t="n"/>
+      <c r="B28" s="25" t="n"/>
+      <c r="C28" s="25" t="n"/>
+      <c r="D28" s="25" t="n"/>
+      <c r="E28" s="25" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="22" t="n"/>
-      <c r="B29" s="22" t="n"/>
-      <c r="C29" s="22" t="n"/>
-      <c r="D29" s="22" t="n"/>
-      <c r="E29" s="22" t="n"/>
+      <c r="A29" s="25" t="n"/>
+      <c r="B29" s="25" t="n"/>
+      <c r="C29" s="25" t="n"/>
+      <c r="D29" s="25" t="n"/>
+      <c r="E29" s="25" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="22" t="n"/>
-      <c r="B30" s="22" t="n"/>
-      <c r="C30" s="22" t="n"/>
-      <c r="D30" s="22" t="n"/>
-      <c r="E30" s="22" t="n"/>
+      <c r="A30" s="25" t="n"/>
+      <c r="B30" s="25" t="n"/>
+      <c r="C30" s="25" t="n"/>
+      <c r="D30" s="25" t="n"/>
+      <c r="E30" s="25" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="22" t="n"/>
-      <c r="B31" s="22" t="n"/>
-      <c r="C31" s="22" t="n"/>
-      <c r="D31" s="22" t="n"/>
-      <c r="E31" s="22" t="n"/>
+      <c r="A31" s="25" t="n"/>
+      <c r="B31" s="25" t="n"/>
+      <c r="C31" s="25" t="n"/>
+      <c r="D31" s="25" t="n"/>
+      <c r="E31" s="25" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="22" t="n"/>
-      <c r="B32" s="22" t="n"/>
-      <c r="C32" s="22" t="n"/>
-      <c r="D32" s="22" t="n"/>
-      <c r="E32" s="22" t="n"/>
+      <c r="A32" s="25" t="n"/>
+      <c r="B32" s="25" t="n"/>
+      <c r="C32" s="25" t="n"/>
+      <c r="D32" s="25" t="n"/>
+      <c r="E32" s="25" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="22" t="n"/>
-      <c r="B33" s="22" t="n"/>
-      <c r="C33" s="22" t="n"/>
-      <c r="D33" s="22" t="n"/>
-      <c r="E33" s="22" t="n"/>
+      <c r="A33" s="25" t="n"/>
+      <c r="B33" s="25" t="n"/>
+      <c r="C33" s="25" t="n"/>
+      <c r="D33" s="25" t="n"/>
+      <c r="E33" s="25" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" s="22" t="n"/>
-      <c r="B34" s="22" t="n"/>
-      <c r="C34" s="22" t="n"/>
-      <c r="D34" s="22" t="n"/>
-      <c r="E34" s="22" t="n"/>
+      <c r="A34" s="25" t="n"/>
+      <c r="B34" s="25" t="n"/>
+      <c r="C34" s="25" t="n"/>
+      <c r="D34" s="25" t="n"/>
+      <c r="E34" s="25" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="22" t="n"/>
-      <c r="B35" s="22" t="n"/>
-      <c r="C35" s="22" t="n"/>
-      <c r="D35" s="22" t="n"/>
-      <c r="E35" s="22" t="n"/>
+      <c r="A35" s="25" t="n"/>
+      <c r="B35" s="25" t="n"/>
+      <c r="C35" s="25" t="n"/>
+      <c r="D35" s="25" t="n"/>
+      <c r="E35" s="25" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" s="22" t="n"/>
-      <c r="B36" s="22" t="n"/>
-      <c r="C36" s="22" t="n"/>
-      <c r="D36" s="22" t="n"/>
-      <c r="E36" s="22" t="n"/>
+      <c r="A36" s="25" t="n"/>
+      <c r="B36" s="25" t="n"/>
+      <c r="C36" s="25" t="n"/>
+      <c r="D36" s="25" t="n"/>
+      <c r="E36" s="25" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="22" t="n"/>
-      <c r="B37" s="22" t="n"/>
-      <c r="C37" s="22" t="n"/>
-      <c r="D37" s="22" t="n"/>
-      <c r="E37" s="22" t="n"/>
+      <c r="A37" s="25" t="n"/>
+      <c r="B37" s="25" t="n"/>
+      <c r="C37" s="25" t="n"/>
+      <c r="D37" s="25" t="n"/>
+      <c r="E37" s="25" t="n"/>
     </row>
     <row r="38">
-      <c r="A38" s="22" t="n"/>
-      <c r="B38" s="22" t="n"/>
-      <c r="C38" s="22" t="n"/>
-      <c r="D38" s="22" t="n"/>
-      <c r="E38" s="22" t="n"/>
+      <c r="A38" s="25" t="n"/>
+      <c r="B38" s="25" t="n"/>
+      <c r="C38" s="25" t="n"/>
+      <c r="D38" s="25" t="n"/>
+      <c r="E38" s="25" t="n"/>
     </row>
     <row r="39">
-      <c r="A39" s="22" t="n"/>
-      <c r="B39" s="22" t="n"/>
-      <c r="C39" s="22" t="n"/>
-      <c r="D39" s="22" t="n"/>
-      <c r="E39" s="22" t="n"/>
+      <c r="A39" s="25" t="n"/>
+      <c r="B39" s="25" t="n"/>
+      <c r="C39" s="25" t="n"/>
+      <c r="D39" s="25" t="n"/>
+      <c r="E39" s="25" t="n"/>
     </row>
     <row r="40">
-      <c r="A40" s="22" t="n"/>
-      <c r="B40" s="22" t="n"/>
-      <c r="C40" s="22" t="n"/>
-      <c r="D40" s="22" t="n"/>
-      <c r="E40" s="22" t="n"/>
+      <c r="A40" s="25" t="n"/>
+      <c r="B40" s="25" t="n"/>
+      <c r="C40" s="25" t="n"/>
+      <c r="D40" s="25" t="n"/>
+      <c r="E40" s="25" t="n"/>
     </row>
     <row r="41">
-      <c r="A41" s="22" t="n"/>
-      <c r="B41" s="22" t="n"/>
-      <c r="C41" s="22" t="n"/>
-      <c r="D41" s="22" t="n"/>
-      <c r="E41" s="22" t="n"/>
+      <c r="A41" s="25" t="n"/>
+      <c r="B41" s="25" t="n"/>
+      <c r="C41" s="25" t="n"/>
+      <c r="D41" s="25" t="n"/>
+      <c r="E41" s="25" t="n"/>
     </row>
     <row r="42">
-      <c r="A42" s="22" t="n"/>
-      <c r="B42" s="22" t="n"/>
-      <c r="C42" s="22" t="n"/>
-      <c r="D42" s="22" t="n"/>
-      <c r="E42" s="22" t="n"/>
+      <c r="A42" s="25" t="n"/>
+      <c r="B42" s="25" t="n"/>
+      <c r="C42" s="25" t="n"/>
+      <c r="D42" s="25" t="n"/>
+      <c r="E42" s="25" t="n"/>
     </row>
     <row r="43">
-      <c r="A43" s="22" t="n"/>
-      <c r="B43" s="22" t="n"/>
-      <c r="C43" s="22" t="n"/>
-      <c r="D43" s="22" t="n"/>
-      <c r="E43" s="22" t="n"/>
+      <c r="A43" s="25" t="n"/>
+      <c r="B43" s="25" t="n"/>
+      <c r="C43" s="25" t="n"/>
+      <c r="D43" s="25" t="n"/>
+      <c r="E43" s="25" t="n"/>
     </row>
     <row r="44">
-      <c r="A44" s="22" t="n"/>
-      <c r="B44" s="22" t="n"/>
-      <c r="C44" s="22" t="n"/>
-      <c r="D44" s="22" t="n"/>
-      <c r="E44" s="22" t="n"/>
+      <c r="A44" s="25" t="n"/>
+      <c r="B44" s="25" t="n"/>
+      <c r="C44" s="25" t="n"/>
+      <c r="D44" s="25" t="n"/>
+      <c r="E44" s="25" t="n"/>
     </row>
     <row r="45">
-      <c r="A45" s="22" t="n"/>
-      <c r="B45" s="22" t="n"/>
-      <c r="C45" s="22" t="n"/>
-      <c r="D45" s="22" t="n"/>
-      <c r="E45" s="22" t="n"/>
+      <c r="A45" s="25" t="n"/>
+      <c r="B45" s="25" t="n"/>
+      <c r="C45" s="25" t="n"/>
+      <c r="D45" s="25" t="n"/>
+      <c r="E45" s="25" t="n"/>
     </row>
     <row r="46">
-      <c r="A46" s="22" t="n"/>
-      <c r="B46" s="22" t="n"/>
-      <c r="C46" s="22" t="n"/>
-      <c r="D46" s="22" t="n"/>
-      <c r="E46" s="22" t="n"/>
+      <c r="A46" s="25" t="n"/>
+      <c r="B46" s="25" t="n"/>
+      <c r="C46" s="25" t="n"/>
+      <c r="D46" s="25" t="n"/>
+      <c r="E46" s="25" t="n"/>
     </row>
     <row r="47">
-      <c r="A47" s="22" t="n"/>
-      <c r="B47" s="22" t="n"/>
-      <c r="C47" s="22" t="n"/>
-      <c r="D47" s="22" t="n"/>
-      <c r="E47" s="22" t="n"/>
+      <c r="A47" s="25" t="n"/>
+      <c r="B47" s="25" t="n"/>
+      <c r="C47" s="25" t="n"/>
+      <c r="D47" s="25" t="n"/>
+      <c r="E47" s="25" t="n"/>
     </row>
     <row r="48">
-      <c r="A48" s="22" t="n"/>
-      <c r="B48" s="22" t="n"/>
-      <c r="C48" s="22" t="n"/>
-      <c r="D48" s="22" t="n"/>
-      <c r="E48" s="22" t="n"/>
+      <c r="A48" s="25" t="n"/>
+      <c r="B48" s="25" t="n"/>
+      <c r="C48" s="25" t="n"/>
+      <c r="D48" s="25" t="n"/>
+      <c r="E48" s="25" t="n"/>
     </row>
     <row r="49">
-      <c r="A49" s="22" t="n"/>
-      <c r="B49" s="22" t="n"/>
-      <c r="C49" s="22" t="n"/>
-      <c r="D49" s="22" t="n"/>
-      <c r="E49" s="22" t="n"/>
+      <c r="A49" s="25" t="n"/>
+      <c r="B49" s="25" t="n"/>
+      <c r="C49" s="25" t="n"/>
+      <c r="D49" s="25" t="n"/>
+      <c r="E49" s="25" t="n"/>
     </row>
     <row r="50">
-      <c r="A50" s="22" t="n"/>
-      <c r="B50" s="22" t="n"/>
-      <c r="C50" s="22" t="n"/>
-      <c r="D50" s="22" t="n"/>
-      <c r="E50" s="22" t="n"/>
+      <c r="A50" s="25" t="n"/>
+      <c r="B50" s="25" t="n"/>
+      <c r="C50" s="25" t="n"/>
+      <c r="D50" s="25" t="n"/>
+      <c r="E50" s="25" t="n"/>
     </row>
     <row r="51">
-      <c r="A51" s="22" t="n"/>
-      <c r="B51" s="22" t="n"/>
-      <c r="C51" s="22" t="n"/>
-      <c r="D51" s="22" t="n"/>
-      <c r="E51" s="22" t="n"/>
+      <c r="A51" s="25" t="n"/>
+      <c r="B51" s="25" t="n"/>
+      <c r="C51" s="25" t="n"/>
+      <c r="D51" s="25" t="n"/>
+      <c r="E51" s="25" t="n"/>
     </row>
     <row r="52">
-      <c r="A52" s="22" t="n"/>
-      <c r="B52" s="22" t="n"/>
-      <c r="C52" s="22" t="n"/>
-      <c r="D52" s="22" t="n"/>
-      <c r="E52" s="22" t="n"/>
+      <c r="A52" s="25" t="n"/>
+      <c r="B52" s="25" t="n"/>
+      <c r="C52" s="25" t="n"/>
+      <c r="D52" s="25" t="n"/>
+      <c r="E52" s="25" t="n"/>
     </row>
     <row r="53">
-      <c r="A53" s="22" t="n"/>
-      <c r="B53" s="22" t="n"/>
-      <c r="C53" s="22" t="n"/>
-      <c r="D53" s="22" t="n"/>
-      <c r="E53" s="22" t="n"/>
+      <c r="A53" s="25" t="n"/>
+      <c r="B53" s="25" t="n"/>
+      <c r="C53" s="25" t="n"/>
+      <c r="D53" s="25" t="n"/>
+      <c r="E53" s="25" t="n"/>
     </row>
     <row r="54">
-      <c r="A54" s="22" t="n"/>
-      <c r="B54" s="22" t="n"/>
-      <c r="C54" s="22" t="n"/>
-      <c r="D54" s="22" t="n"/>
-      <c r="E54" s="22" t="n"/>
+      <c r="A54" s="25" t="n"/>
+      <c r="B54" s="25" t="n"/>
+      <c r="C54" s="25" t="n"/>
+      <c r="D54" s="25" t="n"/>
+      <c r="E54" s="25" t="n"/>
     </row>
     <row r="55">
-      <c r="A55" s="22" t="n"/>
-      <c r="B55" s="22" t="n"/>
-      <c r="C55" s="22" t="n"/>
-      <c r="D55" s="22" t="n"/>
-      <c r="E55" s="22" t="n"/>
+      <c r="A55" s="25" t="n"/>
+      <c r="B55" s="25" t="n"/>
+      <c r="C55" s="25" t="n"/>
+      <c r="D55" s="25" t="n"/>
+      <c r="E55" s="25" t="n"/>
     </row>
     <row r="56">
-      <c r="A56" s="22" t="n"/>
-      <c r="B56" s="22" t="n"/>
-      <c r="C56" s="22" t="n"/>
-      <c r="D56" s="22" t="n"/>
-      <c r="E56" s="22" t="n"/>
+      <c r="A56" s="25" t="n"/>
+      <c r="B56" s="25" t="n"/>
+      <c r="C56" s="25" t="n"/>
+      <c r="D56" s="25" t="n"/>
+      <c r="E56" s="25" t="n"/>
     </row>
     <row r="57">
-      <c r="A57" s="22" t="n"/>
-      <c r="B57" s="22" t="n"/>
-      <c r="C57" s="22" t="n"/>
-      <c r="D57" s="22" t="n"/>
-      <c r="E57" s="22" t="n"/>
+      <c r="A57" s="25" t="n"/>
+      <c r="B57" s="25" t="n"/>
+      <c r="C57" s="25" t="n"/>
+      <c r="D57" s="25" t="n"/>
+      <c r="E57" s="25" t="n"/>
     </row>
     <row r="58">
-      <c r="A58" s="22" t="n"/>
-      <c r="B58" s="22" t="n"/>
-      <c r="C58" s="22" t="n"/>
-      <c r="D58" s="22" t="n"/>
-      <c r="E58" s="22" t="n"/>
+      <c r="A58" s="25" t="n"/>
+      <c r="B58" s="25" t="n"/>
+      <c r="C58" s="25" t="n"/>
+      <c r="D58" s="25" t="n"/>
+      <c r="E58" s="25" t="n"/>
     </row>
     <row r="59">
-      <c r="A59" s="22" t="n"/>
-      <c r="B59" s="22" t="n"/>
-      <c r="C59" s="22" t="n"/>
-      <c r="D59" s="22" t="n"/>
-      <c r="E59" s="22" t="n"/>
+      <c r="A59" s="25" t="n"/>
+      <c r="B59" s="25" t="n"/>
+      <c r="C59" s="25" t="n"/>
+      <c r="D59" s="25" t="n"/>
+      <c r="E59" s="25" t="n"/>
     </row>
     <row r="60">
-      <c r="A60" s="22" t="n"/>
-      <c r="B60" s="22" t="n"/>
-      <c r="C60" s="22" t="n"/>
-      <c r="D60" s="22" t="n"/>
-      <c r="E60" s="22" t="n"/>
+      <c r="A60" s="25" t="n"/>
+      <c r="B60" s="25" t="n"/>
+      <c r="C60" s="25" t="n"/>
+      <c r="D60" s="25" t="n"/>
+      <c r="E60" s="25" t="n"/>
     </row>
     <row r="61">
-      <c r="A61" s="22" t="n"/>
-      <c r="B61" s="22" t="n"/>
-      <c r="C61" s="22" t="n"/>
-      <c r="D61" s="22" t="n"/>
-      <c r="E61" s="22" t="n"/>
+      <c r="A61" s="25" t="n"/>
+      <c r="B61" s="25" t="n"/>
+      <c r="C61" s="25" t="n"/>
+      <c r="D61" s="25" t="n"/>
+      <c r="E61" s="25" t="n"/>
     </row>
     <row r="62">
-      <c r="A62" s="22" t="n"/>
-      <c r="B62" s="22" t="n"/>
-      <c r="C62" s="22" t="n"/>
-      <c r="D62" s="22" t="n"/>
-      <c r="E62" s="22" t="n"/>
+      <c r="A62" s="25" t="n"/>
+      <c r="B62" s="25" t="n"/>
+      <c r="C62" s="25" t="n"/>
+      <c r="D62" s="25" t="n"/>
+      <c r="E62" s="25" t="n"/>
     </row>
     <row r="63">
-      <c r="A63" s="22" t="n"/>
-      <c r="B63" s="22" t="n"/>
-      <c r="C63" s="22" t="n"/>
-      <c r="D63" s="22" t="n"/>
-      <c r="E63" s="22" t="n"/>
+      <c r="A63" s="25" t="n"/>
+      <c r="B63" s="25" t="n"/>
+      <c r="C63" s="25" t="n"/>
+      <c r="D63" s="25" t="n"/>
+      <c r="E63" s="25" t="n"/>
     </row>
     <row r="64">
-      <c r="A64" s="22" t="n"/>
-      <c r="B64" s="22" t="n"/>
-      <c r="C64" s="22" t="n"/>
-      <c r="D64" s="22" t="n"/>
-      <c r="E64" s="22" t="n"/>
+      <c r="A64" s="25" t="n"/>
+      <c r="B64" s="25" t="n"/>
+      <c r="C64" s="25" t="n"/>
+      <c r="D64" s="25" t="n"/>
+      <c r="E64" s="25" t="n"/>
     </row>
     <row r="65">
-      <c r="A65" s="22" t="n"/>
-      <c r="B65" s="22" t="n"/>
-      <c r="C65" s="22" t="n"/>
-      <c r="D65" s="22" t="n"/>
-      <c r="E65" s="22" t="n"/>
+      <c r="A65" s="25" t="n"/>
+      <c r="B65" s="25" t="n"/>
+      <c r="C65" s="25" t="n"/>
+      <c r="D65" s="25" t="n"/>
+      <c r="E65" s="25" t="n"/>
     </row>
     <row r="66">
-      <c r="A66" s="22" t="n"/>
-      <c r="B66" s="22" t="n"/>
-      <c r="C66" s="22" t="n"/>
-      <c r="D66" s="22" t="n"/>
-      <c r="E66" s="22" t="n"/>
+      <c r="A66" s="25" t="n"/>
+      <c r="B66" s="25" t="n"/>
+      <c r="C66" s="25" t="n"/>
+      <c r="D66" s="25" t="n"/>
+      <c r="E66" s="25" t="n"/>
     </row>
     <row r="67">
-      <c r="A67" s="22" t="n"/>
-      <c r="B67" s="22" t="n"/>
-      <c r="C67" s="22" t="n"/>
-      <c r="D67" s="22" t="n"/>
-      <c r="E67" s="22" t="n"/>
+      <c r="A67" s="25" t="n"/>
+      <c r="B67" s="25" t="n"/>
+      <c r="C67" s="25" t="n"/>
+      <c r="D67" s="25" t="n"/>
+      <c r="E67" s="25" t="n"/>
     </row>
     <row r="68">
-      <c r="A68" s="22" t="n"/>
-      <c r="B68" s="22" t="n"/>
-      <c r="C68" s="22" t="n"/>
-      <c r="D68" s="22" t="n"/>
-      <c r="E68" s="22" t="n"/>
+      <c r="A68" s="25" t="n"/>
+      <c r="B68" s="25" t="n"/>
+      <c r="C68" s="25" t="n"/>
+      <c r="D68" s="25" t="n"/>
+      <c r="E68" s="25" t="n"/>
     </row>
     <row r="69">
-      <c r="A69" s="22" t="n"/>
-      <c r="B69" s="22" t="n"/>
-      <c r="C69" s="22" t="n"/>
-      <c r="D69" s="22" t="n"/>
-      <c r="E69" s="22" t="n"/>
+      <c r="A69" s="25" t="n"/>
+      <c r="B69" s="25" t="n"/>
+      <c r="C69" s="25" t="n"/>
+      <c r="D69" s="25" t="n"/>
+      <c r="E69" s="25" t="n"/>
     </row>
     <row r="70">
-      <c r="A70" s="22" t="n"/>
-      <c r="B70" s="22" t="n"/>
-      <c r="C70" s="22" t="n"/>
-      <c r="D70" s="22" t="n"/>
-      <c r="E70" s="22" t="n"/>
+      <c r="A70" s="25" t="n"/>
+      <c r="B70" s="25" t="n"/>
+      <c r="C70" s="25" t="n"/>
+      <c r="D70" s="25" t="n"/>
+      <c r="E70" s="25" t="n"/>
     </row>
     <row r="71">
-      <c r="A71" s="22" t="n"/>
-      <c r="B71" s="22" t="n"/>
-      <c r="C71" s="22" t="n"/>
-      <c r="D71" s="22" t="n"/>
-      <c r="E71" s="22" t="n"/>
+      <c r="A71" s="25" t="n"/>
+      <c r="B71" s="25" t="n"/>
+      <c r="C71" s="25" t="n"/>
+      <c r="D71" s="25" t="n"/>
+      <c r="E71" s="25" t="n"/>
     </row>
     <row r="72">
-      <c r="A72" s="22" t="n"/>
-      <c r="B72" s="22" t="n"/>
-      <c r="C72" s="22" t="n"/>
-      <c r="D72" s="22" t="n"/>
-      <c r="E72" s="22" t="n"/>
+      <c r="A72" s="25" t="n"/>
+      <c r="B72" s="25" t="n"/>
+      <c r="C72" s="25" t="n"/>
+      <c r="D72" s="25" t="n"/>
+      <c r="E72" s="25" t="n"/>
     </row>
     <row r="73">
-      <c r="A73" s="22" t="n"/>
-      <c r="B73" s="22" t="n"/>
-      <c r="C73" s="22" t="n"/>
-      <c r="D73" s="22" t="n"/>
-      <c r="E73" s="22" t="n"/>
+      <c r="A73" s="25" t="n"/>
+      <c r="B73" s="25" t="n"/>
+      <c r="C73" s="25" t="n"/>
+      <c r="D73" s="25" t="n"/>
+      <c r="E73" s="25" t="n"/>
     </row>
     <row r="74">
-      <c r="A74" s="22" t="n"/>
-      <c r="B74" s="22" t="n"/>
-      <c r="C74" s="22" t="n"/>
-      <c r="D74" s="22" t="n"/>
-      <c r="E74" s="22" t="n"/>
+      <c r="A74" s="25" t="n"/>
+      <c r="B74" s="25" t="n"/>
+      <c r="C74" s="25" t="n"/>
+      <c r="D74" s="25" t="n"/>
+      <c r="E74" s="25" t="n"/>
     </row>
     <row r="75">
-      <c r="A75" s="22" t="n"/>
-      <c r="B75" s="22" t="n"/>
-      <c r="C75" s="22" t="n"/>
-      <c r="D75" s="22" t="n"/>
-      <c r="E75" s="22" t="n"/>
+      <c r="A75" s="25" t="n"/>
+      <c r="B75" s="25" t="n"/>
+      <c r="C75" s="25" t="n"/>
+      <c r="D75" s="25" t="n"/>
+      <c r="E75" s="25" t="n"/>
     </row>
     <row r="76">
-      <c r="A76" s="22" t="n"/>
-      <c r="B76" s="22" t="n"/>
-      <c r="C76" s="22" t="n"/>
-      <c r="D76" s="22" t="n"/>
-      <c r="E76" s="22" t="n"/>
+      <c r="A76" s="25" t="n"/>
+      <c r="B76" s="25" t="n"/>
+      <c r="C76" s="25" t="n"/>
+      <c r="D76" s="25" t="n"/>
+      <c r="E76" s="25" t="n"/>
     </row>
     <row r="77">
-      <c r="A77" s="22" t="n"/>
-      <c r="B77" s="22" t="n"/>
-      <c r="C77" s="22" t="n"/>
-      <c r="D77" s="22" t="n"/>
-      <c r="E77" s="22" t="n"/>
+      <c r="A77" s="25" t="n"/>
+      <c r="B77" s="25" t="n"/>
+      <c r="C77" s="25" t="n"/>
+      <c r="D77" s="25" t="n"/>
+      <c r="E77" s="25" t="n"/>
     </row>
     <row r="78">
-      <c r="A78" s="22" t="n"/>
-      <c r="B78" s="22" t="n"/>
-      <c r="C78" s="22" t="n"/>
-      <c r="D78" s="22" t="n"/>
-      <c r="E78" s="22" t="n"/>
+      <c r="A78" s="25" t="n"/>
+      <c r="B78" s="25" t="n"/>
+      <c r="C78" s="25" t="n"/>
+      <c r="D78" s="25" t="n"/>
+      <c r="E78" s="25" t="n"/>
     </row>
     <row r="79">
-      <c r="A79" s="22" t="n"/>
-      <c r="B79" s="22" t="n"/>
-      <c r="C79" s="22" t="n"/>
-      <c r="D79" s="22" t="n"/>
-      <c r="E79" s="22" t="n"/>
+      <c r="A79" s="25" t="n"/>
+      <c r="B79" s="25" t="n"/>
+      <c r="C79" s="25" t="n"/>
+      <c r="D79" s="25" t="n"/>
+      <c r="E79" s="25" t="n"/>
     </row>
     <row r="80">
-      <c r="A80" s="22" t="n"/>
-      <c r="B80" s="22" t="n"/>
-      <c r="C80" s="22" t="n"/>
-      <c r="D80" s="22" t="n"/>
-      <c r="E80" s="22" t="n"/>
+      <c r="A80" s="25" t="n"/>
+      <c r="B80" s="25" t="n"/>
+      <c r="C80" s="25" t="n"/>
+      <c r="D80" s="25" t="n"/>
+      <c r="E80" s="25" t="n"/>
     </row>
     <row r="81">
-      <c r="A81" s="22" t="n"/>
-      <c r="B81" s="22" t="n"/>
-      <c r="C81" s="22" t="n"/>
-      <c r="D81" s="22" t="n"/>
-      <c r="E81" s="22" t="n"/>
+      <c r="A81" s="25" t="n"/>
+      <c r="B81" s="25" t="n"/>
+      <c r="C81" s="25" t="n"/>
+      <c r="D81" s="25" t="n"/>
+      <c r="E81" s="25" t="n"/>
     </row>
     <row r="82">
-      <c r="A82" s="22" t="n"/>
-      <c r="B82" s="22" t="n"/>
-      <c r="C82" s="22" t="n"/>
-      <c r="D82" s="22" t="n"/>
-      <c r="E82" s="22" t="n"/>
+      <c r="A82" s="25" t="n"/>
+      <c r="B82" s="25" t="n"/>
+      <c r="C82" s="25" t="n"/>
+      <c r="D82" s="25" t="n"/>
+      <c r="E82" s="25" t="n"/>
     </row>
     <row r="83">
-      <c r="A83" s="22" t="n"/>
-      <c r="B83" s="22" t="n"/>
-      <c r="C83" s="22" t="n"/>
-      <c r="D83" s="22" t="n"/>
-      <c r="E83" s="22" t="n"/>
+      <c r="A83" s="25" t="n"/>
+      <c r="B83" s="25" t="n"/>
+      <c r="C83" s="25" t="n"/>
+      <c r="D83" s="25" t="n"/>
+      <c r="E83" s="25" t="n"/>
     </row>
     <row r="84">
-      <c r="A84" s="22" t="n"/>
-      <c r="B84" s="22" t="n"/>
-      <c r="C84" s="22" t="n"/>
-      <c r="D84" s="22" t="n"/>
-      <c r="E84" s="22" t="n"/>
+      <c r="A84" s="25" t="n"/>
+      <c r="B84" s="25" t="n"/>
+      <c r="C84" s="25" t="n"/>
+      <c r="D84" s="25" t="n"/>
+      <c r="E84" s="25" t="n"/>
     </row>
     <row r="85">
-      <c r="A85" s="22" t="n"/>
-      <c r="B85" s="22" t="n"/>
-      <c r="C85" s="22" t="n"/>
-      <c r="D85" s="22" t="n"/>
-      <c r="E85" s="22" t="n"/>
+      <c r="A85" s="25" t="n"/>
+      <c r="B85" s="25" t="n"/>
+      <c r="C85" s="25" t="n"/>
+      <c r="D85" s="25" t="n"/>
+      <c r="E85" s="25" t="n"/>
     </row>
     <row r="86">
-      <c r="A86" s="22" t="n"/>
-      <c r="B86" s="22" t="n"/>
-      <c r="C86" s="22" t="n"/>
-      <c r="D86" s="22" t="n"/>
-      <c r="E86" s="22" t="n"/>
+      <c r="A86" s="25" t="n"/>
+      <c r="B86" s="25" t="n"/>
+      <c r="C86" s="25" t="n"/>
+      <c r="D86" s="25" t="n"/>
+      <c r="E86" s="25" t="n"/>
     </row>
     <row r="87">
-      <c r="A87" s="22" t="n"/>
-      <c r="B87" s="22" t="n"/>
-      <c r="C87" s="22" t="n"/>
-      <c r="D87" s="22" t="n"/>
-      <c r="E87" s="22" t="n"/>
+      <c r="A87" s="25" t="n"/>
+      <c r="B87" s="25" t="n"/>
+      <c r="C87" s="25" t="n"/>
+      <c r="D87" s="25" t="n"/>
+      <c r="E87" s="25" t="n"/>
     </row>
     <row r="88">
-      <c r="A88" s="22" t="n"/>
-      <c r="B88" s="22" t="n"/>
-      <c r="C88" s="22" t="n"/>
-      <c r="D88" s="22" t="n"/>
-      <c r="E88" s="22" t="n"/>
+      <c r="A88" s="25" t="n"/>
+      <c r="B88" s="25" t="n"/>
+      <c r="C88" s="25" t="n"/>
+      <c r="D88" s="25" t="n"/>
+      <c r="E88" s="25" t="n"/>
     </row>
     <row r="89">
-      <c r="A89" s="22" t="n"/>
-      <c r="B89" s="22" t="n"/>
-      <c r="C89" s="22" t="n"/>
-      <c r="D89" s="22" t="n"/>
-      <c r="E89" s="22" t="n"/>
+      <c r="A89" s="25" t="n"/>
+      <c r="B89" s="25" t="n"/>
+      <c r="C89" s="25" t="n"/>
+      <c r="D89" s="25" t="n"/>
+      <c r="E89" s="25" t="n"/>
     </row>
     <row r="90">
-      <c r="A90" s="22" t="n"/>
-      <c r="B90" s="22" t="n"/>
-      <c r="C90" s="22" t="n"/>
-      <c r="D90" s="22" t="n"/>
-      <c r="E90" s="22" t="n"/>
+      <c r="A90" s="25" t="n"/>
+      <c r="B90" s="25" t="n"/>
+      <c r="C90" s="25" t="n"/>
+      <c r="D90" s="25" t="n"/>
+      <c r="E90" s="25" t="n"/>
     </row>
     <row r="91">
-      <c r="A91" s="22" t="n"/>
-      <c r="B91" s="22" t="n"/>
-      <c r="C91" s="22" t="n"/>
-      <c r="D91" s="22" t="n"/>
-      <c r="E91" s="22" t="n"/>
+      <c r="A91" s="25" t="n"/>
+      <c r="B91" s="25" t="n"/>
+      <c r="C91" s="25" t="n"/>
+      <c r="D91" s="25" t="n"/>
+      <c r="E91" s="25" t="n"/>
     </row>
     <row r="92">
-      <c r="A92" s="22" t="n"/>
-      <c r="B92" s="22" t="n"/>
-      <c r="C92" s="22" t="n"/>
-      <c r="D92" s="22" t="n"/>
-      <c r="E92" s="22" t="n"/>
+      <c r="A92" s="25" t="n"/>
+      <c r="B92" s="25" t="n"/>
+      <c r="C92" s="25" t="n"/>
+      <c r="D92" s="25" t="n"/>
+      <c r="E92" s="25" t="n"/>
     </row>
     <row r="93">
-      <c r="A93" s="22" t="n"/>
-      <c r="B93" s="22" t="n"/>
-      <c r="C93" s="22" t="n"/>
-      <c r="D93" s="22" t="n"/>
-      <c r="E93" s="22" t="n"/>
+      <c r="A93" s="25" t="n"/>
+      <c r="B93" s="25" t="n"/>
+      <c r="C93" s="25" t="n"/>
+      <c r="D93" s="25" t="n"/>
+      <c r="E93" s="25" t="n"/>
     </row>
     <row r="94">
-      <c r="A94" s="22" t="n"/>
-      <c r="B94" s="22" t="n"/>
-      <c r="C94" s="22" t="n"/>
-      <c r="D94" s="22" t="n"/>
-      <c r="E94" s="22" t="n"/>
+      <c r="A94" s="25" t="n"/>
+      <c r="B94" s="25" t="n"/>
+      <c r="C94" s="25" t="n"/>
+      <c r="D94" s="25" t="n"/>
+      <c r="E94" s="25" t="n"/>
     </row>
     <row r="95">
-      <c r="A95" s="22" t="n"/>
-      <c r="B95" s="22" t="n"/>
-      <c r="C95" s="22" t="n"/>
-      <c r="D95" s="22" t="n"/>
-      <c r="E95" s="22" t="n"/>
+      <c r="A95" s="25" t="n"/>
+      <c r="B95" s="25" t="n"/>
+      <c r="C95" s="25" t="n"/>
+      <c r="D95" s="25" t="n"/>
+      <c r="E95" s="25" t="n"/>
     </row>
     <row r="96">
-      <c r="A96" s="22" t="n"/>
-      <c r="B96" s="22" t="n"/>
-      <c r="C96" s="22" t="n"/>
-      <c r="D96" s="22" t="n"/>
-      <c r="E96" s="22" t="n"/>
+      <c r="A96" s="25" t="n"/>
+      <c r="B96" s="25" t="n"/>
+      <c r="C96" s="25" t="n"/>
+      <c r="D96" s="25" t="n"/>
+      <c r="E96" s="25" t="n"/>
     </row>
     <row r="97">
-      <c r="A97" s="22" t="n"/>
-      <c r="B97" s="22" t="n"/>
-      <c r="C97" s="22" t="n"/>
-      <c r="D97" s="22" t="n"/>
-      <c r="E97" s="22" t="n"/>
+      <c r="A97" s="25" t="n"/>
+      <c r="B97" s="25" t="n"/>
+      <c r="C97" s="25" t="n"/>
+      <c r="D97" s="25" t="n"/>
+      <c r="E97" s="25" t="n"/>
     </row>
     <row r="98">
-      <c r="A98" s="22" t="n"/>
-      <c r="B98" s="22" t="n"/>
-      <c r="C98" s="22" t="n"/>
-      <c r="D98" s="22" t="n"/>
-      <c r="E98" s="22" t="n"/>
+      <c r="A98" s="25" t="n"/>
+      <c r="B98" s="25" t="n"/>
+      <c r="C98" s="25" t="n"/>
+      <c r="D98" s="25" t="n"/>
+      <c r="E98" s="25" t="n"/>
     </row>
     <row r="99">
-      <c r="A99" s="22" t="n"/>
-      <c r="B99" s="22" t="n"/>
-      <c r="C99" s="22" t="n"/>
-      <c r="D99" s="22" t="n"/>
-      <c r="E99" s="22" t="n"/>
+      <c r="A99" s="25" t="n"/>
+      <c r="B99" s="25" t="n"/>
+      <c r="C99" s="25" t="n"/>
+      <c r="D99" s="25" t="n"/>
+      <c r="E99" s="25" t="n"/>
     </row>
     <row r="100">
-      <c r="A100" s="22" t="n"/>
-      <c r="B100" s="22" t="n"/>
-      <c r="C100" s="22" t="n"/>
-      <c r="D100" s="22" t="n"/>
-      <c r="E100" s="22" t="n"/>
+      <c r="A100" s="25" t="n"/>
+      <c r="B100" s="25" t="n"/>
+      <c r="C100" s="25" t="n"/>
+      <c r="D100" s="25" t="n"/>
+      <c r="E100" s="25" t="n"/>
     </row>
     <row r="101">
-      <c r="A101" s="22" t="n"/>
-      <c r="B101" s="22" t="n"/>
-      <c r="C101" s="22" t="n"/>
-      <c r="D101" s="22" t="n"/>
-      <c r="E101" s="22" t="n"/>
+      <c r="A101" s="25" t="n"/>
+      <c r="B101" s="25" t="n"/>
+      <c r="C101" s="25" t="n"/>
+      <c r="D101" s="25" t="n"/>
+      <c r="E101" s="25" t="n"/>
     </row>
     <row r="102">
-      <c r="A102" s="22" t="n"/>
-      <c r="B102" s="22" t="n"/>
-      <c r="C102" s="22" t="n"/>
-      <c r="D102" s="22" t="n"/>
-      <c r="E102" s="22" t="n"/>
+      <c r="A102" s="25" t="n"/>
+      <c r="B102" s="25" t="n"/>
+      <c r="C102" s="25" t="n"/>
+      <c r="D102" s="25" t="n"/>
+      <c r="E102" s="25" t="n"/>
     </row>
     <row r="103">
-      <c r="A103" s="22" t="n"/>
-      <c r="B103" s="22" t="n"/>
-      <c r="C103" s="22" t="n"/>
-      <c r="D103" s="22" t="n"/>
-      <c r="E103" s="22" t="n"/>
+      <c r="A103" s="25" t="n"/>
+      <c r="B103" s="25" t="n"/>
+      <c r="C103" s="25" t="n"/>
+      <c r="D103" s="25" t="n"/>
+      <c r="E103" s="25" t="n"/>
     </row>
     <row r="104">
-      <c r="A104" s="22" t="n"/>
-      <c r="B104" s="22" t="n"/>
-      <c r="C104" s="22" t="n"/>
-      <c r="D104" s="22" t="n"/>
-      <c r="E104" s="22" t="n"/>
+      <c r="A104" s="25" t="n"/>
+      <c r="B104" s="25" t="n"/>
+      <c r="C104" s="25" t="n"/>
+      <c r="D104" s="25" t="n"/>
+      <c r="E104" s="25" t="n"/>
     </row>
     <row r="105">
-      <c r="A105" s="22" t="n"/>
-      <c r="B105" s="22" t="n"/>
-      <c r="C105" s="22" t="n"/>
-      <c r="D105" s="22" t="n"/>
-      <c r="E105" s="22" t="n"/>
+      <c r="A105" s="25" t="n"/>
+      <c r="B105" s="25" t="n"/>
+      <c r="C105" s="25" t="n"/>
+      <c r="D105" s="25" t="n"/>
+      <c r="E105" s="25" t="n"/>
     </row>
     <row r="106">
-      <c r="A106" s="22" t="n"/>
-      <c r="B106" s="22" t="n"/>
-      <c r="C106" s="22" t="n"/>
-      <c r="D106" s="22" t="n"/>
-      <c r="E106" s="22" t="n"/>
+      <c r="A106" s="25" t="n"/>
+      <c r="B106" s="25" t="n"/>
+      <c r="C106" s="25" t="n"/>
+      <c r="D106" s="25" t="n"/>
+      <c r="E106" s="25" t="n"/>
     </row>
     <row r="107">
-      <c r="A107" s="22" t="n"/>
-      <c r="B107" s="22" t="n"/>
-      <c r="C107" s="22" t="n"/>
-      <c r="D107" s="22" t="n"/>
-      <c r="E107" s="22" t="n"/>
+      <c r="A107" s="25" t="n"/>
+      <c r="B107" s="25" t="n"/>
+      <c r="C107" s="25" t="n"/>
+      <c r="D107" s="25" t="n"/>
+      <c r="E107" s="25" t="n"/>
     </row>
     <row r="108">
-      <c r="A108" s="22" t="n"/>
-      <c r="B108" s="22" t="n"/>
-      <c r="C108" s="22" t="n"/>
-      <c r="D108" s="22" t="n"/>
-      <c r="E108" s="22" t="n"/>
+      <c r="A108" s="25" t="n"/>
+      <c r="B108" s="25" t="n"/>
+      <c r="C108" s="25" t="n"/>
+      <c r="D108" s="25" t="n"/>
+      <c r="E108" s="25" t="n"/>
     </row>
     <row r="109">
-      <c r="A109" s="22" t="n"/>
-      <c r="B109" s="22" t="n"/>
-      <c r="C109" s="22" t="n"/>
-      <c r="D109" s="22" t="n"/>
-      <c r="E109" s="22" t="n"/>
+      <c r="A109" s="25" t="n"/>
+      <c r="B109" s="25" t="n"/>
+      <c r="C109" s="25" t="n"/>
+      <c r="D109" s="25" t="n"/>
+      <c r="E109" s="25" t="n"/>
     </row>
     <row r="110">
-      <c r="A110" s="22" t="n"/>
-      <c r="B110" s="22" t="n"/>
-      <c r="C110" s="22" t="n"/>
-      <c r="D110" s="22" t="n"/>
-      <c r="E110" s="22" t="n"/>
+      <c r="A110" s="25" t="n"/>
+      <c r="B110" s="25" t="n"/>
+      <c r="C110" s="25" t="n"/>
+      <c r="D110" s="25" t="n"/>
+      <c r="E110" s="25" t="n"/>
     </row>
     <row r="111">
-      <c r="A111" s="22" t="n"/>
-      <c r="B111" s="22" t="n"/>
-      <c r="C111" s="22" t="n"/>
-      <c r="D111" s="22" t="n"/>
-      <c r="E111" s="22" t="n"/>
+      <c r="A111" s="25" t="n"/>
+      <c r="B111" s="25" t="n"/>
+      <c r="C111" s="25" t="n"/>
+      <c r="D111" s="25" t="n"/>
+      <c r="E111" s="25" t="n"/>
     </row>
     <row r="112">
-      <c r="A112" s="22" t="n"/>
-      <c r="B112" s="22" t="n"/>
-      <c r="C112" s="22" t="n"/>
-      <c r="D112" s="22" t="n"/>
-      <c r="E112" s="22" t="n"/>
+      <c r="A112" s="25" t="n"/>
+      <c r="B112" s="25" t="n"/>
+      <c r="C112" s="25" t="n"/>
+      <c r="D112" s="25" t="n"/>
+      <c r="E112" s="25" t="n"/>
     </row>
     <row r="113">
-      <c r="A113" s="22" t="n"/>
-      <c r="B113" s="22" t="n"/>
-      <c r="C113" s="22" t="n"/>
-      <c r="D113" s="22" t="n"/>
-      <c r="E113" s="22" t="n"/>
+      <c r="A113" s="25" t="n"/>
+      <c r="B113" s="25" t="n"/>
+      <c r="C113" s="25" t="n"/>
+      <c r="D113" s="25" t="n"/>
+      <c r="E113" s="25" t="n"/>
     </row>
     <row r="114">
-      <c r="A114" s="22" t="n"/>
-      <c r="B114" s="22" t="n"/>
-      <c r="C114" s="22" t="n"/>
-      <c r="D114" s="22" t="n"/>
-      <c r="E114" s="22" t="n"/>
+      <c r="A114" s="25" t="n"/>
+      <c r="B114" s="25" t="n"/>
+      <c r="C114" s="25" t="n"/>
+      <c r="D114" s="25" t="n"/>
+      <c r="E114" s="25" t="n"/>
     </row>
     <row r="115">
-      <c r="A115" s="22" t="n"/>
-      <c r="B115" s="22" t="n"/>
-      <c r="C115" s="22" t="n"/>
-      <c r="D115" s="22" t="n"/>
-      <c r="E115" s="22" t="n"/>
+      <c r="A115" s="25" t="n"/>
+      <c r="B115" s="25" t="n"/>
+      <c r="C115" s="25" t="n"/>
+      <c r="D115" s="25" t="n"/>
+      <c r="E115" s="25" t="n"/>
     </row>
     <row r="116">
-      <c r="A116" s="22" t="n"/>
-      <c r="B116" s="22" t="n"/>
-      <c r="C116" s="22" t="n"/>
-      <c r="D116" s="22" t="n"/>
-      <c r="E116" s="22" t="n"/>
+      <c r="A116" s="25" t="n"/>
+      <c r="B116" s="25" t="n"/>
+      <c r="C116" s="25" t="n"/>
+      <c r="D116" s="25" t="n"/>
+      <c r="E116" s="25" t="n"/>
     </row>
     <row r="117">
-      <c r="A117" s="22" t="n"/>
-      <c r="B117" s="22" t="n"/>
-      <c r="C117" s="22" t="n"/>
-      <c r="D117" s="22" t="n"/>
-      <c r="E117" s="22" t="n"/>
+      <c r="A117" s="25" t="n"/>
+      <c r="B117" s="25" t="n"/>
+      <c r="C117" s="25" t="n"/>
+      <c r="D117" s="25" t="n"/>
+      <c r="E117" s="25" t="n"/>
     </row>
     <row r="118">
-      <c r="A118" s="22" t="n"/>
-      <c r="B118" s="22" t="n"/>
-      <c r="C118" s="22" t="n"/>
-      <c r="D118" s="22" t="n"/>
-      <c r="E118" s="22" t="n"/>
+      <c r="A118" s="25" t="n"/>
+      <c r="B118" s="25" t="n"/>
+      <c r="C118" s="25" t="n"/>
+      <c r="D118" s="25" t="n"/>
+      <c r="E118" s="25" t="n"/>
     </row>
     <row r="119">
-      <c r="A119" s="22" t="n"/>
-      <c r="B119" s="22" t="n"/>
-      <c r="C119" s="22" t="n"/>
-      <c r="D119" s="22" t="n"/>
-      <c r="E119" s="22" t="n"/>
+      <c r="A119" s="25" t="n"/>
+      <c r="B119" s="25" t="n"/>
+      <c r="C119" s="25" t="n"/>
+      <c r="D119" s="25" t="n"/>
+      <c r="E119" s="25" t="n"/>
     </row>
     <row r="120">
-      <c r="A120" s="22" t="n"/>
-      <c r="B120" s="22" t="n"/>
-      <c r="C120" s="22" t="n"/>
-      <c r="D120" s="22" t="n"/>
-      <c r="E120" s="22" t="n"/>
+      <c r="A120" s="25" t="n"/>
+      <c r="B120" s="25" t="n"/>
+      <c r="C120" s="25" t="n"/>
+      <c r="D120" s="25" t="n"/>
+      <c r="E120" s="25" t="n"/>
     </row>
     <row r="121">
-      <c r="A121" s="22" t="n"/>
-      <c r="B121" s="22" t="n"/>
-      <c r="C121" s="22" t="n"/>
-      <c r="D121" s="22" t="n"/>
-      <c r="E121" s="22" t="n"/>
+      <c r="A121" s="25" t="n"/>
+      <c r="B121" s="25" t="n"/>
+      <c r="C121" s="25" t="n"/>
+      <c r="D121" s="25" t="n"/>
+      <c r="E121" s="25" t="n"/>
     </row>
     <row r="122">
-      <c r="A122" s="22" t="n"/>
-      <c r="B122" s="22" t="n"/>
-      <c r="C122" s="22" t="n"/>
-      <c r="D122" s="22" t="n"/>
-      <c r="E122" s="22" t="n"/>
+      <c r="A122" s="25" t="n"/>
+      <c r="B122" s="25" t="n"/>
+      <c r="C122" s="25" t="n"/>
+      <c r="D122" s="25" t="n"/>
+      <c r="E122" s="25" t="n"/>
     </row>
     <row r="123">
-      <c r="A123" s="22" t="n"/>
-      <c r="B123" s="22" t="n"/>
-      <c r="C123" s="22" t="n"/>
-      <c r="D123" s="22" t="n"/>
-      <c r="E123" s="22" t="n"/>
+      <c r="A123" s="25" t="n"/>
+      <c r="B123" s="25" t="n"/>
+      <c r="C123" s="25" t="n"/>
+      <c r="D123" s="25" t="n"/>
+      <c r="E123" s="25" t="n"/>
     </row>
     <row r="124">
-      <c r="A124" s="22" t="n"/>
-      <c r="B124" s="22" t="n"/>
-      <c r="C124" s="22" t="n"/>
-      <c r="D124" s="22" t="n"/>
-      <c r="E124" s="22" t="n"/>
+      <c r="A124" s="25" t="n"/>
+      <c r="B124" s="25" t="n"/>
+      <c r="C124" s="25" t="n"/>
+      <c r="D124" s="25" t="n"/>
+      <c r="E124" s="25" t="n"/>
     </row>
     <row r="125">
-      <c r="A125" s="22" t="n"/>
-      <c r="B125" s="22" t="n"/>
-      <c r="C125" s="22" t="n"/>
-      <c r="D125" s="22" t="n"/>
-      <c r="E125" s="22" t="n"/>
+      <c r="A125" s="25" t="n"/>
+      <c r="B125" s="25" t="n"/>
+      <c r="C125" s="25" t="n"/>
+      <c r="D125" s="25" t="n"/>
+      <c r="E125" s="25" t="n"/>
     </row>
     <row r="126">
-      <c r="A126" s="22" t="n"/>
-      <c r="B126" s="22" t="n"/>
-      <c r="C126" s="22" t="n"/>
-      <c r="D126" s="22" t="n"/>
-      <c r="E126" s="22" t="n"/>
+      <c r="A126" s="25" t="n"/>
+      <c r="B126" s="25" t="n"/>
+      <c r="C126" s="25" t="n"/>
+      <c r="D126" s="25" t="n"/>
+      <c r="E126" s="25" t="n"/>
     </row>
     <row r="127">
-      <c r="A127" s="22" t="n"/>
-      <c r="B127" s="22" t="n"/>
-      <c r="C127" s="22" t="n"/>
-      <c r="D127" s="22" t="n"/>
-      <c r="E127" s="22" t="n"/>
+      <c r="A127" s="25" t="n"/>
+      <c r="B127" s="25" t="n"/>
+      <c r="C127" s="25" t="n"/>
+      <c r="D127" s="25" t="n"/>
+      <c r="E127" s="25" t="n"/>
     </row>
     <row r="128">
-      <c r="A128" s="22" t="n"/>
-      <c r="B128" s="22" t="n"/>
-      <c r="C128" s="22" t="n"/>
-      <c r="D128" s="22" t="n"/>
-      <c r="E128" s="22" t="n"/>
+      <c r="A128" s="25" t="n"/>
+      <c r="B128" s="25" t="n"/>
+      <c r="C128" s="25" t="n"/>
+      <c r="D128" s="25" t="n"/>
+      <c r="E128" s="25" t="n"/>
     </row>
     <row r="129">
-      <c r="A129" s="22" t="n"/>
-      <c r="B129" s="22" t="n"/>
-      <c r="C129" s="22" t="n"/>
-      <c r="D129" s="22" t="n"/>
-      <c r="E129" s="22" t="n"/>
+      <c r="A129" s="25" t="n"/>
+      <c r="B129" s="25" t="n"/>
+      <c r="C129" s="25" t="n"/>
+      <c r="D129" s="25" t="n"/>
+      <c r="E129" s="25" t="n"/>
     </row>
     <row r="130">
-      <c r="A130" s="22" t="n"/>
-      <c r="B130" s="22" t="n"/>
-      <c r="C130" s="22" t="n"/>
-      <c r="D130" s="22" t="n"/>
-      <c r="E130" s="22" t="n"/>
+      <c r="A130" s="25" t="n"/>
+      <c r="B130" s="25" t="n"/>
+      <c r="C130" s="25" t="n"/>
+      <c r="D130" s="25" t="n"/>
+      <c r="E130" s="25" t="n"/>
     </row>
     <row r="131">
-      <c r="A131" s="22" t="n"/>
-      <c r="B131" s="22" t="n"/>
-      <c r="C131" s="22" t="n"/>
-      <c r="D131" s="22" t="n"/>
-      <c r="E131" s="22" t="n"/>
+      <c r="A131" s="25" t="n"/>
+      <c r="B131" s="25" t="n"/>
+      <c r="C131" s="25" t="n"/>
+      <c r="D131" s="25" t="n"/>
+      <c r="E131" s="25" t="n"/>
     </row>
     <row r="132">
-      <c r="A132" s="22" t="n"/>
-      <c r="B132" s="22" t="n"/>
-      <c r="C132" s="22" t="n"/>
-      <c r="D132" s="22" t="n"/>
-      <c r="E132" s="22" t="n"/>
+      <c r="A132" s="25" t="n"/>
+      <c r="B132" s="25" t="n"/>
+      <c r="C132" s="25" t="n"/>
+      <c r="D132" s="25" t="n"/>
+      <c r="E132" s="25" t="n"/>
     </row>
     <row r="133">
-      <c r="A133" s="22" t="n"/>
-      <c r="B133" s="22" t="n"/>
-      <c r="C133" s="22" t="n"/>
-      <c r="D133" s="22" t="n"/>
-      <c r="E133" s="22" t="n"/>
+      <c r="A133" s="25" t="n"/>
+      <c r="B133" s="25" t="n"/>
+      <c r="C133" s="25" t="n"/>
+      <c r="D133" s="25" t="n"/>
+      <c r="E133" s="25" t="n"/>
     </row>
     <row r="134">
-      <c r="A134" s="22" t="n"/>
-      <c r="B134" s="22" t="n"/>
-      <c r="C134" s="22" t="n"/>
-      <c r="D134" s="22" t="n"/>
-      <c r="E134" s="22" t="n"/>
+      <c r="A134" s="25" t="n"/>
+      <c r="B134" s="25" t="n"/>
+      <c r="C134" s="25" t="n"/>
+      <c r="D134" s="25" t="n"/>
+      <c r="E134" s="25" t="n"/>
     </row>
     <row r="135">
-      <c r="A135" s="22" t="n"/>
-      <c r="B135" s="22" t="n"/>
-      <c r="C135" s="22" t="n"/>
-      <c r="D135" s="22" t="n"/>
-      <c r="E135" s="22" t="n"/>
+      <c r="A135" s="25" t="n"/>
+      <c r="B135" s="25" t="n"/>
+      <c r="C135" s="25" t="n"/>
+      <c r="D135" s="25" t="n"/>
+      <c r="E135" s="25" t="n"/>
     </row>
     <row r="136">
-      <c r="A136" s="22" t="n"/>
-      <c r="B136" s="22" t="n"/>
-      <c r="C136" s="22" t="n"/>
-      <c r="D136" s="22" t="n"/>
-      <c r="E136" s="22" t="n"/>
+      <c r="A136" s="25" t="n"/>
+      <c r="B136" s="25" t="n"/>
+      <c r="C136" s="25" t="n"/>
+      <c r="D136" s="25" t="n"/>
+      <c r="E136" s="25" t="n"/>
     </row>
     <row r="137">
-      <c r="A137" s="22" t="n"/>
-      <c r="B137" s="22" t="n"/>
-      <c r="C137" s="22" t="n"/>
-      <c r="D137" s="22" t="n"/>
-      <c r="E137" s="22" t="n"/>
+      <c r="A137" s="25" t="n"/>
+      <c r="B137" s="25" t="n"/>
+      <c r="C137" s="25" t="n"/>
+      <c r="D137" s="25" t="n"/>
+      <c r="E137" s="25" t="n"/>
     </row>
     <row r="138">
-      <c r="A138" s="22" t="n"/>
-      <c r="B138" s="22" t="n"/>
-      <c r="C138" s="22" t="n"/>
-      <c r="D138" s="22" t="n"/>
-      <c r="E138" s="22" t="n"/>
+      <c r="A138" s="25" t="n"/>
+      <c r="B138" s="25" t="n"/>
+      <c r="C138" s="25" t="n"/>
+      <c r="D138" s="25" t="n"/>
+      <c r="E138" s="25" t="n"/>
     </row>
     <row r="139">
-      <c r="A139" s="22" t="n"/>
-      <c r="B139" s="22" t="n"/>
-      <c r="C139" s="22" t="n"/>
-      <c r="D139" s="22" t="n"/>
-      <c r="E139" s="22" t="n"/>
+      <c r="A139" s="25" t="n"/>
+      <c r="B139" s="25" t="n"/>
+      <c r="C139" s="25" t="n"/>
+      <c r="D139" s="25" t="n"/>
+      <c r="E139" s="25" t="n"/>
     </row>
     <row r="140">
-      <c r="A140" s="22" t="n"/>
-      <c r="B140" s="22" t="n"/>
-      <c r="C140" s="22" t="n"/>
-      <c r="D140" s="22" t="n"/>
-      <c r="E140" s="22" t="n"/>
+      <c r="A140" s="25" t="n"/>
+      <c r="B140" s="25" t="n"/>
+      <c r="C140" s="25" t="n"/>
+      <c r="D140" s="25" t="n"/>
+      <c r="E140" s="25" t="n"/>
     </row>
     <row r="141">
-      <c r="A141" s="22" t="n"/>
-      <c r="B141" s="22" t="n"/>
-      <c r="C141" s="22" t="n"/>
-      <c r="D141" s="22" t="n"/>
-      <c r="E141" s="22" t="n"/>
+      <c r="A141" s="25" t="n"/>
+      <c r="B141" s="25" t="n"/>
+      <c r="C141" s="25" t="n"/>
+      <c r="D141" s="25" t="n"/>
+      <c r="E141" s="25" t="n"/>
     </row>
     <row r="142">
-      <c r="A142" s="22" t="n"/>
-      <c r="B142" s="22" t="n"/>
-      <c r="C142" s="22" t="n"/>
-      <c r="D142" s="22" t="n"/>
-      <c r="E142" s="22" t="n"/>
+      <c r="A142" s="25" t="n"/>
+      <c r="B142" s="25" t="n"/>
+      <c r="C142" s="25" t="n"/>
+      <c r="D142" s="25" t="n"/>
+      <c r="E142" s="25" t="n"/>
     </row>
     <row r="143">
-      <c r="A143" s="22" t="n"/>
-      <c r="B143" s="22" t="n"/>
-      <c r="C143" s="22" t="n"/>
-      <c r="D143" s="22" t="n"/>
-      <c r="E143" s="22" t="n"/>
+      <c r="A143" s="25" t="n"/>
+      <c r="B143" s="25" t="n"/>
+      <c r="C143" s="25" t="n"/>
+      <c r="D143" s="25" t="n"/>
+      <c r="E143" s="25" t="n"/>
     </row>
     <row r="144">
-      <c r="A144" s="22" t="n"/>
-      <c r="B144" s="22" t="n"/>
-      <c r="C144" s="22" t="n"/>
-      <c r="D144" s="22" t="n"/>
-      <c r="E144" s="22" t="n"/>
+      <c r="A144" s="25" t="n"/>
+      <c r="B144" s="25" t="n"/>
+      <c r="C144" s="25" t="n"/>
+      <c r="D144" s="25" t="n"/>
+      <c r="E144" s="25" t="n"/>
     </row>
     <row r="145">
-      <c r="A145" s="22" t="n"/>
-      <c r="B145" s="22" t="n"/>
-      <c r="C145" s="22" t="n"/>
-      <c r="D145" s="22" t="n"/>
-      <c r="E145" s="22" t="n"/>
+      <c r="A145" s="25" t="n"/>
+      <c r="B145" s="25" t="n"/>
+      <c r="C145" s="25" t="n"/>
+      <c r="D145" s="25" t="n"/>
+      <c r="E145" s="25" t="n"/>
     </row>
     <row r="146">
-      <c r="A146" s="22" t="n"/>
-      <c r="B146" s="22" t="n"/>
-      <c r="C146" s="22" t="n"/>
-      <c r="D146" s="22" t="n"/>
-      <c r="E146" s="22" t="n"/>
+      <c r="A146" s="25" t="n"/>
+      <c r="B146" s="25" t="n"/>
+      <c r="C146" s="25" t="n"/>
+      <c r="D146" s="25" t="n"/>
+      <c r="E146" s="25" t="n"/>
     </row>
     <row r="147">
-      <c r="A147" s="22" t="n"/>
-      <c r="B147" s="22" t="n"/>
-      <c r="C147" s="22" t="n"/>
-      <c r="D147" s="22" t="n"/>
-      <c r="E147" s="22" t="n"/>
+      <c r="A147" s="25" t="n"/>
+      <c r="B147" s="25" t="n"/>
+      <c r="C147" s="25" t="n"/>
+      <c r="D147" s="25" t="n"/>
+      <c r="E147" s="25" t="n"/>
     </row>
     <row r="148">
-      <c r="A148" s="22" t="n"/>
-      <c r="B148" s="22" t="n"/>
-      <c r="C148" s="22" t="n"/>
-      <c r="D148" s="22" t="n"/>
-      <c r="E148" s="22" t="n"/>
+      <c r="A148" s="25" t="n"/>
+      <c r="B148" s="25" t="n"/>
+      <c r="C148" s="25" t="n"/>
+      <c r="D148" s="25" t="n"/>
+      <c r="E148" s="25" t="n"/>
     </row>
     <row r="149">
-      <c r="A149" s="22" t="n"/>
-      <c r="B149" s="22" t="n"/>
-      <c r="C149" s="22" t="n"/>
-      <c r="D149" s="22" t="n"/>
-      <c r="E149" s="22" t="n"/>
+      <c r="A149" s="25" t="n"/>
+      <c r="B149" s="25" t="n"/>
+      <c r="C149" s="25" t="n"/>
+      <c r="D149" s="25" t="n"/>
+      <c r="E149" s="25" t="n"/>
     </row>
     <row r="150">
-      <c r="A150" s="22" t="n"/>
-      <c r="B150" s="22" t="n"/>
-      <c r="C150" s="22" t="n"/>
-      <c r="D150" s="22" t="n"/>
-      <c r="E150" s="22" t="n"/>
+      <c r="A150" s="25" t="n"/>
+      <c r="B150" s="25" t="n"/>
+      <c r="C150" s="25" t="n"/>
+      <c r="D150" s="25" t="n"/>
+      <c r="E150" s="25" t="n"/>
     </row>
     <row r="151">
-      <c r="A151" s="22" t="n"/>
-      <c r="B151" s="22" t="n"/>
-      <c r="C151" s="22" t="n"/>
-      <c r="D151" s="22" t="n"/>
-      <c r="E151" s="22" t="n"/>
+      <c r="A151" s="25" t="n"/>
+      <c r="B151" s="25" t="n"/>
+      <c r="C151" s="25" t="n"/>
+      <c r="D151" s="25" t="n"/>
+      <c r="E151" s="25" t="n"/>
     </row>
     <row r="152">
-      <c r="A152" s="22" t="n"/>
-      <c r="B152" s="22" t="n"/>
-      <c r="C152" s="22" t="n"/>
-      <c r="D152" s="22" t="n"/>
-      <c r="E152" s="22" t="n"/>
+      <c r="A152" s="25" t="n"/>
+      <c r="B152" s="25" t="n"/>
+      <c r="C152" s="25" t="n"/>
+      <c r="D152" s="25" t="n"/>
+      <c r="E152" s="25" t="n"/>
     </row>
     <row r="153">
-      <c r="A153" s="22" t="n"/>
-      <c r="B153" s="22" t="n"/>
-      <c r="C153" s="22" t="n"/>
-      <c r="D153" s="22" t="n"/>
-      <c r="E153" s="22" t="n"/>
+      <c r="A153" s="25" t="n"/>
+      <c r="B153" s="25" t="n"/>
+      <c r="C153" s="25" t="n"/>
+      <c r="D153" s="25" t="n"/>
+      <c r="E153" s="25" t="n"/>
     </row>
     <row r="154">
-      <c r="A154" s="22" t="n"/>
-      <c r="B154" s="22" t="n"/>
-      <c r="C154" s="22" t="n"/>
-      <c r="D154" s="22" t="n"/>
-      <c r="E154" s="22" t="n"/>
+      <c r="A154" s="25" t="n"/>
+      <c r="B154" s="25" t="n"/>
+      <c r="C154" s="25" t="n"/>
+      <c r="D154" s="25" t="n"/>
+      <c r="E154" s="25" t="n"/>
     </row>
     <row r="155">
-      <c r="A155" s="22" t="n"/>
-      <c r="B155" s="22" t="n"/>
-      <c r="C155" s="22" t="n"/>
-      <c r="D155" s="22" t="n"/>
-      <c r="E155" s="22" t="n"/>
+      <c r="A155" s="25" t="n"/>
+      <c r="B155" s="25" t="n"/>
+      <c r="C155" s="25" t="n"/>
+      <c r="D155" s="25" t="n"/>
+      <c r="E155" s="25" t="n"/>
     </row>
     <row r="156">
-      <c r="A156" s="22" t="n"/>
-      <c r="B156" s="22" t="n"/>
-      <c r="C156" s="22" t="n"/>
-      <c r="D156" s="22" t="n"/>
-      <c r="E156" s="22" t="n"/>
+      <c r="A156" s="25" t="n"/>
+      <c r="B156" s="25" t="n"/>
+      <c r="C156" s="25" t="n"/>
+      <c r="D156" s="25" t="n"/>
+      <c r="E156" s="25" t="n"/>
     </row>
     <row r="157">
-      <c r="A157" s="22" t="n"/>
-      <c r="B157" s="22" t="n"/>
-      <c r="C157" s="22" t="n"/>
-      <c r="D157" s="22" t="n"/>
-      <c r="E157" s="22" t="n"/>
+      <c r="A157" s="25" t="n"/>
+      <c r="B157" s="25" t="n"/>
+      <c r="C157" s="25" t="n"/>
+      <c r="D157" s="25" t="n"/>
+      <c r="E157" s="25" t="n"/>
     </row>
     <row r="158">
-      <c r="A158" s="22" t="n"/>
-      <c r="B158" s="22" t="n"/>
-      <c r="C158" s="22" t="n"/>
-      <c r="D158" s="22" t="n"/>
-      <c r="E158" s="22" t="n"/>
+      <c r="A158" s="25" t="n"/>
+      <c r="B158" s="25" t="n"/>
+      <c r="C158" s="25" t="n"/>
+      <c r="D158" s="25" t="n"/>
+      <c r="E158" s="25" t="n"/>
     </row>
     <row r="159">
-      <c r="A159" s="22" t="n"/>
-      <c r="B159" s="22" t="n"/>
-      <c r="C159" s="22" t="n"/>
-      <c r="D159" s="22" t="n"/>
-      <c r="E159" s="22" t="n"/>
+      <c r="A159" s="25" t="n"/>
+      <c r="B159" s="25" t="n"/>
+      <c r="C159" s="25" t="n"/>
+      <c r="D159" s="25" t="n"/>
+      <c r="E159" s="25" t="n"/>
     </row>
     <row r="160">
-      <c r="A160" s="22" t="n"/>
-      <c r="B160" s="22" t="n"/>
-      <c r="C160" s="22" t="n"/>
-      <c r="D160" s="22" t="n"/>
-      <c r="E160" s="22" t="n"/>
+      <c r="A160" s="25" t="n"/>
+      <c r="B160" s="25" t="n"/>
+      <c r="C160" s="25" t="n"/>
+      <c r="D160" s="25" t="n"/>
+      <c r="E160" s="25" t="n"/>
     </row>
     <row r="161">
-      <c r="A161" s="22" t="n"/>
-      <c r="B161" s="22" t="n"/>
-      <c r="C161" s="22" t="n"/>
-      <c r="D161" s="22" t="n"/>
-      <c r="E161" s="22" t="n"/>
+      <c r="A161" s="25" t="n"/>
+      <c r="B161" s="25" t="n"/>
+      <c r="C161" s="25" t="n"/>
+      <c r="D161" s="25" t="n"/>
+      <c r="E161" s="25" t="n"/>
     </row>
     <row r="162">
-      <c r="A162" s="22" t="n"/>
-      <c r="B162" s="22" t="n"/>
-      <c r="C162" s="22" t="n"/>
-      <c r="D162" s="22" t="n"/>
-      <c r="E162" s="22" t="n"/>
+      <c r="A162" s="25" t="n"/>
+      <c r="B162" s="25" t="n"/>
+      <c r="C162" s="25" t="n"/>
+      <c r="D162" s="25" t="n"/>
+      <c r="E162" s="25" t="n"/>
     </row>
     <row r="163">
-      <c r="A163" s="22" t="n"/>
-      <c r="B163" s="22" t="n"/>
-      <c r="C163" s="22" t="n"/>
-      <c r="D163" s="22" t="n"/>
-      <c r="E163" s="22" t="n"/>
+      <c r="A163" s="25" t="n"/>
+      <c r="B163" s="25" t="n"/>
+      <c r="C163" s="25" t="n"/>
+      <c r="D163" s="25" t="n"/>
+      <c r="E163" s="25" t="n"/>
     </row>
     <row r="164">
-      <c r="A164" s="22" t="n"/>
-      <c r="B164" s="22" t="n"/>
-      <c r="C164" s="22" t="n"/>
-      <c r="D164" s="22" t="n"/>
-      <c r="E164" s="22" t="n"/>
+      <c r="A164" s="25" t="n"/>
+      <c r="B164" s="25" t="n"/>
+      <c r="C164" s="25" t="n"/>
+      <c r="D164" s="25" t="n"/>
+      <c r="E164" s="25" t="n"/>
     </row>
     <row r="165">
-      <c r="A165" s="22" t="n"/>
-      <c r="B165" s="22" t="n"/>
-      <c r="C165" s="22" t="n"/>
-      <c r="D165" s="22" t="n"/>
-      <c r="E165" s="22" t="n"/>
+      <c r="A165" s="25" t="n"/>
+      <c r="B165" s="25" t="n"/>
+      <c r="C165" s="25" t="n"/>
+      <c r="D165" s="25" t="n"/>
+      <c r="E165" s="25" t="n"/>
     </row>
     <row r="166">
-      <c r="A166" s="22" t="n"/>
-      <c r="B166" s="22" t="n"/>
-      <c r="C166" s="22" t="n"/>
-      <c r="D166" s="22" t="n"/>
-      <c r="E166" s="22" t="n"/>
+      <c r="A166" s="25" t="n"/>
+      <c r="B166" s="25" t="n"/>
+      <c r="C166" s="25" t="n"/>
+      <c r="D166" s="25" t="n"/>
+      <c r="E166" s="25" t="n"/>
     </row>
     <row r="167">
-      <c r="A167" s="22" t="n"/>
-      <c r="B167" s="22" t="n"/>
-      <c r="C167" s="22" t="n"/>
-      <c r="D167" s="22" t="n"/>
-      <c r="E167" s="22" t="n"/>
+      <c r="A167" s="25" t="n"/>
+      <c r="B167" s="25" t="n"/>
+      <c r="C167" s="25" t="n"/>
+      <c r="D167" s="25" t="n"/>
+      <c r="E167" s="25" t="n"/>
     </row>
     <row r="168">
-      <c r="A168" s="22" t="n"/>
-      <c r="B168" s="22" t="n"/>
-      <c r="C168" s="22" t="n"/>
-      <c r="D168" s="22" t="n"/>
-      <c r="E168" s="22" t="n"/>
+      <c r="A168" s="25" t="n"/>
+      <c r="B168" s="25" t="n"/>
+      <c r="C168" s="25" t="n"/>
+      <c r="D168" s="25" t="n"/>
+      <c r="E168" s="25" t="n"/>
     </row>
     <row r="169">
-      <c r="A169" s="22" t="n"/>
-      <c r="B169" s="22" t="n"/>
-      <c r="C169" s="22" t="n"/>
-      <c r="D169" s="22" t="n"/>
-      <c r="E169" s="22" t="n"/>
+      <c r="A169" s="25" t="n"/>
+      <c r="B169" s="25" t="n"/>
+      <c r="C169" s="25" t="n"/>
+      <c r="D169" s="25" t="n"/>
+      <c r="E169" s="25" t="n"/>
     </row>
     <row r="170">
-      <c r="A170" s="22" t="n"/>
-      <c r="B170" s="22" t="n"/>
-      <c r="C170" s="22" t="n"/>
-      <c r="D170" s="22" t="n"/>
-      <c r="E170" s="22" t="n"/>
+      <c r="A170" s="25" t="n"/>
+      <c r="B170" s="25" t="n"/>
+      <c r="C170" s="25" t="n"/>
+      <c r="D170" s="25" t="n"/>
+      <c r="E170" s="25" t="n"/>
     </row>
     <row r="171">
-      <c r="A171" s="22" t="n"/>
-      <c r="B171" s="22" t="n"/>
-      <c r="C171" s="22" t="n"/>
-      <c r="D171" s="22" t="n"/>
-      <c r="E171" s="22" t="n"/>
+      <c r="A171" s="25" t="n"/>
+      <c r="B171" s="25" t="n"/>
+      <c r="C171" s="25" t="n"/>
+      <c r="D171" s="25" t="n"/>
+      <c r="E171" s="25" t="n"/>
     </row>
     <row r="172">
-      <c r="A172" s="22" t="n"/>
-      <c r="B172" s="22" t="n"/>
-      <c r="C172" s="22" t="n"/>
-      <c r="D172" s="22" t="n"/>
-      <c r="E172" s="22" t="n"/>
+      <c r="A172" s="25" t="n"/>
+      <c r="B172" s="25" t="n"/>
+      <c r="C172" s="25" t="n"/>
+      <c r="D172" s="25" t="n"/>
+      <c r="E172" s="25" t="n"/>
     </row>
     <row r="173">
-      <c r="A173" s="22" t="n"/>
-      <c r="B173" s="22" t="n"/>
-      <c r="C173" s="22" t="n"/>
-      <c r="D173" s="22" t="n"/>
-      <c r="E173" s="22" t="n"/>
+      <c r="A173" s="25" t="n"/>
+      <c r="B173" s="25" t="n"/>
+      <c r="C173" s="25" t="n"/>
+      <c r="D173" s="25" t="n"/>
+      <c r="E173" s="25" t="n"/>
     </row>
     <row r="174">
-      <c r="A174" s="22" t="n"/>
-      <c r="B174" s="22" t="n"/>
-      <c r="C174" s="22" t="n"/>
-      <c r="D174" s="22" t="n"/>
-      <c r="E174" s="22" t="n"/>
+      <c r="A174" s="25" t="n"/>
+      <c r="B174" s="25" t="n"/>
+      <c r="C174" s="25" t="n"/>
+      <c r="D174" s="25" t="n"/>
+      <c r="E174" s="25" t="n"/>
     </row>
     <row r="175">
-      <c r="A175" s="22" t="n"/>
-      <c r="B175" s="22" t="n"/>
-      <c r="C175" s="22" t="n"/>
-      <c r="D175" s="22" t="n"/>
-      <c r="E175" s="22" t="n"/>
+      <c r="A175" s="25" t="n"/>
+      <c r="B175" s="25" t="n"/>
+      <c r="C175" s="25" t="n"/>
+      <c r="D175" s="25" t="n"/>
+      <c r="E175" s="25" t="n"/>
     </row>
     <row r="176">
-      <c r="A176" s="22" t="n"/>
-      <c r="B176" s="22" t="n"/>
-      <c r="C176" s="22" t="n"/>
-      <c r="D176" s="22" t="n"/>
-      <c r="E176" s="22" t="n"/>
+      <c r="A176" s="25" t="n"/>
+      <c r="B176" s="25" t="n"/>
+      <c r="C176" s="25" t="n"/>
+      <c r="D176" s="25" t="n"/>
+      <c r="E176" s="25" t="n"/>
     </row>
     <row r="177">
-      <c r="A177" s="22" t="n"/>
-      <c r="B177" s="22" t="n"/>
-      <c r="C177" s="22" t="n"/>
-      <c r="D177" s="22" t="n"/>
-      <c r="E177" s="22" t="n"/>
+      <c r="A177" s="25" t="n"/>
+      <c r="B177" s="25" t="n"/>
+      <c r="C177" s="25" t="n"/>
+      <c r="D177" s="25" t="n"/>
+      <c r="E177" s="25" t="n"/>
     </row>
     <row r="178">
-      <c r="A178" s="22" t="n"/>
-      <c r="B178" s="22" t="n"/>
-      <c r="C178" s="22" t="n"/>
-      <c r="D178" s="22" t="n"/>
-      <c r="E178" s="22" t="n"/>
+      <c r="A178" s="25" t="n"/>
+      <c r="B178" s="25" t="n"/>
+      <c r="C178" s="25" t="n"/>
+      <c r="D178" s="25" t="n"/>
+      <c r="E178" s="25" t="n"/>
     </row>
     <row r="179">
-      <c r="A179" s="22" t="n"/>
-      <c r="B179" s="22" t="n"/>
-      <c r="C179" s="22" t="n"/>
-      <c r="D179" s="22" t="n"/>
-      <c r="E179" s="22" t="n"/>
+      <c r="A179" s="25" t="n"/>
+      <c r="B179" s="25" t="n"/>
+      <c r="C179" s="25" t="n"/>
+      <c r="D179" s="25" t="n"/>
+      <c r="E179" s="25" t="n"/>
     </row>
     <row r="180">
-      <c r="A180" s="22" t="n"/>
-      <c r="B180" s="22" t="n"/>
-      <c r="C180" s="22" t="n"/>
-      <c r="D180" s="22" t="n"/>
-      <c r="E180" s="22" t="n"/>
+      <c r="A180" s="25" t="n"/>
+      <c r="B180" s="25" t="n"/>
+      <c r="C180" s="25" t="n"/>
+      <c r="D180" s="25" t="n"/>
+      <c r="E180" s="25" t="n"/>
     </row>
     <row r="181">
-      <c r="A181" s="22" t="n"/>
-      <c r="B181" s="22" t="n"/>
-      <c r="C181" s="22" t="n"/>
-      <c r="D181" s="22" t="n"/>
-      <c r="E181" s="22" t="n"/>
+      <c r="A181" s="25" t="n"/>
+      <c r="B181" s="25" t="n"/>
+      <c r="C181" s="25" t="n"/>
+      <c r="D181" s="25" t="n"/>
+      <c r="E181" s="25" t="n"/>
     </row>
     <row r="182">
-      <c r="A182" s="22" t="n"/>
-      <c r="B182" s="22" t="n"/>
-      <c r="C182" s="22" t="n"/>
-      <c r="D182" s="22" t="n"/>
-      <c r="E182" s="22" t="n"/>
+      <c r="A182" s="25" t="n"/>
+      <c r="B182" s="25" t="n"/>
+      <c r="C182" s="25" t="n"/>
+      <c r="D182" s="25" t="n"/>
+      <c r="E182" s="25" t="n"/>
     </row>
     <row r="183">
-      <c r="A183" s="22" t="n"/>
-      <c r="B183" s="22" t="n"/>
-      <c r="C183" s="22" t="n"/>
-      <c r="D183" s="22" t="n"/>
-      <c r="E183" s="22" t="n"/>
+      <c r="A183" s="25" t="n"/>
+      <c r="B183" s="25" t="n"/>
+      <c r="C183" s="25" t="n"/>
+      <c r="D183" s="25" t="n"/>
+      <c r="E183" s="25" t="n"/>
     </row>
     <row r="184">
-      <c r="A184" s="22" t="n"/>
-      <c r="B184" s="22" t="n"/>
-      <c r="C184" s="22" t="n"/>
-      <c r="D184" s="22" t="n"/>
-      <c r="E184" s="22" t="n"/>
+      <c r="A184" s="25" t="n"/>
+      <c r="B184" s="25" t="n"/>
+      <c r="C184" s="25" t="n"/>
+      <c r="D184" s="25" t="n"/>
+      <c r="E184" s="25" t="n"/>
     </row>
     <row r="185">
-      <c r="A185" s="22" t="n"/>
-      <c r="B185" s="22" t="n"/>
-      <c r="C185" s="22" t="n"/>
-      <c r="D185" s="22" t="n"/>
-      <c r="E185" s="22" t="n"/>
+      <c r="A185" s="25" t="n"/>
+      <c r="B185" s="25" t="n"/>
+      <c r="C185" s="25" t="n"/>
+      <c r="D185" s="25" t="n"/>
+      <c r="E185" s="25" t="n"/>
     </row>
     <row r="186">
-      <c r="A186" s="22" t="n"/>
-      <c r="B186" s="22" t="n"/>
-      <c r="C186" s="22" t="n"/>
-      <c r="D186" s="22" t="n"/>
-      <c r="E186" s="22" t="n"/>
+      <c r="A186" s="25" t="n"/>
+      <c r="B186" s="25" t="n"/>
+      <c r="C186" s="25" t="n"/>
+      <c r="D186" s="25" t="n"/>
+      <c r="E186" s="25" t="n"/>
     </row>
     <row r="187">
-      <c r="A187" s="22" t="n"/>
-      <c r="B187" s="22" t="n"/>
-      <c r="C187" s="22" t="n"/>
-      <c r="D187" s="22" t="n"/>
-      <c r="E187" s="22" t="n"/>
+      <c r="A187" s="25" t="n"/>
+      <c r="B187" s="25" t="n"/>
+      <c r="C187" s="25" t="n"/>
+      <c r="D187" s="25" t="n"/>
+      <c r="E187" s="25" t="n"/>
     </row>
     <row r="188">
-      <c r="A188" s="22" t="n"/>
-      <c r="B188" s="22" t="n"/>
-      <c r="C188" s="22" t="n"/>
-      <c r="D188" s="22" t="n"/>
-      <c r="E188" s="22" t="n"/>
+      <c r="A188" s="25" t="n"/>
+      <c r="B188" s="25" t="n"/>
+      <c r="C188" s="25" t="n"/>
+      <c r="D188" s="25" t="n"/>
+      <c r="E188" s="25" t="n"/>
     </row>
     <row r="189">
-      <c r="A189" s="22" t="n"/>
-      <c r="B189" s="22" t="n"/>
-      <c r="C189" s="22" t="n"/>
-      <c r="D189" s="22" t="n"/>
-      <c r="E189" s="22" t="n"/>
+      <c r="A189" s="25" t="n"/>
+      <c r="B189" s="25" t="n"/>
+      <c r="C189" s="25" t="n"/>
+      <c r="D189" s="25" t="n"/>
+      <c r="E189" s="25" t="n"/>
     </row>
     <row r="190">
-      <c r="A190" s="22" t="n"/>
-      <c r="B190" s="22" t="n"/>
-      <c r="C190" s="22" t="n"/>
-      <c r="D190" s="22" t="n"/>
-      <c r="E190" s="22" t="n"/>
+      <c r="A190" s="25" t="n"/>
+      <c r="B190" s="25" t="n"/>
+      <c r="C190" s="25" t="n"/>
+      <c r="D190" s="25" t="n"/>
+      <c r="E190" s="25" t="n"/>
     </row>
     <row r="191">
-      <c r="A191" s="22" t="n"/>
-      <c r="B191" s="22" t="n"/>
-      <c r="C191" s="22" t="n"/>
-      <c r="D191" s="22" t="n"/>
-      <c r="E191" s="22" t="n"/>
+      <c r="A191" s="25" t="n"/>
+      <c r="B191" s="25" t="n"/>
+      <c r="C191" s="25" t="n"/>
+      <c r="D191" s="25" t="n"/>
+      <c r="E191" s="25" t="n"/>
     </row>
     <row r="192">
-      <c r="A192" s="22" t="n"/>
-      <c r="B192" s="22" t="n"/>
-      <c r="C192" s="22" t="n"/>
-      <c r="D192" s="22" t="n"/>
-      <c r="E192" s="22" t="n"/>
+      <c r="A192" s="25" t="n"/>
+      <c r="B192" s="25" t="n"/>
+      <c r="C192" s="25" t="n"/>
+      <c r="D192" s="25" t="n"/>
+      <c r="E192" s="25" t="n"/>
     </row>
     <row r="193">
-      <c r="A193" s="22" t="n"/>
-      <c r="B193" s="22" t="n"/>
-      <c r="C193" s="22" t="n"/>
-      <c r="D193" s="22" t="n"/>
-      <c r="E193" s="22" t="n"/>
+      <c r="A193" s="25" t="n"/>
+      <c r="B193" s="25" t="n"/>
+      <c r="C193" s="25" t="n"/>
+      <c r="D193" s="25" t="n"/>
+      <c r="E193" s="25" t="n"/>
     </row>
     <row r="194">
-      <c r="A194" s="22" t="n"/>
-      <c r="B194" s="22" t="n"/>
-      <c r="C194" s="22" t="n"/>
-      <c r="D194" s="22" t="n"/>
-      <c r="E194" s="22" t="n"/>
+      <c r="A194" s="25" t="n"/>
+      <c r="B194" s="25" t="n"/>
+      <c r="C194" s="25" t="n"/>
+      <c r="D194" s="25" t="n"/>
+      <c r="E194" s="25" t="n"/>
     </row>
     <row r="195">
-      <c r="A195" s="22" t="n"/>
-      <c r="B195" s="22" t="n"/>
-      <c r="C195" s="22" t="n"/>
-      <c r="D195" s="22" t="n"/>
-      <c r="E195" s="22" t="n"/>
+      <c r="A195" s="25" t="n"/>
+      <c r="B195" s="25" t="n"/>
+      <c r="C195" s="25" t="n"/>
+      <c r="D195" s="25" t="n"/>
+      <c r="E195" s="25" t="n"/>
     </row>
     <row r="196">
-      <c r="A196" s="22" t="n"/>
-      <c r="B196" s="22" t="n"/>
-      <c r="C196" s="22" t="n"/>
-      <c r="D196" s="22" t="n"/>
-      <c r="E196" s="22" t="n"/>
+      <c r="A196" s="25" t="n"/>
+      <c r="B196" s="25" t="n"/>
+      <c r="C196" s="25" t="n"/>
+      <c r="D196" s="25" t="n"/>
+      <c r="E196" s="25" t="n"/>
     </row>
     <row r="197">
-      <c r="A197" s="22" t="n"/>
-      <c r="B197" s="22" t="n"/>
-      <c r="C197" s="22" t="n"/>
-      <c r="D197" s="22" t="n"/>
-      <c r="E197" s="22" t="n"/>
+      <c r="A197" s="25" t="n"/>
+      <c r="B197" s="25" t="n"/>
+      <c r="C197" s="25" t="n"/>
+      <c r="D197" s="25" t="n"/>
+      <c r="E197" s="25" t="n"/>
     </row>
     <row r="198">
-      <c r="A198" s="22" t="n"/>
-      <c r="B198" s="22" t="n"/>
-      <c r="C198" s="22" t="n"/>
-      <c r="D198" s="22" t="n"/>
-      <c r="E198" s="22" t="n"/>
+      <c r="A198" s="25" t="n"/>
+      <c r="B198" s="25" t="n"/>
+      <c r="C198" s="25" t="n"/>
+      <c r="D198" s="25" t="n"/>
+      <c r="E198" s="25" t="n"/>
     </row>
     <row r="199">
-      <c r="A199" s="22" t="n"/>
-      <c r="B199" s="22" t="n"/>
-      <c r="C199" s="22" t="n"/>
-      <c r="D199" s="22" t="n"/>
-      <c r="E199" s="22" t="n"/>
+      <c r="A199" s="25" t="n"/>
+      <c r="B199" s="25" t="n"/>
+      <c r="C199" s="25" t="n"/>
+      <c r="D199" s="25" t="n"/>
+      <c r="E199" s="25" t="n"/>
     </row>
     <row r="200">
-      <c r="A200" s="22" t="n"/>
-      <c r="B200" s="22" t="n"/>
-      <c r="C200" s="22" t="n"/>
-      <c r="D200" s="22" t="n"/>
-      <c r="E200" s="22" t="n"/>
+      <c r="A200" s="25" t="n"/>
+      <c r="B200" s="25" t="n"/>
+      <c r="C200" s="25" t="n"/>
+      <c r="D200" s="25" t="n"/>
+      <c r="E200" s="25" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -6371,66 +6554,66 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="23" t="inlineStr">
+      <c r="A1" s="26" t="inlineStr">
         <is>
           <t>HOW TO USE  使用方法</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="24" t="inlineStr">
+      <c r="A2" s="27" t="inlineStr">
         <is>
           <t>1. Client sheet: fill client name, income, review date. Review standard is RM1m for Life, CI, Retirement, Medical - adjust if needed.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="24" t="inlineStr">
+      <c r="A3" s="27" t="inlineStr">
         <is>
           <t>2. Policies sheet: one row per policy. Use the dropdowns for Type, Status, Payment Mode.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="24" t="inlineStr">
+      <c r="A4" s="27" t="inlineStr">
         <is>
           <t>3. Leave a cell BLANK if you don't know it. Never type a guess - the app flags blanks for you to confirm.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="24" t="inlineStr">
+      <c r="A5" s="27" t="inlineStr">
         <is>
           <t>4. Dashboard sheet updates automatically (Excel-only version).</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="24" t="inlineStr">
+      <c r="A6" s="27" t="inlineStr">
         <is>
           <t>5. For the visual PDF report: open 'Policy Review Snapshot.html', load this file, click 'Generate'.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="24" t="inlineStr"/>
+      <c r="A7" s="27" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="24" t="inlineStr">
+      <c r="A8" s="27" t="inlineStr">
         <is>
           <t>Pink nominee cell = inforce policy without nominee recorded.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="24" t="inlineStr">
+      <c r="A9" s="27" t="inlineStr">
         <is>
           <t>Only Inforce policies count toward coverage totals. Lapsed/Paid-up are listed separately.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="24" t="inlineStr">
+      <c r="A10" s="27" t="inlineStr">
         <is>
           <t>The rows marked (sample) are fictional - delete them before using with a real client.</t>
         </is>

</xml_diff>

<commit_message>
Family reports, nominee shares, payout routes and estate checklist
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Policy_Review_Template.xlsx
+++ b/Policy_Review_Template.xlsx
@@ -931,7 +931,7 @@
         </is>
       </c>
       <c r="B15" s="9">
-        <f>SUMIFS(Policies!$AA$2:$AA$100,Policies!$G$2:$G$100,"Inforce")+SUMIFS(Policies!$AA$2:$AA$100,Policies!$G$2:$G$100,"Paid-up")</f>
+        <f>SUMIFS(Policies!$AB$2:$AB$100,Policies!$G$2:$G$100,"Inforce")+SUMIFS(Policies!$AB$2:$AB$100,Policies!$G$2:$G$100,"Paid-up")</f>
         <v/>
       </c>
     </row>
@@ -1453,7 +1453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA100"/>
+  <dimension ref="A1:AB100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1483,6 +1483,7 @@
     <col width="15" customWidth="1" min="25" max="25"/>
     <col width="12" customWidth="1" min="26" max="26"/>
     <col width="14" customWidth="1" min="27" max="27"/>
+    <col width="14" customWidth="1" min="28" max="28"/>
   </cols>
   <sheetData>
     <row r="1" ht="42" customHeight="1">
@@ -1616,7 +1617,12 @@
           <t>Trust Created</t>
         </is>
       </c>
-      <c r="AA1" s="23" t="inlineStr">
+      <c r="AA1" s="22" t="inlineStr">
+        <is>
+          <t>Nominee Share (%)</t>
+        </is>
+      </c>
+      <c r="AB1" s="23" t="inlineStr">
         <is>
           <t>Annual Premium (auto)</t>
         </is>
@@ -1711,7 +1717,8 @@
       <c r="X2" s="12" t="inlineStr"/>
       <c r="Y2" s="9" t="n"/>
       <c r="Z2" s="12" t="n"/>
-      <c r="AA2" s="24">
+      <c r="AA2" s="12" t="n"/>
+      <c r="AB2" s="24">
         <f>IF(J2="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J2,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K2,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -1801,7 +1808,8 @@
       </c>
       <c r="Y3" s="9" t="n"/>
       <c r="Z3" s="12" t="n"/>
-      <c r="AA3" s="24">
+      <c r="AA3" s="12" t="n"/>
+      <c r="AB3" s="24">
         <f>IF(J3="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J3,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K3,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -1897,7 +1905,8 @@
       <c r="X4" s="12" t="inlineStr"/>
       <c r="Y4" s="9" t="n"/>
       <c r="Z4" s="12" t="n"/>
-      <c r="AA4" s="24">
+      <c r="AA4" s="12" t="n"/>
+      <c r="AB4" s="24">
         <f>IF(J4="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J4,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K4,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -1981,7 +1990,8 @@
       </c>
       <c r="Y5" s="9" t="n"/>
       <c r="Z5" s="12" t="n"/>
-      <c r="AA5" s="24">
+      <c r="AA5" s="12" t="n"/>
+      <c r="AB5" s="24">
         <f>IF(J5="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J5,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K5,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2077,7 +2087,8 @@
       </c>
       <c r="Y6" s="9" t="n"/>
       <c r="Z6" s="12" t="n"/>
-      <c r="AA6" s="24">
+      <c r="AA6" s="12" t="n"/>
+      <c r="AB6" s="24">
         <f>IF(J6="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J6,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K6,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2109,7 +2120,8 @@
       <c r="X7" s="12" t="n"/>
       <c r="Y7" s="9" t="n"/>
       <c r="Z7" s="12" t="n"/>
-      <c r="AA7" s="24">
+      <c r="AA7" s="12" t="n"/>
+      <c r="AB7" s="24">
         <f>IF(J7="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J7,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K7,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2141,7 +2153,8 @@
       <c r="X8" s="12" t="n"/>
       <c r="Y8" s="9" t="n"/>
       <c r="Z8" s="12" t="n"/>
-      <c r="AA8" s="24">
+      <c r="AA8" s="12" t="n"/>
+      <c r="AB8" s="24">
         <f>IF(J8="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J8,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K8,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2173,7 +2186,8 @@
       <c r="X9" s="12" t="n"/>
       <c r="Y9" s="9" t="n"/>
       <c r="Z9" s="12" t="n"/>
-      <c r="AA9" s="24">
+      <c r="AA9" s="12" t="n"/>
+      <c r="AB9" s="24">
         <f>IF(J9="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J9,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K9,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2205,7 +2219,8 @@
       <c r="X10" s="12" t="n"/>
       <c r="Y10" s="9" t="n"/>
       <c r="Z10" s="12" t="n"/>
-      <c r="AA10" s="24">
+      <c r="AA10" s="12" t="n"/>
+      <c r="AB10" s="24">
         <f>IF(J10="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J10,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K10,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2237,7 +2252,8 @@
       <c r="X11" s="12" t="n"/>
       <c r="Y11" s="9" t="n"/>
       <c r="Z11" s="12" t="n"/>
-      <c r="AA11" s="24">
+      <c r="AA11" s="12" t="n"/>
+      <c r="AB11" s="24">
         <f>IF(J11="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J11,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K11,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2269,7 +2285,8 @@
       <c r="X12" s="12" t="n"/>
       <c r="Y12" s="9" t="n"/>
       <c r="Z12" s="12" t="n"/>
-      <c r="AA12" s="24">
+      <c r="AA12" s="12" t="n"/>
+      <c r="AB12" s="24">
         <f>IF(J12="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J12,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K12,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2301,7 +2318,8 @@
       <c r="X13" s="12" t="n"/>
       <c r="Y13" s="9" t="n"/>
       <c r="Z13" s="12" t="n"/>
-      <c r="AA13" s="24">
+      <c r="AA13" s="12" t="n"/>
+      <c r="AB13" s="24">
         <f>IF(J13="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J13,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K13,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2333,7 +2351,8 @@
       <c r="X14" s="12" t="n"/>
       <c r="Y14" s="9" t="n"/>
       <c r="Z14" s="12" t="n"/>
-      <c r="AA14" s="24">
+      <c r="AA14" s="12" t="n"/>
+      <c r="AB14" s="24">
         <f>IF(J14="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J14,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K14,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2365,7 +2384,8 @@
       <c r="X15" s="12" t="n"/>
       <c r="Y15" s="9" t="n"/>
       <c r="Z15" s="12" t="n"/>
-      <c r="AA15" s="24">
+      <c r="AA15" s="12" t="n"/>
+      <c r="AB15" s="24">
         <f>IF(J15="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J15,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K15,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2397,7 +2417,8 @@
       <c r="X16" s="12" t="n"/>
       <c r="Y16" s="9" t="n"/>
       <c r="Z16" s="12" t="n"/>
-      <c r="AA16" s="24">
+      <c r="AA16" s="12" t="n"/>
+      <c r="AB16" s="24">
         <f>IF(J16="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J16,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K16,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2429,7 +2450,8 @@
       <c r="X17" s="12" t="n"/>
       <c r="Y17" s="9" t="n"/>
       <c r="Z17" s="12" t="n"/>
-      <c r="AA17" s="24">
+      <c r="AA17" s="12" t="n"/>
+      <c r="AB17" s="24">
         <f>IF(J17="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J17,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K17,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2461,7 +2483,8 @@
       <c r="X18" s="12" t="n"/>
       <c r="Y18" s="9" t="n"/>
       <c r="Z18" s="12" t="n"/>
-      <c r="AA18" s="24">
+      <c r="AA18" s="12" t="n"/>
+      <c r="AB18" s="24">
         <f>IF(J18="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J18,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K18,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2493,7 +2516,8 @@
       <c r="X19" s="12" t="n"/>
       <c r="Y19" s="9" t="n"/>
       <c r="Z19" s="12" t="n"/>
-      <c r="AA19" s="24">
+      <c r="AA19" s="12" t="n"/>
+      <c r="AB19" s="24">
         <f>IF(J19="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J19,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K19,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2525,7 +2549,8 @@
       <c r="X20" s="12" t="n"/>
       <c r="Y20" s="9" t="n"/>
       <c r="Z20" s="12" t="n"/>
-      <c r="AA20" s="24">
+      <c r="AA20" s="12" t="n"/>
+      <c r="AB20" s="24">
         <f>IF(J20="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J20,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K20,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2557,7 +2582,8 @@
       <c r="X21" s="12" t="n"/>
       <c r="Y21" s="9" t="n"/>
       <c r="Z21" s="12" t="n"/>
-      <c r="AA21" s="24">
+      <c r="AA21" s="12" t="n"/>
+      <c r="AB21" s="24">
         <f>IF(J21="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J21,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K21,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2589,7 +2615,8 @@
       <c r="X22" s="12" t="n"/>
       <c r="Y22" s="9" t="n"/>
       <c r="Z22" s="12" t="n"/>
-      <c r="AA22" s="24">
+      <c r="AA22" s="12" t="n"/>
+      <c r="AB22" s="24">
         <f>IF(J22="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J22,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K22,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2621,7 +2648,8 @@
       <c r="X23" s="12" t="n"/>
       <c r="Y23" s="9" t="n"/>
       <c r="Z23" s="12" t="n"/>
-      <c r="AA23" s="24">
+      <c r="AA23" s="12" t="n"/>
+      <c r="AB23" s="24">
         <f>IF(J23="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J23,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K23,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2653,7 +2681,8 @@
       <c r="X24" s="12" t="n"/>
       <c r="Y24" s="9" t="n"/>
       <c r="Z24" s="12" t="n"/>
-      <c r="AA24" s="24">
+      <c r="AA24" s="12" t="n"/>
+      <c r="AB24" s="24">
         <f>IF(J24="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J24,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K24,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2685,7 +2714,8 @@
       <c r="X25" s="12" t="n"/>
       <c r="Y25" s="9" t="n"/>
       <c r="Z25" s="12" t="n"/>
-      <c r="AA25" s="24">
+      <c r="AA25" s="12" t="n"/>
+      <c r="AB25" s="24">
         <f>IF(J25="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J25,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K25,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2717,7 +2747,8 @@
       <c r="X26" s="12" t="n"/>
       <c r="Y26" s="9" t="n"/>
       <c r="Z26" s="12" t="n"/>
-      <c r="AA26" s="24">
+      <c r="AA26" s="12" t="n"/>
+      <c r="AB26" s="24">
         <f>IF(J26="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J26,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K26,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2749,7 +2780,8 @@
       <c r="X27" s="12" t="n"/>
       <c r="Y27" s="9" t="n"/>
       <c r="Z27" s="12" t="n"/>
-      <c r="AA27" s="24">
+      <c r="AA27" s="12" t="n"/>
+      <c r="AB27" s="24">
         <f>IF(J27="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J27,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K27,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2781,7 +2813,8 @@
       <c r="X28" s="12" t="n"/>
       <c r="Y28" s="9" t="n"/>
       <c r="Z28" s="12" t="n"/>
-      <c r="AA28" s="24">
+      <c r="AA28" s="12" t="n"/>
+      <c r="AB28" s="24">
         <f>IF(J28="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J28,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K28,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2813,7 +2846,8 @@
       <c r="X29" s="12" t="n"/>
       <c r="Y29" s="9" t="n"/>
       <c r="Z29" s="12" t="n"/>
-      <c r="AA29" s="24">
+      <c r="AA29" s="12" t="n"/>
+      <c r="AB29" s="24">
         <f>IF(J29="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J29,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K29,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2845,7 +2879,8 @@
       <c r="X30" s="12" t="n"/>
       <c r="Y30" s="9" t="n"/>
       <c r="Z30" s="12" t="n"/>
-      <c r="AA30" s="24">
+      <c r="AA30" s="12" t="n"/>
+      <c r="AB30" s="24">
         <f>IF(J30="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J30,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K30,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2877,7 +2912,8 @@
       <c r="X31" s="12" t="n"/>
       <c r="Y31" s="9" t="n"/>
       <c r="Z31" s="12" t="n"/>
-      <c r="AA31" s="24">
+      <c r="AA31" s="12" t="n"/>
+      <c r="AB31" s="24">
         <f>IF(J31="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J31,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K31,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2909,7 +2945,8 @@
       <c r="X32" s="12" t="n"/>
       <c r="Y32" s="9" t="n"/>
       <c r="Z32" s="12" t="n"/>
-      <c r="AA32" s="24">
+      <c r="AA32" s="12" t="n"/>
+      <c r="AB32" s="24">
         <f>IF(J32="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J32,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K32,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2941,7 +2978,8 @@
       <c r="X33" s="12" t="n"/>
       <c r="Y33" s="9" t="n"/>
       <c r="Z33" s="12" t="n"/>
-      <c r="AA33" s="24">
+      <c r="AA33" s="12" t="n"/>
+      <c r="AB33" s="24">
         <f>IF(J33="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J33,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K33,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2973,7 +3011,8 @@
       <c r="X34" s="12" t="n"/>
       <c r="Y34" s="9" t="n"/>
       <c r="Z34" s="12" t="n"/>
-      <c r="AA34" s="24">
+      <c r="AA34" s="12" t="n"/>
+      <c r="AB34" s="24">
         <f>IF(J34="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J34,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K34,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3005,7 +3044,8 @@
       <c r="X35" s="12" t="n"/>
       <c r="Y35" s="9" t="n"/>
       <c r="Z35" s="12" t="n"/>
-      <c r="AA35" s="24">
+      <c r="AA35" s="12" t="n"/>
+      <c r="AB35" s="24">
         <f>IF(J35="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J35,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K35,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3037,7 +3077,8 @@
       <c r="X36" s="12" t="n"/>
       <c r="Y36" s="9" t="n"/>
       <c r="Z36" s="12" t="n"/>
-      <c r="AA36" s="24">
+      <c r="AA36" s="12" t="n"/>
+      <c r="AB36" s="24">
         <f>IF(J36="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J36,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K36,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3069,7 +3110,8 @@
       <c r="X37" s="12" t="n"/>
       <c r="Y37" s="9" t="n"/>
       <c r="Z37" s="12" t="n"/>
-      <c r="AA37" s="24">
+      <c r="AA37" s="12" t="n"/>
+      <c r="AB37" s="24">
         <f>IF(J37="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J37,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K37,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3101,7 +3143,8 @@
       <c r="X38" s="12" t="n"/>
       <c r="Y38" s="9" t="n"/>
       <c r="Z38" s="12" t="n"/>
-      <c r="AA38" s="24">
+      <c r="AA38" s="12" t="n"/>
+      <c r="AB38" s="24">
         <f>IF(J38="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J38,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K38,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3133,7 +3176,8 @@
       <c r="X39" s="12" t="n"/>
       <c r="Y39" s="9" t="n"/>
       <c r="Z39" s="12" t="n"/>
-      <c r="AA39" s="24">
+      <c r="AA39" s="12" t="n"/>
+      <c r="AB39" s="24">
         <f>IF(J39="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J39,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K39,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3165,7 +3209,8 @@
       <c r="X40" s="12" t="n"/>
       <c r="Y40" s="9" t="n"/>
       <c r="Z40" s="12" t="n"/>
-      <c r="AA40" s="24">
+      <c r="AA40" s="12" t="n"/>
+      <c r="AB40" s="24">
         <f>IF(J40="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J40,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K40,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3197,7 +3242,8 @@
       <c r="X41" s="12" t="n"/>
       <c r="Y41" s="9" t="n"/>
       <c r="Z41" s="12" t="n"/>
-      <c r="AA41" s="24">
+      <c r="AA41" s="12" t="n"/>
+      <c r="AB41" s="24">
         <f>IF(J41="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J41,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K41,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3229,7 +3275,8 @@
       <c r="X42" s="12" t="n"/>
       <c r="Y42" s="9" t="n"/>
       <c r="Z42" s="12" t="n"/>
-      <c r="AA42" s="24">
+      <c r="AA42" s="12" t="n"/>
+      <c r="AB42" s="24">
         <f>IF(J42="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J42,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K42,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3261,7 +3308,8 @@
       <c r="X43" s="12" t="n"/>
       <c r="Y43" s="9" t="n"/>
       <c r="Z43" s="12" t="n"/>
-      <c r="AA43" s="24">
+      <c r="AA43" s="12" t="n"/>
+      <c r="AB43" s="24">
         <f>IF(J43="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J43,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K43,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3293,7 +3341,8 @@
       <c r="X44" s="12" t="n"/>
       <c r="Y44" s="9" t="n"/>
       <c r="Z44" s="12" t="n"/>
-      <c r="AA44" s="24">
+      <c r="AA44" s="12" t="n"/>
+      <c r="AB44" s="24">
         <f>IF(J44="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J44,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K44,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3325,7 +3374,8 @@
       <c r="X45" s="12" t="n"/>
       <c r="Y45" s="9" t="n"/>
       <c r="Z45" s="12" t="n"/>
-      <c r="AA45" s="24">
+      <c r="AA45" s="12" t="n"/>
+      <c r="AB45" s="24">
         <f>IF(J45="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J45,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K45,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3357,7 +3407,8 @@
       <c r="X46" s="12" t="n"/>
       <c r="Y46" s="9" t="n"/>
       <c r="Z46" s="12" t="n"/>
-      <c r="AA46" s="24">
+      <c r="AA46" s="12" t="n"/>
+      <c r="AB46" s="24">
         <f>IF(J46="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J46,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K46,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3389,7 +3440,8 @@
       <c r="X47" s="12" t="n"/>
       <c r="Y47" s="9" t="n"/>
       <c r="Z47" s="12" t="n"/>
-      <c r="AA47" s="24">
+      <c r="AA47" s="12" t="n"/>
+      <c r="AB47" s="24">
         <f>IF(J47="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J47,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K47,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3421,7 +3473,8 @@
       <c r="X48" s="12" t="n"/>
       <c r="Y48" s="9" t="n"/>
       <c r="Z48" s="12" t="n"/>
-      <c r="AA48" s="24">
+      <c r="AA48" s="12" t="n"/>
+      <c r="AB48" s="24">
         <f>IF(J48="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J48,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K48,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3453,7 +3506,8 @@
       <c r="X49" s="12" t="n"/>
       <c r="Y49" s="9" t="n"/>
       <c r="Z49" s="12" t="n"/>
-      <c r="AA49" s="24">
+      <c r="AA49" s="12" t="n"/>
+      <c r="AB49" s="24">
         <f>IF(J49="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J49,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K49,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3485,7 +3539,8 @@
       <c r="X50" s="12" t="n"/>
       <c r="Y50" s="9" t="n"/>
       <c r="Z50" s="12" t="n"/>
-      <c r="AA50" s="24">
+      <c r="AA50" s="12" t="n"/>
+      <c r="AB50" s="24">
         <f>IF(J50="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J50,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K50,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3517,7 +3572,8 @@
       <c r="X51" s="12" t="n"/>
       <c r="Y51" s="9" t="n"/>
       <c r="Z51" s="12" t="n"/>
-      <c r="AA51" s="24">
+      <c r="AA51" s="12" t="n"/>
+      <c r="AB51" s="24">
         <f>IF(J51="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J51,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K51,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3549,7 +3605,8 @@
       <c r="X52" s="12" t="n"/>
       <c r="Y52" s="9" t="n"/>
       <c r="Z52" s="12" t="n"/>
-      <c r="AA52" s="24">
+      <c r="AA52" s="12" t="n"/>
+      <c r="AB52" s="24">
         <f>IF(J52="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J52,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K52,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3581,7 +3638,8 @@
       <c r="X53" s="12" t="n"/>
       <c r="Y53" s="9" t="n"/>
       <c r="Z53" s="12" t="n"/>
-      <c r="AA53" s="24">
+      <c r="AA53" s="12" t="n"/>
+      <c r="AB53" s="24">
         <f>IF(J53="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J53,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K53,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3613,7 +3671,8 @@
       <c r="X54" s="12" t="n"/>
       <c r="Y54" s="9" t="n"/>
       <c r="Z54" s="12" t="n"/>
-      <c r="AA54" s="24">
+      <c r="AA54" s="12" t="n"/>
+      <c r="AB54" s="24">
         <f>IF(J54="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J54,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K54,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3645,7 +3704,8 @@
       <c r="X55" s="12" t="n"/>
       <c r="Y55" s="9" t="n"/>
       <c r="Z55" s="12" t="n"/>
-      <c r="AA55" s="24">
+      <c r="AA55" s="12" t="n"/>
+      <c r="AB55" s="24">
         <f>IF(J55="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J55,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K55,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3677,7 +3737,8 @@
       <c r="X56" s="12" t="n"/>
       <c r="Y56" s="9" t="n"/>
       <c r="Z56" s="12" t="n"/>
-      <c r="AA56" s="24">
+      <c r="AA56" s="12" t="n"/>
+      <c r="AB56" s="24">
         <f>IF(J56="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J56,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K56,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3709,7 +3770,8 @@
       <c r="X57" s="12" t="n"/>
       <c r="Y57" s="9" t="n"/>
       <c r="Z57" s="12" t="n"/>
-      <c r="AA57" s="24">
+      <c r="AA57" s="12" t="n"/>
+      <c r="AB57" s="24">
         <f>IF(J57="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J57,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K57,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3741,7 +3803,8 @@
       <c r="X58" s="12" t="n"/>
       <c r="Y58" s="9" t="n"/>
       <c r="Z58" s="12" t="n"/>
-      <c r="AA58" s="24">
+      <c r="AA58" s="12" t="n"/>
+      <c r="AB58" s="24">
         <f>IF(J58="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J58,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K58,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3773,7 +3836,8 @@
       <c r="X59" s="12" t="n"/>
       <c r="Y59" s="9" t="n"/>
       <c r="Z59" s="12" t="n"/>
-      <c r="AA59" s="24">
+      <c r="AA59" s="12" t="n"/>
+      <c r="AB59" s="24">
         <f>IF(J59="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J59,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K59,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3805,7 +3869,8 @@
       <c r="X60" s="12" t="n"/>
       <c r="Y60" s="9" t="n"/>
       <c r="Z60" s="12" t="n"/>
-      <c r="AA60" s="24">
+      <c r="AA60" s="12" t="n"/>
+      <c r="AB60" s="24">
         <f>IF(J60="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J60,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K60,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3837,7 +3902,8 @@
       <c r="X61" s="12" t="n"/>
       <c r="Y61" s="9" t="n"/>
       <c r="Z61" s="12" t="n"/>
-      <c r="AA61" s="24">
+      <c r="AA61" s="12" t="n"/>
+      <c r="AB61" s="24">
         <f>IF(J61="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J61,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K61,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3869,7 +3935,8 @@
       <c r="X62" s="12" t="n"/>
       <c r="Y62" s="9" t="n"/>
       <c r="Z62" s="12" t="n"/>
-      <c r="AA62" s="24">
+      <c r="AA62" s="12" t="n"/>
+      <c r="AB62" s="24">
         <f>IF(J62="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J62,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K62,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3901,7 +3968,8 @@
       <c r="X63" s="12" t="n"/>
       <c r="Y63" s="9" t="n"/>
       <c r="Z63" s="12" t="n"/>
-      <c r="AA63" s="24">
+      <c r="AA63" s="12" t="n"/>
+      <c r="AB63" s="24">
         <f>IF(J63="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J63,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K63,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3933,7 +4001,8 @@
       <c r="X64" s="12" t="n"/>
       <c r="Y64" s="9" t="n"/>
       <c r="Z64" s="12" t="n"/>
-      <c r="AA64" s="24">
+      <c r="AA64" s="12" t="n"/>
+      <c r="AB64" s="24">
         <f>IF(J64="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J64,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K64,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3965,7 +4034,8 @@
       <c r="X65" s="12" t="n"/>
       <c r="Y65" s="9" t="n"/>
       <c r="Z65" s="12" t="n"/>
-      <c r="AA65" s="24">
+      <c r="AA65" s="12" t="n"/>
+      <c r="AB65" s="24">
         <f>IF(J65="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J65,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K65,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3997,7 +4067,8 @@
       <c r="X66" s="12" t="n"/>
       <c r="Y66" s="9" t="n"/>
       <c r="Z66" s="12" t="n"/>
-      <c r="AA66" s="24">
+      <c r="AA66" s="12" t="n"/>
+      <c r="AB66" s="24">
         <f>IF(J66="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J66,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K66,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -4029,7 +4100,8 @@
       <c r="X67" s="12" t="n"/>
       <c r="Y67" s="9" t="n"/>
       <c r="Z67" s="12" t="n"/>
-      <c r="AA67" s="24">
+      <c r="AA67" s="12" t="n"/>
+      <c r="AB67" s="24">
         <f>IF(J67="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J67,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K67,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -4061,7 +4133,8 @@
       <c r="X68" s="12" t="n"/>
       <c r="Y68" s="9" t="n"/>
       <c r="Z68" s="12" t="n"/>
-      <c r="AA68" s="24">
+      <c r="AA68" s="12" t="n"/>
+      <c r="AB68" s="24">
         <f>IF(J68="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J68,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K68,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -4093,7 +4166,8 @@
       <c r="X69" s="12" t="n"/>
       <c r="Y69" s="9" t="n"/>
       <c r="Z69" s="12" t="n"/>
-      <c r="AA69" s="24">
+      <c r="AA69" s="12" t="n"/>
+      <c r="AB69" s="24">
         <f>IF(J69="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J69,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K69,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -4125,7 +4199,8 @@
       <c r="X70" s="12" t="n"/>
       <c r="Y70" s="9" t="n"/>
       <c r="Z70" s="12" t="n"/>
-      <c r="AA70" s="24">
+      <c r="AA70" s="12" t="n"/>
+      <c r="AB70" s="24">
         <f>IF(J70="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J70,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K70,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -4157,7 +4232,8 @@
       <c r="X71" s="12" t="n"/>
       <c r="Y71" s="9" t="n"/>
       <c r="Z71" s="12" t="n"/>
-      <c r="AA71" s="24">
+      <c r="AA71" s="12" t="n"/>
+      <c r="AB71" s="24">
         <f>IF(J71="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J71,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K71,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -4189,7 +4265,8 @@
       <c r="X72" s="12" t="n"/>
       <c r="Y72" s="9" t="n"/>
       <c r="Z72" s="12" t="n"/>
-      <c r="AA72" s="24">
+      <c r="AA72" s="12" t="n"/>
+      <c r="AB72" s="24">
         <f>IF(J72="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J72,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K72,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -4221,7 +4298,8 @@
       <c r="X73" s="12" t="n"/>
       <c r="Y73" s="9" t="n"/>
       <c r="Z73" s="12" t="n"/>
-      <c r="AA73" s="24">
+      <c r="AA73" s="12" t="n"/>
+      <c r="AB73" s="24">
         <f>IF(J73="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J73,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K73,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -4253,7 +4331,8 @@
       <c r="X74" s="12" t="n"/>
       <c r="Y74" s="9" t="n"/>
       <c r="Z74" s="12" t="n"/>
-      <c r="AA74" s="24">
+      <c r="AA74" s="12" t="n"/>
+      <c r="AB74" s="24">
         <f>IF(J74="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J74,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K74,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -4285,7 +4364,8 @@
       <c r="X75" s="12" t="n"/>
       <c r="Y75" s="9" t="n"/>
       <c r="Z75" s="12" t="n"/>
-      <c r="AA75" s="24">
+      <c r="AA75" s="12" t="n"/>
+      <c r="AB75" s="24">
         <f>IF(J75="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J75,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K75,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -4317,7 +4397,8 @@
       <c r="X76" s="12" t="n"/>
       <c r="Y76" s="9" t="n"/>
       <c r="Z76" s="12" t="n"/>
-      <c r="AA76" s="24">
+      <c r="AA76" s="12" t="n"/>
+      <c r="AB76" s="24">
         <f>IF(J76="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J76,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K76,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -4349,7 +4430,8 @@
       <c r="X77" s="12" t="n"/>
       <c r="Y77" s="9" t="n"/>
       <c r="Z77" s="12" t="n"/>
-      <c r="AA77" s="24">
+      <c r="AA77" s="12" t="n"/>
+      <c r="AB77" s="24">
         <f>IF(J77="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J77,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K77,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -4381,7 +4463,8 @@
       <c r="X78" s="12" t="n"/>
       <c r="Y78" s="9" t="n"/>
       <c r="Z78" s="12" t="n"/>
-      <c r="AA78" s="24">
+      <c r="AA78" s="12" t="n"/>
+      <c r="AB78" s="24">
         <f>IF(J78="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J78,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K78,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -4413,7 +4496,8 @@
       <c r="X79" s="12" t="n"/>
       <c r="Y79" s="9" t="n"/>
       <c r="Z79" s="12" t="n"/>
-      <c r="AA79" s="24">
+      <c r="AA79" s="12" t="n"/>
+      <c r="AB79" s="24">
         <f>IF(J79="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J79,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K79,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -4445,7 +4529,8 @@
       <c r="X80" s="12" t="n"/>
       <c r="Y80" s="9" t="n"/>
       <c r="Z80" s="12" t="n"/>
-      <c r="AA80" s="24">
+      <c r="AA80" s="12" t="n"/>
+      <c r="AB80" s="24">
         <f>IF(J80="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J80,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K80,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -4477,7 +4562,8 @@
       <c r="X81" s="12" t="n"/>
       <c r="Y81" s="9" t="n"/>
       <c r="Z81" s="12" t="n"/>
-      <c r="AA81" s="24">
+      <c r="AA81" s="12" t="n"/>
+      <c r="AB81" s="24">
         <f>IF(J81="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J81,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K81,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -4509,7 +4595,8 @@
       <c r="X82" s="12" t="n"/>
       <c r="Y82" s="9" t="n"/>
       <c r="Z82" s="12" t="n"/>
-      <c r="AA82" s="24">
+      <c r="AA82" s="12" t="n"/>
+      <c r="AB82" s="24">
         <f>IF(J82="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J82,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K82,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -4541,7 +4628,8 @@
       <c r="X83" s="12" t="n"/>
       <c r="Y83" s="9" t="n"/>
       <c r="Z83" s="12" t="n"/>
-      <c r="AA83" s="24">
+      <c r="AA83" s="12" t="n"/>
+      <c r="AB83" s="24">
         <f>IF(J83="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J83,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K83,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -4573,7 +4661,8 @@
       <c r="X84" s="12" t="n"/>
       <c r="Y84" s="9" t="n"/>
       <c r="Z84" s="12" t="n"/>
-      <c r="AA84" s="24">
+      <c r="AA84" s="12" t="n"/>
+      <c r="AB84" s="24">
         <f>IF(J84="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J84,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K84,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -4605,7 +4694,8 @@
       <c r="X85" s="12" t="n"/>
       <c r="Y85" s="9" t="n"/>
       <c r="Z85" s="12" t="n"/>
-      <c r="AA85" s="24">
+      <c r="AA85" s="12" t="n"/>
+      <c r="AB85" s="24">
         <f>IF(J85="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J85,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K85,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -4637,7 +4727,8 @@
       <c r="X86" s="12" t="n"/>
       <c r="Y86" s="9" t="n"/>
       <c r="Z86" s="12" t="n"/>
-      <c r="AA86" s="24">
+      <c r="AA86" s="12" t="n"/>
+      <c r="AB86" s="24">
         <f>IF(J86="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J86,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K86,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -4669,7 +4760,8 @@
       <c r="X87" s="12" t="n"/>
       <c r="Y87" s="9" t="n"/>
       <c r="Z87" s="12" t="n"/>
-      <c r="AA87" s="24">
+      <c r="AA87" s="12" t="n"/>
+      <c r="AB87" s="24">
         <f>IF(J87="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J87,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K87,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -4701,7 +4793,8 @@
       <c r="X88" s="12" t="n"/>
       <c r="Y88" s="9" t="n"/>
       <c r="Z88" s="12" t="n"/>
-      <c r="AA88" s="24">
+      <c r="AA88" s="12" t="n"/>
+      <c r="AB88" s="24">
         <f>IF(J88="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J88,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K88,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -4733,7 +4826,8 @@
       <c r="X89" s="12" t="n"/>
       <c r="Y89" s="9" t="n"/>
       <c r="Z89" s="12" t="n"/>
-      <c r="AA89" s="24">
+      <c r="AA89" s="12" t="n"/>
+      <c r="AB89" s="24">
         <f>IF(J89="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J89,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K89,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -4765,7 +4859,8 @@
       <c r="X90" s="12" t="n"/>
       <c r="Y90" s="9" t="n"/>
       <c r="Z90" s="12" t="n"/>
-      <c r="AA90" s="24">
+      <c r="AA90" s="12" t="n"/>
+      <c r="AB90" s="24">
         <f>IF(J90="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J90,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K90,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -4797,7 +4892,8 @@
       <c r="X91" s="12" t="n"/>
       <c r="Y91" s="9" t="n"/>
       <c r="Z91" s="12" t="n"/>
-      <c r="AA91" s="24">
+      <c r="AA91" s="12" t="n"/>
+      <c r="AB91" s="24">
         <f>IF(J91="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J91,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K91,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -4829,7 +4925,8 @@
       <c r="X92" s="12" t="n"/>
       <c r="Y92" s="9" t="n"/>
       <c r="Z92" s="12" t="n"/>
-      <c r="AA92" s="24">
+      <c r="AA92" s="12" t="n"/>
+      <c r="AB92" s="24">
         <f>IF(J92="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J92,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K92,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -4861,7 +4958,8 @@
       <c r="X93" s="12" t="n"/>
       <c r="Y93" s="9" t="n"/>
       <c r="Z93" s="12" t="n"/>
-      <c r="AA93" s="24">
+      <c r="AA93" s="12" t="n"/>
+      <c r="AB93" s="24">
         <f>IF(J93="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J93,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K93,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -4893,7 +4991,8 @@
       <c r="X94" s="12" t="n"/>
       <c r="Y94" s="9" t="n"/>
       <c r="Z94" s="12" t="n"/>
-      <c r="AA94" s="24">
+      <c r="AA94" s="12" t="n"/>
+      <c r="AB94" s="24">
         <f>IF(J94="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J94,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K94,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -4925,7 +5024,8 @@
       <c r="X95" s="12" t="n"/>
       <c r="Y95" s="9" t="n"/>
       <c r="Z95" s="12" t="n"/>
-      <c r="AA95" s="24">
+      <c r="AA95" s="12" t="n"/>
+      <c r="AB95" s="24">
         <f>IF(J95="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J95,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K95,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -4957,7 +5057,8 @@
       <c r="X96" s="12" t="n"/>
       <c r="Y96" s="9" t="n"/>
       <c r="Z96" s="12" t="n"/>
-      <c r="AA96" s="24">
+      <c r="AA96" s="12" t="n"/>
+      <c r="AB96" s="24">
         <f>IF(J96="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J96,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K96,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -4989,7 +5090,8 @@
       <c r="X97" s="12" t="n"/>
       <c r="Y97" s="9" t="n"/>
       <c r="Z97" s="12" t="n"/>
-      <c r="AA97" s="24">
+      <c r="AA97" s="12" t="n"/>
+      <c r="AB97" s="24">
         <f>IF(J97="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J97,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K97,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -5021,7 +5123,8 @@
       <c r="X98" s="12" t="n"/>
       <c r="Y98" s="9" t="n"/>
       <c r="Z98" s="12" t="n"/>
-      <c r="AA98" s="24">
+      <c r="AA98" s="12" t="n"/>
+      <c r="AB98" s="24">
         <f>IF(J98="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J98,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K98,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -5053,7 +5156,8 @@
       <c r="X99" s="12" t="n"/>
       <c r="Y99" s="9" t="n"/>
       <c r="Z99" s="12" t="n"/>
-      <c r="AA99" s="24">
+      <c r="AA99" s="12" t="n"/>
+      <c r="AB99" s="24">
         <f>IF(J99="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J99,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K99,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -5085,7 +5189,8 @@
       <c r="X100" s="12" t="n"/>
       <c r="Y100" s="9" t="n"/>
       <c r="Z100" s="12" t="n"/>
-      <c r="AA100" s="24">
+      <c r="AA100" s="12" t="n"/>
+      <c r="AB100" s="24">
         <f>IF(J100="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J100,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K100,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Choose whether lapsed policies appear in the report
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Policy_Review_Template.xlsx
+++ b/Policy_Review_Template.xlsx
@@ -931,7 +931,7 @@
         </is>
       </c>
       <c r="B15" s="9">
-        <f>SUMIFS(Policies!$AB$2:$AB$100,Policies!$G$2:$G$100,"Inforce")+SUMIFS(Policies!$AB$2:$AB$100,Policies!$G$2:$G$100,"Paid-up")</f>
+        <f>SUMIFS(Policies!$AC$2:$AC$100,Policies!$G$2:$G$100,"Inforce")+SUMIFS(Policies!$AC$2:$AC$100,Policies!$G$2:$G$100,"Paid-up")</f>
         <v/>
       </c>
     </row>
@@ -1453,7 +1453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB100"/>
+  <dimension ref="A1:AC100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1483,7 +1483,8 @@
     <col width="15" customWidth="1" min="25" max="25"/>
     <col width="12" customWidth="1" min="26" max="26"/>
     <col width="14" customWidth="1" min="27" max="27"/>
-    <col width="14" customWidth="1" min="28" max="28"/>
+    <col width="12" customWidth="1" min="28" max="28"/>
+    <col width="14" customWidth="1" min="29" max="29"/>
   </cols>
   <sheetData>
     <row r="1" ht="42" customHeight="1">
@@ -1622,7 +1623,12 @@
           <t>Nominee Share (%)</t>
         </is>
       </c>
-      <c r="AB1" s="23" t="inlineStr">
+      <c r="AB1" s="22" t="inlineStr">
+        <is>
+          <t>Show in Report</t>
+        </is>
+      </c>
+      <c r="AC1" s="23" t="inlineStr">
         <is>
           <t>Annual Premium (auto)</t>
         </is>
@@ -1718,7 +1724,8 @@
       <c r="Y2" s="9" t="n"/>
       <c r="Z2" s="12" t="n"/>
       <c r="AA2" s="12" t="n"/>
-      <c r="AB2" s="24">
+      <c r="AB2" s="12" t="n"/>
+      <c r="AC2" s="24">
         <f>IF(J2="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J2,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K2,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -1809,7 +1816,8 @@
       <c r="Y3" s="9" t="n"/>
       <c r="Z3" s="12" t="n"/>
       <c r="AA3" s="12" t="n"/>
-      <c r="AB3" s="24">
+      <c r="AB3" s="12" t="n"/>
+      <c r="AC3" s="24">
         <f>IF(J3="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J3,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K3,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -1906,7 +1914,8 @@
       <c r="Y4" s="9" t="n"/>
       <c r="Z4" s="12" t="n"/>
       <c r="AA4" s="12" t="n"/>
-      <c r="AB4" s="24">
+      <c r="AB4" s="12" t="n"/>
+      <c r="AC4" s="24">
         <f>IF(J4="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J4,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K4,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -1991,7 +2000,8 @@
       <c r="Y5" s="9" t="n"/>
       <c r="Z5" s="12" t="n"/>
       <c r="AA5" s="12" t="n"/>
-      <c r="AB5" s="24">
+      <c r="AB5" s="12" t="n"/>
+      <c r="AC5" s="24">
         <f>IF(J5="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J5,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K5,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2088,7 +2098,8 @@
       <c r="Y6" s="9" t="n"/>
       <c r="Z6" s="12" t="n"/>
       <c r="AA6" s="12" t="n"/>
-      <c r="AB6" s="24">
+      <c r="AB6" s="12" t="n"/>
+      <c r="AC6" s="24">
         <f>IF(J6="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J6,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K6,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2121,7 +2132,8 @@
       <c r="Y7" s="9" t="n"/>
       <c r="Z7" s="12" t="n"/>
       <c r="AA7" s="12" t="n"/>
-      <c r="AB7" s="24">
+      <c r="AB7" s="12" t="n"/>
+      <c r="AC7" s="24">
         <f>IF(J7="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J7,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K7,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2154,7 +2166,8 @@
       <c r="Y8" s="9" t="n"/>
       <c r="Z8" s="12" t="n"/>
       <c r="AA8" s="12" t="n"/>
-      <c r="AB8" s="24">
+      <c r="AB8" s="12" t="n"/>
+      <c r="AC8" s="24">
         <f>IF(J8="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J8,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K8,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2187,7 +2200,8 @@
       <c r="Y9" s="9" t="n"/>
       <c r="Z9" s="12" t="n"/>
       <c r="AA9" s="12" t="n"/>
-      <c r="AB9" s="24">
+      <c r="AB9" s="12" t="n"/>
+      <c r="AC9" s="24">
         <f>IF(J9="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J9,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K9,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2220,7 +2234,8 @@
       <c r="Y10" s="9" t="n"/>
       <c r="Z10" s="12" t="n"/>
       <c r="AA10" s="12" t="n"/>
-      <c r="AB10" s="24">
+      <c r="AB10" s="12" t="n"/>
+      <c r="AC10" s="24">
         <f>IF(J10="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J10,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K10,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2253,7 +2268,8 @@
       <c r="Y11" s="9" t="n"/>
       <c r="Z11" s="12" t="n"/>
       <c r="AA11" s="12" t="n"/>
-      <c r="AB11" s="24">
+      <c r="AB11" s="12" t="n"/>
+      <c r="AC11" s="24">
         <f>IF(J11="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J11,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K11,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2286,7 +2302,8 @@
       <c r="Y12" s="9" t="n"/>
       <c r="Z12" s="12" t="n"/>
       <c r="AA12" s="12" t="n"/>
-      <c r="AB12" s="24">
+      <c r="AB12" s="12" t="n"/>
+      <c r="AC12" s="24">
         <f>IF(J12="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J12,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K12,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2319,7 +2336,8 @@
       <c r="Y13" s="9" t="n"/>
       <c r="Z13" s="12" t="n"/>
       <c r="AA13" s="12" t="n"/>
-      <c r="AB13" s="24">
+      <c r="AB13" s="12" t="n"/>
+      <c r="AC13" s="24">
         <f>IF(J13="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J13,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K13,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2352,7 +2370,8 @@
       <c r="Y14" s="9" t="n"/>
       <c r="Z14" s="12" t="n"/>
       <c r="AA14" s="12" t="n"/>
-      <c r="AB14" s="24">
+      <c r="AB14" s="12" t="n"/>
+      <c r="AC14" s="24">
         <f>IF(J14="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J14,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K14,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2385,7 +2404,8 @@
       <c r="Y15" s="9" t="n"/>
       <c r="Z15" s="12" t="n"/>
       <c r="AA15" s="12" t="n"/>
-      <c r="AB15" s="24">
+      <c r="AB15" s="12" t="n"/>
+      <c r="AC15" s="24">
         <f>IF(J15="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J15,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K15,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2418,7 +2438,8 @@
       <c r="Y16" s="9" t="n"/>
       <c r="Z16" s="12" t="n"/>
       <c r="AA16" s="12" t="n"/>
-      <c r="AB16" s="24">
+      <c r="AB16" s="12" t="n"/>
+      <c r="AC16" s="24">
         <f>IF(J16="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J16,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K16,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2451,7 +2472,8 @@
       <c r="Y17" s="9" t="n"/>
       <c r="Z17" s="12" t="n"/>
       <c r="AA17" s="12" t="n"/>
-      <c r="AB17" s="24">
+      <c r="AB17" s="12" t="n"/>
+      <c r="AC17" s="24">
         <f>IF(J17="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J17,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K17,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2484,7 +2506,8 @@
       <c r="Y18" s="9" t="n"/>
       <c r="Z18" s="12" t="n"/>
       <c r="AA18" s="12" t="n"/>
-      <c r="AB18" s="24">
+      <c r="AB18" s="12" t="n"/>
+      <c r="AC18" s="24">
         <f>IF(J18="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J18,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K18,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2517,7 +2540,8 @@
       <c r="Y19" s="9" t="n"/>
       <c r="Z19" s="12" t="n"/>
       <c r="AA19" s="12" t="n"/>
-      <c r="AB19" s="24">
+      <c r="AB19" s="12" t="n"/>
+      <c r="AC19" s="24">
         <f>IF(J19="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J19,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K19,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2550,7 +2574,8 @@
       <c r="Y20" s="9" t="n"/>
       <c r="Z20" s="12" t="n"/>
       <c r="AA20" s="12" t="n"/>
-      <c r="AB20" s="24">
+      <c r="AB20" s="12" t="n"/>
+      <c r="AC20" s="24">
         <f>IF(J20="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J20,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K20,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2583,7 +2608,8 @@
       <c r="Y21" s="9" t="n"/>
       <c r="Z21" s="12" t="n"/>
       <c r="AA21" s="12" t="n"/>
-      <c r="AB21" s="24">
+      <c r="AB21" s="12" t="n"/>
+      <c r="AC21" s="24">
         <f>IF(J21="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J21,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K21,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2616,7 +2642,8 @@
       <c r="Y22" s="9" t="n"/>
       <c r="Z22" s="12" t="n"/>
       <c r="AA22" s="12" t="n"/>
-      <c r="AB22" s="24">
+      <c r="AB22" s="12" t="n"/>
+      <c r="AC22" s="24">
         <f>IF(J22="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J22,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K22,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2649,7 +2676,8 @@
       <c r="Y23" s="9" t="n"/>
       <c r="Z23" s="12" t="n"/>
       <c r="AA23" s="12" t="n"/>
-      <c r="AB23" s="24">
+      <c r="AB23" s="12" t="n"/>
+      <c r="AC23" s="24">
         <f>IF(J23="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J23,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K23,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2682,7 +2710,8 @@
       <c r="Y24" s="9" t="n"/>
       <c r="Z24" s="12" t="n"/>
       <c r="AA24" s="12" t="n"/>
-      <c r="AB24" s="24">
+      <c r="AB24" s="12" t="n"/>
+      <c r="AC24" s="24">
         <f>IF(J24="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J24,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K24,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2715,7 +2744,8 @@
       <c r="Y25" s="9" t="n"/>
       <c r="Z25" s="12" t="n"/>
       <c r="AA25" s="12" t="n"/>
-      <c r="AB25" s="24">
+      <c r="AB25" s="12" t="n"/>
+      <c r="AC25" s="24">
         <f>IF(J25="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J25,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K25,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2748,7 +2778,8 @@
       <c r="Y26" s="9" t="n"/>
       <c r="Z26" s="12" t="n"/>
       <c r="AA26" s="12" t="n"/>
-      <c r="AB26" s="24">
+      <c r="AB26" s="12" t="n"/>
+      <c r="AC26" s="24">
         <f>IF(J26="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J26,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K26,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2781,7 +2812,8 @@
       <c r="Y27" s="9" t="n"/>
       <c r="Z27" s="12" t="n"/>
       <c r="AA27" s="12" t="n"/>
-      <c r="AB27" s="24">
+      <c r="AB27" s="12" t="n"/>
+      <c r="AC27" s="24">
         <f>IF(J27="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J27,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K27,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2814,7 +2846,8 @@
       <c r="Y28" s="9" t="n"/>
       <c r="Z28" s="12" t="n"/>
       <c r="AA28" s="12" t="n"/>
-      <c r="AB28" s="24">
+      <c r="AB28" s="12" t="n"/>
+      <c r="AC28" s="24">
         <f>IF(J28="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J28,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K28,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2847,7 +2880,8 @@
       <c r="Y29" s="9" t="n"/>
       <c r="Z29" s="12" t="n"/>
       <c r="AA29" s="12" t="n"/>
-      <c r="AB29" s="24">
+      <c r="AB29" s="12" t="n"/>
+      <c r="AC29" s="24">
         <f>IF(J29="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J29,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K29,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2880,7 +2914,8 @@
       <c r="Y30" s="9" t="n"/>
       <c r="Z30" s="12" t="n"/>
       <c r="AA30" s="12" t="n"/>
-      <c r="AB30" s="24">
+      <c r="AB30" s="12" t="n"/>
+      <c r="AC30" s="24">
         <f>IF(J30="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J30,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K30,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2913,7 +2948,8 @@
       <c r="Y31" s="9" t="n"/>
       <c r="Z31" s="12" t="n"/>
       <c r="AA31" s="12" t="n"/>
-      <c r="AB31" s="24">
+      <c r="AB31" s="12" t="n"/>
+      <c r="AC31" s="24">
         <f>IF(J31="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J31,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K31,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2946,7 +2982,8 @@
       <c r="Y32" s="9" t="n"/>
       <c r="Z32" s="12" t="n"/>
       <c r="AA32" s="12" t="n"/>
-      <c r="AB32" s="24">
+      <c r="AB32" s="12" t="n"/>
+      <c r="AC32" s="24">
         <f>IF(J32="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J32,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K32,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -2979,7 +3016,8 @@
       <c r="Y33" s="9" t="n"/>
       <c r="Z33" s="12" t="n"/>
       <c r="AA33" s="12" t="n"/>
-      <c r="AB33" s="24">
+      <c r="AB33" s="12" t="n"/>
+      <c r="AC33" s="24">
         <f>IF(J33="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J33,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K33,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3012,7 +3050,8 @@
       <c r="Y34" s="9" t="n"/>
       <c r="Z34" s="12" t="n"/>
       <c r="AA34" s="12" t="n"/>
-      <c r="AB34" s="24">
+      <c r="AB34" s="12" t="n"/>
+      <c r="AC34" s="24">
         <f>IF(J34="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J34,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K34,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3045,7 +3084,8 @@
       <c r="Y35" s="9" t="n"/>
       <c r="Z35" s="12" t="n"/>
       <c r="AA35" s="12" t="n"/>
-      <c r="AB35" s="24">
+      <c r="AB35" s="12" t="n"/>
+      <c r="AC35" s="24">
         <f>IF(J35="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J35,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K35,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3078,7 +3118,8 @@
       <c r="Y36" s="9" t="n"/>
       <c r="Z36" s="12" t="n"/>
       <c r="AA36" s="12" t="n"/>
-      <c r="AB36" s="24">
+      <c r="AB36" s="12" t="n"/>
+      <c r="AC36" s="24">
         <f>IF(J36="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J36,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K36,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3111,7 +3152,8 @@
       <c r="Y37" s="9" t="n"/>
       <c r="Z37" s="12" t="n"/>
       <c r="AA37" s="12" t="n"/>
-      <c r="AB37" s="24">
+      <c r="AB37" s="12" t="n"/>
+      <c r="AC37" s="24">
         <f>IF(J37="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J37,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K37,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3144,7 +3186,8 @@
       <c r="Y38" s="9" t="n"/>
       <c r="Z38" s="12" t="n"/>
       <c r="AA38" s="12" t="n"/>
-      <c r="AB38" s="24">
+      <c r="AB38" s="12" t="n"/>
+      <c r="AC38" s="24">
         <f>IF(J38="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J38,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K38,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3177,7 +3220,8 @@
       <c r="Y39" s="9" t="n"/>
       <c r="Z39" s="12" t="n"/>
       <c r="AA39" s="12" t="n"/>
-      <c r="AB39" s="24">
+      <c r="AB39" s="12" t="n"/>
+      <c r="AC39" s="24">
         <f>IF(J39="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J39,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K39,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3210,7 +3254,8 @@
       <c r="Y40" s="9" t="n"/>
       <c r="Z40" s="12" t="n"/>
       <c r="AA40" s="12" t="n"/>
-      <c r="AB40" s="24">
+      <c r="AB40" s="12" t="n"/>
+      <c r="AC40" s="24">
         <f>IF(J40="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J40,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K40,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3243,7 +3288,8 @@
       <c r="Y41" s="9" t="n"/>
       <c r="Z41" s="12" t="n"/>
       <c r="AA41" s="12" t="n"/>
-      <c r="AB41" s="24">
+      <c r="AB41" s="12" t="n"/>
+      <c r="AC41" s="24">
         <f>IF(J41="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J41,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K41,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3276,7 +3322,8 @@
       <c r="Y42" s="9" t="n"/>
       <c r="Z42" s="12" t="n"/>
       <c r="AA42" s="12" t="n"/>
-      <c r="AB42" s="24">
+      <c r="AB42" s="12" t="n"/>
+      <c r="AC42" s="24">
         <f>IF(J42="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J42,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K42,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3309,7 +3356,8 @@
       <c r="Y43" s="9" t="n"/>
       <c r="Z43" s="12" t="n"/>
       <c r="AA43" s="12" t="n"/>
-      <c r="AB43" s="24">
+      <c r="AB43" s="12" t="n"/>
+      <c r="AC43" s="24">
         <f>IF(J43="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J43,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K43,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3342,7 +3390,8 @@
       <c r="Y44" s="9" t="n"/>
       <c r="Z44" s="12" t="n"/>
       <c r="AA44" s="12" t="n"/>
-      <c r="AB44" s="24">
+      <c r="AB44" s="12" t="n"/>
+      <c r="AC44" s="24">
         <f>IF(J44="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J44,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K44,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3375,7 +3424,8 @@
       <c r="Y45" s="9" t="n"/>
       <c r="Z45" s="12" t="n"/>
       <c r="AA45" s="12" t="n"/>
-      <c r="AB45" s="24">
+      <c r="AB45" s="12" t="n"/>
+      <c r="AC45" s="24">
         <f>IF(J45="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J45,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K45,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3408,7 +3458,8 @@
       <c r="Y46" s="9" t="n"/>
       <c r="Z46" s="12" t="n"/>
       <c r="AA46" s="12" t="n"/>
-      <c r="AB46" s="24">
+      <c r="AB46" s="12" t="n"/>
+      <c r="AC46" s="24">
         <f>IF(J46="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J46,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K46,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3441,7 +3492,8 @@
       <c r="Y47" s="9" t="n"/>
       <c r="Z47" s="12" t="n"/>
       <c r="AA47" s="12" t="n"/>
-      <c r="AB47" s="24">
+      <c r="AB47" s="12" t="n"/>
+      <c r="AC47" s="24">
         <f>IF(J47="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J47,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K47,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3474,7 +3526,8 @@
       <c r="Y48" s="9" t="n"/>
       <c r="Z48" s="12" t="n"/>
       <c r="AA48" s="12" t="n"/>
-      <c r="AB48" s="24">
+      <c r="AB48" s="12" t="n"/>
+      <c r="AC48" s="24">
         <f>IF(J48="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J48,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K48,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3507,7 +3560,8 @@
       <c r="Y49" s="9" t="n"/>
       <c r="Z49" s="12" t="n"/>
       <c r="AA49" s="12" t="n"/>
-      <c r="AB49" s="24">
+      <c r="AB49" s="12" t="n"/>
+      <c r="AC49" s="24">
         <f>IF(J49="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J49,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K49,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3540,7 +3594,8 @@
       <c r="Y50" s="9" t="n"/>
       <c r="Z50" s="12" t="n"/>
       <c r="AA50" s="12" t="n"/>
-      <c r="AB50" s="24">
+      <c r="AB50" s="12" t="n"/>
+      <c r="AC50" s="24">
         <f>IF(J50="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J50,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K50,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3573,7 +3628,8 @@
       <c r="Y51" s="9" t="n"/>
       <c r="Z51" s="12" t="n"/>
       <c r="AA51" s="12" t="n"/>
-      <c r="AB51" s="24">
+      <c r="AB51" s="12" t="n"/>
+      <c r="AC51" s="24">
         <f>IF(J51="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J51,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K51,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3606,7 +3662,8 @@
       <c r="Y52" s="9" t="n"/>
       <c r="Z52" s="12" t="n"/>
       <c r="AA52" s="12" t="n"/>
-      <c r="AB52" s="24">
+      <c r="AB52" s="12" t="n"/>
+      <c r="AC52" s="24">
         <f>IF(J52="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J52,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K52,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3639,7 +3696,8 @@
       <c r="Y53" s="9" t="n"/>
       <c r="Z53" s="12" t="n"/>
       <c r="AA53" s="12" t="n"/>
-      <c r="AB53" s="24">
+      <c r="AB53" s="12" t="n"/>
+      <c r="AC53" s="24">
         <f>IF(J53="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J53,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K53,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3672,7 +3730,8 @@
       <c r="Y54" s="9" t="n"/>
       <c r="Z54" s="12" t="n"/>
       <c r="AA54" s="12" t="n"/>
-      <c r="AB54" s="24">
+      <c r="AB54" s="12" t="n"/>
+      <c r="AC54" s="24">
         <f>IF(J54="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J54,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K54,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3705,7 +3764,8 @@
       <c r="Y55" s="9" t="n"/>
       <c r="Z55" s="12" t="n"/>
       <c r="AA55" s="12" t="n"/>
-      <c r="AB55" s="24">
+      <c r="AB55" s="12" t="n"/>
+      <c r="AC55" s="24">
         <f>IF(J55="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J55,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K55,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3738,7 +3798,8 @@
       <c r="Y56" s="9" t="n"/>
       <c r="Z56" s="12" t="n"/>
       <c r="AA56" s="12" t="n"/>
-      <c r="AB56" s="24">
+      <c r="AB56" s="12" t="n"/>
+      <c r="AC56" s="24">
         <f>IF(J56="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J56,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K56,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3771,7 +3832,8 @@
       <c r="Y57" s="9" t="n"/>
       <c r="Z57" s="12" t="n"/>
       <c r="AA57" s="12" t="n"/>
-      <c r="AB57" s="24">
+      <c r="AB57" s="12" t="n"/>
+      <c r="AC57" s="24">
         <f>IF(J57="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J57,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K57,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3804,7 +3866,8 @@
       <c r="Y58" s="9" t="n"/>
       <c r="Z58" s="12" t="n"/>
       <c r="AA58" s="12" t="n"/>
-      <c r="AB58" s="24">
+      <c r="AB58" s="12" t="n"/>
+      <c r="AC58" s="24">
         <f>IF(J58="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J58,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K58,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3837,7 +3900,8 @@
       <c r="Y59" s="9" t="n"/>
       <c r="Z59" s="12" t="n"/>
       <c r="AA59" s="12" t="n"/>
-      <c r="AB59" s="24">
+      <c r="AB59" s="12" t="n"/>
+      <c r="AC59" s="24">
         <f>IF(J59="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J59,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K59,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3870,7 +3934,8 @@
       <c r="Y60" s="9" t="n"/>
       <c r="Z60" s="12" t="n"/>
       <c r="AA60" s="12" t="n"/>
-      <c r="AB60" s="24">
+      <c r="AB60" s="12" t="n"/>
+      <c r="AC60" s="24">
         <f>IF(J60="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J60,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K60,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3903,7 +3968,8 @@
       <c r="Y61" s="9" t="n"/>
       <c r="Z61" s="12" t="n"/>
       <c r="AA61" s="12" t="n"/>
-      <c r="AB61" s="24">
+      <c r="AB61" s="12" t="n"/>
+      <c r="AC61" s="24">
         <f>IF(J61="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J61,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K61,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3936,7 +4002,8 @@
       <c r="Y62" s="9" t="n"/>
       <c r="Z62" s="12" t="n"/>
       <c r="AA62" s="12" t="n"/>
-      <c r="AB62" s="24">
+      <c r="AB62" s="12" t="n"/>
+      <c r="AC62" s="24">
         <f>IF(J62="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J62,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K62,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -3969,7 +4036,8 @@
       <c r="Y63" s="9" t="n"/>
       <c r="Z63" s="12" t="n"/>
       <c r="AA63" s="12" t="n"/>
-      <c r="AB63" s="24">
+      <c r="AB63" s="12" t="n"/>
+      <c r="AC63" s="24">
         <f>IF(J63="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J63,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K63,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -4002,7 +4070,8 @@
       <c r="Y64" s="9" t="n"/>
       <c r="Z64" s="12" t="n"/>
       <c r="AA64" s="12" t="n"/>
-      <c r="AB64" s="24">
+      <c r="AB64" s="12" t="n"/>
+      <c r="AC64" s="24">
         <f>IF(J64="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J64,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K64,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -4035,7 +4104,8 @@
       <c r="Y65" s="9" t="n"/>
       <c r="Z65" s="12" t="n"/>
       <c r="AA65" s="12" t="n"/>
-      <c r="AB65" s="24">
+      <c r="AB65" s="12" t="n"/>
+      <c r="AC65" s="24">
         <f>IF(J65="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J65,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K65,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -4068,7 +4138,8 @@
       <c r="Y66" s="9" t="n"/>
       <c r="Z66" s="12" t="n"/>
       <c r="AA66" s="12" t="n"/>
-      <c r="AB66" s="24">
+      <c r="AB66" s="12" t="n"/>
+      <c r="AC66" s="24">
         <f>IF(J66="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J66,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K66,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -4101,7 +4172,8 @@
       <c r="Y67" s="9" t="n"/>
       <c r="Z67" s="12" t="n"/>
       <c r="AA67" s="12" t="n"/>
-      <c r="AB67" s="24">
+      <c r="AB67" s="12" t="n"/>
+      <c r="AC67" s="24">
         <f>IF(J67="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J67,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K67,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -4134,7 +4206,8 @@
       <c r="Y68" s="9" t="n"/>
       <c r="Z68" s="12" t="n"/>
       <c r="AA68" s="12" t="n"/>
-      <c r="AB68" s="24">
+      <c r="AB68" s="12" t="n"/>
+      <c r="AC68" s="24">
         <f>IF(J68="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J68,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K68,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -4167,7 +4240,8 @@
       <c r="Y69" s="9" t="n"/>
       <c r="Z69" s="12" t="n"/>
       <c r="AA69" s="12" t="n"/>
-      <c r="AB69" s="24">
+      <c r="AB69" s="12" t="n"/>
+      <c r="AC69" s="24">
         <f>IF(J69="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J69,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K69,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -4200,7 +4274,8 @@
       <c r="Y70" s="9" t="n"/>
       <c r="Z70" s="12" t="n"/>
       <c r="AA70" s="12" t="n"/>
-      <c r="AB70" s="24">
+      <c r="AB70" s="12" t="n"/>
+      <c r="AC70" s="24">
         <f>IF(J70="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J70,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K70,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -4233,7 +4308,8 @@
       <c r="Y71" s="9" t="n"/>
       <c r="Z71" s="12" t="n"/>
       <c r="AA71" s="12" t="n"/>
-      <c r="AB71" s="24">
+      <c r="AB71" s="12" t="n"/>
+      <c r="AC71" s="24">
         <f>IF(J71="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J71,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K71,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -4266,7 +4342,8 @@
       <c r="Y72" s="9" t="n"/>
       <c r="Z72" s="12" t="n"/>
       <c r="AA72" s="12" t="n"/>
-      <c r="AB72" s="24">
+      <c r="AB72" s="12" t="n"/>
+      <c r="AC72" s="24">
         <f>IF(J72="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J72,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K72,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -4299,7 +4376,8 @@
       <c r="Y73" s="9" t="n"/>
       <c r="Z73" s="12" t="n"/>
       <c r="AA73" s="12" t="n"/>
-      <c r="AB73" s="24">
+      <c r="AB73" s="12" t="n"/>
+      <c r="AC73" s="24">
         <f>IF(J73="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J73,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K73,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -4332,7 +4410,8 @@
       <c r="Y74" s="9" t="n"/>
       <c r="Z74" s="12" t="n"/>
       <c r="AA74" s="12" t="n"/>
-      <c r="AB74" s="24">
+      <c r="AB74" s="12" t="n"/>
+      <c r="AC74" s="24">
         <f>IF(J74="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J74,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K74,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -4365,7 +4444,8 @@
       <c r="Y75" s="9" t="n"/>
       <c r="Z75" s="12" t="n"/>
       <c r="AA75" s="12" t="n"/>
-      <c r="AB75" s="24">
+      <c r="AB75" s="12" t="n"/>
+      <c r="AC75" s="24">
         <f>IF(J75="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J75,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K75,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -4398,7 +4478,8 @@
       <c r="Y76" s="9" t="n"/>
       <c r="Z76" s="12" t="n"/>
       <c r="AA76" s="12" t="n"/>
-      <c r="AB76" s="24">
+      <c r="AB76" s="12" t="n"/>
+      <c r="AC76" s="24">
         <f>IF(J76="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J76,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K76,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -4431,7 +4512,8 @@
       <c r="Y77" s="9" t="n"/>
       <c r="Z77" s="12" t="n"/>
       <c r="AA77" s="12" t="n"/>
-      <c r="AB77" s="24">
+      <c r="AB77" s="12" t="n"/>
+      <c r="AC77" s="24">
         <f>IF(J77="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J77,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K77,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -4464,7 +4546,8 @@
       <c r="Y78" s="9" t="n"/>
       <c r="Z78" s="12" t="n"/>
       <c r="AA78" s="12" t="n"/>
-      <c r="AB78" s="24">
+      <c r="AB78" s="12" t="n"/>
+      <c r="AC78" s="24">
         <f>IF(J78="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J78,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K78,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -4497,7 +4580,8 @@
       <c r="Y79" s="9" t="n"/>
       <c r="Z79" s="12" t="n"/>
       <c r="AA79" s="12" t="n"/>
-      <c r="AB79" s="24">
+      <c r="AB79" s="12" t="n"/>
+      <c r="AC79" s="24">
         <f>IF(J79="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J79,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K79,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -4530,7 +4614,8 @@
       <c r="Y80" s="9" t="n"/>
       <c r="Z80" s="12" t="n"/>
       <c r="AA80" s="12" t="n"/>
-      <c r="AB80" s="24">
+      <c r="AB80" s="12" t="n"/>
+      <c r="AC80" s="24">
         <f>IF(J80="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J80,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K80,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -4563,7 +4648,8 @@
       <c r="Y81" s="9" t="n"/>
       <c r="Z81" s="12" t="n"/>
       <c r="AA81" s="12" t="n"/>
-      <c r="AB81" s="24">
+      <c r="AB81" s="12" t="n"/>
+      <c r="AC81" s="24">
         <f>IF(J81="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J81,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K81,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -4596,7 +4682,8 @@
       <c r="Y82" s="9" t="n"/>
       <c r="Z82" s="12" t="n"/>
       <c r="AA82" s="12" t="n"/>
-      <c r="AB82" s="24">
+      <c r="AB82" s="12" t="n"/>
+      <c r="AC82" s="24">
         <f>IF(J82="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J82,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K82,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -4629,7 +4716,8 @@
       <c r="Y83" s="9" t="n"/>
       <c r="Z83" s="12" t="n"/>
       <c r="AA83" s="12" t="n"/>
-      <c r="AB83" s="24">
+      <c r="AB83" s="12" t="n"/>
+      <c r="AC83" s="24">
         <f>IF(J83="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J83,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K83,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -4662,7 +4750,8 @@
       <c r="Y84" s="9" t="n"/>
       <c r="Z84" s="12" t="n"/>
       <c r="AA84" s="12" t="n"/>
-      <c r="AB84" s="24">
+      <c r="AB84" s="12" t="n"/>
+      <c r="AC84" s="24">
         <f>IF(J84="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J84,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K84,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -4695,7 +4784,8 @@
       <c r="Y85" s="9" t="n"/>
       <c r="Z85" s="12" t="n"/>
       <c r="AA85" s="12" t="n"/>
-      <c r="AB85" s="24">
+      <c r="AB85" s="12" t="n"/>
+      <c r="AC85" s="24">
         <f>IF(J85="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J85,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K85,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -4728,7 +4818,8 @@
       <c r="Y86" s="9" t="n"/>
       <c r="Z86" s="12" t="n"/>
       <c r="AA86" s="12" t="n"/>
-      <c r="AB86" s="24">
+      <c r="AB86" s="12" t="n"/>
+      <c r="AC86" s="24">
         <f>IF(J86="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J86,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K86,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -4761,7 +4852,8 @@
       <c r="Y87" s="9" t="n"/>
       <c r="Z87" s="12" t="n"/>
       <c r="AA87" s="12" t="n"/>
-      <c r="AB87" s="24">
+      <c r="AB87" s="12" t="n"/>
+      <c r="AC87" s="24">
         <f>IF(J87="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J87,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K87,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -4794,7 +4886,8 @@
       <c r="Y88" s="9" t="n"/>
       <c r="Z88" s="12" t="n"/>
       <c r="AA88" s="12" t="n"/>
-      <c r="AB88" s="24">
+      <c r="AB88" s="12" t="n"/>
+      <c r="AC88" s="24">
         <f>IF(J88="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J88,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K88,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -4827,7 +4920,8 @@
       <c r="Y89" s="9" t="n"/>
       <c r="Z89" s="12" t="n"/>
       <c r="AA89" s="12" t="n"/>
-      <c r="AB89" s="24">
+      <c r="AB89" s="12" t="n"/>
+      <c r="AC89" s="24">
         <f>IF(J89="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J89,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K89,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -4860,7 +4954,8 @@
       <c r="Y90" s="9" t="n"/>
       <c r="Z90" s="12" t="n"/>
       <c r="AA90" s="12" t="n"/>
-      <c r="AB90" s="24">
+      <c r="AB90" s="12" t="n"/>
+      <c r="AC90" s="24">
         <f>IF(J90="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J90,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K90,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -4893,7 +4988,8 @@
       <c r="Y91" s="9" t="n"/>
       <c r="Z91" s="12" t="n"/>
       <c r="AA91" s="12" t="n"/>
-      <c r="AB91" s="24">
+      <c r="AB91" s="12" t="n"/>
+      <c r="AC91" s="24">
         <f>IF(J91="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J91,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K91,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -4926,7 +5022,8 @@
       <c r="Y92" s="9" t="n"/>
       <c r="Z92" s="12" t="n"/>
       <c r="AA92" s="12" t="n"/>
-      <c r="AB92" s="24">
+      <c r="AB92" s="12" t="n"/>
+      <c r="AC92" s="24">
         <f>IF(J92="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J92,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K92,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -4959,7 +5056,8 @@
       <c r="Y93" s="9" t="n"/>
       <c r="Z93" s="12" t="n"/>
       <c r="AA93" s="12" t="n"/>
-      <c r="AB93" s="24">
+      <c r="AB93" s="12" t="n"/>
+      <c r="AC93" s="24">
         <f>IF(J93="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J93,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K93,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -4992,7 +5090,8 @@
       <c r="Y94" s="9" t="n"/>
       <c r="Z94" s="12" t="n"/>
       <c r="AA94" s="12" t="n"/>
-      <c r="AB94" s="24">
+      <c r="AB94" s="12" t="n"/>
+      <c r="AC94" s="24">
         <f>IF(J94="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J94,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K94,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -5025,7 +5124,8 @@
       <c r="Y95" s="9" t="n"/>
       <c r="Z95" s="12" t="n"/>
       <c r="AA95" s="12" t="n"/>
-      <c r="AB95" s="24">
+      <c r="AB95" s="12" t="n"/>
+      <c r="AC95" s="24">
         <f>IF(J95="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J95,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K95,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -5058,7 +5158,8 @@
       <c r="Y96" s="9" t="n"/>
       <c r="Z96" s="12" t="n"/>
       <c r="AA96" s="12" t="n"/>
-      <c r="AB96" s="24">
+      <c r="AB96" s="12" t="n"/>
+      <c r="AC96" s="24">
         <f>IF(J96="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J96,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K96,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -5091,7 +5192,8 @@
       <c r="Y97" s="9" t="n"/>
       <c r="Z97" s="12" t="n"/>
       <c r="AA97" s="12" t="n"/>
-      <c r="AB97" s="24">
+      <c r="AB97" s="12" t="n"/>
+      <c r="AC97" s="24">
         <f>IF(J97="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J97,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K97,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -5124,7 +5226,8 @@
       <c r="Y98" s="9" t="n"/>
       <c r="Z98" s="12" t="n"/>
       <c r="AA98" s="12" t="n"/>
-      <c r="AB98" s="24">
+      <c r="AB98" s="12" t="n"/>
+      <c r="AC98" s="24">
         <f>IF(J98="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J98,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K98,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -5157,7 +5260,8 @@
       <c r="Y99" s="9" t="n"/>
       <c r="Z99" s="12" t="n"/>
       <c r="AA99" s="12" t="n"/>
-      <c r="AB99" s="24">
+      <c r="AB99" s="12" t="n"/>
+      <c r="AC99" s="24">
         <f>IF(J99="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J99,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K99,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -5190,7 +5294,8 @@
       <c r="Y100" s="9" t="n"/>
       <c r="Z100" s="12" t="n"/>
       <c r="AA100" s="12" t="n"/>
-      <c r="AB100" s="24">
+      <c r="AB100" s="12" t="n"/>
+      <c r="AC100" s="24">
         <f>IF(J100="","",IFERROR(VALUE(SUBSTITUTE(SUBSTITUTE(J100,"RM",""),",",""))*IFERROR(INDEX({12,4,2,1,0},MATCH(K100,{"Monthly","Quarterly","Half-yearly","Yearly","Single"},0)),0),0))</f>
         <v/>
       </c>
@@ -5201,7 +5306,7 @@
       <formula>AND($G2="Inforce",$T2="",$A2&lt;&gt;"")</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="8">
+  <dataValidations count="9">
     <dataValidation sqref="D2:D100" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Whole Life,Term Life,Investment-Linked,Medical,Critical Illness,Personal Accident,Endowment / Savings,Other"</formula1>
     </dataValidation>
@@ -5219,6 +5324,9 @@
     </dataValidation>
     <dataValidation sqref="Z2:Z100" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Yes,No,Not sure"</formula1>
+    </dataValidation>
+    <dataValidation sqref="AB2:AB100" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Yes,No"</formula1>
     </dataValidation>
     <dataValidation sqref="W2:W100" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Family income protection,Medical &amp; hospital bills,Critical illness recovery,Retirement,Children's education,Savings &amp; wealth,Mortgage / loan protection,Estate &amp; legacy,Accident cover,Business protection"</formula1>

</xml_diff>

<commit_message>
Nominee details: IC, phone, birthday
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Policy_Review_Template.xlsx
+++ b/Policy_Review_Template.xlsx
@@ -1032,7 +1032,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E45"/>
+  <dimension ref="A1:F45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -1040,6 +1040,7 @@
     <col width="40" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
     <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1328,6 +1329,11 @@
       <c r="E30" s="19" t="inlineStr">
         <is>
           <t>Notes  备注</t>
+        </is>
+      </c>
+      <c r="F30" s="19" t="inlineStr">
+        <is>
+          <t>IC No  身份证</t>
         </is>
       </c>
     </row>
@@ -1337,6 +1343,7 @@
       <c r="C31" s="20" t="n"/>
       <c r="D31" s="21" t="n"/>
       <c r="E31" s="12" t="n"/>
+      <c r="F31" s="21" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="12" t="n"/>
@@ -1344,6 +1351,7 @@
       <c r="C32" s="20" t="n"/>
       <c r="D32" s="21" t="n"/>
       <c r="E32" s="12" t="n"/>
+      <c r="F32" s="21" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="12" t="n"/>
@@ -1351,6 +1359,7 @@
       <c r="C33" s="20" t="n"/>
       <c r="D33" s="21" t="n"/>
       <c r="E33" s="12" t="n"/>
+      <c r="F33" s="21" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="12" t="n"/>
@@ -1358,6 +1367,7 @@
       <c r="C34" s="20" t="n"/>
       <c r="D34" s="21" t="n"/>
       <c r="E34" s="12" t="n"/>
+      <c r="F34" s="21" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="12" t="n"/>
@@ -1365,6 +1375,7 @@
       <c r="C35" s="20" t="n"/>
       <c r="D35" s="21" t="n"/>
       <c r="E35" s="12" t="n"/>
+      <c r="F35" s="21" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="12" t="n"/>
@@ -1372,6 +1383,7 @@
       <c r="C36" s="20" t="n"/>
       <c r="D36" s="21" t="n"/>
       <c r="E36" s="12" t="n"/>
+      <c r="F36" s="21" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="12" t="n"/>
@@ -1379,6 +1391,7 @@
       <c r="C37" s="20" t="n"/>
       <c r="D37" s="21" t="n"/>
       <c r="E37" s="12" t="n"/>
+      <c r="F37" s="21" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="12" t="n"/>
@@ -1386,6 +1399,7 @@
       <c r="C38" s="20" t="n"/>
       <c r="D38" s="21" t="n"/>
       <c r="E38" s="12" t="n"/>
+      <c r="F38" s="21" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="12" t="n"/>
@@ -1393,6 +1407,7 @@
       <c r="C39" s="20" t="n"/>
       <c r="D39" s="21" t="n"/>
       <c r="E39" s="12" t="n"/>
+      <c r="F39" s="21" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="12" t="n"/>
@@ -1400,6 +1415,7 @@
       <c r="C40" s="20" t="n"/>
       <c r="D40" s="21" t="n"/>
       <c r="E40" s="12" t="n"/>
+      <c r="F40" s="21" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="12" t="n"/>
@@ -1407,6 +1423,7 @@
       <c r="C41" s="20" t="n"/>
       <c r="D41" s="21" t="n"/>
       <c r="E41" s="12" t="n"/>
+      <c r="F41" s="21" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="12" t="n"/>
@@ -1414,6 +1431,7 @@
       <c r="C42" s="20" t="n"/>
       <c r="D42" s="21" t="n"/>
       <c r="E42" s="12" t="n"/>
+      <c r="F42" s="21" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="12" t="n"/>
@@ -1421,6 +1439,7 @@
       <c r="C43" s="20" t="n"/>
       <c r="D43" s="21" t="n"/>
       <c r="E43" s="12" t="n"/>
+      <c r="F43" s="21" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="12" t="n"/>
@@ -1428,6 +1447,7 @@
       <c r="C44" s="20" t="n"/>
       <c r="D44" s="21" t="n"/>
       <c r="E44" s="12" t="n"/>
+      <c r="F44" s="21" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="12" t="n"/>
@@ -1435,6 +1455,7 @@
       <c r="C45" s="20" t="n"/>
       <c r="D45" s="21" t="n"/>
       <c r="E45" s="12" t="n"/>
+      <c r="F45" s="21" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="1">

</xml_diff>

<commit_message>
Template: dropdowns match the app (nomination type, relationship, status, report style)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Policy_Review_Template.xlsx
+++ b/Policy_Review_Template.xlsx
@@ -1121,6 +1121,19 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>Report style (DISC)</t>
+        </is>
+      </c>
+      <c r="B10" s="14" t="n"/>
+      <c r="C10" s="16" t="inlineStr">
+        <is>
+          <t>Blank = standard; D, I, S or C changes the report layout</t>
+        </is>
+      </c>
+    </row>
     <row r="11">
       <c r="A11" s="10" t="inlineStr">
         <is>
@@ -1458,7 +1471,10 @@
       <c r="F45" s="21" t="n"/>
     </row>
   </sheetData>
-  <dataValidations count="1">
+  <dataValidations count="2">
+    <dataValidation sqref="B10" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"D,I,S,C"</formula1>
+    </dataValidation>
     <dataValidation sqref="B31 B32 B33 B34 B35 B36 B37 B38 B39 B40 B41 B42 B43 B44 B45" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Spouse 配偶,Son 儿子,Daughter 女儿,Father 父亲,Mother 母亲,Brother 兄弟,Sister 姐妹,Other 其他"</formula1>
     </dataValidation>
@@ -5327,12 +5343,12 @@
       <formula>AND($G2="Inforce",$T2="",$A2&lt;&gt;"")</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="9">
+  <dataValidations count="10">
     <dataValidation sqref="D2:D100" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Whole Life,Term Life,Investment-Linked,Medical,Critical Illness,Personal Accident,Endowment / Savings,Other"</formula1>
     </dataValidation>
     <dataValidation sqref="G2:G100" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Inforce,Lapsed,Paid-up,Surrendered,Matured"</formula1>
+      <formula1>"Inforce,Lapsed,Paid-up,Surrendered,Matured,Terminated,Withdrawn"</formula1>
     </dataValidation>
     <dataValidation sqref="K2:K100" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Monthly,Quarterly,Half-yearly,Yearly,Single"</formula1>
@@ -5340,8 +5356,11 @@
     <dataValidation sqref="S2:S100" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
+    <dataValidation sqref="U2:U100" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Spouse,Husband,Wife,Son,Daughter,Father,Mother,Brother,Sister,Grandchild,Other"</formula1>
+    </dataValidation>
     <dataValidation sqref="V2:V100" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Beneficiary,Hibah,Trustee,Conditional Hibah,None"</formula1>
+      <formula1>"Trust,Hibah,Beneficiary,Executor,Not sure"</formula1>
     </dataValidation>
     <dataValidation sqref="Z2:Z100" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Yes,No,Not sure"</formula1>

</xml_diff>